<commit_message>
Add 02 Oct 2026 data: 4 berth reassignments, 20C reopening slips to 5 Oct; update history and Excel export
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="29 Sep 2026" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30 Sep 2026" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 Oct 2026" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 Oct 2026" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -505,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -513,6 +514,7 @@
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="32" customWidth="1" min="4" max="4"/>
     <col width="36" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -555,6 +557,11 @@
           <t>01 Oct 2026</t>
         </is>
       </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>02 Oct 2026</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -578,6 +585,7 @@
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -605,6 +613,7 @@
           <t>sailed (01/04)</t>
         </is>
       </c>
+      <c r="F6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -624,6 +633,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr"/>
       <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -647,6 +657,7 @@
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -670,6 +681,7 @@
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr"/>
+      <c r="F9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -689,6 +701,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr"/>
       <c r="E10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -716,6 +729,7 @@
           <t>sailed (30/16)</t>
         </is>
       </c>
+      <c r="F11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -735,6 +749,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr"/>
       <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -762,6 +777,7 @@
           <t>sailed (30/18)</t>
         </is>
       </c>
+      <c r="F13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -789,6 +805,11 @@
           <t>alongside · 20AB</t>
         </is>
       </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20AB (ETD now 02/15)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -816,6 +837,7 @@
           <t>sailed (01/05)</t>
         </is>
       </c>
+      <c r="F15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -839,6 +861,11 @@
           <t>alongside · 20B (marked)</t>
         </is>
       </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20B (marked)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -860,6 +887,11 @@
       <c r="E17" s="6" t="inlineStr">
         <is>
           <t>expected · 20D (marked, 1C)</t>
+        </is>
+      </c>
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20D (marked, 1C)</t>
         </is>
       </c>
     </row>
@@ -881,6 +913,11 @@
           <t>expected · 20AB</t>
         </is>
       </c>
+      <c r="F18" s="6" t="inlineStr">
+        <is>
+          <t>alongside → 20F</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -898,6 +935,11 @@
       <c r="E19" s="5" t="inlineStr">
         <is>
           <t>expected · 20F</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20E</t>
         </is>
       </c>
     </row>
@@ -915,6 +957,11 @@
           <t>expected · 20B (new)</t>
         </is>
       </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20AB</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -925,9 +972,14 @@
       <c r="B21" s="5" t="inlineStr"/>
       <c r="C21" s="5" t="inlineStr"/>
       <c r="D21" s="5" t="inlineStr"/>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>expected → 20C (new, first since reopening)</t>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C (new)</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20B</t>
         </is>
       </c>
     </row>
@@ -943,6 +995,75 @@
       <c r="E22" s="5" t="inlineStr">
         <is>
           <t>expected · 20E (new)</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20AB</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>JOSCO LUCKY</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr"/>
+      <c r="C23" s="5" t="inlineStr"/>
+      <c r="D23" s="5" t="inlineStr"/>
+      <c r="E23" s="5" t="inlineStr"/>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>SAWASDEE DENEB</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr"/>
+      <c r="C24" s="5" t="inlineStr"/>
+      <c r="D24" s="5" t="inlineStr"/>
+      <c r="E24" s="5" t="inlineStr"/>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C (new, first since reopening)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>HARI BHUM (Barge)</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr"/>
+      <c r="C25" s="5" t="inlineStr"/>
+      <c r="D25" s="5" t="inlineStr"/>
+      <c r="E25" s="5" t="inlineStr"/>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D (new, barge)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 98</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr"/>
+      <c r="C26" s="5" t="inlineStr"/>
+      <c r="D26" s="5" t="inlineStr"/>
+      <c r="E26" s="5" t="inlineStr"/>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F (new)</t>
         </is>
       </c>
     </row>
@@ -987,7 +1108,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Period (as of 01 Oct sheet)</t>
+          <t>Period (as of 02 Oct sheet)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -1041,7 +1162,7 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Closed until 3 Oct 2026 (slipped from 1 Oct)</t>
+          <t>Closed until 5 Oct 2026 (slipped 1→3→5 Oct)</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
@@ -1051,7 +1172,7 @@
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>Wharf to be utilised from 3 Oct 2026</t>
+          <t>Wharf to be utilised from 5 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1189,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>3–24 Oct 2026 (slipped from 1–21 Oct)</t>
+          <t>4–24 Oct 2026 (slipped 1–21→3–24→4–24 Oct)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -1078,7 +1199,7 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>Berth closed 3–24 Oct 2026 to renovate electric channel</t>
+          <t>Berth closed 4–24 Oct 2026 to renovate electric channel</t>
         </is>
       </c>
     </row>
@@ -1095,7 +1216,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>3–18 Oct 2026 (slipped from 1–15 Oct)</t>
+          <t>5–18 Oct 2026 (slipped 1–15→3–18→5–18 Oct)</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
@@ -1105,7 +1226,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>G.25 stops working 3–18 Oct 2026 to change trolley rail</t>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail</t>
         </is>
       </c>
     </row>
@@ -2740,4 +2861,499 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 02 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>CAPE FAWLEY</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>558</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>46295.875</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>46296.25</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>46297.625</v>
+      </c>
+      <c r="G4" s="9">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="7" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>RESURGENCE</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>458</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>46298.54166666666</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>46298.54166666666</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>46299.5</v>
+      </c>
+      <c r="G5" s="9">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>ZHONG GU BEI HAI</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>561</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>46299.45833333334</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>46301.45833333334</v>
+      </c>
+      <c r="G6" s="9">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>KHARIS HERITAGE</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>482</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46296.45833333334</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46296.75</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46297.70833333334</v>
+      </c>
+      <c r="G7" s="12">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>YM IMPROVEMENT</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>46298.83333333334</v>
+      </c>
+      <c r="E8" s="8" t="n">
+        <v>46298.83333333334</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>46300.41666666666</v>
+      </c>
+      <c r="G8" s="9">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>JOSCO LUCKY</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>46300.91666666666</v>
+      </c>
+      <c r="E9" s="8" t="n">
+        <v>46301.5</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="G9" s="9">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE DENEB</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E10" s="8" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="F10" s="8" t="n">
+        <v>46302.5</v>
+      </c>
+      <c r="G10" s="9">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>ALS SUMIRE</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>537</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>46296.25</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>46296.66666666666</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>46297.70833333334</v>
+      </c>
+      <c r="G11" s="12">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>1C</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>HARI BHUM (Barge)</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>259</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>46298.20833333334</v>
+      </c>
+      <c r="E12" s="8" t="n">
+        <v>46298.20833333334</v>
+      </c>
+      <c r="F12" s="8" t="n">
+        <v>46298.66666666666</v>
+      </c>
+      <c r="G12" s="9">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 278</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>46297.75</v>
+      </c>
+      <c r="E13" s="8" t="n">
+        <v>46298.41666666666</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>46300.45833333334</v>
+      </c>
+      <c r="G13" s="9">
+        <f>(F13-E13)*24</f>
+        <v/>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>KMTC BANGKOK</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>565</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>46297.29166666666</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>46297.33333333334</v>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>46298.70833333334</v>
+      </c>
+      <c r="G14" s="9">
+        <f>(F14-E14)*24</f>
+        <v/>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 98</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>564</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="E15" s="8" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>46300.375</v>
+      </c>
+      <c r="G15" s="9">
+        <f>(F15-E15)*24</f>
+        <v/>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I15" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add 06 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -17,9 +17,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 Oct 2026" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Oct 2026" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Oct 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Oct 2026" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -626,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:J37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -638,6 +639,7 @@
     <col width="40" customWidth="1" min="7" max="7"/>
     <col width="40" customWidth="1" min="8" max="8"/>
     <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="44" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -698,6 +700,11 @@
       <c r="I4" s="3" t="inlineStr">
         <is>
           <t>05 Oct 2026</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>06 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -727,6 +734,7 @@
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr"/>
       <c r="I5" s="5" t="inlineStr"/>
+      <c r="J5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -758,6 +766,7 @@
       <c r="G6" s="5" t="inlineStr"/>
       <c r="H6" s="5" t="inlineStr"/>
       <c r="I6" s="5" t="inlineStr"/>
+      <c r="J6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -781,6 +790,7 @@
       <c r="G7" s="5" t="inlineStr"/>
       <c r="H7" s="5" t="inlineStr"/>
       <c r="I7" s="5" t="inlineStr"/>
+      <c r="J7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -808,6 +818,7 @@
       <c r="G8" s="5" t="inlineStr"/>
       <c r="H8" s="5" t="inlineStr"/>
       <c r="I8" s="5" t="inlineStr"/>
+      <c r="J8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -835,6 +846,7 @@
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr"/>
       <c r="I9" s="5" t="inlineStr"/>
+      <c r="J9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -858,6 +870,7 @@
       <c r="G10" s="5" t="inlineStr"/>
       <c r="H10" s="5" t="inlineStr"/>
       <c r="I10" s="5" t="inlineStr"/>
+      <c r="J10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -889,6 +902,7 @@
       <c r="G11" s="5" t="inlineStr"/>
       <c r="H11" s="5" t="inlineStr"/>
       <c r="I11" s="5" t="inlineStr"/>
+      <c r="J11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -912,6 +926,7 @@
       <c r="G12" s="5" t="inlineStr"/>
       <c r="H12" s="5" t="inlineStr"/>
       <c r="I12" s="5" t="inlineStr"/>
+      <c r="J12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -943,6 +958,7 @@
       <c r="G13" s="5" t="inlineStr"/>
       <c r="H13" s="5" t="inlineStr"/>
       <c r="I13" s="5" t="inlineStr"/>
+      <c r="J13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -982,6 +998,7 @@
       </c>
       <c r="H14" s="5" t="inlineStr"/>
       <c r="I14" s="5" t="inlineStr"/>
+      <c r="J14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1013,6 +1030,7 @@
       <c r="G15" s="5" t="inlineStr"/>
       <c r="H15" s="5" t="inlineStr"/>
       <c r="I15" s="5" t="inlineStr"/>
+      <c r="J15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1048,6 +1066,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr"/>
       <c r="I16" s="5" t="inlineStr"/>
+      <c r="J16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1083,6 +1102,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr"/>
       <c r="I17" s="5" t="inlineStr"/>
+      <c r="J17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1118,6 +1138,7 @@
         </is>
       </c>
       <c r="I18" s="5" t="inlineStr"/>
+      <c r="J18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1155,6 +1176,11 @@
       <c r="I19" s="5" t="inlineStr">
         <is>
           <t>alongside · 20E (ETD 05/11)</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>sailed (05/11)</t>
         </is>
       </c>
     </row>
@@ -1192,6 +1218,11 @@
           <t>alongside · 20AB (ETD slipped to 06/11)</t>
         </is>
       </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20AB (ETD 06/11)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1227,6 +1258,11 @@
           <t>alongside · 20B (ETD 05/12)</t>
         </is>
       </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>sailed (05/12)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1262,6 +1298,7 @@
           <t>sailed (04/17)</t>
         </is>
       </c>
+      <c r="J22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1293,6 +1330,11 @@
           <t>expected → 20D (P.B 06/18)</t>
         </is>
       </c>
+      <c r="J23" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20C (P.B 07/13)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1324,6 +1366,11 @@
           <t>at anchorage · 20C (P.B 05/12)</t>
         </is>
       </c>
+      <c r="J24" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20C (ETD now 07/11)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1351,6 +1398,7 @@
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr"/>
+      <c r="J25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1382,6 +1430,7 @@
           <t>sailed (05/09)</t>
         </is>
       </c>
+      <c r="J26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1407,6 +1456,11 @@
       <c r="I27" s="5" t="inlineStr">
         <is>
           <t>expected · 20B</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B (P.B 06/13)</t>
         </is>
       </c>
     </row>
@@ -1430,6 +1484,11 @@
       <c r="I28" s="6" t="inlineStr">
         <is>
           <t>expected → 20AB (ETA 06/13)</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20AB (P.B 06/13)</t>
         </is>
       </c>
     </row>
@@ -1451,6 +1510,11 @@
           <t>expected · 20AB (new, marked)</t>
         </is>
       </c>
+      <c r="J29" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20B</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1470,6 +1534,11 @@
           <t>expected · 20C (new)</t>
         </is>
       </c>
+      <c r="J30" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20C (P.B 08/15→09/15, ETD 10/13→11/03)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1489,6 +1558,11 @@
           <t>expected · 20D (new, marked)</t>
         </is>
       </c>
+      <c r="J31" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20D (P.B 07/17→07/14)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1506,6 +1580,111 @@
       <c r="I32" s="6" t="inlineStr">
         <is>
           <t>expected · 20F (new, marked)</t>
+        </is>
+      </c>
+      <c r="J32" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20F (P.B 07/17→07/14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>SITC HOCHIMINH</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr"/>
+      <c r="C33" s="5" t="inlineStr"/>
+      <c r="D33" s="5" t="inlineStr"/>
+      <c r="E33" s="5" t="inlineStr"/>
+      <c r="F33" s="5" t="inlineStr"/>
+      <c r="G33" s="5" t="inlineStr"/>
+      <c r="H33" s="5" t="inlineStr"/>
+      <c r="I33" s="5" t="inlineStr"/>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20AB (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>YM INCEPTION</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr"/>
+      <c r="C34" s="5" t="inlineStr"/>
+      <c r="D34" s="5" t="inlineStr"/>
+      <c r="E34" s="5" t="inlineStr"/>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="5" t="inlineStr"/>
+      <c r="H34" s="5" t="inlineStr"/>
+      <c r="I34" s="5" t="inlineStr"/>
+      <c r="J34" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20AB (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>HE JIN</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr"/>
+      <c r="C35" s="5" t="inlineStr"/>
+      <c r="D35" s="5" t="inlineStr"/>
+      <c r="E35" s="5" t="inlineStr"/>
+      <c r="F35" s="5" t="inlineStr"/>
+      <c r="G35" s="5" t="inlineStr"/>
+      <c r="H35" s="5" t="inlineStr"/>
+      <c r="I35" s="5" t="inlineStr"/>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>ZHONG GU DONG HAI</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr"/>
+      <c r="C36" s="5" t="inlineStr"/>
+      <c r="D36" s="5" t="inlineStr"/>
+      <c r="E36" s="5" t="inlineStr"/>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr"/>
+      <c r="H36" s="5" t="inlineStr"/>
+      <c r="I36" s="5" t="inlineStr"/>
+      <c r="J36" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>KANWAY FORTUNE</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr"/>
+      <c r="C37" s="5" t="inlineStr"/>
+      <c r="D37" s="5" t="inlineStr"/>
+      <c r="E37" s="5" t="inlineStr"/>
+      <c r="F37" s="5" t="inlineStr"/>
+      <c r="G37" s="5" t="inlineStr"/>
+      <c r="H37" s="5" t="inlineStr"/>
+      <c r="I37" s="5" t="inlineStr"/>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D (new)</t>
         </is>
       </c>
     </row>
@@ -2108,13 +2287,665 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 06 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>ZHONG GU BEI HAI</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>561</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>46299.625</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>46301.45833333334</v>
+      </c>
+      <c r="G4" s="26">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>KMTC TOKYO</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46301.54166666666</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46301.54166666666</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46303.5</v>
+      </c>
+      <c r="G5" s="26">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>SITC HOCHIMINH</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>470</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46302.79166666666</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46303.58333333334</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46304.70833333334</v>
+      </c>
+      <c r="G6" s="26">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>YM INCEPTION</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46304.625</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="G7" s="26">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE SPICA</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>46300.875</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>46301.54166666666</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="G8" s="26">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>GREEN PARK</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>482</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>46302.45833333334</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>46303.625</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="G9" s="26">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>HE JIN</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>552</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>46302.875</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>46304.625</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>46305.625</v>
+      </c>
+      <c r="G10" s="26">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE DENEB</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>46302.45833333334</v>
+      </c>
+      <c r="G11" s="26">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="23" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>JOSCO LUCKY</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>46301.875</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>46303.5</v>
+      </c>
+      <c r="G12" s="26">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="23" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>ZHONG GU DONG HAI</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>46302.66666666666</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>46303.58333333334</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="G13" s="26">
+        <f>(F13-E13)*24</f>
+        <v/>
+      </c>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I13" s="23" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE ATLANTIC</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>46302.91666666666</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>46304.625</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>46306.125</v>
+      </c>
+      <c r="G14" s="26">
+        <f>(F14-E14)*24</f>
+        <v/>
+      </c>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I14" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>MTT BANGKOK</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>46302.5</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>46302.58333333334</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="G15" s="26">
+        <f>(F15-E15)*24</f>
+        <v/>
+      </c>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>KANWAY FORTUNE</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>46303.75</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>46304.625</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>46306.125</v>
+      </c>
+      <c r="G16" s="26">
+        <f>(F16-E16)*24</f>
+        <v/>
+      </c>
+      <c r="H16" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I16" s="23" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>XIN AN</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>46302.58333333334</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="G17" s="26">
+        <f>(F17-E17)*24</f>
+        <v/>
+      </c>
+      <c r="H17" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I17" s="23" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="28" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G21" s="29" t="n"/>
+      <c r="H21" s="29" t="n"/>
+      <c r="I21" s="30" t="n"/>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C22" s="32" t="n"/>
+      <c r="D22" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E22" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (MTT BANGKOK and KANWAY FORTUNE are still booked at 20D from 07/12)  —  Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+      <c r="G22" s="32" t="n"/>
+      <c r="H22" s="32" t="n"/>
+      <c r="I22" s="32" t="n"/>
+    </row>
+    <row r="23" ht="42" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C23" s="31" t="n"/>
+      <c r="D23" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E23" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail (in progress)  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G23" s="31" t="n"/>
+      <c r="H23" s="31" t="n"/>
+      <c r="I23" s="31" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="F21:I21"/>
+    <mergeCell ref="F22:I22"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3065,8 +3896,70 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="12" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D33" s="14" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E33" s="14" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F33" s="13" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (MTT BANGKOK and KANWAY FORTUNE are still booked at 20D from 07/12)</t>
+        </is>
+      </c>
+      <c r="G33" s="13" t="inlineStr">
+        <is>
+          <t>Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="C34" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E34" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail (in progress)</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G32"/>
+  <autoFilter ref="A4:G34"/>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add 07 Oct 2026 ship movement data, widen timeline to 13 Oct, update Excel and history
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -18,9 +18,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Oct 2026" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Oct 2026" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Oct 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Oct 2026" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -627,7 +628,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:K41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -640,6 +641,7 @@
     <col width="40" customWidth="1" min="8" max="8"/>
     <col width="42" customWidth="1" min="9" max="9"/>
     <col width="44" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -705,6 +707,11 @@
       <c r="J4" s="3" t="inlineStr">
         <is>
           <t>06 Oct 2026</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>07 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -735,6 +742,7 @@
       <c r="H5" s="5" t="inlineStr"/>
       <c r="I5" s="5" t="inlineStr"/>
       <c r="J5" s="5" t="inlineStr"/>
+      <c r="K5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -767,6 +775,7 @@
       <c r="H6" s="5" t="inlineStr"/>
       <c r="I6" s="5" t="inlineStr"/>
       <c r="J6" s="5" t="inlineStr"/>
+      <c r="K6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -791,6 +800,7 @@
       <c r="H7" s="5" t="inlineStr"/>
       <c r="I7" s="5" t="inlineStr"/>
       <c r="J7" s="5" t="inlineStr"/>
+      <c r="K7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -819,6 +829,7 @@
       <c r="H8" s="5" t="inlineStr"/>
       <c r="I8" s="5" t="inlineStr"/>
       <c r="J8" s="5" t="inlineStr"/>
+      <c r="K8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -847,6 +858,7 @@
       <c r="H9" s="5" t="inlineStr"/>
       <c r="I9" s="5" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr"/>
+      <c r="K9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -871,6 +883,7 @@
       <c r="H10" s="5" t="inlineStr"/>
       <c r="I10" s="5" t="inlineStr"/>
       <c r="J10" s="5" t="inlineStr"/>
+      <c r="K10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -903,6 +916,7 @@
       <c r="H11" s="5" t="inlineStr"/>
       <c r="I11" s="5" t="inlineStr"/>
       <c r="J11" s="5" t="inlineStr"/>
+      <c r="K11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -927,6 +941,7 @@
       <c r="H12" s="5" t="inlineStr"/>
       <c r="I12" s="5" t="inlineStr"/>
       <c r="J12" s="5" t="inlineStr"/>
+      <c r="K12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -959,6 +974,7 @@
       <c r="H13" s="5" t="inlineStr"/>
       <c r="I13" s="5" t="inlineStr"/>
       <c r="J13" s="5" t="inlineStr"/>
+      <c r="K13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -999,6 +1015,7 @@
       <c r="H14" s="5" t="inlineStr"/>
       <c r="I14" s="5" t="inlineStr"/>
       <c r="J14" s="5" t="inlineStr"/>
+      <c r="K14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1031,6 +1048,7 @@
       <c r="H15" s="5" t="inlineStr"/>
       <c r="I15" s="5" t="inlineStr"/>
       <c r="J15" s="5" t="inlineStr"/>
+      <c r="K15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1067,6 +1085,7 @@
       <c r="H16" s="5" t="inlineStr"/>
       <c r="I16" s="5" t="inlineStr"/>
       <c r="J16" s="5" t="inlineStr"/>
+      <c r="K16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1103,6 +1122,7 @@
       <c r="H17" s="5" t="inlineStr"/>
       <c r="I17" s="5" t="inlineStr"/>
       <c r="J17" s="5" t="inlineStr"/>
+      <c r="K17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1139,6 +1159,7 @@
       </c>
       <c r="I18" s="5" t="inlineStr"/>
       <c r="J18" s="5" t="inlineStr"/>
+      <c r="K18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1183,6 +1204,7 @@
           <t>sailed (05/11)</t>
         </is>
       </c>
+      <c r="K19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1223,6 +1245,11 @@
           <t>alongside · 20AB (ETD 06/11)</t>
         </is>
       </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>sailed (06/11)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1263,6 +1290,7 @@
           <t>sailed (05/12)</t>
         </is>
       </c>
+      <c r="K21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1299,6 +1327,7 @@
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr"/>
+      <c r="K22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1335,6 +1364,11 @@
           <t>expected → 20C (P.B 07/13)</t>
         </is>
       </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>at anchorage · 20C (P.B 07/13, ETD 08/12→08/13)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1371,6 +1405,11 @@
           <t>alongside · 20C (ETD now 07/11)</t>
         </is>
       </c>
+      <c r="K24" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20C (ETD 07/11)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1399,6 +1438,7 @@
       </c>
       <c r="I25" s="5" t="inlineStr"/>
       <c r="J25" s="5" t="inlineStr"/>
+      <c r="K25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1431,6 +1471,7 @@
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr"/>
+      <c r="K26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1461,6 +1502,11 @@
       <c r="J27" s="5" t="inlineStr">
         <is>
           <t>expected · 20B (P.B 06/13)</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20B (ETD 08/13)</t>
         </is>
       </c>
     </row>
@@ -1489,6 +1535,11 @@
       <c r="J28" s="5" t="inlineStr">
         <is>
           <t>expected · 20AB (P.B 06/13)</t>
+        </is>
+      </c>
+      <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20AB (ETD 08/12)</t>
         </is>
       </c>
     </row>
@@ -1515,6 +1566,11 @@
           <t>expected → 20B</t>
         </is>
       </c>
+      <c r="K29" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20AB (P.B 08/15→08/13)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1539,6 +1595,11 @@
           <t>expected · 20C (P.B 08/15→09/15, ETD 10/13→11/03)</t>
         </is>
       </c>
+      <c r="K30" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20D</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1563,6 +1624,11 @@
           <t>expected · 20D (P.B 07/17→07/14)</t>
         </is>
       </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D (ETA 07/12)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1585,6 +1651,11 @@
       <c r="J32" s="6" t="inlineStr">
         <is>
           <t>expected · 20F (P.B 07/17→07/14)</t>
+        </is>
+      </c>
+      <c r="K32" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F (ETA 07/13)</t>
         </is>
       </c>
     </row>
@@ -1607,6 +1678,11 @@
           <t>expected · 20AB (new)</t>
         </is>
       </c>
+      <c r="K33" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20B (ETA 07/19→07/18)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -1627,6 +1703,11 @@
           <t>expected · 20AB (new)</t>
         </is>
       </c>
+      <c r="K34" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20C (P.B 09/15→09/13, ETD 10/16→11/01)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -1647,6 +1728,11 @@
           <t>expected · 20B (new)</t>
         </is>
       </c>
+      <c r="K35" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20AB</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -1667,6 +1753,11 @@
           <t>expected · 20C (new)</t>
         </is>
       </c>
+      <c r="K36" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20C (ETA 07/16→07/13)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -1685,6 +1776,95 @@
       <c r="J37" s="5" t="inlineStr">
         <is>
           <t>expected · 20D (new)</t>
+        </is>
+      </c>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20F (P.B 09/15→09/14, ETD 11/03→10/15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>CNC MARS</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr"/>
+      <c r="C38" s="5" t="inlineStr"/>
+      <c r="D38" s="5" t="inlineStr"/>
+      <c r="E38" s="5" t="inlineStr"/>
+      <c r="F38" s="5" t="inlineStr"/>
+      <c r="G38" s="5" t="inlineStr"/>
+      <c r="H38" s="5" t="inlineStr"/>
+      <c r="I38" s="5" t="inlineStr"/>
+      <c r="J38" s="5" t="inlineStr"/>
+      <c r="K38" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20AB (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>INDURO</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr"/>
+      <c r="C39" s="5" t="inlineStr"/>
+      <c r="D39" s="5" t="inlineStr"/>
+      <c r="E39" s="5" t="inlineStr"/>
+      <c r="F39" s="5" t="inlineStr"/>
+      <c r="G39" s="5" t="inlineStr"/>
+      <c r="H39" s="5" t="inlineStr"/>
+      <c r="I39" s="5" t="inlineStr"/>
+      <c r="J39" s="5" t="inlineStr"/>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>CUL HAIPHONG</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr"/>
+      <c r="C40" s="5" t="inlineStr"/>
+      <c r="D40" s="5" t="inlineStr"/>
+      <c r="E40" s="5" t="inlineStr"/>
+      <c r="F40" s="5" t="inlineStr"/>
+      <c r="G40" s="5" t="inlineStr"/>
+      <c r="H40" s="5" t="inlineStr"/>
+      <c r="I40" s="5" t="inlineStr"/>
+      <c r="J40" s="5" t="inlineStr"/>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B (new, shift 4A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 102</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr"/>
+      <c r="C41" s="5" t="inlineStr"/>
+      <c r="D41" s="5" t="inlineStr"/>
+      <c r="E41" s="5" t="inlineStr"/>
+      <c r="F41" s="5" t="inlineStr"/>
+      <c r="G41" s="5" t="inlineStr"/>
+      <c r="H41" s="5" t="inlineStr"/>
+      <c r="I41" s="5" t="inlineStr"/>
+      <c r="J41" s="5" t="inlineStr"/>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F (new)</t>
         </is>
       </c>
     </row>
@@ -2939,13 +3119,767 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 07 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>KMTC TOKYO</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>46301.54166666666</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>46301.54166666666</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>46303.5</v>
+      </c>
+      <c r="G4" s="26">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>GREEN PARK</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>482</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46302.45833333334</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="G5" s="26">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>HE JIN</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>552</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46302.83333333334</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46304.625</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46305.625</v>
+      </c>
+      <c r="G6" s="26">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>CNC MARS</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46304.41666666666</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46305.58333333334</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46307.16666666666</v>
+      </c>
+      <c r="G7" s="26">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE SPICA</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>46300.875</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>46301.54166666666</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="G8" s="26">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>SITC HOCHIMINH</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>470</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>46302.75</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>46303.58333333334</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>46304.70833333334</v>
+      </c>
+      <c r="G9" s="26">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>INDURO</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>46304.375</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>46304.625</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>46306.125</v>
+      </c>
+      <c r="G10" s="26">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>CUL HAIPHONG</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>458</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>46304.75</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>46306.20833333334</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>46307.20833333334</v>
+      </c>
+      <c r="G11" s="26">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="I11" s="23" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE DENEB</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>46302.45833333334</v>
+      </c>
+      <c r="G12" s="26">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="23" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>JOSCO LUCKY</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>46301.875</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="G13" s="26">
+        <f>(F13-E13)*24</f>
+        <v/>
+      </c>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I13" s="23" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>ZHONG GU DONG HAI</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>46303.58333333334</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="G14" s="26">
+        <f>(F14-E14)*24</f>
+        <v/>
+      </c>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I14" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>YM INCEPTION</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>46306.04166666666</v>
+      </c>
+      <c r="G15" s="26">
+        <f>(F15-E15)*24</f>
+        <v/>
+      </c>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>MTT BANGKOK</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>46302.5</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>46302.58333333334</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="G16" s="26">
+        <f>(F16-E16)*24</f>
+        <v/>
+      </c>
+      <c r="H16" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I16" s="23" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE ATLANTIC</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>46302.91666666666</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>46304.625</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>46306.125</v>
+      </c>
+      <c r="G17" s="26">
+        <f>(F17-E17)*24</f>
+        <v/>
+      </c>
+      <c r="H17" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I17" s="23" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>XIN AN</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>46302.58333333334</v>
+      </c>
+      <c r="F18" s="11" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="G18" s="26">
+        <f>(F18-E18)*24</f>
+        <v/>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I18" s="23" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>KANWAY FORTUNE</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>46303.75</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>46305.625</v>
+      </c>
+      <c r="G19" s="26">
+        <f>(F19-E19)*24</f>
+        <v/>
+      </c>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I19" s="23" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 102</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>46305.58333333334</v>
+      </c>
+      <c r="F20" s="11" t="n">
+        <v>46306.125</v>
+      </c>
+      <c r="G20" s="26">
+        <f>(F20-E20)*24</f>
+        <v/>
+      </c>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I20" s="23" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="28" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G24" s="29" t="n"/>
+      <c r="H24" s="29" t="n"/>
+      <c r="I24" s="30" t="n"/>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C25" s="32" t="n"/>
+      <c r="D25" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E25" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (MTT BANGKOK and SAWASDEE ATLANTIC are still booked at 20D)  —  Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+      <c r="G25" s="32" t="n"/>
+      <c r="H25" s="32" t="n"/>
+      <c r="I25" s="32" t="n"/>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C26" s="31" t="n"/>
+      <c r="D26" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E26" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail (in progress)  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G26" s="31" t="n"/>
+      <c r="H26" s="31" t="n"/>
+      <c r="I26" s="31" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="F26:I26"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3958,8 +4892,70 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="12" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C35" s="13" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E35" s="14" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (MTT BANGKOK and SAWASDEE ATLANTIC are still booked at 20D)</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="inlineStr">
+        <is>
+          <t>Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="C36" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D36" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E36" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F36" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail (in progress)</t>
+        </is>
+      </c>
+      <c r="G36" s="9" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G34"/>
+  <autoFilter ref="A4:G36"/>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add 08 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -19,9 +19,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 Oct 2026" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Oct 2026" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Oct 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Oct 2026" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -628,7 +629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -642,6 +643,7 @@
     <col width="42" customWidth="1" min="9" max="9"/>
     <col width="44" customWidth="1" min="10" max="10"/>
     <col width="44" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -712,6 +714,11 @@
       <c r="K4" s="3" t="inlineStr">
         <is>
           <t>07 Oct 2026</t>
+        </is>
+      </c>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>08 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -743,6 +750,7 @@
       <c r="I5" s="5" t="inlineStr"/>
       <c r="J5" s="5" t="inlineStr"/>
       <c r="K5" s="5" t="inlineStr"/>
+      <c r="L5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -776,6 +784,7 @@
       <c r="I6" s="5" t="inlineStr"/>
       <c r="J6" s="5" t="inlineStr"/>
       <c r="K6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -801,6 +810,7 @@
       <c r="I7" s="5" t="inlineStr"/>
       <c r="J7" s="5" t="inlineStr"/>
       <c r="K7" s="5" t="inlineStr"/>
+      <c r="L7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -830,6 +840,7 @@
       <c r="I8" s="5" t="inlineStr"/>
       <c r="J8" s="5" t="inlineStr"/>
       <c r="K8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -859,6 +870,7 @@
       <c r="I9" s="5" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr"/>
       <c r="K9" s="5" t="inlineStr"/>
+      <c r="L9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -884,6 +896,7 @@
       <c r="I10" s="5" t="inlineStr"/>
       <c r="J10" s="5" t="inlineStr"/>
       <c r="K10" s="5" t="inlineStr"/>
+      <c r="L10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -917,6 +930,7 @@
       <c r="I11" s="5" t="inlineStr"/>
       <c r="J11" s="5" t="inlineStr"/>
       <c r="K11" s="5" t="inlineStr"/>
+      <c r="L11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -942,6 +956,7 @@
       <c r="I12" s="5" t="inlineStr"/>
       <c r="J12" s="5" t="inlineStr"/>
       <c r="K12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -975,6 +990,7 @@
       <c r="I13" s="5" t="inlineStr"/>
       <c r="J13" s="5" t="inlineStr"/>
       <c r="K13" s="5" t="inlineStr"/>
+      <c r="L13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1016,6 +1032,7 @@
       <c r="I14" s="5" t="inlineStr"/>
       <c r="J14" s="5" t="inlineStr"/>
       <c r="K14" s="5" t="inlineStr"/>
+      <c r="L14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1049,6 +1066,7 @@
       <c r="I15" s="5" t="inlineStr"/>
       <c r="J15" s="5" t="inlineStr"/>
       <c r="K15" s="5" t="inlineStr"/>
+      <c r="L15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1086,6 +1104,7 @@
       <c r="I16" s="5" t="inlineStr"/>
       <c r="J16" s="5" t="inlineStr"/>
       <c r="K16" s="5" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1123,6 +1142,7 @@
       <c r="I17" s="5" t="inlineStr"/>
       <c r="J17" s="5" t="inlineStr"/>
       <c r="K17" s="5" t="inlineStr"/>
+      <c r="L17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1160,6 +1180,7 @@
       <c r="I18" s="5" t="inlineStr"/>
       <c r="J18" s="5" t="inlineStr"/>
       <c r="K18" s="5" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1205,6 +1226,7 @@
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr"/>
+      <c r="L19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1250,6 +1272,7 @@
           <t>sailed (06/11)</t>
         </is>
       </c>
+      <c r="L20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1291,6 +1314,7 @@
         </is>
       </c>
       <c r="K21" s="5" t="inlineStr"/>
+      <c r="L21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1328,6 +1352,7 @@
       </c>
       <c r="J22" s="5" t="inlineStr"/>
       <c r="K22" s="5" t="inlineStr"/>
+      <c r="L22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1369,6 +1394,11 @@
           <t>at anchorage · 20C (P.B 07/13, ETD 08/12→08/13)</t>
         </is>
       </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20C (ETD 08/13)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1410,6 +1440,11 @@
           <t>alongside · 20C (ETD 07/11)</t>
         </is>
       </c>
+      <c r="L24" s="5" t="inlineStr">
+        <is>
+          <t>sailed (07/11)</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1439,6 +1474,7 @@
       <c r="I25" s="5" t="inlineStr"/>
       <c r="J25" s="5" t="inlineStr"/>
       <c r="K25" s="5" t="inlineStr"/>
+      <c r="L25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1472,6 +1508,7 @@
       </c>
       <c r="J26" s="5" t="inlineStr"/>
       <c r="K26" s="5" t="inlineStr"/>
+      <c r="L26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1505,6 +1542,11 @@
         </is>
       </c>
       <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20B (ETD 08/13)</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
         <is>
           <t>alongside · 20B (ETD 08/13)</t>
         </is>
@@ -1538,6 +1580,11 @@
         </is>
       </c>
       <c r="K28" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20AB (ETD 08/12)</t>
+        </is>
+      </c>
+      <c r="L28" s="5" t="inlineStr">
         <is>
           <t>alongside · 20AB (ETD 08/12)</t>
         </is>
@@ -1571,6 +1618,11 @@
           <t>expected → 20AB (P.B 08/15→08/13)</t>
         </is>
       </c>
+      <c r="L29" s="6" t="inlineStr">
+        <is>
+          <t>at anchorage · 20AB (ETA 07/11→07/10, P.B 08/13)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1600,6 +1652,11 @@
           <t>expected → 20D</t>
         </is>
       </c>
+      <c r="L30" s="6" t="inlineStr">
+        <is>
+          <t>at anchorage → 20F (ETA 07/22→07/20)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1629,6 +1686,11 @@
           <t>expected · 20D (ETA 07/12)</t>
         </is>
       </c>
+      <c r="L31" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20D (ETD 09/13→09/02)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1656,6 +1718,11 @@
       <c r="K32" s="5" t="inlineStr">
         <is>
           <t>expected · 20F (ETA 07/13)</t>
+        </is>
+      </c>
+      <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20F (ETD 09/13)</t>
         </is>
       </c>
     </row>
@@ -1683,6 +1750,11 @@
           <t>expected → 20B (ETA 07/19→07/18)</t>
         </is>
       </c>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>at anchorage · 20B (ETA 07/18→07/15)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -1708,6 +1780,11 @@
           <t>expected → 20C (P.B 09/15→09/13, ETD 10/16→11/01)</t>
         </is>
       </c>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -1733,6 +1810,11 @@
           <t>expected → 20AB</t>
         </is>
       </c>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>at anchorage → 22A (shifts to 20D 09/02, ETD 10/13)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -1758,6 +1840,11 @@
           <t>expected · 20C (ETA 07/16→07/13)</t>
         </is>
       </c>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>at anchorage · 20C (ETA 07/13→07/14)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -1781,6 +1868,11 @@
       <c r="K37" s="6" t="inlineStr">
         <is>
           <t>expected → 20F (P.B 09/15→09/14, ETD 11/03→10/15)</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20AB</t>
         </is>
       </c>
     </row>
@@ -1804,6 +1896,11 @@
           <t>expected · 20AB (new)</t>
         </is>
       </c>
+      <c r="L38" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20AB (ETA 09/10→09/22, ETD 12/04→11/15)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -1825,6 +1922,11 @@
           <t>expected · 20B (new)</t>
         </is>
       </c>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20B (P.B 09/15→09/16, ETD 11/03→11/14)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -1846,6 +1948,11 @@
           <t>expected · 20B (new, shift 4A)</t>
         </is>
       </c>
+      <c r="L40" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20D (shift 4A, ETA 09/20)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -1865,6 +1972,55 @@
       <c r="K41" s="5" t="inlineStr">
         <is>
           <t>expected · 20F (new)</t>
+        </is>
+      </c>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20F (ETA 09/13→10/21, ETD 11/03→12/02)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>STARSHIP AQUILA</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr"/>
+      <c r="C42" s="5" t="inlineStr"/>
+      <c r="D42" s="5" t="inlineStr"/>
+      <c r="E42" s="5" t="inlineStr"/>
+      <c r="F42" s="5" t="inlineStr"/>
+      <c r="G42" s="5" t="inlineStr"/>
+      <c r="H42" s="5" t="inlineStr"/>
+      <c r="I42" s="5" t="inlineStr"/>
+      <c r="J42" s="5" t="inlineStr"/>
+      <c r="K42" s="5" t="inlineStr"/>
+      <c r="L42" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>INCEDA</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr"/>
+      <c r="C43" s="5" t="inlineStr"/>
+      <c r="D43" s="5" t="inlineStr"/>
+      <c r="E43" s="5" t="inlineStr"/>
+      <c r="F43" s="5" t="inlineStr"/>
+      <c r="G43" s="5" t="inlineStr"/>
+      <c r="H43" s="5" t="inlineStr"/>
+      <c r="I43" s="5" t="inlineStr"/>
+      <c r="J43" s="5" t="inlineStr"/>
+      <c r="K43" s="5" t="inlineStr"/>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D (new)</t>
         </is>
       </c>
     </row>
@@ -3873,13 +4029,835 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 08 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>KMTC TOKYO</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>46301.54166666666</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>46301.54166666666</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>46303.5</v>
+      </c>
+      <c r="G4" s="26">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>GREEN PARK</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>482</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46302.41666666666</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="G5" s="26">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>KANWAY FORTUNE</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46303.75</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46305.625</v>
+      </c>
+      <c r="G6" s="26">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>CNC MARS</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46304.91666666666</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46305.625</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46306.625</v>
+      </c>
+      <c r="G7" s="26">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE SPICA</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>46300.875</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>46301.54166666666</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="G8" s="26">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>SITC HOCHIMINH</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>470</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>46302.625</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>46303.58333333334</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>46304.70833333334</v>
+      </c>
+      <c r="G9" s="26">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>INDURO</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>46304.375</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>46304.66666666666</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>46306.58333333334</v>
+      </c>
+      <c r="G10" s="26">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>JOSCO LUCKY</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>46301.875</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="G11" s="26">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="23" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>ZHONG GU DONG HAI</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>46302.58333333334</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>46303.58333333334</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="G12" s="26">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="23" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>YM INCEPTION</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>46306.04166666666</v>
+      </c>
+      <c r="G13" s="26">
+        <f>(F13-E13)*24</f>
+        <v/>
+      </c>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I13" s="23" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>STARSHIP AQUILA</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>46304.91666666666</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>46306.16666666666</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>46307.54166666666</v>
+      </c>
+      <c r="G14" s="26">
+        <f>(F14-E14)*24</f>
+        <v/>
+      </c>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I14" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>MTT BANGKOK</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>46302.58333333334</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>46304.08333333334</v>
+      </c>
+      <c r="G15" s="26">
+        <f>(F15-E15)*24</f>
+        <v/>
+      </c>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>HE JIN</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>552</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>46304.08333333334</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>46304.08333333334</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>46305.54166666666</v>
+      </c>
+      <c r="G16" s="26">
+        <f>(F16-E16)*24</f>
+        <v/>
+      </c>
+      <c r="H16" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I16" s="23" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>CUL HAIPHONG</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>458</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>46304.83333333334</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>46306.25</v>
+      </c>
+      <c r="G17" s="26">
+        <f>(F17-E17)*24</f>
+        <v/>
+      </c>
+      <c r="H17" s="23" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="I17" s="23" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>INCEDA</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>46305.70833333334</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>46306.20833333334</v>
+      </c>
+      <c r="F18" s="11" t="n">
+        <v>46307.58333333334</v>
+      </c>
+      <c r="G18" s="26">
+        <f>(F18-E18)*24</f>
+        <v/>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I18" s="23" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>XIN AN</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>46302.58333333334</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="G19" s="26">
+        <f>(F19-E19)*24</f>
+        <v/>
+      </c>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I19" s="23" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE ATLANTIC</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>46302.83333333334</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>46304.625</v>
+      </c>
+      <c r="F20" s="11" t="n">
+        <v>46306.125</v>
+      </c>
+      <c r="G20" s="26">
+        <f>(F20-E20)*24</f>
+        <v/>
+      </c>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I20" s="23" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 102</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D21" s="11" t="n">
+        <v>46305.875</v>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>46306.20833333334</v>
+      </c>
+      <c r="F21" s="11" t="n">
+        <v>46307.08333333334</v>
+      </c>
+      <c r="G21" s="26">
+        <f>(F21-E21)*24</f>
+        <v/>
+      </c>
+      <c r="H21" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I21" s="23" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>22A</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>HE JIN</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="n">
+        <v>552</v>
+      </c>
+      <c r="D22" s="11" t="n">
+        <v>46302.79166666666</v>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>46303.66666666666</v>
+      </c>
+      <c r="F22" s="11" t="n">
+        <v>46304.08333333334</v>
+      </c>
+      <c r="G22" s="26">
+        <f>(F22-E22)*24</f>
+        <v/>
+      </c>
+      <c r="H22" s="23" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="I22" s="23" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="28" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G26" s="29" t="n"/>
+      <c r="H26" s="29" t="n"/>
+      <c r="I26" s="30" t="n"/>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C27" s="32" t="n"/>
+      <c r="D27" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E27" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (MTT BANGKOK has been alongside at 20D since 07/14, HE JIN shifts in on 09/02)  —  Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+      <c r="G27" s="32" t="n"/>
+      <c r="H27" s="32" t="n"/>
+      <c r="I27" s="32" t="n"/>
+    </row>
+    <row r="28" ht="42" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C28" s="31" t="n"/>
+      <c r="D28" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E28" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail (in progress)  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G28" s="31" t="n"/>
+      <c r="H28" s="31" t="n"/>
+      <c r="I28" s="31" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="F27:I27"/>
+    <mergeCell ref="F28:I28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4954,8 +5932,70 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="12" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D37" s="14" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E37" s="14" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F37" s="13" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (MTT BANGKOK has been alongside at 20D since 07/14, HE JIN shifts in on 09/02)</t>
+        </is>
+      </c>
+      <c r="G37" s="13" t="inlineStr">
+        <is>
+          <t>Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B38" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="C38" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D38" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E38" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F38" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail (in progress)</t>
+        </is>
+      </c>
+      <c r="G38" s="9" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G36"/>
+  <autoFilter ref="A4:G38"/>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add 09 Oct 2026 ship movement data, widen timeline to 15 Oct, update Excel and history
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -21,10 +21,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 Oct 2026" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Oct 2026" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Oct 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Oct 2026" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$N$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$N$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -668,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:M47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -683,6 +684,7 @@
     <col width="44" customWidth="1" min="10" max="10"/>
     <col width="44" customWidth="1" min="11" max="11"/>
     <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="44" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -758,6 +760,11 @@
       <c r="L4" s="3" t="inlineStr">
         <is>
           <t>08 Oct 2026</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>09 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -790,6 +797,7 @@
       <c r="J5" s="5" t="inlineStr"/>
       <c r="K5" s="5" t="inlineStr"/>
       <c r="L5" s="5" t="inlineStr"/>
+      <c r="M5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -824,6 +832,7 @@
       <c r="J6" s="5" t="inlineStr"/>
       <c r="K6" s="5" t="inlineStr"/>
       <c r="L6" s="5" t="inlineStr"/>
+      <c r="M6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -850,6 +859,7 @@
       <c r="J7" s="5" t="inlineStr"/>
       <c r="K7" s="5" t="inlineStr"/>
       <c r="L7" s="5" t="inlineStr"/>
+      <c r="M7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -880,6 +890,7 @@
       <c r="J8" s="5" t="inlineStr"/>
       <c r="K8" s="5" t="inlineStr"/>
       <c r="L8" s="5" t="inlineStr"/>
+      <c r="M8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -910,6 +921,7 @@
       <c r="J9" s="5" t="inlineStr"/>
       <c r="K9" s="5" t="inlineStr"/>
       <c r="L9" s="5" t="inlineStr"/>
+      <c r="M9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -936,6 +948,7 @@
       <c r="J10" s="5" t="inlineStr"/>
       <c r="K10" s="5" t="inlineStr"/>
       <c r="L10" s="5" t="inlineStr"/>
+      <c r="M10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -970,6 +983,7 @@
       <c r="J11" s="5" t="inlineStr"/>
       <c r="K11" s="5" t="inlineStr"/>
       <c r="L11" s="5" t="inlineStr"/>
+      <c r="M11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -996,6 +1010,7 @@
       <c r="J12" s="5" t="inlineStr"/>
       <c r="K12" s="5" t="inlineStr"/>
       <c r="L12" s="5" t="inlineStr"/>
+      <c r="M12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1030,6 +1045,7 @@
       <c r="J13" s="5" t="inlineStr"/>
       <c r="K13" s="5" t="inlineStr"/>
       <c r="L13" s="5" t="inlineStr"/>
+      <c r="M13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1072,6 +1088,7 @@
       <c r="J14" s="5" t="inlineStr"/>
       <c r="K14" s="5" t="inlineStr"/>
       <c r="L14" s="5" t="inlineStr"/>
+      <c r="M14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1106,6 +1123,7 @@
       <c r="J15" s="5" t="inlineStr"/>
       <c r="K15" s="5" t="inlineStr"/>
       <c r="L15" s="5" t="inlineStr"/>
+      <c r="M15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1144,6 +1162,7 @@
       <c r="J16" s="5" t="inlineStr"/>
       <c r="K16" s="5" t="inlineStr"/>
       <c r="L16" s="5" t="inlineStr"/>
+      <c r="M16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1182,6 +1201,11 @@
       <c r="J17" s="5" t="inlineStr"/>
       <c r="K17" s="5" t="inlineStr"/>
       <c r="L17" s="5" t="inlineStr"/>
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20C (returns for a new call, ETA 12/18, shift 1C)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1220,6 +1244,7 @@
       <c r="J18" s="5" t="inlineStr"/>
       <c r="K18" s="5" t="inlineStr"/>
       <c r="L18" s="5" t="inlineStr"/>
+      <c r="M18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1266,6 +1291,7 @@
       </c>
       <c r="K19" s="5" t="inlineStr"/>
       <c r="L19" s="5" t="inlineStr"/>
+      <c r="M19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1312,6 +1338,7 @@
         </is>
       </c>
       <c r="L20" s="5" t="inlineStr"/>
+      <c r="M20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1354,6 +1381,7 @@
       </c>
       <c r="K21" s="5" t="inlineStr"/>
       <c r="L21" s="5" t="inlineStr"/>
+      <c r="M21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1392,6 +1420,7 @@
       <c r="J22" s="5" t="inlineStr"/>
       <c r="K22" s="5" t="inlineStr"/>
       <c r="L22" s="5" t="inlineStr"/>
+      <c r="M22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1438,6 +1467,11 @@
           <t>alongside · 20C (ETD 08/13)</t>
         </is>
       </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>sailed (08/13)</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1484,6 +1518,7 @@
           <t>sailed (07/11)</t>
         </is>
       </c>
+      <c r="M24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1514,6 +1549,7 @@
       <c r="J25" s="5" t="inlineStr"/>
       <c r="K25" s="5" t="inlineStr"/>
       <c r="L25" s="5" t="inlineStr"/>
+      <c r="M25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1548,6 +1584,7 @@
       <c r="J26" s="5" t="inlineStr"/>
       <c r="K26" s="5" t="inlineStr"/>
       <c r="L26" s="5" t="inlineStr"/>
+      <c r="M26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1588,6 +1625,11 @@
       <c r="L27" s="5" t="inlineStr">
         <is>
           <t>alongside · 20B (ETD 08/13)</t>
+        </is>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>sailed (08/13)</t>
         </is>
       </c>
     </row>
@@ -1626,6 +1668,11 @@
       <c r="L28" s="5" t="inlineStr">
         <is>
           <t>alongside · 20AB (ETD 08/12)</t>
+        </is>
+      </c>
+      <c r="M28" s="5" t="inlineStr">
+        <is>
+          <t>sailed (08/12)</t>
         </is>
       </c>
     </row>
@@ -1662,6 +1709,11 @@
           <t>at anchorage · 20AB (ETA 07/11→07/10, P.B 08/13)</t>
         </is>
       </c>
+      <c r="M29" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20AB (P.B 08/13→08/14, ETD 09/14→09/16)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1696,6 +1748,11 @@
           <t>at anchorage → 20F (ETA 07/22→07/20)</t>
         </is>
       </c>
+      <c r="M30" s="5" t="inlineStr">
+        <is>
+          <t>at anchorage · 20F (P.B 09/15)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1730,6 +1787,11 @@
           <t>alongside · 20D (ETD 09/13→09/02)</t>
         </is>
       </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>sailed (09/02)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1760,6 +1822,11 @@
         </is>
       </c>
       <c r="L32" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20F (ETD 09/13)</t>
+        </is>
+      </c>
+      <c r="M32" s="5" t="inlineStr">
         <is>
           <t>alongside · 20F (ETD 09/13)</t>
         </is>
@@ -1794,6 +1861,11 @@
           <t>at anchorage · 20B (ETA 07/18→07/15)</t>
         </is>
       </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20B (ETD 09/17)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -1824,6 +1896,11 @@
           <t>expected · 20C</t>
         </is>
       </c>
+      <c r="M34" s="6" t="inlineStr">
+        <is>
+          <t>at anchorage · 20C (ETD 11/01→10/16)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -1854,6 +1931,11 @@
           <t>at anchorage → 22A (shifts to 20D 09/02, ETD 10/13)</t>
         </is>
       </c>
+      <c r="M35" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20D (shifted in from 22A, P.B 09/02→08/24)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -1884,6 +1966,11 @@
           <t>at anchorage · 20C (ETA 07/13→07/14)</t>
         </is>
       </c>
+      <c r="M36" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20C (ETD 09/14)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -1912,6 +1999,11 @@
       <c r="L37" s="6" t="inlineStr">
         <is>
           <t>expected → 20AB</t>
+        </is>
+      </c>
+      <c r="M37" s="6" t="inlineStr">
+        <is>
+          <t>at anchorage · 20AB (ETA 08/18→08/16)</t>
         </is>
       </c>
     </row>
@@ -1940,6 +2032,11 @@
           <t>expected · 20AB (ETA 09/10→09/22, ETD 12/04→11/15)</t>
         </is>
       </c>
+      <c r="M38" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20AB</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -1966,6 +2063,11 @@
           <t>expected · 20B (P.B 09/15→09/16, ETD 11/03→11/14)</t>
         </is>
       </c>
+      <c r="M39" s="6" t="inlineStr">
+        <is>
+          <t>at anchorage · 20B (ETA 09/09→09/06)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -1992,6 +2094,11 @@
           <t>expected → 20D (shift 4A, ETA 09/20)</t>
         </is>
       </c>
+      <c r="M40" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D (ETA 09/20)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2016,6 +2123,11 @@
       <c r="L41" s="6" t="inlineStr">
         <is>
           <t>expected · 20F (ETA 09/13→10/21, ETD 11/03→12/02)</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F</t>
         </is>
       </c>
     </row>
@@ -2040,6 +2152,11 @@
           <t>expected · 20C (new)</t>
         </is>
       </c>
+      <c r="M42" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20C (P.B 11/04→10/16, ETD 12/13→12/05)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2060,6 +2177,103 @@
       <c r="L43" s="5" t="inlineStr">
         <is>
           <t>expected · 20D (new)</t>
+        </is>
+      </c>
+      <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>SAMAL</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr"/>
+      <c r="C44" s="5" t="inlineStr"/>
+      <c r="D44" s="5" t="inlineStr"/>
+      <c r="E44" s="5" t="inlineStr"/>
+      <c r="F44" s="5" t="inlineStr"/>
+      <c r="G44" s="5" t="inlineStr"/>
+      <c r="H44" s="5" t="inlineStr"/>
+      <c r="I44" s="5" t="inlineStr"/>
+      <c r="J44" s="5" t="inlineStr"/>
+      <c r="K44" s="5" t="inlineStr"/>
+      <c r="L44" s="5" t="inlineStr"/>
+      <c r="M44" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20AB (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>JOSCO SHINE</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr"/>
+      <c r="C45" s="5" t="inlineStr"/>
+      <c r="D45" s="5" t="inlineStr"/>
+      <c r="E45" s="5" t="inlineStr"/>
+      <c r="F45" s="5" t="inlineStr"/>
+      <c r="G45" s="5" t="inlineStr"/>
+      <c r="H45" s="5" t="inlineStr"/>
+      <c r="I45" s="5" t="inlineStr"/>
+      <c r="J45" s="5" t="inlineStr"/>
+      <c r="K45" s="5" t="inlineStr"/>
+      <c r="L45" s="5" t="inlineStr"/>
+      <c r="M45" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>KMTC TAIPEIS</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr"/>
+      <c r="C46" s="5" t="inlineStr"/>
+      <c r="D46" s="5" t="inlineStr"/>
+      <c r="E46" s="5" t="inlineStr"/>
+      <c r="F46" s="5" t="inlineStr"/>
+      <c r="G46" s="5" t="inlineStr"/>
+      <c r="H46" s="5" t="inlineStr"/>
+      <c r="I46" s="5" t="inlineStr"/>
+      <c r="J46" s="5" t="inlineStr"/>
+      <c r="K46" s="5" t="inlineStr"/>
+      <c r="L46" s="5" t="inlineStr"/>
+      <c r="M46" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>SAWASDEE SUNRISE</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr"/>
+      <c r="C47" s="5" t="inlineStr"/>
+      <c r="D47" s="5" t="inlineStr"/>
+      <c r="E47" s="5" t="inlineStr"/>
+      <c r="F47" s="5" t="inlineStr"/>
+      <c r="G47" s="5" t="inlineStr"/>
+      <c r="H47" s="5" t="inlineStr"/>
+      <c r="I47" s="5" t="inlineStr"/>
+      <c r="J47" s="5" t="inlineStr"/>
+      <c r="K47" s="5" t="inlineStr"/>
+      <c r="L47" s="5" t="inlineStr"/>
+      <c r="M47" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F (new)</t>
         </is>
       </c>
     </row>
@@ -5402,13 +5616,835 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 09 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>GREEN PARK</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>482</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>46302.41666666666</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>46303.58333333334</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>46304.66666666666</v>
+      </c>
+      <c r="G4" s="28">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>KANWAY FORTUNE</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46303.66666666666</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46305.625</v>
+      </c>
+      <c r="G5" s="28">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>CNC MARS</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46304.91666666666</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46305.625</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46306.625</v>
+      </c>
+      <c r="G6" s="28">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>SAMAL</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46307.16666666666</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46307.20833333334</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46308.58333333334</v>
+      </c>
+      <c r="G7" s="28">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>SITC HOCHIMINH</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>470</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>46302.625</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>46303.58333333334</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>46304.70833333334</v>
+      </c>
+      <c r="G8" s="28">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>INDURO</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>46304.25</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>46304.66666666666</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>46306.58333333334</v>
+      </c>
+      <c r="G9" s="28">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>JOSCO SHINE</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>46306.70833333334</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>46306.70833333334</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>46307.58333333334</v>
+      </c>
+      <c r="G10" s="28">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>ZHONG GU DONG HAI</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>46302.58333333334</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>46303.58333333334</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="G11" s="28">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="23" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>YM INCEPTION</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="G12" s="28">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="23" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>STARSHIP AQUILA</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>46304.91666666666</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>46307.20833333334</v>
+      </c>
+      <c r="G13" s="28">
+        <f>(F13-E13)*24</f>
+        <v/>
+      </c>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I13" s="23" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>ALS SUMIRE</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>537</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>46307.75</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>46307.75</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>46309.20833333334</v>
+      </c>
+      <c r="G14" s="28">
+        <f>(F14-E14)*24</f>
+        <v/>
+      </c>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>1C</t>
+        </is>
+      </c>
+      <c r="I14" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>HE JIN</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>552</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>46305.54166666666</v>
+      </c>
+      <c r="G15" s="28">
+        <f>(F15-E15)*24</f>
+        <v/>
+      </c>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>CUL HAIPHONG</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>458</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>46304.83333333334</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>46306.25</v>
+      </c>
+      <c r="G16" s="28">
+        <f>(F16-E16)*24</f>
+        <v/>
+      </c>
+      <c r="H16" s="23" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="I16" s="23" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>INCEDA</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>46305.70833333334</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>46306.20833333334</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>46307.58333333334</v>
+      </c>
+      <c r="G17" s="28">
+        <f>(F17-E17)*24</f>
+        <v/>
+      </c>
+      <c r="H17" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I17" s="23" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>KMTC TAIPEIS</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>46307.95833333334</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>46308.20833333334</v>
+      </c>
+      <c r="F18" s="11" t="n">
+        <v>46309.625</v>
+      </c>
+      <c r="G18" s="28">
+        <f>(F18-E18)*24</f>
+        <v/>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I18" s="23" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>XIN AN</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>46302.58333333334</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="G19" s="28">
+        <f>(F19-E19)*24</f>
+        <v/>
+      </c>
+      <c r="H19" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I19" s="23" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE ATLANTIC</t>
+        </is>
+      </c>
+      <c r="C20" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D20" s="11" t="n">
+        <v>46302.83333333334</v>
+      </c>
+      <c r="E20" s="11" t="n">
+        <v>46304.625</v>
+      </c>
+      <c r="F20" s="11" t="n">
+        <v>46306.125</v>
+      </c>
+      <c r="G20" s="28">
+        <f>(F20-E20)*24</f>
+        <v/>
+      </c>
+      <c r="H20" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I20" s="23" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 102</t>
+        </is>
+      </c>
+      <c r="C21" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D21" s="11" t="n">
+        <v>46305.875</v>
+      </c>
+      <c r="E21" s="11" t="n">
+        <v>46306.20833333334</v>
+      </c>
+      <c r="F21" s="11" t="n">
+        <v>46307.08333333334</v>
+      </c>
+      <c r="G21" s="28">
+        <f>(F21-E21)*24</f>
+        <v/>
+      </c>
+      <c r="H21" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I21" s="23" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE SUNRISE</t>
+        </is>
+      </c>
+      <c r="C22" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D22" s="11" t="n">
+        <v>46307.20833333334</v>
+      </c>
+      <c r="E22" s="11" t="n">
+        <v>46307.20833333334</v>
+      </c>
+      <c r="F22" s="11" t="n">
+        <v>46308.625</v>
+      </c>
+      <c r="G22" s="28">
+        <f>(F22-E22)*24</f>
+        <v/>
+      </c>
+      <c r="H22" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I22" s="23" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="39" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G26" s="40" t="n"/>
+      <c r="H26" s="40" t="n"/>
+      <c r="I26" s="41" t="n"/>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C27" s="43" t="n"/>
+      <c r="D27" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E27" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F27" s="16" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (HE JIN has shifted in to 20D, other vessels are booked from 10/16)  —  Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+      <c r="G27" s="43" t="n"/>
+      <c r="H27" s="43" t="n"/>
+      <c r="I27" s="43" t="n"/>
+    </row>
+    <row r="28" ht="42" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C28" s="42" t="n"/>
+      <c r="D28" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E28" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail (in progress)  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G28" s="42" t="n"/>
+      <c r="H28" s="42" t="n"/>
+      <c r="I28" s="42" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="F27:I27"/>
+    <mergeCell ref="F28:I28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6545,8 +7581,70 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" s="12" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E39" s="14" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (HE JIN has shifted in to 20D, other vessels are booked from 10/16)</t>
+        </is>
+      </c>
+      <c r="G39" s="13" t="inlineStr">
+        <is>
+          <t>Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B40" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="C40" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D40" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E40" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F40" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail (in progress)</t>
+        </is>
+      </c>
+      <c r="G40" s="9" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G38"/>
+  <autoFilter ref="A4:G40"/>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
@@ -6560,7 +7658,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:N50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6600,7 +7698,7 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>46303.375</v>
+        <v>46304.375</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -6992,9 +8090,10 @@
         </is>
       </c>
       <c r="M11" s="23" t="inlineStr"/>
-      <c r="N11" s="23">
-        <f>IF(J11&lt;=$B$3,"Sailed",IF(I11&lt;=$B$3,"Alongside",IF(H11&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N11" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -7015,10 +8114,10 @@
         <v>46300</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="F12" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -7029,10 +8128,10 @@
         <v>46302.41666666666</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>46303.54166666666</v>
+        <v>46303.58333333334</v>
       </c>
       <c r="J12" s="11" t="n">
-        <v>46304.58333333334</v>
+        <v>46304.66666666666</v>
       </c>
       <c r="K12" s="28">
         <f>(J12-I12)*24</f>
@@ -7067,10 +8166,10 @@
         <v>46301</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="F13" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -7078,7 +8177,7 @@
         </is>
       </c>
       <c r="H13" s="11" t="n">
-        <v>46303.75</v>
+        <v>46303.66666666666</v>
       </c>
       <c r="I13" s="11" t="n">
         <v>46304.58333333334</v>
@@ -7119,10 +8218,10 @@
         <v>46302</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="F14" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
@@ -7154,106 +8253,105 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>SAMAL</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F15" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="n">
+        <v>46307.16666666666</v>
+      </c>
+      <c r="I15" s="11" t="n">
+        <v>46307.20833333334</v>
+      </c>
+      <c r="J15" s="11" t="n">
+        <v>46308.58333333334</v>
+      </c>
+      <c r="K15" s="28">
+        <f>(J15-I15)*24</f>
+        <v/>
+      </c>
+      <c r="L15" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M15" s="23" t="inlineStr"/>
+      <c r="N15" s="23">
+        <f>IF(J15&lt;=$B$3,"Sailed",IF(I15&lt;=$B$3,"Alongside",IF(H15&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="29" t="inlineStr">
         <is>
           <t>20B</t>
         </is>
       </c>
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B16" s="29" t="inlineStr">
         <is>
           <t>KMTC GWANGYANG</t>
         </is>
       </c>
-      <c r="C15" s="24" t="n">
+      <c r="C16" s="24" t="n">
         <v>564</v>
       </c>
-      <c r="D15" s="21" t="n">
+      <c r="D16" s="21" t="n">
         <v>46293</v>
       </c>
-      <c r="E15" s="21" t="n">
+      <c r="E16" s="21" t="n">
         <v>46293</v>
       </c>
-      <c r="F15" s="24" t="n">
+      <c r="F16" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="30" t="inlineStr">
+      <c r="G16" s="30" t="inlineStr">
         <is>
           <t>20B</t>
         </is>
       </c>
-      <c r="H15" s="31" t="n">
+      <c r="H16" s="31" t="n">
         <v>46292.79166666666</v>
       </c>
-      <c r="I15" s="31" t="n">
+      <c r="I16" s="31" t="n">
         <v>46292.79166666666</v>
       </c>
-      <c r="J15" s="31" t="n">
+      <c r="J16" s="31" t="n">
         <v>46294.20833333334</v>
       </c>
-      <c r="K15" s="32">
-        <f>(J15-I15)*24</f>
-        <v/>
-      </c>
-      <c r="L15" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M15" s="24" t="inlineStr"/>
-      <c r="N15" s="24" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>20B</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>MILLENNIUM BRIGHT</t>
-        </is>
-      </c>
-      <c r="C16" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D16" s="10" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E16" s="10" t="n">
-        <v>46294</v>
-      </c>
-      <c r="F16" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="n">
-        <v>46293.45833333334</v>
-      </c>
-      <c r="I16" s="11" t="n">
-        <v>46294.20833333334</v>
-      </c>
-      <c r="J16" s="11" t="n">
-        <v>46295.16666666666</v>
-      </c>
-      <c r="K16" s="28">
+      <c r="K16" s="32">
         <f>(J16-I16)*24</f>
         <v/>
       </c>
-      <c r="L16" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M16" s="23" t="inlineStr"/>
-      <c r="N16" s="23" t="inlineStr">
+      <c r="L16" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M16" s="24" t="inlineStr"/>
+      <c r="N16" s="24" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -7267,20 +8365,20 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>M ODYSSEY</t>
+          <t>MILLENNIUM BRIGHT</t>
         </is>
       </c>
       <c r="C17" s="23" t="n">
-        <v>449</v>
+        <v>564</v>
       </c>
       <c r="D17" s="10" t="n">
         <v>46293</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>46295</v>
+        <v>46294</v>
       </c>
       <c r="F17" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
@@ -7288,13 +8386,13 @@
         </is>
       </c>
       <c r="H17" s="11" t="n">
+        <v>46293.45833333334</v>
+      </c>
+      <c r="I17" s="11" t="n">
+        <v>46294.20833333334</v>
+      </c>
+      <c r="J17" s="11" t="n">
         <v>46295.16666666666</v>
-      </c>
-      <c r="I17" s="11" t="n">
-        <v>46295.20833333334</v>
-      </c>
-      <c r="J17" s="11" t="n">
-        <v>46296.20833333334</v>
       </c>
       <c r="K17" s="28">
         <f>(J17-I17)*24</f>
@@ -7302,7 +8400,7 @@
       </c>
       <c r="L17" s="23" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>–</t>
         </is>
       </c>
       <c r="M17" s="23" t="inlineStr"/>
@@ -7313,110 +8411,110 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="33" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>20B</t>
         </is>
       </c>
-      <c r="B18" s="33" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>M ODYSSEY</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="n">
+        <v>449</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F18" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="n">
+        <v>46295.16666666666</v>
+      </c>
+      <c r="I18" s="11" t="n">
+        <v>46295.20833333334</v>
+      </c>
+      <c r="J18" s="11" t="n">
+        <v>46296.20833333334</v>
+      </c>
+      <c r="K18" s="28">
+        <f>(J18-I18)*24</f>
+        <v/>
+      </c>
+      <c r="L18" s="23" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="M18" s="23" t="inlineStr"/>
+      <c r="N18" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="33" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B19" s="33" t="inlineStr">
         <is>
           <t>KHARIS HERITAGE</t>
         </is>
       </c>
-      <c r="C18" s="17" t="n">
+      <c r="C19" s="17" t="n">
         <v>482</v>
       </c>
-      <c r="D18" s="18" t="n">
+      <c r="D19" s="18" t="n">
         <v>46294</v>
       </c>
-      <c r="E18" s="18" t="n">
+      <c r="E19" s="18" t="n">
         <v>46297</v>
       </c>
-      <c r="F18" s="17" t="n">
+      <c r="F19" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>20AB → 20B</t>
         </is>
       </c>
-      <c r="H18" s="25" t="n">
+      <c r="H19" s="25" t="n">
         <v>46296.45833333334</v>
       </c>
-      <c r="I18" s="25" t="n">
+      <c r="I19" s="25" t="n">
         <v>46296.75</v>
       </c>
-      <c r="J18" s="25" t="n">
+      <c r="J19" s="25" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="K18" s="34">
-        <f>(J18-I18)*24</f>
-        <v/>
-      </c>
-      <c r="L18" s="17" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M18" s="17" t="inlineStr">
+      <c r="K19" s="34">
+        <f>(J19-I19)*24</f>
+        <v/>
+      </c>
+      <c r="L19" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M19" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N18" s="17" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>20B</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>YM IMPROVEMENT</t>
-        </is>
-      </c>
-      <c r="C19" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D19" s="10" t="n">
-        <v>46296</v>
-      </c>
-      <c r="E19" s="10" t="n">
-        <v>46300</v>
-      </c>
-      <c r="F19" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>20C → 20B</t>
-        </is>
-      </c>
-      <c r="H19" s="11" t="n">
-        <v>46298.95833333334</v>
-      </c>
-      <c r="I19" s="11" t="n">
-        <v>46299.41666666666</v>
-      </c>
-      <c r="J19" s="11" t="n">
-        <v>46300.5</v>
-      </c>
-      <c r="K19" s="28">
-        <f>(J19-I19)*24</f>
-        <v/>
-      </c>
-      <c r="L19" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M19" s="23" t="inlineStr"/>
-      <c r="N19" s="23" t="inlineStr">
+      <c r="N19" s="17" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -7430,34 +8528,34 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE SPICA</t>
+          <t>YM IMPROVEMENT</t>
         </is>
       </c>
       <c r="C20" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>46299</v>
+        <v>46296</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>46303</v>
+        <v>46300</v>
       </c>
       <c r="F20" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>20C → 20B</t>
         </is>
       </c>
       <c r="H20" s="11" t="n">
-        <v>46300.875</v>
+        <v>46298.95833333334</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>46301.54166666666</v>
+        <v>46299.41666666666</v>
       </c>
       <c r="J20" s="11" t="n">
-        <v>46303.54166666666</v>
+        <v>46300.5</v>
       </c>
       <c r="K20" s="28">
         <f>(J20-I20)*24</f>
@@ -7469,9 +8567,10 @@
         </is>
       </c>
       <c r="M20" s="23" t="inlineStr"/>
-      <c r="N20" s="23">
-        <f>IF(J20&lt;=$B$3,"Sailed",IF(I20&lt;=$B$3,"Alongside",IF(H20&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N20" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -7482,34 +8581,34 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>SITC HOCHIMINH</t>
+          <t>SAWASDEE SPICA</t>
         </is>
       </c>
       <c r="C21" s="23" t="n">
-        <v>470</v>
+        <v>564</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>46301</v>
+        <v>46299</v>
       </c>
       <c r="E21" s="10" t="n">
         <v>46303</v>
       </c>
       <c r="F21" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20B</t>
+        <v>5</v>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H21" s="11" t="n">
-        <v>46302.625</v>
+        <v>46300.875</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>46303.58333333334</v>
+        <v>46301.54166666666</v>
       </c>
       <c r="J21" s="11" t="n">
-        <v>46304.70833333334</v>
+        <v>46303.54166666666</v>
       </c>
       <c r="K21" s="28">
         <f>(J21-I21)*24</f>
@@ -7521,9 +8620,10 @@
         </is>
       </c>
       <c r="M21" s="23" t="inlineStr"/>
-      <c r="N21" s="23">
-        <f>IF(J21&lt;=$B$3,"Sailed",IF(I21&lt;=$B$3,"Alongside",IF(H21&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N21" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -7534,34 +8634,34 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>INDURO</t>
+          <t>SITC HOCHIMINH</t>
         </is>
       </c>
       <c r="C22" s="23" t="n">
-        <v>565</v>
+        <v>470</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="F22" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>4</v>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20B</t>
         </is>
       </c>
       <c r="H22" s="11" t="n">
-        <v>46304.375</v>
+        <v>46302.625</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>46304.66666666666</v>
+        <v>46303.58333333334</v>
       </c>
       <c r="J22" s="11" t="n">
-        <v>46306.58333333334</v>
+        <v>46304.70833333334</v>
       </c>
       <c r="K22" s="28">
         <f>(J22-I22)*24</f>
@@ -7579,94 +8679,93 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="29" t="inlineStr">
-        <is>
-          <t>20C</t>
-        </is>
-      </c>
-      <c r="B23" s="29" t="inlineStr">
-        <is>
-          <t>SAWASDEE DENEB</t>
-        </is>
-      </c>
-      <c r="C23" s="24" t="n">
-        <v>564</v>
-      </c>
-      <c r="D23" s="21" t="n">
-        <v>46297</v>
-      </c>
-      <c r="E23" s="21" t="n">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>INDURO</t>
+        </is>
+      </c>
+      <c r="C23" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D23" s="10" t="n">
         <v>46302</v>
       </c>
-      <c r="F23" s="24" t="n">
-        <v>6</v>
-      </c>
-      <c r="G23" s="30" t="inlineStr">
-        <is>
-          <t>20C</t>
-        </is>
-      </c>
-      <c r="H23" s="31" t="n">
-        <v>46300</v>
-      </c>
-      <c r="I23" s="31" t="n">
-        <v>46300.5</v>
-      </c>
-      <c r="J23" s="31" t="n">
-        <v>46302.45833333334</v>
-      </c>
-      <c r="K23" s="32">
+      <c r="E23" s="10" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F23" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="H23" s="11" t="n">
+        <v>46304.25</v>
+      </c>
+      <c r="I23" s="11" t="n">
+        <v>46304.66666666666</v>
+      </c>
+      <c r="J23" s="11" t="n">
+        <v>46306.58333333334</v>
+      </c>
+      <c r="K23" s="28">
         <f>(J23-I23)*24</f>
         <v/>
       </c>
-      <c r="L23" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M23" s="24" t="inlineStr"/>
-      <c r="N23" s="24" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="L23" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M23" s="23" t="inlineStr"/>
+      <c r="N23" s="23">
+        <f>IF(J23&lt;=$B$3,"Sailed",IF(I23&lt;=$B$3,"Alongside",IF(H23&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>20C</t>
+          <t>20B</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>JOSCO LUCKY</t>
+          <t>JOSCO SHINE</t>
         </is>
       </c>
       <c r="C24" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
       <c r="E24" s="10" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="F24" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="G24" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 20D → 20C</t>
+        <v>1</v>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H24" s="11" t="n">
-        <v>46301.875</v>
+        <v>46306.70833333334</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>46302.54166666666</v>
+        <v>46306.70833333334</v>
       </c>
       <c r="J24" s="11" t="n">
-        <v>46303.54166666666</v>
+        <v>46307.58333333334</v>
       </c>
       <c r="K24" s="28">
         <f>(J24-I24)*24</f>
@@ -7684,55 +8783,56 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="29" t="inlineStr">
         <is>
           <t>20C</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>ZHONG GU DONG HAI</t>
-        </is>
-      </c>
-      <c r="C25" s="23" t="n">
+      <c r="B25" s="29" t="inlineStr">
+        <is>
+          <t>SAWASDEE DENEB</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="n">
         <v>564</v>
       </c>
-      <c r="D25" s="10" t="n">
-        <v>46301</v>
-      </c>
-      <c r="E25" s="10" t="n">
-        <v>46303</v>
-      </c>
-      <c r="F25" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="D25" s="21" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E25" s="21" t="n">
+        <v>46302</v>
+      </c>
+      <c r="F25" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="G25" s="30" t="inlineStr">
         <is>
           <t>20C</t>
         </is>
       </c>
-      <c r="H25" s="11" t="n">
-        <v>46302.58333333334</v>
-      </c>
-      <c r="I25" s="11" t="n">
-        <v>46303.58333333334</v>
-      </c>
-      <c r="J25" s="11" t="n">
-        <v>46304.58333333334</v>
-      </c>
-      <c r="K25" s="28">
+      <c r="H25" s="31" t="n">
+        <v>46300</v>
+      </c>
+      <c r="I25" s="31" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="J25" s="31" t="n">
+        <v>46302.45833333334</v>
+      </c>
+      <c r="K25" s="32">
         <f>(J25-I25)*24</f>
         <v/>
       </c>
-      <c r="L25" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M25" s="23" t="inlineStr"/>
-      <c r="N25" s="23">
-        <f>IF(J25&lt;=$B$3,"Sailed",IF(I25&lt;=$B$3,"Alongside",IF(H25&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="L25" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M25" s="24" t="inlineStr"/>
+      <c r="N25" s="24" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -7743,34 +8843,34 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>YM INCEPTION</t>
+          <t>JOSCO LUCKY</t>
         </is>
       </c>
       <c r="C26" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D26" s="10" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="E26" s="10" t="n">
         <v>46303</v>
       </c>
       <c r="F26" s="23" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20C</t>
+          <t>20B → 20AB → 20D → 20C</t>
         </is>
       </c>
       <c r="H26" s="11" t="n">
+        <v>46301.875</v>
+      </c>
+      <c r="I26" s="11" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="J26" s="11" t="n">
         <v>46303.54166666666</v>
-      </c>
-      <c r="I26" s="11" t="n">
-        <v>46304.54166666666</v>
-      </c>
-      <c r="J26" s="11" t="n">
-        <v>46306.04166666666</v>
       </c>
       <c r="K26" s="28">
         <f>(J26-I26)*24</f>
@@ -7782,9 +8882,10 @@
         </is>
       </c>
       <c r="M26" s="23" t="inlineStr"/>
-      <c r="N26" s="23">
-        <f>IF(J26&lt;=$B$3,"Sailed",IF(I26&lt;=$B$3,"Alongside",IF(H26&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N26" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -7795,20 +8896,20 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>STARSHIP AQUILA</t>
+          <t>ZHONG GU DONG HAI</t>
         </is>
       </c>
       <c r="C27" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D27" s="10" t="n">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E27" s="10" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="F27" s="23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
@@ -7816,13 +8917,13 @@
         </is>
       </c>
       <c r="H27" s="11" t="n">
-        <v>46304.91666666666</v>
+        <v>46302.58333333334</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>46306.16666666666</v>
+        <v>46303.58333333334</v>
       </c>
       <c r="J27" s="11" t="n">
-        <v>46307.54166666666</v>
+        <v>46304.58333333334</v>
       </c>
       <c r="K27" s="28">
         <f>(J27-I27)*24</f>
@@ -7840,151 +8941,145 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="29" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="B28" s="29" t="inlineStr">
-        <is>
-          <t>BANGKOK</t>
-        </is>
-      </c>
-      <c r="C28" s="24" t="n">
-        <v>551</v>
-      </c>
-      <c r="D28" s="21" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E28" s="21" t="n">
-        <v>46294</v>
-      </c>
-      <c r="F28" s="24" t="n">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>YM INCEPTION</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D28" s="10" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E28" s="10" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F28" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20C</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="I28" s="11" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="J28" s="11" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="K28" s="28">
+        <f>(J28-I28)*24</f>
+        <v/>
+      </c>
+      <c r="L28" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M28" s="23" t="inlineStr"/>
+      <c r="N28" s="23">
+        <f>IF(J28&lt;=$B$3,"Sailed",IF(I28&lt;=$B$3,"Alongside",IF(H28&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>STARSHIP AQUILA</t>
+        </is>
+      </c>
+      <c r="C29" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D29" s="10" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E29" s="10" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F29" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="30" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="H28" s="31" t="n">
-        <v>46292.54166666666</v>
-      </c>
-      <c r="I28" s="31" t="n">
-        <v>46292.625</v>
-      </c>
-      <c r="J28" s="31" t="n">
-        <v>46294.58333333334</v>
-      </c>
-      <c r="K28" s="32">
-        <f>(J28-I28)*24</f>
-        <v/>
-      </c>
-      <c r="L28" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M28" s="24" t="inlineStr"/>
-      <c r="N28" s="24" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="33" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="B29" s="33" t="inlineStr">
-        <is>
-          <t>ALS SUMIRE</t>
-        </is>
-      </c>
-      <c r="C29" s="17" t="n">
-        <v>537</v>
-      </c>
-      <c r="D29" s="18" t="n">
-        <v>46294</v>
-      </c>
-      <c r="E29" s="18" t="n">
-        <v>46297</v>
-      </c>
-      <c r="F29" s="17" t="n">
-        <v>4</v>
-      </c>
-      <c r="G29" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20D</t>
-        </is>
-      </c>
-      <c r="H29" s="25" t="n">
-        <v>46296.25</v>
-      </c>
-      <c r="I29" s="25" t="n">
-        <v>46296.66666666666</v>
-      </c>
-      <c r="J29" s="25" t="n">
-        <v>46297.70833333334</v>
-      </c>
-      <c r="K29" s="34">
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="H29" s="11" t="n">
+        <v>46304.91666666666</v>
+      </c>
+      <c r="I29" s="11" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="J29" s="11" t="n">
+        <v>46307.20833333334</v>
+      </c>
+      <c r="K29" s="28">
         <f>(J29-I29)*24</f>
         <v/>
       </c>
-      <c r="L29" s="17" t="inlineStr">
-        <is>
-          <t>1C</t>
-        </is>
-      </c>
-      <c r="M29" s="17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N29" s="17" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="L29" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M29" s="23" t="inlineStr"/>
+      <c r="N29" s="23">
+        <f>IF(J29&lt;=$B$3,"Sailed",IF(I29&lt;=$B$3,"Alongside",IF(H29&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>20D</t>
+          <t>20C</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>HARI BHUM (Barge)</t>
+          <t>ALS SUMIRE</t>
         </is>
       </c>
       <c r="C30" s="23" t="n">
-        <v>259</v>
+        <v>537</v>
       </c>
       <c r="D30" s="10" t="n">
-        <v>46297</v>
+        <v>46294</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>46298</v>
+        <v>46304</v>
       </c>
       <c r="F30" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G30" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
+        <v>5</v>
+      </c>
+      <c r="G30" s="6" t="inlineStr">
+        <is>
+          <t>20F → 20D → 20C</t>
         </is>
       </c>
       <c r="H30" s="11" t="n">
-        <v>46298.20833333334</v>
+        <v>46307.75</v>
       </c>
       <c r="I30" s="11" t="n">
-        <v>46298.29166666666</v>
+        <v>46307.75</v>
       </c>
       <c r="J30" s="11" t="n">
-        <v>46298.66666666666</v>
+        <v>46309.20833333334</v>
       </c>
       <c r="K30" s="28">
         <f>(J30-I30)*24</f>
@@ -7992,66 +9087,66 @@
       </c>
       <c r="L30" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>1C</t>
         </is>
       </c>
       <c r="M30" s="23" t="inlineStr"/>
-      <c r="N30" s="23" t="inlineStr">
+      <c r="N30" s="23">
+        <f>IF(J30&lt;=$B$3,"Sailed",IF(I30&lt;=$B$3,"Alongside",IF(H30&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="29" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B31" s="29" t="inlineStr">
+        <is>
+          <t>BANGKOK</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="n">
+        <v>551</v>
+      </c>
+      <c r="D31" s="21" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E31" s="21" t="n">
+        <v>46294</v>
+      </c>
+      <c r="F31" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" s="30" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="H31" s="31" t="n">
+        <v>46292.54166666666</v>
+      </c>
+      <c r="I31" s="31" t="n">
+        <v>46292.625</v>
+      </c>
+      <c r="J31" s="31" t="n">
+        <v>46294.58333333334</v>
+      </c>
+      <c r="K31" s="32">
+        <f>(J31-I31)*24</f>
+        <v/>
+      </c>
+      <c r="L31" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M31" s="24" t="inlineStr"/>
+      <c r="N31" s="24" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>MTT BANGKOK</t>
-        </is>
-      </c>
-      <c r="C31" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D31" s="10" t="n">
-        <v>46300</v>
-      </c>
-      <c r="E31" s="10" t="n">
-        <v>46303</v>
-      </c>
-      <c r="F31" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="H31" s="11" t="n">
-        <v>46302.54166666666</v>
-      </c>
-      <c r="I31" s="11" t="n">
-        <v>46302.58333333334</v>
-      </c>
-      <c r="J31" s="11" t="n">
-        <v>46304.08333333334</v>
-      </c>
-      <c r="K31" s="28">
-        <f>(J31-I31)*24</f>
-        <v/>
-      </c>
-      <c r="L31" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M31" s="23" t="inlineStr"/>
-      <c r="N31" s="23">
-        <f>IF(J31&lt;=$B$3,"Sailed",IF(I31&lt;=$B$3,"Alongside",IF(H31&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
       </c>
     </row>
     <row r="32">
@@ -8062,34 +9157,34 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>HE JIN</t>
+          <t>HARI BHUM (Barge)</t>
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>552</v>
+        <v>259</v>
       </c>
       <c r="D32" s="10" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>46303</v>
+        <v>46298</v>
       </c>
       <c r="F32" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 22A → 20D</t>
+        <v>2</v>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H32" s="11" t="n">
-        <v>46304.08333333334</v>
+        <v>46298.20833333334</v>
       </c>
       <c r="I32" s="11" t="n">
-        <v>46304.08333333334</v>
+        <v>46298.29166666666</v>
       </c>
       <c r="J32" s="11" t="n">
-        <v>46305.54166666666</v>
+        <v>46298.66666666666</v>
       </c>
       <c r="K32" s="28">
         <f>(J32-I32)*24</f>
@@ -8101,9 +9196,10 @@
         </is>
       </c>
       <c r="M32" s="23" t="inlineStr"/>
-      <c r="N32" s="23">
-        <f>IF(J32&lt;=$B$3,"Sailed",IF(I32&lt;=$B$3,"Alongside",IF(H32&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N32" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -8114,34 +9210,34 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>CUL HAIPHONG</t>
+          <t>MTT BANGKOK</t>
         </is>
       </c>
       <c r="C33" s="23" t="n">
-        <v>458</v>
+        <v>564</v>
       </c>
       <c r="D33" s="10" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="E33" s="10" t="n">
         <v>46303</v>
       </c>
       <c r="F33" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20D</t>
+        <v>4</v>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H33" s="11" t="n">
-        <v>46304.83333333334</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="I33" s="11" t="n">
-        <v>46305.66666666666</v>
+        <v>46302.58333333334</v>
       </c>
       <c r="J33" s="11" t="n">
-        <v>46306.25</v>
+        <v>46304.08333333334</v>
       </c>
       <c r="K33" s="28">
         <f>(J33-I33)*24</f>
@@ -8149,13 +9245,14 @@
       </c>
       <c r="L33" s="23" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>–</t>
         </is>
       </c>
       <c r="M33" s="23" t="inlineStr"/>
-      <c r="N33" s="23">
-        <f>IF(J33&lt;=$B$3,"Sailed",IF(I33&lt;=$B$3,"Alongside",IF(H33&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N33" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="34">
@@ -8166,34 +9263,34 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>INCEDA</t>
+          <t>HE JIN</t>
         </is>
       </c>
       <c r="C34" s="23" t="n">
-        <v>564</v>
+        <v>552</v>
       </c>
       <c r="D34" s="10" t="n">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E34" s="10" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="F34" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
+        <v>4</v>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20AB → 22A → 20D</t>
         </is>
       </c>
       <c r="H34" s="11" t="n">
-        <v>46305.70833333334</v>
+        <v>46304</v>
       </c>
       <c r="I34" s="11" t="n">
-        <v>46306.20833333334</v>
+        <v>46304</v>
       </c>
       <c r="J34" s="11" t="n">
-        <v>46307.58333333334</v>
+        <v>46305.54166666666</v>
       </c>
       <c r="K34" s="28">
         <f>(J34-I34)*24</f>
@@ -8211,94 +9308,93 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="29" t="inlineStr">
-        <is>
-          <t>20E</t>
-        </is>
-      </c>
-      <c r="B35" s="29" t="inlineStr">
-        <is>
-          <t>TS CHIBA</t>
-        </is>
-      </c>
-      <c r="C35" s="24" t="n">
-        <v>485</v>
-      </c>
-      <c r="D35" s="21" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E35" s="21" t="n">
-        <v>46293</v>
-      </c>
-      <c r="F35" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" s="30" t="inlineStr">
-        <is>
-          <t>20E</t>
-        </is>
-      </c>
-      <c r="H35" s="31" t="n">
-        <v>46293.29166666666</v>
-      </c>
-      <c r="I35" s="31" t="n">
-        <v>46293.29166666666</v>
-      </c>
-      <c r="J35" s="31" t="n">
-        <v>46294.16666666666</v>
-      </c>
-      <c r="K35" s="32">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>CUL HAIPHONG</t>
+        </is>
+      </c>
+      <c r="C35" s="23" t="n">
+        <v>458</v>
+      </c>
+      <c r="D35" s="10" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E35" s="10" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F35" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20D</t>
+        </is>
+      </c>
+      <c r="H35" s="11" t="n">
+        <v>46304.83333333334</v>
+      </c>
+      <c r="I35" s="11" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="J35" s="11" t="n">
+        <v>46306.25</v>
+      </c>
+      <c r="K35" s="28">
         <f>(J35-I35)*24</f>
         <v/>
       </c>
-      <c r="L35" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M35" s="24" t="inlineStr"/>
-      <c r="N35" s="24" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="L35" s="23" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="M35" s="23" t="inlineStr"/>
+      <c r="N35" s="23">
+        <f>IF(J35&lt;=$B$3,"Sailed",IF(I35&lt;=$B$3,"Alongside",IF(H35&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>20E</t>
+          <t>20D</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>MITRA BHUM</t>
+          <t>INCEDA</t>
         </is>
       </c>
       <c r="C36" s="23" t="n">
-        <v>485</v>
+        <v>564</v>
       </c>
       <c r="D36" s="10" t="n">
-        <v>46293</v>
+        <v>46303</v>
       </c>
       <c r="E36" s="10" t="n">
-        <v>46295</v>
+        <v>46304</v>
       </c>
       <c r="F36" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G36" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20E</t>
+        <v>2</v>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H36" s="11" t="n">
-        <v>46295.125</v>
+        <v>46305.70833333334</v>
       </c>
       <c r="I36" s="11" t="n">
-        <v>46295.20833333334</v>
+        <v>46306.20833333334</v>
       </c>
       <c r="J36" s="11" t="n">
-        <v>46295.75</v>
+        <v>46307.58333333334</v>
       </c>
       <c r="K36" s="28">
         <f>(J36-I36)*24</f>
@@ -8310,48 +9406,47 @@
         </is>
       </c>
       <c r="M36" s="23" t="inlineStr"/>
-      <c r="N36" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="N36" s="23">
+        <f>IF(J36&lt;=$B$3,"Sailed",IF(I36&lt;=$B$3,"Alongside",IF(H36&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>20E</t>
+          <t>20D</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 278</t>
+          <t>KMTC TAIPEIS</t>
         </is>
       </c>
       <c r="C37" s="23" t="n">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>46295</v>
+        <v>46304</v>
       </c>
       <c r="E37" s="10" t="n">
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="F37" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20E</t>
+        <v>1</v>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H37" s="11" t="n">
-        <v>46297.75</v>
+        <v>46307.95833333334</v>
       </c>
       <c r="I37" s="11" t="n">
-        <v>46298.41666666666</v>
+        <v>46308.20833333334</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>46300.45833333334</v>
+        <v>46309.625</v>
       </c>
       <c r="K37" s="28">
         <f>(J37-I37)*24</f>
@@ -8363,64 +9458,59 @@
         </is>
       </c>
       <c r="M37" s="23" t="inlineStr"/>
-      <c r="N37" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="N37" s="23">
+        <f>IF(J37&lt;=$B$3,"Sailed",IF(I37&lt;=$B$3,"Alongside",IF(H37&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="35" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="B38" s="35" t="inlineStr">
-        <is>
-          <t>JARU BHUM</t>
-        </is>
-      </c>
-      <c r="C38" s="22" t="n">
-        <v>564</v>
-      </c>
-      <c r="D38" s="14" t="n">
+      <c r="A38" s="29" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B38" s="29" t="inlineStr">
+        <is>
+          <t>TS CHIBA</t>
+        </is>
+      </c>
+      <c r="C38" s="24" t="n">
+        <v>485</v>
+      </c>
+      <c r="D38" s="21" t="n">
         <v>46293</v>
       </c>
-      <c r="E38" s="14" t="n">
+      <c r="E38" s="21" t="n">
         <v>46293</v>
       </c>
-      <c r="F38" s="22" t="n">
+      <c r="F38" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="G38" s="36" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="H38" s="37" t="n">
-        <v>46293.33333333334</v>
-      </c>
-      <c r="I38" s="37" t="n">
-        <v>46293.33333333334</v>
-      </c>
-      <c r="J38" s="37" t="n">
+      <c r="G38" s="30" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="H38" s="31" t="n">
+        <v>46293.29166666666</v>
+      </c>
+      <c r="I38" s="31" t="n">
+        <v>46293.29166666666</v>
+      </c>
+      <c r="J38" s="31" t="n">
         <v>46294.16666666666</v>
       </c>
-      <c r="K38" s="38">
+      <c r="K38" s="32">
         <f>(J38-I38)*24</f>
         <v/>
       </c>
-      <c r="L38" s="22" t="inlineStr">
-        <is>
-          <t>7B</t>
-        </is>
-      </c>
-      <c r="M38" s="22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N38" s="22" t="inlineStr">
+      <c r="L38" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M38" s="24" t="inlineStr"/>
+      <c r="N38" s="24" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -8429,16 +9519,16 @@
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>20F</t>
+          <t>20E</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>HOPE C</t>
+          <t>MITRA BHUM</t>
         </is>
       </c>
       <c r="C39" s="23" t="n">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="D39" s="10" t="n">
         <v>46293</v>
@@ -8451,17 +9541,17 @@
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>20E → 20F</t>
+          <t>20F → 20E</t>
         </is>
       </c>
       <c r="H39" s="11" t="n">
-        <v>46294.70833333334</v>
+        <v>46295.125</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>46294.70833333334</v>
+        <v>46295.20833333334</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>46295.66666666666</v>
+        <v>46295.75</v>
       </c>
       <c r="K39" s="28">
         <f>(J39-I39)*24</f>
@@ -8482,12 +9572,12 @@
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>20F</t>
+          <t>20E</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>KMTC BANGKOK</t>
+          <t>WAN HAI 278</t>
         </is>
       </c>
       <c r="C40" s="23" t="n">
@@ -8497,24 +9587,24 @@
         <v>46295</v>
       </c>
       <c r="E40" s="10" t="n">
-        <v>46298</v>
+        <v>46300</v>
       </c>
       <c r="F40" s="23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20F</t>
+          <t>20F → 20E</t>
         </is>
       </c>
       <c r="H40" s="11" t="n">
-        <v>46297.29166666666</v>
+        <v>46297.75</v>
       </c>
       <c r="I40" s="11" t="n">
-        <v>46297.45833333334</v>
+        <v>46298.41666666666</v>
       </c>
       <c r="J40" s="11" t="n">
-        <v>46298.70833333334</v>
+        <v>46300.45833333334</v>
       </c>
       <c r="K40" s="28">
         <f>(J40-I40)*24</f>
@@ -8533,53 +9623,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="A41" s="35" t="inlineStr">
         <is>
           <t>20F</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>XIN MING ZHOU 98</t>
-        </is>
-      </c>
-      <c r="C41" s="23" t="n">
+      <c r="B41" s="35" t="inlineStr">
+        <is>
+          <t>JARU BHUM</t>
+        </is>
+      </c>
+      <c r="C41" s="22" t="n">
         <v>564</v>
       </c>
-      <c r="D41" s="10" t="n">
-        <v>46297</v>
-      </c>
-      <c r="E41" s="10" t="n">
-        <v>46299</v>
-      </c>
-      <c r="F41" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
+      <c r="D41" s="14" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E41" s="14" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F41" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="36" t="inlineStr">
         <is>
           <t>20F</t>
         </is>
       </c>
-      <c r="H41" s="11" t="n">
-        <v>46299.375</v>
-      </c>
-      <c r="I41" s="11" t="n">
-        <v>46299.375</v>
-      </c>
-      <c r="J41" s="11" t="n">
-        <v>46300.375</v>
-      </c>
-      <c r="K41" s="28">
+      <c r="H41" s="37" t="n">
+        <v>46293.33333333334</v>
+      </c>
+      <c r="I41" s="37" t="n">
+        <v>46293.33333333334</v>
+      </c>
+      <c r="J41" s="37" t="n">
+        <v>46294.16666666666</v>
+      </c>
+      <c r="K41" s="38">
         <f>(J41-I41)*24</f>
         <v/>
       </c>
-      <c r="L41" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M41" s="23" t="inlineStr"/>
-      <c r="N41" s="23" t="inlineStr">
+      <c r="L41" s="22" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="M41" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N41" s="22" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -8593,34 +9687,34 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>XIN AN</t>
+          <t>HOPE C</t>
         </is>
       </c>
       <c r="C42" s="23" t="n">
-        <v>564</v>
+        <v>481</v>
       </c>
       <c r="D42" s="10" t="n">
-        <v>46300</v>
+        <v>46293</v>
       </c>
       <c r="E42" s="10" t="n">
-        <v>46303</v>
+        <v>46295</v>
       </c>
       <c r="F42" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G42" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+        <v>3</v>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>20E → 20F</t>
         </is>
       </c>
       <c r="H42" s="11" t="n">
-        <v>46302.54166666666</v>
+        <v>46294.70833333334</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>46302.58333333334</v>
+        <v>46294.70833333334</v>
       </c>
       <c r="J42" s="11" t="n">
-        <v>46304.54166666666</v>
+        <v>46295.66666666666</v>
       </c>
       <c r="K42" s="28">
         <f>(J42-I42)*24</f>
@@ -8632,9 +9726,10 @@
         </is>
       </c>
       <c r="M42" s="23" t="inlineStr"/>
-      <c r="N42" s="23">
-        <f>IF(J42&lt;=$B$3,"Sailed",IF(I42&lt;=$B$3,"Alongside",IF(H42&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N42" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -8645,34 +9740,34 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE ATLANTIC</t>
+          <t>KMTC BANGKOK</t>
         </is>
       </c>
       <c r="C43" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>46300</v>
+        <v>46295</v>
       </c>
       <c r="E43" s="10" t="n">
-        <v>46303</v>
+        <v>46298</v>
       </c>
       <c r="F43" s="23" t="n">
         <v>4</v>
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>20C → 20D → 20F</t>
+          <t>20AB → 20F</t>
         </is>
       </c>
       <c r="H43" s="11" t="n">
-        <v>46302.83333333334</v>
+        <v>46297.29166666666</v>
       </c>
       <c r="I43" s="11" t="n">
-        <v>46304.625</v>
+        <v>46297.45833333334</v>
       </c>
       <c r="J43" s="11" t="n">
-        <v>46306.125</v>
+        <v>46298.70833333334</v>
       </c>
       <c r="K43" s="28">
         <f>(J43-I43)*24</f>
@@ -8684,9 +9779,10 @@
         </is>
       </c>
       <c r="M43" s="23" t="inlineStr"/>
-      <c r="N43" s="23">
-        <f>IF(J43&lt;=$B$3,"Sailed",IF(I43&lt;=$B$3,"Alongside",IF(H43&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N43" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -8697,20 +9793,20 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 102</t>
+          <t>XIN MING ZHOU 98</t>
         </is>
       </c>
       <c r="C44" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D44" s="10" t="n">
-        <v>46302</v>
+        <v>46297</v>
       </c>
       <c r="E44" s="10" t="n">
-        <v>46303</v>
+        <v>46299</v>
       </c>
       <c r="F44" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
@@ -8718,13 +9814,13 @@
         </is>
       </c>
       <c r="H44" s="11" t="n">
-        <v>46305.875</v>
+        <v>46299.375</v>
       </c>
       <c r="I44" s="11" t="n">
-        <v>46306.20833333334</v>
+        <v>46299.375</v>
       </c>
       <c r="J44" s="11" t="n">
-        <v>46307.08333333334</v>
+        <v>46300.375</v>
       </c>
       <c r="K44" s="28">
         <f>(J44-I44)*24</f>
@@ -8736,20 +9832,229 @@
         </is>
       </c>
       <c r="M44" s="23" t="inlineStr"/>
-      <c r="N44" s="23">
-        <f>IF(J44&lt;=$B$3,"Sailed",IF(I44&lt;=$B$3,"Alongside",IF(H44&lt;=$B$3,"At anchorage","Expected")))</f>
+      <c r="N44" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>XIN AN</t>
+        </is>
+      </c>
+      <c r="C45" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D45" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E45" s="10" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F45" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="H45" s="11" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="I45" s="11" t="n">
+        <v>46302.58333333334</v>
+      </c>
+      <c r="J45" s="11" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="K45" s="28">
+        <f>(J45-I45)*24</f>
+        <v/>
+      </c>
+      <c r="L45" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M45" s="23" t="inlineStr"/>
+      <c r="N45" s="23">
+        <f>IF(J45&lt;=$B$3,"Sailed",IF(I45&lt;=$B$3,"Alongside",IF(H45&lt;=$B$3,"At anchorage","Expected")))</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>39 vessels in total. Orange cells: marked on sheet, or the vessel changed berth.</t>
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>SAWASDEE ATLANTIC</t>
+        </is>
+      </c>
+      <c r="C46" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D46" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E46" s="10" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F46" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G46" s="6" t="inlineStr">
+        <is>
+          <t>20C → 20D → 20F</t>
+        </is>
+      </c>
+      <c r="H46" s="11" t="n">
+        <v>46302.83333333334</v>
+      </c>
+      <c r="I46" s="11" t="n">
+        <v>46304.625</v>
+      </c>
+      <c r="J46" s="11" t="n">
+        <v>46306.125</v>
+      </c>
+      <c r="K46" s="28">
+        <f>(J46-I46)*24</f>
+        <v/>
+      </c>
+      <c r="L46" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M46" s="23" t="inlineStr"/>
+      <c r="N46" s="23">
+        <f>IF(J46&lt;=$B$3,"Sailed",IF(I46&lt;=$B$3,"Alongside",IF(H46&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 102</t>
+        </is>
+      </c>
+      <c r="C47" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D47" s="10" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E47" s="10" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F47" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="H47" s="11" t="n">
+        <v>46305.875</v>
+      </c>
+      <c r="I47" s="11" t="n">
+        <v>46306.20833333334</v>
+      </c>
+      <c r="J47" s="11" t="n">
+        <v>46307.08333333334</v>
+      </c>
+      <c r="K47" s="28">
+        <f>(J47-I47)*24</f>
+        <v/>
+      </c>
+      <c r="L47" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M47" s="23" t="inlineStr"/>
+      <c r="N47" s="23">
+        <f>IF(J47&lt;=$B$3,"Sailed",IF(I47&lt;=$B$3,"Alongside",IF(H47&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>SAWASDEE SUNRISE</t>
+        </is>
+      </c>
+      <c r="C48" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D48" s="10" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E48" s="10" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F48" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="H48" s="11" t="n">
+        <v>46307.20833333334</v>
+      </c>
+      <c r="I48" s="11" t="n">
+        <v>46307.20833333334</v>
+      </c>
+      <c r="J48" s="11" t="n">
+        <v>46308.625</v>
+      </c>
+      <c r="K48" s="28">
+        <f>(J48-I48)*24</f>
+        <v/>
+      </c>
+      <c r="L48" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M48" s="23" t="inlineStr"/>
+      <c r="N48" s="23">
+        <f>IF(J48&lt;=$B$3,"Sailed",IF(I48&lt;=$B$3,"Alongside",IF(H48&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>43 vessels in total. Orange cells: marked on sheet, or the vessel changed berth.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:N44"/>
+  <autoFilter ref="A5:N48"/>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add 10 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -22,10 +22,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 Oct 2026" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Oct 2026" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Oct 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Oct 2026" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$N$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$N$50</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -669,7 +670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:N49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -685,6 +686,7 @@
     <col width="44" customWidth="1" min="11" max="11"/>
     <col width="44" customWidth="1" min="12" max="12"/>
     <col width="44" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -765,6 +767,11 @@
       <c r="M4" s="3" t="inlineStr">
         <is>
           <t>09 Oct 2026</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>10 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -798,6 +805,7 @@
       <c r="K5" s="5" t="inlineStr"/>
       <c r="L5" s="5" t="inlineStr"/>
       <c r="M5" s="5" t="inlineStr"/>
+      <c r="N5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -833,6 +841,7 @@
       <c r="K6" s="5" t="inlineStr"/>
       <c r="L6" s="5" t="inlineStr"/>
       <c r="M6" s="5" t="inlineStr"/>
+      <c r="N6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -860,6 +869,7 @@
       <c r="K7" s="5" t="inlineStr"/>
       <c r="L7" s="5" t="inlineStr"/>
       <c r="M7" s="5" t="inlineStr"/>
+      <c r="N7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -891,6 +901,7 @@
       <c r="K8" s="5" t="inlineStr"/>
       <c r="L8" s="5" t="inlineStr"/>
       <c r="M8" s="5" t="inlineStr"/>
+      <c r="N8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -922,6 +933,7 @@
       <c r="K9" s="5" t="inlineStr"/>
       <c r="L9" s="5" t="inlineStr"/>
       <c r="M9" s="5" t="inlineStr"/>
+      <c r="N9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -949,6 +961,7 @@
       <c r="K10" s="5" t="inlineStr"/>
       <c r="L10" s="5" t="inlineStr"/>
       <c r="M10" s="5" t="inlineStr"/>
+      <c r="N10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -984,6 +997,7 @@
       <c r="K11" s="5" t="inlineStr"/>
       <c r="L11" s="5" t="inlineStr"/>
       <c r="M11" s="5" t="inlineStr"/>
+      <c r="N11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1011,6 +1025,7 @@
       <c r="K12" s="5" t="inlineStr"/>
       <c r="L12" s="5" t="inlineStr"/>
       <c r="M12" s="5" t="inlineStr"/>
+      <c r="N12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1046,6 +1061,7 @@
       <c r="K13" s="5" t="inlineStr"/>
       <c r="L13" s="5" t="inlineStr"/>
       <c r="M13" s="5" t="inlineStr"/>
+      <c r="N13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1089,6 +1105,7 @@
       <c r="K14" s="5" t="inlineStr"/>
       <c r="L14" s="5" t="inlineStr"/>
       <c r="M14" s="5" t="inlineStr"/>
+      <c r="N14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1124,6 +1141,7 @@
       <c r="K15" s="5" t="inlineStr"/>
       <c r="L15" s="5" t="inlineStr"/>
       <c r="M15" s="5" t="inlineStr"/>
+      <c r="N15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1163,6 +1181,7 @@
       <c r="K16" s="5" t="inlineStr"/>
       <c r="L16" s="5" t="inlineStr"/>
       <c r="M16" s="5" t="inlineStr"/>
+      <c r="N16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1206,6 +1225,11 @@
           <t>expected → 20C (returns for a new call, ETA 12/18, shift 1C)</t>
         </is>
       </c>
+      <c r="N17" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20B (marked, 1C; ETA 12/18→12/22, ETD 14/05→14/06)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1245,6 +1269,7 @@
       <c r="K18" s="5" t="inlineStr"/>
       <c r="L18" s="5" t="inlineStr"/>
       <c r="M18" s="5" t="inlineStr"/>
+      <c r="N18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1292,6 +1317,7 @@
       <c r="K19" s="5" t="inlineStr"/>
       <c r="L19" s="5" t="inlineStr"/>
       <c r="M19" s="5" t="inlineStr"/>
+      <c r="N19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1339,6 +1365,7 @@
       </c>
       <c r="L20" s="5" t="inlineStr"/>
       <c r="M20" s="5" t="inlineStr"/>
+      <c r="N20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1382,6 +1409,7 @@
       <c r="K21" s="5" t="inlineStr"/>
       <c r="L21" s="5" t="inlineStr"/>
       <c r="M21" s="5" t="inlineStr"/>
+      <c r="N21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1421,6 +1449,7 @@
       <c r="K22" s="5" t="inlineStr"/>
       <c r="L22" s="5" t="inlineStr"/>
       <c r="M22" s="5" t="inlineStr"/>
+      <c r="N22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1472,6 +1501,7 @@
           <t>sailed (08/13)</t>
         </is>
       </c>
+      <c r="N23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1519,6 +1549,7 @@
         </is>
       </c>
       <c r="M24" s="5" t="inlineStr"/>
+      <c r="N24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1550,6 +1581,7 @@
       <c r="K25" s="5" t="inlineStr"/>
       <c r="L25" s="5" t="inlineStr"/>
       <c r="M25" s="5" t="inlineStr"/>
+      <c r="N25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1585,6 +1617,7 @@
       <c r="K26" s="5" t="inlineStr"/>
       <c r="L26" s="5" t="inlineStr"/>
       <c r="M26" s="5" t="inlineStr"/>
+      <c r="N26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1632,6 +1665,7 @@
           <t>sailed (08/13)</t>
         </is>
       </c>
+      <c r="N27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1675,6 +1709,7 @@
           <t>sailed (08/12)</t>
         </is>
       </c>
+      <c r="N28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1714,6 +1749,11 @@
           <t>alongside · 20AB (P.B 08/13→08/14, ETD 09/14→09/16)</t>
         </is>
       </c>
+      <c r="N29" s="5" t="inlineStr">
+        <is>
+          <t>sailed (09/16)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1753,6 +1793,11 @@
           <t>at anchorage · 20F (P.B 09/15)</t>
         </is>
       </c>
+      <c r="N30" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20F (ETD 11/03→11/13)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1792,6 +1837,7 @@
           <t>sailed (09/02)</t>
         </is>
       </c>
+      <c r="N31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1829,6 +1875,11 @@
       <c r="M32" s="5" t="inlineStr">
         <is>
           <t>alongside · 20F (ETD 09/13)</t>
+        </is>
+      </c>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t>sailed (09/13)</t>
         </is>
       </c>
     </row>
@@ -1866,6 +1917,11 @@
           <t>alongside · 20B (ETD 09/17)</t>
         </is>
       </c>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>sailed (09/17)</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -1901,6 +1957,11 @@
           <t>at anchorage · 20C (ETD 11/01→10/16)</t>
         </is>
       </c>
+      <c r="N34" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20C (marked, ETD 10/16→10/14)</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -1936,6 +1997,11 @@
           <t>alongside · 20D (shifted in from 22A, P.B 09/02→08/24)</t>
         </is>
       </c>
+      <c r="N35" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20D (ETD 10/13)</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -1971,6 +2037,11 @@
           <t>alongside · 20C (ETD 09/14)</t>
         </is>
       </c>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t>sailed (09/14)</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2004,6 +2075,11 @@
       <c r="M37" s="6" t="inlineStr">
         <is>
           <t>at anchorage · 20AB (ETA 08/18→08/16)</t>
+        </is>
+      </c>
+      <c r="N37" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20AB (ETD 10/15)</t>
         </is>
       </c>
     </row>
@@ -2037,6 +2113,11 @@
           <t>expected · 20AB</t>
         </is>
       </c>
+      <c r="N38" s="5" t="inlineStr">
+        <is>
+          <t>at anchorage · 20AB (P.B 10/15)</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2068,6 +2149,11 @@
           <t>at anchorage · 20B (ETA 09/09→09/06)</t>
         </is>
       </c>
+      <c r="N39" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20B (ETD 11/14→11/04)</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -2099,6 +2185,11 @@
           <t>expected · 20D (ETA 09/20)</t>
         </is>
       </c>
+      <c r="N40" s="5" t="inlineStr">
+        <is>
+          <t>at anchorage · 20D (P.B 10/16)</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2128,6 +2219,11 @@
       <c r="M41" s="5" t="inlineStr">
         <is>
           <t>expected · 20F</t>
+        </is>
+      </c>
+      <c r="N41" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20B (marked)</t>
         </is>
       </c>
     </row>
@@ -2157,6 +2253,11 @@
           <t>expected · 20C (P.B 11/04→10/16, ETD 12/13→12/05)</t>
         </is>
       </c>
+      <c r="N42" s="6" t="inlineStr">
+        <is>
+          <t>at anchorage · 20C (marked, P.B 10/16→10/14, ETD 12/05→12/02)</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2180,6 +2281,11 @@
         </is>
       </c>
       <c r="M43" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D</t>
+        </is>
+      </c>
+      <c r="N43" s="5" t="inlineStr">
         <is>
           <t>expected · 20D</t>
         </is>
@@ -2207,6 +2313,11 @@
           <t>expected · 20AB (new)</t>
         </is>
       </c>
+      <c r="N44" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20F (marked, ETA 12/04→12/01, P.B 12/05→12/06)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -2230,6 +2341,11 @@
           <t>expected · 20B (new)</t>
         </is>
       </c>
+      <c r="N45" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20AB (ETA 11/17→12/13, P.B 11/17→12/16)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -2253,6 +2369,11 @@
           <t>expected · 20D (new)</t>
         </is>
       </c>
+      <c r="N46" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20C</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -2274,6 +2395,59 @@
       <c r="M47" s="5" t="inlineStr">
         <is>
           <t>expected · 20F (new)</t>
+        </is>
+      </c>
+      <c r="N47" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20D (ETA 12/05→12/09, P.B 12/05→12/16, ETD 13/15→14/05)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
+        <is>
+          <t>KHUNA BHUM</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr"/>
+      <c r="C48" s="5" t="inlineStr"/>
+      <c r="D48" s="5" t="inlineStr"/>
+      <c r="E48" s="5" t="inlineStr"/>
+      <c r="F48" s="5" t="inlineStr"/>
+      <c r="G48" s="5" t="inlineStr"/>
+      <c r="H48" s="5" t="inlineStr"/>
+      <c r="I48" s="5" t="inlineStr"/>
+      <c r="J48" s="5" t="inlineStr"/>
+      <c r="K48" s="5" t="inlineStr"/>
+      <c r="L48" s="5" t="inlineStr"/>
+      <c r="M48" s="5" t="inlineStr"/>
+      <c r="N48" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20AB (new, shift 7B)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>WAN HAI 277</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr"/>
+      <c r="C49" s="5" t="inlineStr"/>
+      <c r="D49" s="5" t="inlineStr"/>
+      <c r="E49" s="5" t="inlineStr"/>
+      <c r="F49" s="5" t="inlineStr"/>
+      <c r="G49" s="5" t="inlineStr"/>
+      <c r="H49" s="5" t="inlineStr"/>
+      <c r="I49" s="5" t="inlineStr"/>
+      <c r="J49" s="5" t="inlineStr"/>
+      <c r="K49" s="5" t="inlineStr"/>
+      <c r="L49" s="5" t="inlineStr"/>
+      <c r="M49" s="5" t="inlineStr"/>
+      <c r="N49" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20F (new, marked)</t>
         </is>
       </c>
     </row>
@@ -6438,13 +6612,791 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 10 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>KANWAY FORTUNE</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>46303.66666666666</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>46305.625</v>
+      </c>
+      <c r="G4" s="28">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>CNC MARS</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46304.91666666666</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46305.625</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46306.625</v>
+      </c>
+      <c r="G5" s="28">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>JOSCO SHINE</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46307.54166666666</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46307.66666666666</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46308.58333333334</v>
+      </c>
+      <c r="G6" s="28">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>KHUNA BHUM</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46308.29166666666</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46308.54166666666</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46309.29166666666</v>
+      </c>
+      <c r="G7" s="28">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="I7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>INDURO</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>46304.25</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>46304.66666666666</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>46306.16666666666</v>
+      </c>
+      <c r="G8" s="28">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 102</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>564</v>
+      </c>
+      <c r="D9" s="25" t="n">
+        <v>46305.875</v>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>46306.20833333334</v>
+      </c>
+      <c r="F9" s="25" t="n">
+        <v>46307.08333333334</v>
+      </c>
+      <c r="G9" s="34">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>ALS SUMIRE</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>537</v>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>46307.91666666666</v>
+      </c>
+      <c r="E10" s="25" t="n">
+        <v>46308.25</v>
+      </c>
+      <c r="F10" s="25" t="n">
+        <v>46309.25</v>
+      </c>
+      <c r="G10" s="34">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="17" t="inlineStr">
+        <is>
+          <t>1C</t>
+        </is>
+      </c>
+      <c r="I10" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>YM INCEPTION</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>564</v>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="E11" s="25" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="F11" s="25" t="n">
+        <v>46305.58333333334</v>
+      </c>
+      <c r="G11" s="34">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>STARSHIP AQUILA</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>565</v>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>46304.91666666666</v>
+      </c>
+      <c r="E12" s="25" t="n">
+        <v>46305.58333333334</v>
+      </c>
+      <c r="F12" s="25" t="n">
+        <v>46307.08333333334</v>
+      </c>
+      <c r="G12" s="34">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I12" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>KMTC TAIPEIS</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>46307.95833333334</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>46308.20833333334</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>46309.625</v>
+      </c>
+      <c r="G13" s="28">
+        <f>(F13-E13)*24</f>
+        <v/>
+      </c>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I13" s="23" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>HE JIN</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>552</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>46305.54166666666</v>
+      </c>
+      <c r="G14" s="28">
+        <f>(F14-E14)*24</f>
+        <v/>
+      </c>
+      <c r="H14" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I14" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>CUL HAIPHONG</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>458</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>46304.83333333334</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>46306.25</v>
+      </c>
+      <c r="G15" s="28">
+        <f>(F15-E15)*24</f>
+        <v/>
+      </c>
+      <c r="H15" s="23" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="I15" s="23" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>INCEDA</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>46305.70833333334</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>46306.20833333334</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>46307.58333333334</v>
+      </c>
+      <c r="G16" s="28">
+        <f>(F16-E16)*24</f>
+        <v/>
+      </c>
+      <c r="H16" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I16" s="23" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE SUNRISE</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>46307.375</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>46307.66666666666</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>46309.20833333334</v>
+      </c>
+      <c r="G17" s="28">
+        <f>(F17-E17)*24</f>
+        <v/>
+      </c>
+      <c r="H17" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I17" s="23" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE ATLANTIC</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>46302.83333333334</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>46304.625</v>
+      </c>
+      <c r="F18" s="11" t="n">
+        <v>46306.54166666666</v>
+      </c>
+      <c r="G18" s="28">
+        <f>(F18-E18)*24</f>
+        <v/>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I18" s="23" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>SAMAL</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="n">
+        <v>564</v>
+      </c>
+      <c r="D19" s="25" t="n">
+        <v>46307.04166666666</v>
+      </c>
+      <c r="E19" s="25" t="n">
+        <v>46307.25</v>
+      </c>
+      <c r="F19" s="25" t="n">
+        <v>46308.58333333334</v>
+      </c>
+      <c r="G19" s="34">
+        <f>(F19-E19)*24</f>
+        <v/>
+      </c>
+      <c r="H19" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I19" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>WAN HAI 277</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="n">
+        <v>564</v>
+      </c>
+      <c r="D20" s="25" t="n">
+        <v>46308.16666666666</v>
+      </c>
+      <c r="E20" s="25" t="n">
+        <v>46308.66666666666</v>
+      </c>
+      <c r="F20" s="25" t="n">
+        <v>46310.20833333334</v>
+      </c>
+      <c r="G20" s="34">
+        <f>(F20-E20)*24</f>
+        <v/>
+      </c>
+      <c r="H20" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="I20" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n"/>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G24" s="40" t="n"/>
+      <c r="H24" s="40" t="n"/>
+      <c r="I24" s="41" t="n"/>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C25" s="43" t="n"/>
+      <c r="D25" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E25" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F25" s="16" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (HE JIN is alongside at 20D; other vessels are booked from 10/16)  —  Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+      <c r="G25" s="43" t="n"/>
+      <c r="H25" s="43" t="n"/>
+      <c r="I25" s="43" t="n"/>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="B26" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C26" s="42" t="n"/>
+      <c r="D26" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E26" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail (in progress)  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G26" s="42" t="n"/>
+      <c r="H26" s="42" t="n"/>
+      <c r="I26" s="42" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="F26:I26"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7643,8 +8595,70 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="12" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E41" s="14" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F41" s="13" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (HE JIN is alongside at 20D; other vessels are booked from 10/16)</t>
+        </is>
+      </c>
+      <c r="G41" s="13" t="inlineStr">
+        <is>
+          <t>Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B42" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="C42" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E42" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail (in progress)</t>
+        </is>
+      </c>
+      <c r="G42" s="9" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G40"/>
+  <autoFilter ref="A4:G42"/>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
@@ -7658,7 +8672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N50"/>
+  <dimension ref="A1:N52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -7698,7 +8712,7 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>46304.375</v>
+        <v>46305.375</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -8143,9 +9157,10 @@
         </is>
       </c>
       <c r="M12" s="23" t="inlineStr"/>
-      <c r="N12" s="23">
-        <f>IF(J12&lt;=$B$3,"Sailed",IF(I12&lt;=$B$3,"Alongside",IF(H12&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N12" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -8166,10 +9181,10 @@
         <v>46301</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="F13" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -8218,10 +9233,10 @@
         <v>46302</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="F14" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
@@ -8260,7 +9275,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>SAMAL</t>
+          <t>JOSCO SHINE</t>
         </is>
       </c>
       <c r="C15" s="23" t="n">
@@ -8270,21 +9285,21 @@
         <v>46304</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="F15" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="5" t="inlineStr">
-        <is>
-          <t>20AB</t>
+        <v>2</v>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20AB</t>
         </is>
       </c>
       <c r="H15" s="11" t="n">
-        <v>46307.16666666666</v>
+        <v>46307.54166666666</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>46307.20833333334</v>
+        <v>46307.66666666666</v>
       </c>
       <c r="J15" s="11" t="n">
         <v>46308.58333333334</v>
@@ -8305,106 +9320,105 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>KHUNA BHUM</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F16" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="n">
+        <v>46308.29166666666</v>
+      </c>
+      <c r="I16" s="11" t="n">
+        <v>46308.54166666666</v>
+      </c>
+      <c r="J16" s="11" t="n">
+        <v>46309.29166666666</v>
+      </c>
+      <c r="K16" s="28">
+        <f>(J16-I16)*24</f>
+        <v/>
+      </c>
+      <c r="L16" s="23" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="M16" s="23" t="inlineStr"/>
+      <c r="N16" s="23">
+        <f>IF(J16&lt;=$B$3,"Sailed",IF(I16&lt;=$B$3,"Alongside",IF(H16&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>20B</t>
         </is>
       </c>
-      <c r="B16" s="29" t="inlineStr">
+      <c r="B17" s="29" t="inlineStr">
         <is>
           <t>KMTC GWANGYANG</t>
         </is>
       </c>
-      <c r="C16" s="24" t="n">
+      <c r="C17" s="24" t="n">
         <v>564</v>
       </c>
-      <c r="D16" s="21" t="n">
+      <c r="D17" s="21" t="n">
         <v>46293</v>
       </c>
-      <c r="E16" s="21" t="n">
+      <c r="E17" s="21" t="n">
         <v>46293</v>
       </c>
-      <c r="F16" s="24" t="n">
+      <c r="F17" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="G16" s="30" t="inlineStr">
+      <c r="G17" s="30" t="inlineStr">
         <is>
           <t>20B</t>
         </is>
       </c>
-      <c r="H16" s="31" t="n">
+      <c r="H17" s="31" t="n">
         <v>46292.79166666666</v>
       </c>
-      <c r="I16" s="31" t="n">
+      <c r="I17" s="31" t="n">
         <v>46292.79166666666</v>
       </c>
-      <c r="J16" s="31" t="n">
+      <c r="J17" s="31" t="n">
         <v>46294.20833333334</v>
       </c>
-      <c r="K16" s="32">
-        <f>(J16-I16)*24</f>
-        <v/>
-      </c>
-      <c r="L16" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M16" s="24" t="inlineStr"/>
-      <c r="N16" s="24" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>20B</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>MILLENNIUM BRIGHT</t>
-        </is>
-      </c>
-      <c r="C17" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D17" s="10" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E17" s="10" t="n">
-        <v>46294</v>
-      </c>
-      <c r="F17" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G17" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
-        </is>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>46293.45833333334</v>
-      </c>
-      <c r="I17" s="11" t="n">
-        <v>46294.20833333334</v>
-      </c>
-      <c r="J17" s="11" t="n">
-        <v>46295.16666666666</v>
-      </c>
-      <c r="K17" s="28">
+      <c r="K17" s="32">
         <f>(J17-I17)*24</f>
         <v/>
       </c>
-      <c r="L17" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M17" s="23" t="inlineStr"/>
-      <c r="N17" s="23" t="inlineStr">
+      <c r="L17" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M17" s="24" t="inlineStr"/>
+      <c r="N17" s="24" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -8418,20 +9432,20 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>M ODYSSEY</t>
+          <t>MILLENNIUM BRIGHT</t>
         </is>
       </c>
       <c r="C18" s="23" t="n">
-        <v>449</v>
+        <v>564</v>
       </c>
       <c r="D18" s="10" t="n">
         <v>46293</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>46295</v>
+        <v>46294</v>
       </c>
       <c r="F18" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
@@ -8439,13 +9453,13 @@
         </is>
       </c>
       <c r="H18" s="11" t="n">
+        <v>46293.45833333334</v>
+      </c>
+      <c r="I18" s="11" t="n">
+        <v>46294.20833333334</v>
+      </c>
+      <c r="J18" s="11" t="n">
         <v>46295.16666666666</v>
-      </c>
-      <c r="I18" s="11" t="n">
-        <v>46295.20833333334</v>
-      </c>
-      <c r="J18" s="11" t="n">
-        <v>46296.20833333334</v>
       </c>
       <c r="K18" s="28">
         <f>(J18-I18)*24</f>
@@ -8453,7 +9467,7 @@
       </c>
       <c r="L18" s="23" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>–</t>
         </is>
       </c>
       <c r="M18" s="23" t="inlineStr"/>
@@ -8464,110 +9478,110 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="33" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>20B</t>
         </is>
       </c>
-      <c r="B19" s="33" t="inlineStr">
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>M ODYSSEY</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="n">
+        <v>449</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F19" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="H19" s="11" t="n">
+        <v>46295.16666666666</v>
+      </c>
+      <c r="I19" s="11" t="n">
+        <v>46295.20833333334</v>
+      </c>
+      <c r="J19" s="11" t="n">
+        <v>46296.20833333334</v>
+      </c>
+      <c r="K19" s="28">
+        <f>(J19-I19)*24</f>
+        <v/>
+      </c>
+      <c r="L19" s="23" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="M19" s="23" t="inlineStr"/>
+      <c r="N19" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B20" s="33" t="inlineStr">
         <is>
           <t>KHARIS HERITAGE</t>
         </is>
       </c>
-      <c r="C19" s="17" t="n">
+      <c r="C20" s="17" t="n">
         <v>482</v>
       </c>
-      <c r="D19" s="18" t="n">
+      <c r="D20" s="18" t="n">
         <v>46294</v>
       </c>
-      <c r="E19" s="18" t="n">
+      <c r="E20" s="18" t="n">
         <v>46297</v>
       </c>
-      <c r="F19" s="17" t="n">
+      <c r="F20" s="17" t="n">
         <v>4</v>
       </c>
-      <c r="G19" s="6" t="inlineStr">
+      <c r="G20" s="6" t="inlineStr">
         <is>
           <t>20AB → 20B</t>
         </is>
       </c>
-      <c r="H19" s="25" t="n">
+      <c r="H20" s="25" t="n">
         <v>46296.45833333334</v>
       </c>
-      <c r="I19" s="25" t="n">
+      <c r="I20" s="25" t="n">
         <v>46296.75</v>
       </c>
-      <c r="J19" s="25" t="n">
+      <c r="J20" s="25" t="n">
         <v>46297.70833333334</v>
       </c>
-      <c r="K19" s="34">
-        <f>(J19-I19)*24</f>
-        <v/>
-      </c>
-      <c r="L19" s="17" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M19" s="17" t="inlineStr">
+      <c r="K20" s="34">
+        <f>(J20-I20)*24</f>
+        <v/>
+      </c>
+      <c r="L20" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M20" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="N19" s="17" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>20B</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>YM IMPROVEMENT</t>
-        </is>
-      </c>
-      <c r="C20" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D20" s="10" t="n">
-        <v>46296</v>
-      </c>
-      <c r="E20" s="10" t="n">
-        <v>46300</v>
-      </c>
-      <c r="F20" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>20C → 20B</t>
-        </is>
-      </c>
-      <c r="H20" s="11" t="n">
-        <v>46298.95833333334</v>
-      </c>
-      <c r="I20" s="11" t="n">
-        <v>46299.41666666666</v>
-      </c>
-      <c r="J20" s="11" t="n">
-        <v>46300.5</v>
-      </c>
-      <c r="K20" s="28">
-        <f>(J20-I20)*24</f>
-        <v/>
-      </c>
-      <c r="L20" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M20" s="23" t="inlineStr"/>
-      <c r="N20" s="23" t="inlineStr">
+      <c r="N20" s="17" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -8581,34 +9595,34 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE SPICA</t>
+          <t>YM IMPROVEMENT</t>
         </is>
       </c>
       <c r="C21" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>46299</v>
+        <v>46296</v>
       </c>
       <c r="E21" s="10" t="n">
-        <v>46303</v>
+        <v>46300</v>
       </c>
       <c r="F21" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>20C → 20B</t>
         </is>
       </c>
       <c r="H21" s="11" t="n">
-        <v>46300.875</v>
+        <v>46298.95833333334</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>46301.54166666666</v>
+        <v>46299.41666666666</v>
       </c>
       <c r="J21" s="11" t="n">
-        <v>46303.54166666666</v>
+        <v>46300.5</v>
       </c>
       <c r="K21" s="28">
         <f>(J21-I21)*24</f>
@@ -8634,34 +9648,34 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>SITC HOCHIMINH</t>
+          <t>SAWASDEE SPICA</t>
         </is>
       </c>
       <c r="C22" s="23" t="n">
-        <v>470</v>
+        <v>564</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>46301</v>
+        <v>46299</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="F22" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20B</t>
+        <v>5</v>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H22" s="11" t="n">
-        <v>46302.625</v>
+        <v>46300.875</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>46303.58333333334</v>
+        <v>46301.54166666666</v>
       </c>
       <c r="J22" s="11" t="n">
-        <v>46304.70833333334</v>
+        <v>46303.54166666666</v>
       </c>
       <c r="K22" s="28">
         <f>(J22-I22)*24</f>
@@ -8673,9 +9687,10 @@
         </is>
       </c>
       <c r="M22" s="23" t="inlineStr"/>
-      <c r="N22" s="23">
-        <f>IF(J22&lt;=$B$3,"Sailed",IF(I22&lt;=$B$3,"Alongside",IF(H22&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N22" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -8686,34 +9701,34 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>INDURO</t>
+          <t>SITC HOCHIMINH</t>
         </is>
       </c>
       <c r="C23" s="23" t="n">
-        <v>565</v>
+        <v>470</v>
       </c>
       <c r="D23" s="10" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E23" s="10" t="n">
         <v>46304</v>
       </c>
       <c r="F23" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>4</v>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20B</t>
         </is>
       </c>
       <c r="H23" s="11" t="n">
-        <v>46304.25</v>
+        <v>46302.625</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>46304.66666666666</v>
+        <v>46303.58333333334</v>
       </c>
       <c r="J23" s="11" t="n">
-        <v>46306.58333333334</v>
+        <v>46304.70833333334</v>
       </c>
       <c r="K23" s="28">
         <f>(J23-I23)*24</f>
@@ -8725,9 +9740,10 @@
         </is>
       </c>
       <c r="M23" s="23" t="inlineStr"/>
-      <c r="N23" s="23">
-        <f>IF(J23&lt;=$B$3,"Sailed",IF(I23&lt;=$B$3,"Alongside",IF(H23&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N23" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -8738,20 +9754,20 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>JOSCO SHINE</t>
+          <t>INDURO</t>
         </is>
       </c>
       <c r="C24" s="23" t="n">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E24" s="10" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="F24" s="23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
@@ -8759,13 +9775,13 @@
         </is>
       </c>
       <c r="H24" s="11" t="n">
-        <v>46306.70833333334</v>
+        <v>46304.25</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>46306.70833333334</v>
+        <v>46304.66666666666</v>
       </c>
       <c r="J24" s="11" t="n">
-        <v>46307.58333333334</v>
+        <v>46306.16666666666</v>
       </c>
       <c r="K24" s="28">
         <f>(J24-I24)*24</f>
@@ -8783,161 +9799,168 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="29" t="inlineStr">
+      <c r="A25" s="33" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B25" s="33" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 102</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="n">
+        <v>564</v>
+      </c>
+      <c r="D25" s="18" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E25" s="18" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F25" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>20F → 20B</t>
+        </is>
+      </c>
+      <c r="H25" s="25" t="n">
+        <v>46305.875</v>
+      </c>
+      <c r="I25" s="25" t="n">
+        <v>46306.20833333334</v>
+      </c>
+      <c r="J25" s="25" t="n">
+        <v>46307.08333333334</v>
+      </c>
+      <c r="K25" s="34">
+        <f>(J25-I25)*24</f>
+        <v/>
+      </c>
+      <c r="L25" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M25" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N25" s="17">
+        <f>IF(J25&lt;=$B$3,"Sailed",IF(I25&lt;=$B$3,"Alongside",IF(H25&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="33" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B26" s="33" t="inlineStr">
+        <is>
+          <t>ALS SUMIRE</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="n">
+        <v>537</v>
+      </c>
+      <c r="D26" s="18" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E26" s="18" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F26" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>20F → 20D → 20C → 20B</t>
+        </is>
+      </c>
+      <c r="H26" s="25" t="n">
+        <v>46307.91666666666</v>
+      </c>
+      <c r="I26" s="25" t="n">
+        <v>46308.25</v>
+      </c>
+      <c r="J26" s="25" t="n">
+        <v>46309.25</v>
+      </c>
+      <c r="K26" s="34">
+        <f>(J26-I26)*24</f>
+        <v/>
+      </c>
+      <c r="L26" s="17" t="inlineStr">
+        <is>
+          <t>1C</t>
+        </is>
+      </c>
+      <c r="M26" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N26" s="17">
+        <f>IF(J26&lt;=$B$3,"Sailed",IF(I26&lt;=$B$3,"Alongside",IF(H26&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="29" t="inlineStr">
         <is>
           <t>20C</t>
         </is>
       </c>
-      <c r="B25" s="29" t="inlineStr">
+      <c r="B27" s="29" t="inlineStr">
         <is>
           <t>SAWASDEE DENEB</t>
         </is>
       </c>
-      <c r="C25" s="24" t="n">
+      <c r="C27" s="24" t="n">
         <v>564</v>
       </c>
-      <c r="D25" s="21" t="n">
+      <c r="D27" s="21" t="n">
         <v>46297</v>
       </c>
-      <c r="E25" s="21" t="n">
+      <c r="E27" s="21" t="n">
         <v>46302</v>
       </c>
-      <c r="F25" s="24" t="n">
+      <c r="F27" s="24" t="n">
         <v>6</v>
       </c>
-      <c r="G25" s="30" t="inlineStr">
+      <c r="G27" s="30" t="inlineStr">
         <is>
           <t>20C</t>
         </is>
       </c>
-      <c r="H25" s="31" t="n">
+      <c r="H27" s="31" t="n">
         <v>46300</v>
       </c>
-      <c r="I25" s="31" t="n">
+      <c r="I27" s="31" t="n">
         <v>46300.5</v>
       </c>
-      <c r="J25" s="31" t="n">
+      <c r="J27" s="31" t="n">
         <v>46302.45833333334</v>
       </c>
-      <c r="K25" s="32">
-        <f>(J25-I25)*24</f>
-        <v/>
-      </c>
-      <c r="L25" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M25" s="24" t="inlineStr"/>
-      <c r="N25" s="24" t="inlineStr">
+      <c r="K27" s="32">
+        <f>(J27-I27)*24</f>
+        <v/>
+      </c>
+      <c r="L27" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M27" s="24" t="inlineStr"/>
+      <c r="N27" s="24" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>20C</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>JOSCO LUCKY</t>
-        </is>
-      </c>
-      <c r="C26" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D26" s="10" t="n">
-        <v>46297</v>
-      </c>
-      <c r="E26" s="10" t="n">
-        <v>46303</v>
-      </c>
-      <c r="F26" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="G26" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 20D → 20C</t>
-        </is>
-      </c>
-      <c r="H26" s="11" t="n">
-        <v>46301.875</v>
-      </c>
-      <c r="I26" s="11" t="n">
-        <v>46302.54166666666</v>
-      </c>
-      <c r="J26" s="11" t="n">
-        <v>46303.54166666666</v>
-      </c>
-      <c r="K26" s="28">
-        <f>(J26-I26)*24</f>
-        <v/>
-      </c>
-      <c r="L26" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M26" s="23" t="inlineStr"/>
-      <c r="N26" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>20C</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>ZHONG GU DONG HAI</t>
-        </is>
-      </c>
-      <c r="C27" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D27" s="10" t="n">
-        <v>46301</v>
-      </c>
-      <c r="E27" s="10" t="n">
-        <v>46304</v>
-      </c>
-      <c r="F27" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G27" s="5" t="inlineStr">
-        <is>
-          <t>20C</t>
-        </is>
-      </c>
-      <c r="H27" s="11" t="n">
-        <v>46302.58333333334</v>
-      </c>
-      <c r="I27" s="11" t="n">
-        <v>46303.58333333334</v>
-      </c>
-      <c r="J27" s="11" t="n">
-        <v>46304.58333333334</v>
-      </c>
-      <c r="K27" s="28">
-        <f>(J27-I27)*24</f>
-        <v/>
-      </c>
-      <c r="L27" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M27" s="23" t="inlineStr"/>
-      <c r="N27" s="23">
-        <f>IF(J27&lt;=$B$3,"Sailed",IF(I27&lt;=$B$3,"Alongside",IF(H27&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
       </c>
     </row>
     <row r="28">
@@ -8948,34 +9971,34 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>YM INCEPTION</t>
+          <t>JOSCO LUCKY</t>
         </is>
       </c>
       <c r="C28" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D28" s="10" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="F28" s="23" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20C</t>
+          <t>20B → 20AB → 20D → 20C</t>
         </is>
       </c>
       <c r="H28" s="11" t="n">
+        <v>46301.875</v>
+      </c>
+      <c r="I28" s="11" t="n">
+        <v>46302.54166666666</v>
+      </c>
+      <c r="J28" s="11" t="n">
         <v>46303.54166666666</v>
-      </c>
-      <c r="I28" s="11" t="n">
-        <v>46304.54166666666</v>
-      </c>
-      <c r="J28" s="11" t="n">
-        <v>46305.66666666666</v>
       </c>
       <c r="K28" s="28">
         <f>(J28-I28)*24</f>
@@ -8987,9 +10010,10 @@
         </is>
       </c>
       <c r="M28" s="23" t="inlineStr"/>
-      <c r="N28" s="23">
-        <f>IF(J28&lt;=$B$3,"Sailed",IF(I28&lt;=$B$3,"Alongside",IF(H28&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N28" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -9000,20 +10024,20 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>STARSHIP AQUILA</t>
+          <t>ZHONG GU DONG HAI</t>
         </is>
       </c>
       <c r="C29" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D29" s="10" t="n">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E29" s="10" t="n">
         <v>46304</v>
       </c>
       <c r="F29" s="23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
@@ -9021,13 +10045,13 @@
         </is>
       </c>
       <c r="H29" s="11" t="n">
-        <v>46304.91666666666</v>
+        <v>46302.58333333334</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>46305.66666666666</v>
+        <v>46303.58333333334</v>
       </c>
       <c r="J29" s="11" t="n">
-        <v>46307.20833333334</v>
+        <v>46304.58333333334</v>
       </c>
       <c r="K29" s="28">
         <f>(J29-I29)*24</f>
@@ -9039,152 +10063,160 @@
         </is>
       </c>
       <c r="M29" s="23" t="inlineStr"/>
-      <c r="N29" s="23">
-        <f>IF(J29&lt;=$B$3,"Sailed",IF(I29&lt;=$B$3,"Alongside",IF(H29&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N29" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+      <c r="A30" s="33" t="inlineStr">
         <is>
           <t>20C</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>ALS SUMIRE</t>
-        </is>
-      </c>
-      <c r="C30" s="23" t="n">
-        <v>537</v>
-      </c>
-      <c r="D30" s="10" t="n">
-        <v>46294</v>
-      </c>
-      <c r="E30" s="10" t="n">
-        <v>46304</v>
-      </c>
-      <c r="F30" s="23" t="n">
+      <c r="B30" s="33" t="inlineStr">
+        <is>
+          <t>YM INCEPTION</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="n">
+        <v>564</v>
+      </c>
+      <c r="D30" s="18" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E30" s="18" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F30" s="17" t="n">
         <v>5</v>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>20F → 20D → 20C</t>
-        </is>
-      </c>
-      <c r="H30" s="11" t="n">
-        <v>46307.75</v>
-      </c>
-      <c r="I30" s="11" t="n">
-        <v>46307.75</v>
-      </c>
-      <c r="J30" s="11" t="n">
-        <v>46309.20833333334</v>
-      </c>
-      <c r="K30" s="28">
+          <t>20AB → 20C</t>
+        </is>
+      </c>
+      <c r="H30" s="25" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="I30" s="25" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="J30" s="25" t="n">
+        <v>46305.58333333334</v>
+      </c>
+      <c r="K30" s="34">
         <f>(J30-I30)*24</f>
         <v/>
       </c>
-      <c r="L30" s="23" t="inlineStr">
-        <is>
-          <t>1C</t>
-        </is>
-      </c>
-      <c r="M30" s="23" t="inlineStr"/>
-      <c r="N30" s="23">
+      <c r="L30" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M30" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N30" s="17">
         <f>IF(J30&lt;=$B$3,"Sailed",IF(I30&lt;=$B$3,"Alongside",IF(H30&lt;=$B$3,"At anchorage","Expected")))</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="29" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="B31" s="29" t="inlineStr">
-        <is>
-          <t>BANGKOK</t>
-        </is>
-      </c>
-      <c r="C31" s="24" t="n">
-        <v>551</v>
-      </c>
-      <c r="D31" s="21" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E31" s="21" t="n">
-        <v>46294</v>
-      </c>
-      <c r="F31" s="24" t="n">
-        <v>2</v>
-      </c>
-      <c r="G31" s="30" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="H31" s="31" t="n">
-        <v>46292.54166666666</v>
-      </c>
-      <c r="I31" s="31" t="n">
-        <v>46292.625</v>
-      </c>
-      <c r="J31" s="31" t="n">
-        <v>46294.58333333334</v>
-      </c>
-      <c r="K31" s="32">
+      <c r="A31" s="33" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B31" s="33" t="inlineStr">
+        <is>
+          <t>STARSHIP AQUILA</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="n">
+        <v>565</v>
+      </c>
+      <c r="D31" s="18" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E31" s="18" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F31" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="H31" s="25" t="n">
+        <v>46304.91666666666</v>
+      </c>
+      <c r="I31" s="25" t="n">
+        <v>46305.58333333334</v>
+      </c>
+      <c r="J31" s="25" t="n">
+        <v>46307.08333333334</v>
+      </c>
+      <c r="K31" s="34">
         <f>(J31-I31)*24</f>
         <v/>
       </c>
-      <c r="L31" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M31" s="24" t="inlineStr"/>
-      <c r="N31" s="24" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="L31" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M31" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N31" s="17">
+        <f>IF(J31&lt;=$B$3,"Sailed",IF(I31&lt;=$B$3,"Alongside",IF(H31&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>20D</t>
+          <t>20C</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>HARI BHUM (Barge)</t>
+          <t>KMTC TAIPEIS</t>
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>259</v>
+        <v>565</v>
       </c>
       <c r="D32" s="10" t="n">
-        <v>46297</v>
+        <v>46304</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>46298</v>
+        <v>46305</v>
       </c>
       <c r="F32" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>20D → 20C</t>
         </is>
       </c>
       <c r="H32" s="11" t="n">
-        <v>46298.20833333334</v>
+        <v>46307.95833333334</v>
       </c>
       <c r="I32" s="11" t="n">
-        <v>46298.29166666666</v>
+        <v>46308.20833333334</v>
       </c>
       <c r="J32" s="11" t="n">
-        <v>46298.66666666666</v>
+        <v>46309.625</v>
       </c>
       <c r="K32" s="28">
         <f>(J32-I32)*24</f>
@@ -9196,60 +10228,59 @@
         </is>
       </c>
       <c r="M32" s="23" t="inlineStr"/>
-      <c r="N32" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="N32" s="23">
+        <f>IF(J32&lt;=$B$3,"Sailed",IF(I32&lt;=$B$3,"Alongside",IF(H32&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="A33" s="29" t="inlineStr">
         <is>
           <t>20D</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>MTT BANGKOK</t>
-        </is>
-      </c>
-      <c r="C33" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D33" s="10" t="n">
-        <v>46300</v>
-      </c>
-      <c r="E33" s="10" t="n">
-        <v>46303</v>
-      </c>
-      <c r="F33" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="B33" s="29" t="inlineStr">
+        <is>
+          <t>BANGKOK</t>
+        </is>
+      </c>
+      <c r="C33" s="24" t="n">
+        <v>551</v>
+      </c>
+      <c r="D33" s="21" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E33" s="21" t="n">
+        <v>46294</v>
+      </c>
+      <c r="F33" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="G33" s="30" t="inlineStr">
         <is>
           <t>20D</t>
         </is>
       </c>
-      <c r="H33" s="11" t="n">
-        <v>46302.54166666666</v>
-      </c>
-      <c r="I33" s="11" t="n">
-        <v>46302.58333333334</v>
-      </c>
-      <c r="J33" s="11" t="n">
-        <v>46304.08333333334</v>
-      </c>
-      <c r="K33" s="28">
+      <c r="H33" s="31" t="n">
+        <v>46292.54166666666</v>
+      </c>
+      <c r="I33" s="31" t="n">
+        <v>46292.625</v>
+      </c>
+      <c r="J33" s="31" t="n">
+        <v>46294.58333333334</v>
+      </c>
+      <c r="K33" s="32">
         <f>(J33-I33)*24</f>
         <v/>
       </c>
-      <c r="L33" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M33" s="23" t="inlineStr"/>
-      <c r="N33" s="23" t="inlineStr">
+      <c r="L33" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M33" s="24" t="inlineStr"/>
+      <c r="N33" s="24" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -9263,34 +10294,34 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>HE JIN</t>
+          <t>HARI BHUM (Barge)</t>
         </is>
       </c>
       <c r="C34" s="23" t="n">
-        <v>552</v>
+        <v>259</v>
       </c>
       <c r="D34" s="10" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="E34" s="10" t="n">
-        <v>46304</v>
+        <v>46298</v>
       </c>
       <c r="F34" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G34" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 22A → 20D</t>
+        <v>2</v>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H34" s="11" t="n">
-        <v>46304</v>
+        <v>46298.20833333334</v>
       </c>
       <c r="I34" s="11" t="n">
-        <v>46304</v>
+        <v>46298.29166666666</v>
       </c>
       <c r="J34" s="11" t="n">
-        <v>46305.54166666666</v>
+        <v>46298.66666666666</v>
       </c>
       <c r="K34" s="28">
         <f>(J34-I34)*24</f>
@@ -9302,9 +10333,10 @@
         </is>
       </c>
       <c r="M34" s="23" t="inlineStr"/>
-      <c r="N34" s="23">
-        <f>IF(J34&lt;=$B$3,"Sailed",IF(I34&lt;=$B$3,"Alongside",IF(H34&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N34" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -9315,34 +10347,34 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>CUL HAIPHONG</t>
+          <t>MTT BANGKOK</t>
         </is>
       </c>
       <c r="C35" s="23" t="n">
-        <v>458</v>
+        <v>564</v>
       </c>
       <c r="D35" s="10" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="E35" s="10" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="F35" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20D</t>
+        <v>4</v>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H35" s="11" t="n">
-        <v>46304.83333333334</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="I35" s="11" t="n">
-        <v>46305.66666666666</v>
+        <v>46302.58333333334</v>
       </c>
       <c r="J35" s="11" t="n">
-        <v>46306.25</v>
+        <v>46304.08333333334</v>
       </c>
       <c r="K35" s="28">
         <f>(J35-I35)*24</f>
@@ -9350,13 +10382,14 @@
       </c>
       <c r="L35" s="23" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>–</t>
         </is>
       </c>
       <c r="M35" s="23" t="inlineStr"/>
-      <c r="N35" s="23">
-        <f>IF(J35&lt;=$B$3,"Sailed",IF(I35&lt;=$B$3,"Alongside",IF(H35&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N35" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="36">
@@ -9367,34 +10400,34 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>INCEDA</t>
+          <t>HE JIN</t>
         </is>
       </c>
       <c r="C36" s="23" t="n">
-        <v>564</v>
+        <v>552</v>
       </c>
       <c r="D36" s="10" t="n">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="E36" s="10" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F36" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20AB → 22A → 20D</t>
+        </is>
+      </c>
+      <c r="H36" s="11" t="n">
         <v>46304</v>
       </c>
-      <c r="F36" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="H36" s="11" t="n">
-        <v>46305.70833333334</v>
-      </c>
       <c r="I36" s="11" t="n">
-        <v>46306.20833333334</v>
+        <v>46304</v>
       </c>
       <c r="J36" s="11" t="n">
-        <v>46307.58333333334</v>
+        <v>46305.54166666666</v>
       </c>
       <c r="K36" s="28">
         <f>(J36-I36)*24</f>
@@ -9419,34 +10452,34 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>KMTC TAIPEIS</t>
+          <t>CUL HAIPHONG</t>
         </is>
       </c>
       <c r="C37" s="23" t="n">
-        <v>565</v>
+        <v>458</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>46304</v>
+        <v>46302</v>
       </c>
       <c r="E37" s="10" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="F37" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
+        <v>4</v>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20D</t>
         </is>
       </c>
       <c r="H37" s="11" t="n">
-        <v>46307.95833333334</v>
+        <v>46304.83333333334</v>
       </c>
       <c r="I37" s="11" t="n">
-        <v>46308.20833333334</v>
+        <v>46305.66666666666</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>46309.625</v>
+        <v>46306.25</v>
       </c>
       <c r="K37" s="28">
         <f>(J37-I37)*24</f>
@@ -9454,7 +10487,7 @@
       </c>
       <c r="L37" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="M37" s="23" t="inlineStr"/>
@@ -9464,94 +10497,93 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="29" t="inlineStr">
-        <is>
-          <t>20E</t>
-        </is>
-      </c>
-      <c r="B38" s="29" t="inlineStr">
-        <is>
-          <t>TS CHIBA</t>
-        </is>
-      </c>
-      <c r="C38" s="24" t="n">
-        <v>485</v>
-      </c>
-      <c r="D38" s="21" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E38" s="21" t="n">
-        <v>46293</v>
-      </c>
-      <c r="F38" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" s="30" t="inlineStr">
-        <is>
-          <t>20E</t>
-        </is>
-      </c>
-      <c r="H38" s="31" t="n">
-        <v>46293.29166666666</v>
-      </c>
-      <c r="I38" s="31" t="n">
-        <v>46293.29166666666</v>
-      </c>
-      <c r="J38" s="31" t="n">
-        <v>46294.16666666666</v>
-      </c>
-      <c r="K38" s="32">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>INCEDA</t>
+        </is>
+      </c>
+      <c r="C38" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D38" s="10" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E38" s="10" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F38" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="H38" s="11" t="n">
+        <v>46305.70833333334</v>
+      </c>
+      <c r="I38" s="11" t="n">
+        <v>46306.20833333334</v>
+      </c>
+      <c r="J38" s="11" t="n">
+        <v>46307.58333333334</v>
+      </c>
+      <c r="K38" s="28">
         <f>(J38-I38)*24</f>
         <v/>
       </c>
-      <c r="L38" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M38" s="24" t="inlineStr"/>
-      <c r="N38" s="24" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="L38" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M38" s="23" t="inlineStr"/>
+      <c r="N38" s="23">
+        <f>IF(J38&lt;=$B$3,"Sailed",IF(I38&lt;=$B$3,"Alongside",IF(H38&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>20E</t>
+          <t>20D</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>MITRA BHUM</t>
+          <t>SAWASDEE SUNRISE</t>
         </is>
       </c>
       <c r="C39" s="23" t="n">
-        <v>485</v>
+        <v>564</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>46293</v>
+        <v>46304</v>
       </c>
       <c r="E39" s="10" t="n">
-        <v>46295</v>
+        <v>46305</v>
       </c>
       <c r="F39" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>20F → 20E</t>
+          <t>20F → 20D</t>
         </is>
       </c>
       <c r="H39" s="11" t="n">
-        <v>46295.125</v>
+        <v>46307.375</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>46295.20833333334</v>
+        <v>46307.66666666666</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>46295.75</v>
+        <v>46309.20833333334</v>
       </c>
       <c r="K39" s="28">
         <f>(J39-I39)*24</f>
@@ -9563,117 +10595,112 @@
         </is>
       </c>
       <c r="M39" s="23" t="inlineStr"/>
-      <c r="N39" s="23" t="inlineStr">
+      <c r="N39" s="23">
+        <f>IF(J39&lt;=$B$3,"Sailed",IF(I39&lt;=$B$3,"Alongside",IF(H39&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="29" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B40" s="29" t="inlineStr">
+        <is>
+          <t>TS CHIBA</t>
+        </is>
+      </c>
+      <c r="C40" s="24" t="n">
+        <v>485</v>
+      </c>
+      <c r="D40" s="21" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E40" s="21" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F40" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="30" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="H40" s="31" t="n">
+        <v>46293.29166666666</v>
+      </c>
+      <c r="I40" s="31" t="n">
+        <v>46293.29166666666</v>
+      </c>
+      <c r="J40" s="31" t="n">
+        <v>46294.16666666666</v>
+      </c>
+      <c r="K40" s="32">
+        <f>(J40-I40)*24</f>
+        <v/>
+      </c>
+      <c r="L40" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M40" s="24" t="inlineStr"/>
+      <c r="N40" s="24" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>20E</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>WAN HAI 278</t>
-        </is>
-      </c>
-      <c r="C40" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D40" s="10" t="n">
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>MITRA BHUM</t>
+        </is>
+      </c>
+      <c r="C41" s="23" t="n">
+        <v>485</v>
+      </c>
+      <c r="D41" s="10" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E41" s="10" t="n">
         <v>46295</v>
       </c>
-      <c r="E40" s="10" t="n">
-        <v>46300</v>
-      </c>
-      <c r="F40" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="G40" s="6" t="inlineStr">
+      <c r="F41" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
         <is>
           <t>20F → 20E</t>
         </is>
       </c>
-      <c r="H40" s="11" t="n">
-        <v>46297.75</v>
-      </c>
-      <c r="I40" s="11" t="n">
-        <v>46298.41666666666</v>
-      </c>
-      <c r="J40" s="11" t="n">
-        <v>46300.45833333334</v>
-      </c>
-      <c r="K40" s="28">
-        <f>(J40-I40)*24</f>
-        <v/>
-      </c>
-      <c r="L40" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M40" s="23" t="inlineStr"/>
-      <c r="N40" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="35" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="B41" s="35" t="inlineStr">
-        <is>
-          <t>JARU BHUM</t>
-        </is>
-      </c>
-      <c r="C41" s="22" t="n">
-        <v>564</v>
-      </c>
-      <c r="D41" s="14" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E41" s="14" t="n">
-        <v>46293</v>
-      </c>
-      <c r="F41" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G41" s="36" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="H41" s="37" t="n">
-        <v>46293.33333333334</v>
-      </c>
-      <c r="I41" s="37" t="n">
-        <v>46293.33333333334</v>
-      </c>
-      <c r="J41" s="37" t="n">
-        <v>46294.16666666666</v>
-      </c>
-      <c r="K41" s="38">
+      <c r="H41" s="11" t="n">
+        <v>46295.125</v>
+      </c>
+      <c r="I41" s="11" t="n">
+        <v>46295.20833333334</v>
+      </c>
+      <c r="J41" s="11" t="n">
+        <v>46295.75</v>
+      </c>
+      <c r="K41" s="28">
         <f>(J41-I41)*24</f>
         <v/>
       </c>
-      <c r="L41" s="22" t="inlineStr">
-        <is>
-          <t>7B</t>
-        </is>
-      </c>
-      <c r="M41" s="22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="N41" s="22" t="inlineStr">
+      <c r="L41" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M41" s="23" t="inlineStr"/>
+      <c r="N41" s="23" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -9682,39 +10709,39 @@
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>20F</t>
+          <t>20E</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>HOPE C</t>
+          <t>WAN HAI 278</t>
         </is>
       </c>
       <c r="C42" s="23" t="n">
-        <v>481</v>
+        <v>564</v>
       </c>
       <c r="D42" s="10" t="n">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="E42" s="10" t="n">
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="F42" s="23" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>20E → 20F</t>
+          <t>20F → 20E</t>
         </is>
       </c>
       <c r="H42" s="11" t="n">
-        <v>46294.70833333334</v>
+        <v>46297.75</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>46294.70833333334</v>
+        <v>46298.41666666666</v>
       </c>
       <c r="J42" s="11" t="n">
-        <v>46295.66666666666</v>
+        <v>46300.45833333334</v>
       </c>
       <c r="K42" s="28">
         <f>(J42-I42)*24</f>
@@ -9733,53 +10760,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+      <c r="A43" s="35" t="inlineStr">
         <is>
           <t>20F</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="C43" s="23" t="n">
+      <c r="B43" s="35" t="inlineStr">
+        <is>
+          <t>JARU BHUM</t>
+        </is>
+      </c>
+      <c r="C43" s="22" t="n">
         <v>564</v>
       </c>
-      <c r="D43" s="10" t="n">
-        <v>46295</v>
-      </c>
-      <c r="E43" s="10" t="n">
-        <v>46298</v>
-      </c>
-      <c r="F43" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20F</t>
-        </is>
-      </c>
-      <c r="H43" s="11" t="n">
-        <v>46297.29166666666</v>
-      </c>
-      <c r="I43" s="11" t="n">
-        <v>46297.45833333334</v>
-      </c>
-      <c r="J43" s="11" t="n">
-        <v>46298.70833333334</v>
-      </c>
-      <c r="K43" s="28">
+      <c r="D43" s="14" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E43" s="14" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F43" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="36" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="H43" s="37" t="n">
+        <v>46293.33333333334</v>
+      </c>
+      <c r="I43" s="37" t="n">
+        <v>46293.33333333334</v>
+      </c>
+      <c r="J43" s="37" t="n">
+        <v>46294.16666666666</v>
+      </c>
+      <c r="K43" s="38">
         <f>(J43-I43)*24</f>
         <v/>
       </c>
-      <c r="L43" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="M43" s="23" t="inlineStr"/>
-      <c r="N43" s="23" t="inlineStr">
+      <c r="L43" s="22" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="M43" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N43" s="22" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -9793,34 +10824,34 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 98</t>
+          <t>HOPE C</t>
         </is>
       </c>
       <c r="C44" s="23" t="n">
-        <v>564</v>
+        <v>481</v>
       </c>
       <c r="D44" s="10" t="n">
-        <v>46297</v>
+        <v>46293</v>
       </c>
       <c r="E44" s="10" t="n">
-        <v>46299</v>
+        <v>46295</v>
       </c>
       <c r="F44" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="G44" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+      <c r="G44" s="6" t="inlineStr">
+        <is>
+          <t>20E → 20F</t>
         </is>
       </c>
       <c r="H44" s="11" t="n">
-        <v>46299.375</v>
+        <v>46294.70833333334</v>
       </c>
       <c r="I44" s="11" t="n">
-        <v>46299.375</v>
+        <v>46294.70833333334</v>
       </c>
       <c r="J44" s="11" t="n">
-        <v>46300.375</v>
+        <v>46295.66666666666</v>
       </c>
       <c r="K44" s="28">
         <f>(J44-I44)*24</f>
@@ -9846,34 +10877,34 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>XIN AN</t>
+          <t>KMTC BANGKOK</t>
         </is>
       </c>
       <c r="C45" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D45" s="10" t="n">
-        <v>46300</v>
+        <v>46295</v>
       </c>
       <c r="E45" s="10" t="n">
-        <v>46304</v>
+        <v>46298</v>
       </c>
       <c r="F45" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G45" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+        <v>4</v>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20F</t>
         </is>
       </c>
       <c r="H45" s="11" t="n">
-        <v>46302.54166666666</v>
+        <v>46297.29166666666</v>
       </c>
       <c r="I45" s="11" t="n">
-        <v>46302.58333333334</v>
+        <v>46297.45833333334</v>
       </c>
       <c r="J45" s="11" t="n">
-        <v>46304.54166666666</v>
+        <v>46298.70833333334</v>
       </c>
       <c r="K45" s="28">
         <f>(J45-I45)*24</f>
@@ -9885,9 +10916,10 @@
         </is>
       </c>
       <c r="M45" s="23" t="inlineStr"/>
-      <c r="N45" s="23">
-        <f>IF(J45&lt;=$B$3,"Sailed",IF(I45&lt;=$B$3,"Alongside",IF(H45&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N45" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -9898,34 +10930,34 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE ATLANTIC</t>
+          <t>XIN MING ZHOU 98</t>
         </is>
       </c>
       <c r="C46" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D46" s="10" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="E46" s="10" t="n">
-        <v>46304</v>
+        <v>46299</v>
       </c>
       <c r="F46" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G46" s="6" t="inlineStr">
-        <is>
-          <t>20C → 20D → 20F</t>
+        <v>3</v>
+      </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
         </is>
       </c>
       <c r="H46" s="11" t="n">
-        <v>46302.83333333334</v>
+        <v>46299.375</v>
       </c>
       <c r="I46" s="11" t="n">
-        <v>46304.625</v>
+        <v>46299.375</v>
       </c>
       <c r="J46" s="11" t="n">
-        <v>46306.125</v>
+        <v>46300.375</v>
       </c>
       <c r="K46" s="28">
         <f>(J46-I46)*24</f>
@@ -9937,9 +10969,10 @@
         </is>
       </c>
       <c r="M46" s="23" t="inlineStr"/>
-      <c r="N46" s="23">
-        <f>IF(J46&lt;=$B$3,"Sailed",IF(I46&lt;=$B$3,"Alongside",IF(H46&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N46" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -9950,20 +10983,20 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 102</t>
+          <t>XIN AN</t>
         </is>
       </c>
       <c r="C47" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D47" s="10" t="n">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="E47" s="10" t="n">
         <v>46304</v>
       </c>
       <c r="F47" s="23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
@@ -9971,13 +11004,13 @@
         </is>
       </c>
       <c r="H47" s="11" t="n">
-        <v>46305.875</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="I47" s="11" t="n">
-        <v>46306.20833333334</v>
+        <v>46302.58333333334</v>
       </c>
       <c r="J47" s="11" t="n">
-        <v>46307.08333333334</v>
+        <v>46304.54166666666</v>
       </c>
       <c r="K47" s="28">
         <f>(J47-I47)*24</f>
@@ -9989,9 +11022,10 @@
         </is>
       </c>
       <c r="M47" s="23" t="inlineStr"/>
-      <c r="N47" s="23">
-        <f>IF(J47&lt;=$B$3,"Sailed",IF(I47&lt;=$B$3,"Alongside",IF(H47&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="N47" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -10002,34 +11036,34 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE SUNRISE</t>
+          <t>SAWASDEE ATLANTIC</t>
         </is>
       </c>
       <c r="C48" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D48" s="10" t="n">
-        <v>46304</v>
+        <v>46300</v>
       </c>
       <c r="E48" s="10" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="F48" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+        <v>6</v>
+      </c>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>20C → 20D → 20F</t>
         </is>
       </c>
       <c r="H48" s="11" t="n">
-        <v>46307.20833333334</v>
+        <v>46302.83333333334</v>
       </c>
       <c r="I48" s="11" t="n">
-        <v>46307.20833333334</v>
+        <v>46304.625</v>
       </c>
       <c r="J48" s="11" t="n">
-        <v>46308.625</v>
+        <v>46306.54166666666</v>
       </c>
       <c r="K48" s="28">
         <f>(J48-I48)*24</f>
@@ -10046,15 +11080,127 @@
         <v/>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="33" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B49" s="33" t="inlineStr">
+        <is>
+          <t>SAMAL</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="n">
+        <v>564</v>
+      </c>
+      <c r="D49" s="18" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E49" s="18" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F49" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20F</t>
+        </is>
+      </c>
+      <c r="H49" s="25" t="n">
+        <v>46307.04166666666</v>
+      </c>
+      <c r="I49" s="25" t="n">
+        <v>46307.25</v>
+      </c>
+      <c r="J49" s="25" t="n">
+        <v>46308.58333333334</v>
+      </c>
+      <c r="K49" s="34">
+        <f>(J49-I49)*24</f>
+        <v/>
+      </c>
+      <c r="L49" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M49" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N49" s="17">
+        <f>IF(J49&lt;=$B$3,"Sailed",IF(I49&lt;=$B$3,"Alongside",IF(H49&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>43 vessels in total. Orange cells: marked on sheet, or the vessel changed berth.</t>
+      <c r="A50" s="33" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B50" s="33" t="inlineStr">
+        <is>
+          <t>WAN HAI 277</t>
+        </is>
+      </c>
+      <c r="C50" s="17" t="n">
+        <v>564</v>
+      </c>
+      <c r="D50" s="18" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E50" s="18" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F50" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="H50" s="25" t="n">
+        <v>46308.16666666666</v>
+      </c>
+      <c r="I50" s="25" t="n">
+        <v>46308.66666666666</v>
+      </c>
+      <c r="J50" s="25" t="n">
+        <v>46310.20833333334</v>
+      </c>
+      <c r="K50" s="34">
+        <f>(J50-I50)*24</f>
+        <v/>
+      </c>
+      <c r="L50" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="M50" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N50" s="17">
+        <f>IF(J50&lt;=$B$3,"Sailed",IF(I50&lt;=$B$3,"Alongside",IF(H50&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>45 vessels in total. Orange cells: marked on sheet, or the vessel changed berth.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:N48"/>
+  <autoFilter ref="A5:N50"/>
   <mergeCells count="1">
     <mergeCell ref="A2:N2"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add 13 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -25,10 +25,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Oct 2026" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Oct 2026" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Oct 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Oct 2026" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$46</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$O$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$O$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -672,7 +673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P52"/>
+  <dimension ref="A1:Q54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -691,6 +692,7 @@
     <col width="44" customWidth="1" min="14" max="14"/>
     <col width="44" customWidth="1" min="15" max="15"/>
     <col width="44" customWidth="1" min="16" max="16"/>
+    <col width="44" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -786,6 +788,11 @@
       <c r="P4" s="3" t="inlineStr">
         <is>
           <t>12 Oct 2026</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>13 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -822,6 +829,7 @@
       <c r="N5" s="5" t="inlineStr"/>
       <c r="O5" s="5" t="inlineStr"/>
       <c r="P5" s="5" t="inlineStr"/>
+      <c r="Q5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -860,6 +868,7 @@
       <c r="N6" s="5" t="inlineStr"/>
       <c r="O6" s="5" t="inlineStr"/>
       <c r="P6" s="5" t="inlineStr"/>
+      <c r="Q6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -890,6 +899,7 @@
       <c r="N7" s="5" t="inlineStr"/>
       <c r="O7" s="5" t="inlineStr"/>
       <c r="P7" s="5" t="inlineStr"/>
+      <c r="Q7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -924,6 +934,7 @@
       <c r="N8" s="5" t="inlineStr"/>
       <c r="O8" s="5" t="inlineStr"/>
       <c r="P8" s="5" t="inlineStr"/>
+      <c r="Q8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -958,6 +969,7 @@
       <c r="N9" s="5" t="inlineStr"/>
       <c r="O9" s="5" t="inlineStr"/>
       <c r="P9" s="5" t="inlineStr"/>
+      <c r="Q9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -988,6 +1000,7 @@
       <c r="N10" s="5" t="inlineStr"/>
       <c r="O10" s="5" t="inlineStr"/>
       <c r="P10" s="5" t="inlineStr"/>
+      <c r="Q10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1026,6 +1039,7 @@
       <c r="N11" s="5" t="inlineStr"/>
       <c r="O11" s="5" t="inlineStr"/>
       <c r="P11" s="5" t="inlineStr"/>
+      <c r="Q11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1056,6 +1070,7 @@
       <c r="N12" s="5" t="inlineStr"/>
       <c r="O12" s="5" t="inlineStr"/>
       <c r="P12" s="5" t="inlineStr"/>
+      <c r="Q12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1094,6 +1109,7 @@
       <c r="N13" s="5" t="inlineStr"/>
       <c r="O13" s="5" t="inlineStr"/>
       <c r="P13" s="5" t="inlineStr"/>
+      <c r="Q13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1140,6 +1156,7 @@
       <c r="N14" s="5" t="inlineStr"/>
       <c r="O14" s="5" t="inlineStr"/>
       <c r="P14" s="5" t="inlineStr"/>
+      <c r="Q14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1182,6 +1199,11 @@
           <t>expected → 20C (returns for a new call, shift 4A)</t>
         </is>
       </c>
+      <c r="Q15" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C (shift 4A no longer shown)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1224,6 +1246,11 @@
       <c r="N16" s="5" t="inlineStr"/>
       <c r="O16" s="5" t="inlineStr"/>
       <c r="P16" s="5" t="inlineStr"/>
+      <c r="Q16" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20C (returns for a new call, ETA 15/01)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1280,6 +1307,11 @@
       <c r="P17" s="5" t="inlineStr">
         <is>
           <t>expected · 20F (1C)</t>
+        </is>
+      </c>
+      <c r="Q17" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20F (P.B 13/06, ETD 14/06, 1C)</t>
         </is>
       </c>
     </row>
@@ -1324,6 +1356,7 @@
       <c r="N18" s="5" t="inlineStr"/>
       <c r="O18" s="5" t="inlineStr"/>
       <c r="P18" s="5" t="inlineStr"/>
+      <c r="Q18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1374,6 +1407,7 @@
       <c r="N19" s="5" t="inlineStr"/>
       <c r="O19" s="5" t="inlineStr"/>
       <c r="P19" s="5" t="inlineStr"/>
+      <c r="Q19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1424,6 +1458,7 @@
       <c r="N20" s="5" t="inlineStr"/>
       <c r="O20" s="5" t="inlineStr"/>
       <c r="P20" s="5" t="inlineStr"/>
+      <c r="Q20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1470,6 +1505,7 @@
       <c r="N21" s="5" t="inlineStr"/>
       <c r="O21" s="5" t="inlineStr"/>
       <c r="P21" s="5" t="inlineStr"/>
+      <c r="Q21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1512,6 +1548,7 @@
       <c r="N22" s="5" t="inlineStr"/>
       <c r="O22" s="5" t="inlineStr"/>
       <c r="P22" s="5" t="inlineStr"/>
+      <c r="Q22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1566,6 +1603,7 @@
       <c r="N23" s="5" t="inlineStr"/>
       <c r="O23" s="5" t="inlineStr"/>
       <c r="P23" s="5" t="inlineStr"/>
+      <c r="Q23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1616,6 +1654,7 @@
       <c r="N24" s="5" t="inlineStr"/>
       <c r="O24" s="5" t="inlineStr"/>
       <c r="P24" s="5" t="inlineStr"/>
+      <c r="Q24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1650,6 +1689,7 @@
       <c r="N25" s="5" t="inlineStr"/>
       <c r="O25" s="5" t="inlineStr"/>
       <c r="P25" s="5" t="inlineStr"/>
+      <c r="Q25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1688,6 +1728,7 @@
       <c r="N26" s="5" t="inlineStr"/>
       <c r="O26" s="5" t="inlineStr"/>
       <c r="P26" s="5" t="inlineStr"/>
+      <c r="Q26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1738,6 +1779,7 @@
       <c r="N27" s="5" t="inlineStr"/>
       <c r="O27" s="5" t="inlineStr"/>
       <c r="P27" s="5" t="inlineStr"/>
+      <c r="Q27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1784,6 +1826,7 @@
       <c r="N28" s="5" t="inlineStr"/>
       <c r="O28" s="5" t="inlineStr"/>
       <c r="P28" s="5" t="inlineStr"/>
+      <c r="Q28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1830,6 +1873,7 @@
       </c>
       <c r="O29" s="5" t="inlineStr"/>
       <c r="P29" s="5" t="inlineStr"/>
+      <c r="Q29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1884,6 +1928,7 @@
           <t>sailed (11/12)</t>
         </is>
       </c>
+      <c r="Q30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1926,6 +1971,7 @@
       <c r="N31" s="5" t="inlineStr"/>
       <c r="O31" s="5" t="inlineStr"/>
       <c r="P31" s="5" t="inlineStr"/>
+      <c r="Q31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -1972,6 +2018,7 @@
       </c>
       <c r="O32" s="5" t="inlineStr"/>
       <c r="P32" s="5" t="inlineStr"/>
+      <c r="Q32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2014,6 +2061,7 @@
       </c>
       <c r="O33" s="5" t="inlineStr"/>
       <c r="P33" s="5" t="inlineStr"/>
+      <c r="Q33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2060,6 +2108,7 @@
         </is>
       </c>
       <c r="P34" s="5" t="inlineStr"/>
+      <c r="Q34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2106,6 +2155,7 @@
         </is>
       </c>
       <c r="P35" s="5" t="inlineStr"/>
+      <c r="Q35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2148,6 +2198,7 @@
       </c>
       <c r="O36" s="5" t="inlineStr"/>
       <c r="P36" s="5" t="inlineStr"/>
+      <c r="Q36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2194,6 +2245,7 @@
         </is>
       </c>
       <c r="P37" s="5" t="inlineStr"/>
+      <c r="Q37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2240,6 +2292,7 @@
           <t>sailed (11/15)</t>
         </is>
       </c>
+      <c r="Q38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2282,6 +2335,7 @@
         </is>
       </c>
       <c r="P39" s="5" t="inlineStr"/>
+      <c r="Q39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -2324,6 +2378,7 @@
         </is>
       </c>
       <c r="P40" s="5" t="inlineStr"/>
+      <c r="Q40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2370,6 +2425,7 @@
           <t>sailed (12/02)</t>
         </is>
       </c>
+      <c r="Q41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -2412,6 +2468,7 @@
           <t>sailed (12/02)</t>
         </is>
       </c>
+      <c r="Q42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2452,6 +2509,11 @@
       <c r="P43" s="5" t="inlineStr">
         <is>
           <t>alongside · 20D (ETD 12/14)</t>
+        </is>
+      </c>
+      <c r="Q43" s="5" t="inlineStr">
+        <is>
+          <t>sailed (12/14)</t>
         </is>
       </c>
     </row>
@@ -2492,6 +2554,11 @@
           <t>at anchorage · 20AB (ETA 12/09→12/08)</t>
         </is>
       </c>
+      <c r="Q44" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20AB (ETA 12/08→12/09, ETD 14/05)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -2530,6 +2597,11 @@
           <t>expected · 20F (ETA 12/09→12/11)</t>
         </is>
       </c>
+      <c r="Q45" s="5" t="inlineStr">
+        <is>
+          <t>sailed (13/06)</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -2568,6 +2640,11 @@
           <t>expected → 20AB (P.B 13/05→14/05, ETD 14/15→15/15)</t>
         </is>
       </c>
+      <c r="Q46" s="6" t="inlineStr">
+        <is>
+          <t>at anchorage · 20AB (ETA 13/01→13/02)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -2604,6 +2681,11 @@
       <c r="P47" s="6" t="inlineStr">
         <is>
           <t>at anchorage · 20D (ETA 12/09→12/04)</t>
+        </is>
+      </c>
+      <c r="Q47" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20D (P.B 12/16, ETD 14/05)</t>
         </is>
       </c>
     </row>
@@ -2640,6 +2722,11 @@
           <t>expected · 20D (shift 7B)</t>
         </is>
       </c>
+      <c r="Q48" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20D (ETA 13/07→13/11, shift 7B)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -2672,6 +2759,11 @@
       <c r="P49" s="6" t="inlineStr">
         <is>
           <t>expected → 20C (ETA 12/23→12/21)</t>
+        </is>
+      </c>
+      <c r="Q49" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20C (P.B 13/06, ETD 14/15)</t>
         </is>
       </c>
     </row>
@@ -2702,6 +2794,11 @@
       <c r="P50" s="6" t="inlineStr">
         <is>
           <t>expected → 20B (ETA 12/24→12/22, P.B 14/06→13/06, ETD 15/16→14/16)</t>
+        </is>
+      </c>
+      <c r="Q50" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20B (ETD 14/16)</t>
         </is>
       </c>
     </row>
@@ -2730,6 +2827,11 @@
           <t>expected · 20B (new)</t>
         </is>
       </c>
+      <c r="Q51" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20B (ETA 14/08→14/01)</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -2754,6 +2856,65 @@
       <c r="P52" s="5" t="inlineStr">
         <is>
           <t>expected · 20F (new)</t>
+        </is>
+      </c>
+      <c r="Q52" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F (ETA 13/15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>WAN HAI 176</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr"/>
+      <c r="C53" s="5" t="inlineStr"/>
+      <c r="D53" s="5" t="inlineStr"/>
+      <c r="E53" s="5" t="inlineStr"/>
+      <c r="F53" s="5" t="inlineStr"/>
+      <c r="G53" s="5" t="inlineStr"/>
+      <c r="H53" s="5" t="inlineStr"/>
+      <c r="I53" s="5" t="inlineStr"/>
+      <c r="J53" s="5" t="inlineStr"/>
+      <c r="K53" s="5" t="inlineStr"/>
+      <c r="L53" s="5" t="inlineStr"/>
+      <c r="M53" s="5" t="inlineStr"/>
+      <c r="N53" s="5" t="inlineStr"/>
+      <c r="O53" s="5" t="inlineStr"/>
+      <c r="P53" s="5" t="inlineStr"/>
+      <c r="Q53" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>WAN HAI 175</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr"/>
+      <c r="C54" s="5" t="inlineStr"/>
+      <c r="D54" s="5" t="inlineStr"/>
+      <c r="E54" s="5" t="inlineStr"/>
+      <c r="F54" s="5" t="inlineStr"/>
+      <c r="G54" s="5" t="inlineStr"/>
+      <c r="H54" s="5" t="inlineStr"/>
+      <c r="I54" s="5" t="inlineStr"/>
+      <c r="J54" s="5" t="inlineStr"/>
+      <c r="K54" s="5" t="inlineStr"/>
+      <c r="L54" s="5" t="inlineStr"/>
+      <c r="M54" s="5" t="inlineStr"/>
+      <c r="N54" s="5" t="inlineStr"/>
+      <c r="O54" s="5" t="inlineStr"/>
+      <c r="P54" s="5" t="inlineStr"/>
+      <c r="Q54" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D (new)</t>
         </is>
       </c>
     </row>
@@ -9521,13 +9682,692 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 13 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Waiting for Berth (h)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>SAMAL</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>46307.375</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>46307.66666666666</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>46309.20833333334</v>
+      </c>
+      <c r="G4" s="28">
+        <f>(E4-D4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="28">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>KMTC TAIPEIS</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46308.08333333334</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46309.20833333334</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46310.625</v>
+      </c>
+      <c r="G5" s="28">
+        <f>(E5-D5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="28">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>CEBU</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46307.91666666666</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46308.25</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46309.66666666666</v>
+      </c>
+      <c r="G6" s="28">
+        <f>(E6-D6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="28">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 173</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46309.04166666666</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46309.66666666666</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46310.29166666666</v>
+      </c>
+      <c r="G7" s="28">
+        <f>(E7-D7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="28">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 176</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>46310.45833333334</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>46310.45833333334</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>46311.66666666666</v>
+      </c>
+      <c r="G8" s="28">
+        <f>(E8-D8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="28">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 277</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>46307.875</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>46308.25</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>46309.625</v>
+      </c>
+      <c r="G9" s="28">
+        <f>(E9-D9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="28">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>M ODYSSEY</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>449</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>46309.125</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>46309.58333333334</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>46310.20833333334</v>
+      </c>
+      <c r="G10" s="28">
+        <f>(E10-D10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="28">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>KHARIS HERITAGE</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>482</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>46310.04166666666</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>46310.29166666666</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>46311.29166666666</v>
+      </c>
+      <c r="G11" s="28">
+        <f>(E11-D11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="28">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J11" s="23" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE SUNRISE</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>46307.16666666666</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>46307.66666666666</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>46309.20833333334</v>
+      </c>
+      <c r="G12" s="28">
+        <f>(E12-D12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="28">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J12" s="23" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>KHUNA BHUM</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>46308.45833333334</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>46309.20833333334</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>46309.91666666666</v>
+      </c>
+      <c r="G13" s="28">
+        <f>(E13-D13)*24</f>
+        <v/>
+      </c>
+      <c r="H13" s="28">
+        <f>(F13-E13)*24</f>
+        <v/>
+      </c>
+      <c r="I13" s="23" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="J13" s="23" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 175</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>46310.04166666666</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>46310.29166666666</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>46311.70833333334</v>
+      </c>
+      <c r="G14" s="28">
+        <f>(E14-D14)*24</f>
+        <v/>
+      </c>
+      <c r="H14" s="28">
+        <f>(F14-E14)*24</f>
+        <v/>
+      </c>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J14" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>ALS SUMIRE</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>537</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>46307.91666666666</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>46308.25</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>46309.25</v>
+      </c>
+      <c r="G15" s="28">
+        <f>(E15-D15)*24</f>
+        <v/>
+      </c>
+      <c r="H15" s="28">
+        <f>(F15-E15)*24</f>
+        <v/>
+      </c>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>1C</t>
+        </is>
+      </c>
+      <c r="J15" s="23" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE INCHEON</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>46308.625</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>46309.25</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>46310.625</v>
+      </c>
+      <c r="G16" s="28">
+        <f>(E16-D16)*24</f>
+        <v/>
+      </c>
+      <c r="H16" s="28">
+        <f>(F16-E16)*24</f>
+        <v/>
+      </c>
+      <c r="I16" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J16" s="23" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="39" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G20" s="40" t="n"/>
+      <c r="H20" s="40" t="n"/>
+      <c r="I20" s="40" t="n"/>
+      <c r="J20" s="41" t="n"/>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C21" s="43" t="n"/>
+      <c r="D21" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E21" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (SAWASDEE SUNRISE is alongside at 20D; other vessels are booked from 14/05)  —  Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+      <c r="G21" s="43" t="n"/>
+      <c r="H21" s="43" t="n"/>
+      <c r="I21" s="43" t="n"/>
+      <c r="J21" s="43" t="n"/>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C22" s="42" t="n"/>
+      <c r="D22" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E22" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail (in progress)  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G22" s="42" t="n"/>
+      <c r="H22" s="42" t="n"/>
+      <c r="I22" s="42" t="n"/>
+      <c r="J22" s="42" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="F22:J22"/>
+    <mergeCell ref="F20:J20"/>
+    <mergeCell ref="F21:J21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G46"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10912,8 +11752,70 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="12" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B47" s="13" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C47" s="13" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D47" s="14" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E47" s="14" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F47" s="13" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (SAWASDEE SUNRISE is alongside at 20D; other vessels are booked from 14/05)</t>
+        </is>
+      </c>
+      <c r="G47" s="13" t="inlineStr">
+        <is>
+          <t>Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B48" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="C48" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D48" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E48" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F48" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail (in progress)</t>
+        </is>
+      </c>
+      <c r="G48" s="9" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G46"/>
+  <autoFilter ref="A4:G48"/>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
@@ -10927,7 +11829,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O55"/>
+  <dimension ref="A1:O57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10968,7 +11870,7 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>46307.375</v>
+        <v>46308.375</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -11584,10 +12486,10 @@
         <v>46304</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="F15" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
@@ -11595,7 +12497,7 @@
         </is>
       </c>
       <c r="H15" s="11" t="n">
-        <v>46307.33333333334</v>
+        <v>46307.375</v>
       </c>
       <c r="I15" s="11" t="n">
         <v>46307.66666666666</v>
@@ -11640,10 +12542,10 @@
         <v>46304</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="F16" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
@@ -11651,7 +12553,7 @@
         </is>
       </c>
       <c r="H16" s="11" t="n">
-        <v>46308.04166666666</v>
+        <v>46308.08333333334</v>
       </c>
       <c r="I16" s="11" t="n">
         <v>46309.20833333334</v>
@@ -11793,61 +12695,57 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="33" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>20B</t>
         </is>
       </c>
-      <c r="B19" s="33" t="inlineStr">
-        <is>
-          <t>KHARIS HERITAGE</t>
-        </is>
-      </c>
-      <c r="C19" s="17" t="n">
-        <v>482</v>
-      </c>
-      <c r="D19" s="18" t="n">
-        <v>46294</v>
-      </c>
-      <c r="E19" s="18" t="n">
-        <v>46297</v>
-      </c>
-      <c r="F19" s="17" t="n">
-        <v>4</v>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>YM IMPROVEMENT</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D19" s="10" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F19" s="23" t="n">
+        <v>5</v>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20B</t>
-        </is>
-      </c>
-      <c r="H19" s="25" t="n">
-        <v>46296.45833333334</v>
-      </c>
-      <c r="I19" s="25" t="n">
-        <v>46296.75</v>
-      </c>
-      <c r="J19" s="25" t="n">
-        <v>46297.70833333334</v>
-      </c>
-      <c r="K19" s="34">
+          <t>20C → 20B</t>
+        </is>
+      </c>
+      <c r="H19" s="11" t="n">
+        <v>46298.95833333334</v>
+      </c>
+      <c r="I19" s="11" t="n">
+        <v>46299.41666666666</v>
+      </c>
+      <c r="J19" s="11" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="K19" s="28">
         <f>(I19-H19)*24</f>
         <v/>
       </c>
-      <c r="L19" s="34">
+      <c r="L19" s="28">
         <f>(J19-I19)*24</f>
         <v/>
       </c>
-      <c r="M19" s="17" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N19" s="17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O19" s="17" t="inlineStr">
+      <c r="M19" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N19" s="23" t="inlineStr"/>
+      <c r="O19" s="23" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -11861,34 +12759,34 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>YM IMPROVEMENT</t>
+          <t>SAWASDEE SPICA</t>
         </is>
       </c>
       <c r="C20" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>46296</v>
+        <v>46299</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="F20" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>20C → 20B</t>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H20" s="11" t="n">
-        <v>46298.95833333334</v>
+        <v>46300.875</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>46299.41666666666</v>
+        <v>46301.54166666666</v>
       </c>
       <c r="J20" s="11" t="n">
-        <v>46300.5</v>
+        <v>46303.54166666666</v>
       </c>
       <c r="K20" s="28">
         <f>(I20-H20)*24</f>
@@ -11918,34 +12816,34 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE SPICA</t>
+          <t>SITC HOCHIMINH</t>
         </is>
       </c>
       <c r="C21" s="23" t="n">
-        <v>564</v>
+        <v>470</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>46299</v>
+        <v>46301</v>
       </c>
       <c r="E21" s="10" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="F21" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>4</v>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20B</t>
         </is>
       </c>
       <c r="H21" s="11" t="n">
-        <v>46300.875</v>
+        <v>46302.625</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>46301.54166666666</v>
+        <v>46303.58333333334</v>
       </c>
       <c r="J21" s="11" t="n">
-        <v>46303.54166666666</v>
+        <v>46304.70833333334</v>
       </c>
       <c r="K21" s="28">
         <f>(I21-H21)*24</f>
@@ -11975,34 +12873,34 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>SITC HOCHIMINH</t>
+          <t>INDURO</t>
         </is>
       </c>
       <c r="C22" s="23" t="n">
-        <v>470</v>
+        <v>565</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="F22" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20B</t>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H22" s="11" t="n">
-        <v>46302.625</v>
+        <v>46304.25</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>46303.58333333334</v>
+        <v>46304.66666666666</v>
       </c>
       <c r="J22" s="11" t="n">
-        <v>46304.70833333334</v>
+        <v>46306.16666666666</v>
       </c>
       <c r="K22" s="28">
         <f>(I22-H22)*24</f>
@@ -12032,34 +12930,34 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>INDURO</t>
+          <t>XIN MING ZHOU 102</t>
         </is>
       </c>
       <c r="C23" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D23" s="10" t="n">
         <v>46302</v>
       </c>
       <c r="E23" s="10" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="F23" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>5</v>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>20F → 20B</t>
         </is>
       </c>
       <c r="H23" s="11" t="n">
-        <v>46304.25</v>
+        <v>46305.875</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>46304.66666666666</v>
+        <v>46306.20833333334</v>
       </c>
       <c r="J23" s="11" t="n">
-        <v>46306.16666666666</v>
+        <v>46307.08333333334</v>
       </c>
       <c r="K23" s="28">
         <f>(I23-H23)*24</f>
@@ -12089,34 +12987,34 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 102</t>
+          <t>CEBU</t>
         </is>
       </c>
       <c r="C24" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="E24" s="10" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="F24" s="23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>20F → 20B</t>
+          <t>20AB → 20B</t>
         </is>
       </c>
       <c r="H24" s="11" t="n">
-        <v>46305.875</v>
+        <v>46307.91666666666</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>46306.20833333334</v>
+        <v>46308.25</v>
       </c>
       <c r="J24" s="11" t="n">
-        <v>46307.08333333334</v>
+        <v>46309.66666666666</v>
       </c>
       <c r="K24" s="28">
         <f>(I24-H24)*24</f>
@@ -12132,10 +13030,9 @@
         </is>
       </c>
       <c r="N24" s="23" t="inlineStr"/>
-      <c r="O24" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="O24" s="23">
+        <f>IF(J24&lt;=$B$3,"Sailed",IF(I24&lt;=$B$3,"Alongside",IF(H24&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -12146,34 +13043,34 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>CEBU</t>
+          <t>WAN HAI 173</t>
         </is>
       </c>
       <c r="C25" s="23" t="n">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="E25" s="10" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="F25" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20B</t>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H25" s="11" t="n">
-        <v>46307.91666666666</v>
+        <v>46309.04166666666</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>46308.25</v>
+        <v>46309.66666666666</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>46309.66666666666</v>
+        <v>46310.29166666666</v>
       </c>
       <c r="K25" s="28">
         <f>(I25-H25)*24</f>
@@ -12202,17 +13099,17 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 173</t>
+          <t>WAN HAI 176</t>
         </is>
       </c>
       <c r="C26" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D26" s="10" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="E26" s="10" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="F26" s="23" t="n">
         <v>1</v>
@@ -12223,13 +13120,13 @@
         </is>
       </c>
       <c r="H26" s="11" t="n">
-        <v>46309.33333333334</v>
+        <v>46310.45833333334</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>46309.66666666666</v>
+        <v>46310.45833333334</v>
       </c>
       <c r="J26" s="11" t="n">
-        <v>46310.29166666666</v>
+        <v>46311.66666666666</v>
       </c>
       <c r="K26" s="28">
         <f>(I26-H26)*24</f>
@@ -12557,10 +13454,10 @@
         <v>46305</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="F32" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -12613,10 +13510,10 @@
         <v>46293</v>
       </c>
       <c r="E33" s="10" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="F33" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
@@ -12642,7 +13539,7 @@
       </c>
       <c r="M33" s="23" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N33" s="23" t="inlineStr"/>
@@ -12652,114 +13549,113 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="29" t="inlineStr">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>KHARIS HERITAGE</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="n">
+        <v>482</v>
+      </c>
+      <c r="D34" s="10" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E34" s="10" t="n">
+        <v>46308</v>
+      </c>
+      <c r="F34" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G34" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20B → 20C</t>
+        </is>
+      </c>
+      <c r="H34" s="11" t="n">
+        <v>46310.04166666666</v>
+      </c>
+      <c r="I34" s="11" t="n">
+        <v>46310.29166666666</v>
+      </c>
+      <c r="J34" s="11" t="n">
+        <v>46311.29166666666</v>
+      </c>
+      <c r="K34" s="28">
+        <f>(I34-H34)*24</f>
+        <v/>
+      </c>
+      <c r="L34" s="28">
+        <f>(J34-I34)*24</f>
+        <v/>
+      </c>
+      <c r="M34" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N34" s="23" t="inlineStr"/>
+      <c r="O34" s="23">
+        <f>IF(J34&lt;=$B$3,"Sailed",IF(I34&lt;=$B$3,"Alongside",IF(H34&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="29" t="inlineStr">
         <is>
           <t>20D</t>
         </is>
       </c>
-      <c r="B34" s="29" t="inlineStr">
+      <c r="B35" s="29" t="inlineStr">
         <is>
           <t>BANGKOK</t>
         </is>
       </c>
-      <c r="C34" s="24" t="n">
+      <c r="C35" s="24" t="n">
         <v>551</v>
       </c>
-      <c r="D34" s="21" t="n">
+      <c r="D35" s="21" t="n">
         <v>46293</v>
       </c>
-      <c r="E34" s="21" t="n">
+      <c r="E35" s="21" t="n">
         <v>46294</v>
       </c>
-      <c r="F34" s="24" t="n">
+      <c r="F35" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="G34" s="30" t="inlineStr">
+      <c r="G35" s="30" t="inlineStr">
         <is>
           <t>20D</t>
         </is>
       </c>
-      <c r="H34" s="31" t="n">
+      <c r="H35" s="31" t="n">
         <v>46292.54166666666</v>
       </c>
-      <c r="I34" s="31" t="n">
+      <c r="I35" s="31" t="n">
         <v>46292.625</v>
       </c>
-      <c r="J34" s="31" t="n">
+      <c r="J35" s="31" t="n">
         <v>46294.58333333334</v>
       </c>
-      <c r="K34" s="32">
-        <f>(I34-H34)*24</f>
-        <v/>
-      </c>
-      <c r="L34" s="32">
-        <f>(J34-I34)*24</f>
-        <v/>
-      </c>
-      <c r="M34" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N34" s="24" t="inlineStr"/>
-      <c r="O34" s="24" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>HARI BHUM (Barge)</t>
-        </is>
-      </c>
-      <c r="C35" s="23" t="n">
-        <v>259</v>
-      </c>
-      <c r="D35" s="10" t="n">
-        <v>46297</v>
-      </c>
-      <c r="E35" s="10" t="n">
-        <v>46298</v>
-      </c>
-      <c r="F35" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="H35" s="11" t="n">
-        <v>46298.20833333334</v>
-      </c>
-      <c r="I35" s="11" t="n">
-        <v>46298.29166666666</v>
-      </c>
-      <c r="J35" s="11" t="n">
-        <v>46298.66666666666</v>
-      </c>
-      <c r="K35" s="28">
+      <c r="K35" s="32">
         <f>(I35-H35)*24</f>
         <v/>
       </c>
-      <c r="L35" s="28">
+      <c r="L35" s="32">
         <f>(J35-I35)*24</f>
         <v/>
       </c>
-      <c r="M35" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N35" s="23" t="inlineStr"/>
-      <c r="O35" s="23" t="inlineStr">
+      <c r="M35" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N35" s="24" t="inlineStr"/>
+      <c r="O35" s="24" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -12773,20 +13669,20 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>MTT BANGKOK</t>
+          <t>HARI BHUM (Barge)</t>
         </is>
       </c>
       <c r="C36" s="23" t="n">
-        <v>564</v>
+        <v>259</v>
       </c>
       <c r="D36" s="10" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="E36" s="10" t="n">
-        <v>46303</v>
+        <v>46298</v>
       </c>
       <c r="F36" s="23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
@@ -12794,13 +13690,13 @@
         </is>
       </c>
       <c r="H36" s="11" t="n">
-        <v>46302.54166666666</v>
+        <v>46298.20833333334</v>
       </c>
       <c r="I36" s="11" t="n">
-        <v>46302.58333333334</v>
+        <v>46298.29166666666</v>
       </c>
       <c r="J36" s="11" t="n">
-        <v>46304.08333333334</v>
+        <v>46298.66666666666</v>
       </c>
       <c r="K36" s="28">
         <f>(I36-H36)*24</f>
@@ -12830,34 +13726,34 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>HE JIN</t>
+          <t>MTT BANGKOK</t>
         </is>
       </c>
       <c r="C37" s="23" t="n">
-        <v>552</v>
+        <v>564</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="E37" s="10" t="n">
-        <v>46305</v>
+        <v>46303</v>
       </c>
       <c r="F37" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G37" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 22A → 20D</t>
+        <v>4</v>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H37" s="11" t="n">
-        <v>46304</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="I37" s="11" t="n">
-        <v>46304</v>
+        <v>46302.58333333334</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>46305.54166666666</v>
+        <v>46304.08333333334</v>
       </c>
       <c r="K37" s="28">
         <f>(I37-H37)*24</f>
@@ -12887,34 +13783,34 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>CUL HAIPHONG</t>
+          <t>HE JIN</t>
         </is>
       </c>
       <c r="C38" s="23" t="n">
-        <v>458</v>
+        <v>552</v>
       </c>
       <c r="D38" s="10" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E38" s="10" t="n">
         <v>46305</v>
       </c>
       <c r="F38" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>20B → 20D</t>
+          <t>20B → 20AB → 22A → 20D</t>
         </is>
       </c>
       <c r="H38" s="11" t="n">
-        <v>46304.83333333334</v>
+        <v>46304</v>
       </c>
       <c r="I38" s="11" t="n">
-        <v>46305.66666666666</v>
+        <v>46304</v>
       </c>
       <c r="J38" s="11" t="n">
-        <v>46306.25</v>
+        <v>46305.54166666666</v>
       </c>
       <c r="K38" s="28">
         <f>(I38-H38)*24</f>
@@ -12926,7 +13822,7 @@
       </c>
       <c r="M38" s="23" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N38" s="23" t="inlineStr"/>
@@ -12944,34 +13840,34 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>INCEDA</t>
+          <t>CUL HAIPHONG</t>
         </is>
       </c>
       <c r="C39" s="23" t="n">
-        <v>564</v>
+        <v>458</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E39" s="10" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="F39" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
+        <v>4</v>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20D</t>
         </is>
       </c>
       <c r="H39" s="11" t="n">
-        <v>46305.70833333334</v>
+        <v>46304.83333333334</v>
       </c>
       <c r="I39" s="11" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="J39" s="11" t="n">
         <v>46306.25</v>
-      </c>
-      <c r="J39" s="11" t="n">
-        <v>46307.58333333334</v>
       </c>
       <c r="K39" s="28">
         <f>(I39-H39)*24</f>
@@ -12983,13 +13879,14 @@
       </c>
       <c r="M39" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="N39" s="23" t="inlineStr"/>
-      <c r="O39" s="23">
-        <f>IF(J39&lt;=$B$3,"Sailed",IF(I39&lt;=$B$3,"Alongside",IF(H39&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O39" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -13000,34 +13897,34 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE SUNRISE</t>
+          <t>INCEDA</t>
         </is>
       </c>
       <c r="C40" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D40" s="10" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="E40" s="10" t="n">
         <v>46307</v>
       </c>
       <c r="F40" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G40" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20D</t>
+        <v>5</v>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H40" s="11" t="n">
-        <v>46307.16666666666</v>
+        <v>46305.70833333334</v>
       </c>
       <c r="I40" s="11" t="n">
-        <v>46307.66666666666</v>
+        <v>46306.25</v>
       </c>
       <c r="J40" s="11" t="n">
-        <v>46309.20833333334</v>
+        <v>46307.58333333334</v>
       </c>
       <c r="K40" s="28">
         <f>(I40-H40)*24</f>
@@ -13043,9 +13940,10 @@
         </is>
       </c>
       <c r="N40" s="23" t="inlineStr"/>
-      <c r="O40" s="23">
-        <f>IF(J40&lt;=$B$3,"Sailed",IF(I40&lt;=$B$3,"Alongside",IF(H40&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O40" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="41">
@@ -13056,34 +13954,34 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>KHUNA BHUM</t>
+          <t>SAWASDEE SUNRISE</t>
         </is>
       </c>
       <c r="C41" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D41" s="10" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="E41" s="10" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="F41" s="23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20D</t>
+          <t>20F → 20D</t>
         </is>
       </c>
       <c r="H41" s="11" t="n">
-        <v>46308.29166666666</v>
+        <v>46307.16666666666</v>
       </c>
       <c r="I41" s="11" t="n">
+        <v>46307.66666666666</v>
+      </c>
+      <c r="J41" s="11" t="n">
         <v>46309.20833333334</v>
-      </c>
-      <c r="J41" s="11" t="n">
-        <v>46309.91666666666</v>
       </c>
       <c r="K41" s="28">
         <f>(I41-H41)*24</f>
@@ -13095,7 +13993,7 @@
       </c>
       <c r="M41" s="23" t="inlineStr">
         <is>
-          <t>7B</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N41" s="23" t="inlineStr"/>
@@ -13105,98 +14003,97 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="29" t="inlineStr">
-        <is>
-          <t>20E</t>
-        </is>
-      </c>
-      <c r="B42" s="29" t="inlineStr">
-        <is>
-          <t>TS CHIBA</t>
-        </is>
-      </c>
-      <c r="C42" s="24" t="n">
-        <v>485</v>
-      </c>
-      <c r="D42" s="21" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E42" s="21" t="n">
-        <v>46293</v>
-      </c>
-      <c r="F42" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" s="30" t="inlineStr">
-        <is>
-          <t>20E</t>
-        </is>
-      </c>
-      <c r="H42" s="31" t="n">
-        <v>46293.29166666666</v>
-      </c>
-      <c r="I42" s="31" t="n">
-        <v>46293.29166666666</v>
-      </c>
-      <c r="J42" s="31" t="n">
-        <v>46294.16666666666</v>
-      </c>
-      <c r="K42" s="32">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>KHUNA BHUM</t>
+        </is>
+      </c>
+      <c r="C42" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D42" s="10" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E42" s="10" t="n">
+        <v>46308</v>
+      </c>
+      <c r="F42" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="G42" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20D</t>
+        </is>
+      </c>
+      <c r="H42" s="11" t="n">
+        <v>46308.45833333334</v>
+      </c>
+      <c r="I42" s="11" t="n">
+        <v>46309.20833333334</v>
+      </c>
+      <c r="J42" s="11" t="n">
+        <v>46309.91666666666</v>
+      </c>
+      <c r="K42" s="28">
         <f>(I42-H42)*24</f>
         <v/>
       </c>
-      <c r="L42" s="32">
+      <c r="L42" s="28">
         <f>(J42-I42)*24</f>
         <v/>
       </c>
-      <c r="M42" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N42" s="24" t="inlineStr"/>
-      <c r="O42" s="24" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="M42" s="23" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="N42" s="23" t="inlineStr"/>
+      <c r="O42" s="23">
+        <f>IF(J42&lt;=$B$3,"Sailed",IF(I42&lt;=$B$3,"Alongside",IF(H42&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>20E</t>
+          <t>20D</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>MITRA BHUM</t>
+          <t>WAN HAI 175</t>
         </is>
       </c>
       <c r="C43" s="23" t="n">
-        <v>485</v>
+        <v>565</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>46293</v>
+        <v>46308</v>
       </c>
       <c r="E43" s="10" t="n">
-        <v>46295</v>
+        <v>46308</v>
       </c>
       <c r="F43" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G43" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20E</t>
+        <v>1</v>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H43" s="11" t="n">
-        <v>46295.125</v>
+        <v>46310.04166666666</v>
       </c>
       <c r="I43" s="11" t="n">
-        <v>46295.20833333334</v>
+        <v>46310.29166666666</v>
       </c>
       <c r="J43" s="11" t="n">
-        <v>46295.75</v>
+        <v>46311.70833333334</v>
       </c>
       <c r="K43" s="28">
         <f>(I43-H43)*24</f>
@@ -13212,125 +14109,120 @@
         </is>
       </c>
       <c r="N43" s="23" t="inlineStr"/>
-      <c r="O43" s="23" t="inlineStr">
+      <c r="O43" s="23">
+        <f>IF(J43&lt;=$B$3,"Sailed",IF(I43&lt;=$B$3,"Alongside",IF(H43&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="29" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B44" s="29" t="inlineStr">
+        <is>
+          <t>TS CHIBA</t>
+        </is>
+      </c>
+      <c r="C44" s="24" t="n">
+        <v>485</v>
+      </c>
+      <c r="D44" s="21" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E44" s="21" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F44" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="30" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="H44" s="31" t="n">
+        <v>46293.29166666666</v>
+      </c>
+      <c r="I44" s="31" t="n">
+        <v>46293.29166666666</v>
+      </c>
+      <c r="J44" s="31" t="n">
+        <v>46294.16666666666</v>
+      </c>
+      <c r="K44" s="32">
+        <f>(I44-H44)*24</f>
+        <v/>
+      </c>
+      <c r="L44" s="32">
+        <f>(J44-I44)*24</f>
+        <v/>
+      </c>
+      <c r="M44" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N44" s="24" t="inlineStr"/>
+      <c r="O44" s="24" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>20E</t>
         </is>
       </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>WAN HAI 278</t>
-        </is>
-      </c>
-      <c r="C44" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D44" s="10" t="n">
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>MITRA BHUM</t>
+        </is>
+      </c>
+      <c r="C45" s="23" t="n">
+        <v>485</v>
+      </c>
+      <c r="D45" s="10" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E45" s="10" t="n">
         <v>46295</v>
       </c>
-      <c r="E44" s="10" t="n">
-        <v>46300</v>
-      </c>
-      <c r="F44" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="G44" s="6" t="inlineStr">
+      <c r="F45" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
         <is>
           <t>20F → 20E</t>
         </is>
       </c>
-      <c r="H44" s="11" t="n">
-        <v>46297.75</v>
-      </c>
-      <c r="I44" s="11" t="n">
-        <v>46298.41666666666</v>
-      </c>
-      <c r="J44" s="11" t="n">
-        <v>46300.45833333334</v>
-      </c>
-      <c r="K44" s="28">
-        <f>(I44-H44)*24</f>
-        <v/>
-      </c>
-      <c r="L44" s="28">
-        <f>(J44-I44)*24</f>
-        <v/>
-      </c>
-      <c r="M44" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N44" s="23" t="inlineStr"/>
-      <c r="O44" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="35" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="B45" s="35" t="inlineStr">
-        <is>
-          <t>JARU BHUM</t>
-        </is>
-      </c>
-      <c r="C45" s="22" t="n">
-        <v>564</v>
-      </c>
-      <c r="D45" s="14" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E45" s="14" t="n">
-        <v>46293</v>
-      </c>
-      <c r="F45" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G45" s="36" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="H45" s="37" t="n">
-        <v>46293.33333333334</v>
-      </c>
-      <c r="I45" s="37" t="n">
-        <v>46293.33333333334</v>
-      </c>
-      <c r="J45" s="37" t="n">
-        <v>46294.16666666666</v>
-      </c>
-      <c r="K45" s="38">
+      <c r="H45" s="11" t="n">
+        <v>46295.125</v>
+      </c>
+      <c r="I45" s="11" t="n">
+        <v>46295.20833333334</v>
+      </c>
+      <c r="J45" s="11" t="n">
+        <v>46295.75</v>
+      </c>
+      <c r="K45" s="28">
         <f>(I45-H45)*24</f>
         <v/>
       </c>
-      <c r="L45" s="38">
+      <c r="L45" s="28">
         <f>(J45-I45)*24</f>
         <v/>
       </c>
-      <c r="M45" s="22" t="inlineStr">
-        <is>
-          <t>7B</t>
-        </is>
-      </c>
-      <c r="N45" s="22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O45" s="22" t="inlineStr">
+      <c r="M45" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N45" s="23" t="inlineStr"/>
+      <c r="O45" s="23" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -13339,39 +14231,39 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>20F</t>
+          <t>20E</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>HOPE C</t>
+          <t>WAN HAI 278</t>
         </is>
       </c>
       <c r="C46" s="23" t="n">
-        <v>481</v>
+        <v>564</v>
       </c>
       <c r="D46" s="10" t="n">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="E46" s="10" t="n">
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="F46" s="23" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>20E → 20F</t>
+          <t>20F → 20E</t>
         </is>
       </c>
       <c r="H46" s="11" t="n">
-        <v>46294.70833333334</v>
+        <v>46297.75</v>
       </c>
       <c r="I46" s="11" t="n">
-        <v>46294.70833333334</v>
+        <v>46298.41666666666</v>
       </c>
       <c r="J46" s="11" t="n">
-        <v>46295.66666666666</v>
+        <v>46300.45833333334</v>
       </c>
       <c r="K46" s="28">
         <f>(I46-H46)*24</f>
@@ -13394,57 +14286,61 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+      <c r="A47" s="35" t="inlineStr">
         <is>
           <t>20F</t>
         </is>
       </c>
-      <c r="B47" s="4" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="C47" s="23" t="n">
+      <c r="B47" s="35" t="inlineStr">
+        <is>
+          <t>JARU BHUM</t>
+        </is>
+      </c>
+      <c r="C47" s="22" t="n">
         <v>564</v>
       </c>
-      <c r="D47" s="10" t="n">
-        <v>46295</v>
-      </c>
-      <c r="E47" s="10" t="n">
-        <v>46298</v>
-      </c>
-      <c r="F47" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G47" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20F</t>
-        </is>
-      </c>
-      <c r="H47" s="11" t="n">
-        <v>46297.29166666666</v>
-      </c>
-      <c r="I47" s="11" t="n">
-        <v>46297.45833333334</v>
-      </c>
-      <c r="J47" s="11" t="n">
-        <v>46298.70833333334</v>
-      </c>
-      <c r="K47" s="28">
+      <c r="D47" s="14" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E47" s="14" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F47" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="36" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="H47" s="37" t="n">
+        <v>46293.33333333334</v>
+      </c>
+      <c r="I47" s="37" t="n">
+        <v>46293.33333333334</v>
+      </c>
+      <c r="J47" s="37" t="n">
+        <v>46294.16666666666</v>
+      </c>
+      <c r="K47" s="38">
         <f>(I47-H47)*24</f>
         <v/>
       </c>
-      <c r="L47" s="28">
+      <c r="L47" s="38">
         <f>(J47-I47)*24</f>
         <v/>
       </c>
-      <c r="M47" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N47" s="23" t="inlineStr"/>
-      <c r="O47" s="23" t="inlineStr">
+      <c r="M47" s="22" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="N47" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O47" s="22" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -13458,34 +14354,34 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 98</t>
+          <t>HOPE C</t>
         </is>
       </c>
       <c r="C48" s="23" t="n">
-        <v>564</v>
+        <v>481</v>
       </c>
       <c r="D48" s="10" t="n">
-        <v>46297</v>
+        <v>46293</v>
       </c>
       <c r="E48" s="10" t="n">
-        <v>46299</v>
+        <v>46295</v>
       </c>
       <c r="F48" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="G48" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+      <c r="G48" s="6" t="inlineStr">
+        <is>
+          <t>20E → 20F</t>
         </is>
       </c>
       <c r="H48" s="11" t="n">
-        <v>46299.375</v>
+        <v>46294.70833333334</v>
       </c>
       <c r="I48" s="11" t="n">
-        <v>46299.375</v>
+        <v>46294.70833333334</v>
       </c>
       <c r="J48" s="11" t="n">
-        <v>46300.375</v>
+        <v>46295.66666666666</v>
       </c>
       <c r="K48" s="28">
         <f>(I48-H48)*24</f>
@@ -13515,34 +14411,34 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>XIN AN</t>
+          <t>KMTC BANGKOK</t>
         </is>
       </c>
       <c r="C49" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D49" s="10" t="n">
-        <v>46300</v>
+        <v>46295</v>
       </c>
       <c r="E49" s="10" t="n">
-        <v>46304</v>
+        <v>46298</v>
       </c>
       <c r="F49" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G49" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+        <v>4</v>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20F</t>
         </is>
       </c>
       <c r="H49" s="11" t="n">
-        <v>46302.54166666666</v>
+        <v>46297.29166666666</v>
       </c>
       <c r="I49" s="11" t="n">
-        <v>46302.58333333334</v>
+        <v>46297.45833333334</v>
       </c>
       <c r="J49" s="11" t="n">
-        <v>46304.54166666666</v>
+        <v>46298.70833333334</v>
       </c>
       <c r="K49" s="28">
         <f>(I49-H49)*24</f>
@@ -13572,34 +14468,34 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE ATLANTIC</t>
+          <t>XIN MING ZHOU 98</t>
         </is>
       </c>
       <c r="C50" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D50" s="10" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="E50" s="10" t="n">
-        <v>46306</v>
+        <v>46299</v>
       </c>
       <c r="F50" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>20C → 20D → 20F</t>
+        <v>3</v>
+      </c>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
         </is>
       </c>
       <c r="H50" s="11" t="n">
-        <v>46302.83333333334</v>
+        <v>46299.375</v>
       </c>
       <c r="I50" s="11" t="n">
-        <v>46304.625</v>
+        <v>46299.375</v>
       </c>
       <c r="J50" s="11" t="n">
-        <v>46306.5</v>
+        <v>46300.375</v>
       </c>
       <c r="K50" s="28">
         <f>(I50-H50)*24</f>
@@ -13629,34 +14525,34 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>JOSCO SHINE</t>
+          <t>XIN AN</t>
         </is>
       </c>
       <c r="C51" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D51" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E51" s="10" t="n">
         <v>46304</v>
       </c>
-      <c r="E51" s="10" t="n">
-        <v>46307</v>
-      </c>
       <c r="F51" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G51" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 20F</t>
+        <v>5</v>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
         </is>
       </c>
       <c r="H51" s="11" t="n">
-        <v>46307.45833333334</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="I51" s="11" t="n">
-        <v>46307.625</v>
+        <v>46302.58333333334</v>
       </c>
       <c r="J51" s="11" t="n">
-        <v>46308.25</v>
+        <v>46304.54166666666</v>
       </c>
       <c r="K51" s="28">
         <f>(I51-H51)*24</f>
@@ -13672,9 +14568,10 @@
         </is>
       </c>
       <c r="N51" s="23" t="inlineStr"/>
-      <c r="O51" s="23">
-        <f>IF(J51&lt;=$B$3,"Sailed",IF(I51&lt;=$B$3,"Alongside",IF(H51&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O51" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="52">
@@ -13685,34 +14582,34 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>ALS SUMIRE</t>
+          <t>SAWASDEE ATLANTIC</t>
         </is>
       </c>
       <c r="C52" s="23" t="n">
-        <v>537</v>
+        <v>564</v>
       </c>
       <c r="D52" s="10" t="n">
-        <v>46294</v>
+        <v>46300</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="F52" s="23" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>20F → 20D → 20C → 20B → 20F</t>
+          <t>20C → 20D → 20F</t>
         </is>
       </c>
       <c r="H52" s="11" t="n">
-        <v>46307.91666666666</v>
+        <v>46302.83333333334</v>
       </c>
       <c r="I52" s="11" t="n">
-        <v>46308.25</v>
+        <v>46304.625</v>
       </c>
       <c r="J52" s="11" t="n">
-        <v>46309.25</v>
+        <v>46306.5</v>
       </c>
       <c r="K52" s="28">
         <f>(I52-H52)*24</f>
@@ -13724,13 +14621,14 @@
       </c>
       <c r="M52" s="23" t="inlineStr">
         <is>
-          <t>1C</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N52" s="23" t="inlineStr"/>
-      <c r="O52" s="23">
-        <f>IF(J52&lt;=$B$3,"Sailed",IF(I52&lt;=$B$3,"Alongside",IF(H52&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O52" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="53">
@@ -13741,34 +14639,34 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE INCHEON</t>
+          <t>JOSCO SHINE</t>
         </is>
       </c>
       <c r="C53" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D53" s="10" t="n">
-        <v>46307</v>
+        <v>46304</v>
       </c>
       <c r="E53" s="10" t="n">
         <v>46307</v>
       </c>
       <c r="F53" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G53" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+        <v>4</v>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20AB → 20F</t>
         </is>
       </c>
       <c r="H53" s="11" t="n">
-        <v>46308.625</v>
+        <v>46307.45833333334</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>46309.25</v>
+        <v>46307.625</v>
       </c>
       <c r="J53" s="11" t="n">
-        <v>46310.625</v>
+        <v>46308.25</v>
       </c>
       <c r="K53" s="28">
         <f>(I53-H53)*24</f>
@@ -13784,20 +14682,133 @@
         </is>
       </c>
       <c r="N53" s="23" t="inlineStr"/>
-      <c r="O53" s="23">
-        <f>IF(J53&lt;=$B$3,"Sailed",IF(I53&lt;=$B$3,"Alongside",IF(H53&lt;=$B$3,"At anchorage","Expected")))</f>
+      <c r="O53" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>ALS SUMIRE</t>
+        </is>
+      </c>
+      <c r="C54" s="23" t="n">
+        <v>537</v>
+      </c>
+      <c r="D54" s="10" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E54" s="10" t="n">
+        <v>46308</v>
+      </c>
+      <c r="F54" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>20F → 20D → 20C → 20B → 20F</t>
+        </is>
+      </c>
+      <c r="H54" s="11" t="n">
+        <v>46307.91666666666</v>
+      </c>
+      <c r="I54" s="11" t="n">
+        <v>46308.25</v>
+      </c>
+      <c r="J54" s="11" t="n">
+        <v>46309.25</v>
+      </c>
+      <c r="K54" s="28">
+        <f>(I54-H54)*24</f>
+        <v/>
+      </c>
+      <c r="L54" s="28">
+        <f>(J54-I54)*24</f>
+        <v/>
+      </c>
+      <c r="M54" s="23" t="inlineStr">
+        <is>
+          <t>1C</t>
+        </is>
+      </c>
+      <c r="N54" s="23" t="inlineStr"/>
+      <c r="O54" s="23">
+        <f>IF(J54&lt;=$B$3,"Sailed",IF(I54&lt;=$B$3,"Alongside",IF(H54&lt;=$B$3,"At anchorage","Expected")))</f>
         <v/>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>48 vessels in total. Orange cells: marked on sheet, or the vessel changed berth.</t>
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>SAWASDEE INCHEON</t>
+        </is>
+      </c>
+      <c r="C55" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D55" s="10" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E55" s="10" t="n">
+        <v>46308</v>
+      </c>
+      <c r="F55" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="H55" s="11" t="n">
+        <v>46308.625</v>
+      </c>
+      <c r="I55" s="11" t="n">
+        <v>46309.25</v>
+      </c>
+      <c r="J55" s="11" t="n">
+        <v>46310.625</v>
+      </c>
+      <c r="K55" s="28">
+        <f>(I55-H55)*24</f>
+        <v/>
+      </c>
+      <c r="L55" s="28">
+        <f>(J55-I55)*24</f>
+        <v/>
+      </c>
+      <c r="M55" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N55" s="23" t="inlineStr"/>
+      <c r="O55" s="23">
+        <f>IF(J55&lt;=$B$3,"Sailed",IF(I55&lt;=$B$3,"Alongside",IF(H55&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>50 vessels in total. Orange cells: marked on sheet, or the vessel changed berth.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:O53"/>
+  <autoFilter ref="A5:O55"/>
   <mergeCells count="1">
     <mergeCell ref="A2:O2"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add 14 Oct 2026 ship movement data; show vessels listed without times as Schedule TBA
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -26,10 +26,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 Oct 2026" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Oct 2026" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Oct 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 Oct 2026" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$O$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$50</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$O$57</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -673,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q54"/>
+  <dimension ref="A1:R57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -693,6 +694,7 @@
     <col width="44" customWidth="1" min="15" max="15"/>
     <col width="44" customWidth="1" min="16" max="16"/>
     <col width="44" customWidth="1" min="17" max="17"/>
+    <col width="44" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -793,6 +795,11 @@
       <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>13 Oct 2026</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>14 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -830,6 +837,7 @@
       <c r="O5" s="5" t="inlineStr"/>
       <c r="P5" s="5" t="inlineStr"/>
       <c r="Q5" s="5" t="inlineStr"/>
+      <c r="R5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -869,6 +877,7 @@
       <c r="O6" s="5" t="inlineStr"/>
       <c r="P6" s="5" t="inlineStr"/>
       <c r="Q6" s="5" t="inlineStr"/>
+      <c r="R6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -900,6 +909,7 @@
       <c r="O7" s="5" t="inlineStr"/>
       <c r="P7" s="5" t="inlineStr"/>
       <c r="Q7" s="5" t="inlineStr"/>
+      <c r="R7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -935,6 +945,7 @@
       <c r="O8" s="5" t="inlineStr"/>
       <c r="P8" s="5" t="inlineStr"/>
       <c r="Q8" s="5" t="inlineStr"/>
+      <c r="R8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -970,6 +981,11 @@
       <c r="O9" s="5" t="inlineStr"/>
       <c r="P9" s="5" t="inlineStr"/>
       <c r="Q9" s="5" t="inlineStr"/>
+      <c r="R9" s="5" t="inlineStr">
+        <is>
+          <t>listed at 20B without times (returns, schedule TBA)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1001,6 +1017,7 @@
       <c r="O10" s="5" t="inlineStr"/>
       <c r="P10" s="5" t="inlineStr"/>
       <c r="Q10" s="5" t="inlineStr"/>
+      <c r="R10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1040,6 +1057,7 @@
       <c r="O11" s="5" t="inlineStr"/>
       <c r="P11" s="5" t="inlineStr"/>
       <c r="Q11" s="5" t="inlineStr"/>
+      <c r="R11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1071,6 +1089,7 @@
       <c r="O12" s="5" t="inlineStr"/>
       <c r="P12" s="5" t="inlineStr"/>
       <c r="Q12" s="5" t="inlineStr"/>
+      <c r="R12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1110,6 +1129,7 @@
       <c r="O13" s="5" t="inlineStr"/>
       <c r="P13" s="5" t="inlineStr"/>
       <c r="Q13" s="5" t="inlineStr"/>
+      <c r="R13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1157,6 +1177,7 @@
       <c r="O14" s="5" t="inlineStr"/>
       <c r="P14" s="5" t="inlineStr"/>
       <c r="Q14" s="5" t="inlineStr"/>
+      <c r="R14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1204,6 +1225,11 @@
           <t>expected · 20C (shift 4A no longer shown)</t>
         </is>
       </c>
+      <c r="R15" s="6" t="inlineStr">
+        <is>
+          <t>at anchorage → 20B (shift 4A, ETA 14/03→14/01, P.B 14/14→14/15)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1251,6 +1277,11 @@
           <t>expected → 20C (returns for a new call, ETA 15/01)</t>
         </is>
       </c>
+      <c r="R16" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20B</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1312,6 +1343,11 @@
       <c r="Q17" s="5" t="inlineStr">
         <is>
           <t>alongside · 20F (P.B 13/06, ETD 14/06, 1C)</t>
+        </is>
+      </c>
+      <c r="R17" s="5" t="inlineStr">
+        <is>
+          <t>sailed (14/06)</t>
         </is>
       </c>
     </row>
@@ -1357,6 +1393,7 @@
       <c r="O18" s="5" t="inlineStr"/>
       <c r="P18" s="5" t="inlineStr"/>
       <c r="Q18" s="5" t="inlineStr"/>
+      <c r="R18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1408,6 +1445,7 @@
       <c r="O19" s="5" t="inlineStr"/>
       <c r="P19" s="5" t="inlineStr"/>
       <c r="Q19" s="5" t="inlineStr"/>
+      <c r="R19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1459,6 +1497,7 @@
       <c r="O20" s="5" t="inlineStr"/>
       <c r="P20" s="5" t="inlineStr"/>
       <c r="Q20" s="5" t="inlineStr"/>
+      <c r="R20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1506,6 +1545,7 @@
       <c r="O21" s="5" t="inlineStr"/>
       <c r="P21" s="5" t="inlineStr"/>
       <c r="Q21" s="5" t="inlineStr"/>
+      <c r="R21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1549,6 +1589,7 @@
       <c r="O22" s="5" t="inlineStr"/>
       <c r="P22" s="5" t="inlineStr"/>
       <c r="Q22" s="5" t="inlineStr"/>
+      <c r="R22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1604,6 +1645,7 @@
       <c r="O23" s="5" t="inlineStr"/>
       <c r="P23" s="5" t="inlineStr"/>
       <c r="Q23" s="5" t="inlineStr"/>
+      <c r="R23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1655,6 +1697,7 @@
       <c r="O24" s="5" t="inlineStr"/>
       <c r="P24" s="5" t="inlineStr"/>
       <c r="Q24" s="5" t="inlineStr"/>
+      <c r="R24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1690,6 +1733,7 @@
       <c r="O25" s="5" t="inlineStr"/>
       <c r="P25" s="5" t="inlineStr"/>
       <c r="Q25" s="5" t="inlineStr"/>
+      <c r="R25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1729,6 +1773,7 @@
       <c r="O26" s="5" t="inlineStr"/>
       <c r="P26" s="5" t="inlineStr"/>
       <c r="Q26" s="5" t="inlineStr"/>
+      <c r="R26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1780,6 +1825,7 @@
       <c r="O27" s="5" t="inlineStr"/>
       <c r="P27" s="5" t="inlineStr"/>
       <c r="Q27" s="5" t="inlineStr"/>
+      <c r="R27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1827,6 +1873,7 @@
       <c r="O28" s="5" t="inlineStr"/>
       <c r="P28" s="5" t="inlineStr"/>
       <c r="Q28" s="5" t="inlineStr"/>
+      <c r="R28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1874,6 +1921,7 @@
       <c r="O29" s="5" t="inlineStr"/>
       <c r="P29" s="5" t="inlineStr"/>
       <c r="Q29" s="5" t="inlineStr"/>
+      <c r="R29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -1929,6 +1977,7 @@
         </is>
       </c>
       <c r="Q30" s="5" t="inlineStr"/>
+      <c r="R30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1972,6 +2021,7 @@
       <c r="O31" s="5" t="inlineStr"/>
       <c r="P31" s="5" t="inlineStr"/>
       <c r="Q31" s="5" t="inlineStr"/>
+      <c r="R31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2019,6 +2069,7 @@
       <c r="O32" s="5" t="inlineStr"/>
       <c r="P32" s="5" t="inlineStr"/>
       <c r="Q32" s="5" t="inlineStr"/>
+      <c r="R32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2062,6 +2113,7 @@
       <c r="O33" s="5" t="inlineStr"/>
       <c r="P33" s="5" t="inlineStr"/>
       <c r="Q33" s="5" t="inlineStr"/>
+      <c r="R33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2109,6 +2161,7 @@
       </c>
       <c r="P34" s="5" t="inlineStr"/>
       <c r="Q34" s="5" t="inlineStr"/>
+      <c r="R34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2156,6 +2209,7 @@
       </c>
       <c r="P35" s="5" t="inlineStr"/>
       <c r="Q35" s="5" t="inlineStr"/>
+      <c r="R35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2199,6 +2253,7 @@
       <c r="O36" s="5" t="inlineStr"/>
       <c r="P36" s="5" t="inlineStr"/>
       <c r="Q36" s="5" t="inlineStr"/>
+      <c r="R36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2246,6 +2301,7 @@
       </c>
       <c r="P37" s="5" t="inlineStr"/>
       <c r="Q37" s="5" t="inlineStr"/>
+      <c r="R37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2293,6 +2349,7 @@
         </is>
       </c>
       <c r="Q38" s="5" t="inlineStr"/>
+      <c r="R38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2336,6 +2393,7 @@
       </c>
       <c r="P39" s="5" t="inlineStr"/>
       <c r="Q39" s="5" t="inlineStr"/>
+      <c r="R39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -2379,6 +2437,7 @@
       </c>
       <c r="P40" s="5" t="inlineStr"/>
       <c r="Q40" s="5" t="inlineStr"/>
+      <c r="R40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2426,6 +2485,7 @@
         </is>
       </c>
       <c r="Q41" s="5" t="inlineStr"/>
+      <c r="R41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -2469,6 +2529,7 @@
         </is>
       </c>
       <c r="Q42" s="5" t="inlineStr"/>
+      <c r="R42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2516,6 +2577,7 @@
           <t>sailed (12/14)</t>
         </is>
       </c>
+      <c r="R43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -2559,6 +2621,11 @@
           <t>alongside · 20AB (ETA 12/08→12/09, ETD 14/05)</t>
         </is>
       </c>
+      <c r="R44" s="5" t="inlineStr">
+        <is>
+          <t>sailed (14/05)</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -2602,6 +2669,7 @@
           <t>sailed (13/06)</t>
         </is>
       </c>
+      <c r="R45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -2645,6 +2713,11 @@
           <t>at anchorage · 20AB (ETA 13/01→13/02)</t>
         </is>
       </c>
+      <c r="R46" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20AB (P.B 14/05, ETD 15/15→15/08)</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -2686,6 +2759,11 @@
       <c r="Q47" s="5" t="inlineStr">
         <is>
           <t>alongside · 20D (P.B 12/16, ETD 14/05)</t>
+        </is>
+      </c>
+      <c r="R47" s="5" t="inlineStr">
+        <is>
+          <t>sailed (14/05)</t>
         </is>
       </c>
     </row>
@@ -2727,6 +2805,11 @@
           <t>expected · 20D (ETA 13/07→13/11, shift 7B)</t>
         </is>
       </c>
+      <c r="R48" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20D (7B)</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -2764,6 +2847,11 @@
       <c r="Q49" s="5" t="inlineStr">
         <is>
           <t>alongside · 20C (P.B 13/06, ETD 14/15)</t>
+        </is>
+      </c>
+      <c r="R49" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20C (ETD 14/15→14/16)</t>
         </is>
       </c>
     </row>
@@ -2799,6 +2887,11 @@
       <c r="Q50" s="5" t="inlineStr">
         <is>
           <t>alongside · 20B (ETD 14/16)</t>
+        </is>
+      </c>
+      <c r="R50" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20B (ETD 14/16→14/13)</t>
         </is>
       </c>
     </row>
@@ -2832,6 +2925,11 @@
           <t>expected · 20B (ETA 14/08→14/01)</t>
         </is>
       </c>
+      <c r="R51" s="6" t="inlineStr">
+        <is>
+          <t>at anchorage → 20C</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -2861,6 +2959,11 @@
       <c r="Q52" s="5" t="inlineStr">
         <is>
           <t>expected · 20F (ETA 13/15)</t>
+        </is>
+      </c>
+      <c r="R52" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20F (ETD 15/15→16/06)</t>
         </is>
       </c>
     </row>
@@ -2890,6 +2993,11 @@
           <t>expected · 20B (new)</t>
         </is>
       </c>
+      <c r="R53" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20AB</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -2915,6 +3023,95 @@
       <c r="Q54" s="5" t="inlineStr">
         <is>
           <t>expected · 20D (new)</t>
+        </is>
+      </c>
+      <c r="R54" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20C (ETA 15/01→14/23, ETD 16/17→16/15)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>SITC DALIAN</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr"/>
+      <c r="C55" s="5" t="inlineStr"/>
+      <c r="D55" s="5" t="inlineStr"/>
+      <c r="E55" s="5" t="inlineStr"/>
+      <c r="F55" s="5" t="inlineStr"/>
+      <c r="G55" s="5" t="inlineStr"/>
+      <c r="H55" s="5" t="inlineStr"/>
+      <c r="I55" s="5" t="inlineStr"/>
+      <c r="J55" s="5" t="inlineStr"/>
+      <c r="K55" s="5" t="inlineStr"/>
+      <c r="L55" s="5" t="inlineStr"/>
+      <c r="M55" s="5" t="inlineStr"/>
+      <c r="N55" s="5" t="inlineStr"/>
+      <c r="O55" s="5" t="inlineStr"/>
+      <c r="P55" s="5" t="inlineStr"/>
+      <c r="Q55" s="5" t="inlineStr"/>
+      <c r="R55" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>WAN HAI 172</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr"/>
+      <c r="C56" s="5" t="inlineStr"/>
+      <c r="D56" s="5" t="inlineStr"/>
+      <c r="E56" s="5" t="inlineStr"/>
+      <c r="F56" s="5" t="inlineStr"/>
+      <c r="G56" s="5" t="inlineStr"/>
+      <c r="H56" s="5" t="inlineStr"/>
+      <c r="I56" s="5" t="inlineStr"/>
+      <c r="J56" s="5" t="inlineStr"/>
+      <c r="K56" s="5" t="inlineStr"/>
+      <c r="L56" s="5" t="inlineStr"/>
+      <c r="M56" s="5" t="inlineStr"/>
+      <c r="N56" s="5" t="inlineStr"/>
+      <c r="O56" s="5" t="inlineStr"/>
+      <c r="P56" s="5" t="inlineStr"/>
+      <c r="Q56" s="5" t="inlineStr"/>
+      <c r="R56" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>LITTLE DOLPHIN</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr"/>
+      <c r="C57" s="5" t="inlineStr"/>
+      <c r="D57" s="5" t="inlineStr"/>
+      <c r="E57" s="5" t="inlineStr"/>
+      <c r="F57" s="5" t="inlineStr"/>
+      <c r="G57" s="5" t="inlineStr"/>
+      <c r="H57" s="5" t="inlineStr"/>
+      <c r="I57" s="5" t="inlineStr"/>
+      <c r="J57" s="5" t="inlineStr"/>
+      <c r="K57" s="5" t="inlineStr"/>
+      <c r="L57" s="5" t="inlineStr"/>
+      <c r="M57" s="5" t="inlineStr"/>
+      <c r="N57" s="5" t="inlineStr"/>
+      <c r="O57" s="5" t="inlineStr"/>
+      <c r="P57" s="5" t="inlineStr"/>
+      <c r="Q57" s="5" t="inlineStr"/>
+      <c r="R57" s="5" t="inlineStr">
+        <is>
+          <t>listed at 20F without times (new, schedule TBA)</t>
         </is>
       </c>
     </row>
@@ -10367,7 +10564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11814,10 +12011,713 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="12" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B49" s="13" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C49" s="13" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D49" s="14" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E49" s="14" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F49" s="13" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (KHUNA BHUM is alongside at 20D; other vessels are booked from 15/05)</t>
+        </is>
+      </c>
+      <c r="G49" s="13" t="inlineStr">
+        <is>
+          <t>Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B50" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="D50" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E50" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F50" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail (in progress)</t>
+        </is>
+      </c>
+      <c r="G50" s="9" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G48"/>
+  <autoFilter ref="A4:G50"/>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 14 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Waiting for Berth (h)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>KMTC TAIPEIS</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>46308.08333333334</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>46309.20833333334</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>46310.33333333334</v>
+      </c>
+      <c r="G4" s="28">
+        <f>(E4-D4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="28">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 176</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46310.45833333334</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46310.45833333334</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46311.66666666666</v>
+      </c>
+      <c r="G5" s="28">
+        <f>(E5-D5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="28">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>CEBU</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46307.91666666666</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46308.25</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46309.54166666666</v>
+      </c>
+      <c r="G6" s="28">
+        <f>(E6-D6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="28">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>M ODYSSEY</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>449</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46309.04166666666</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46309.625</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46310.20833333334</v>
+      </c>
+      <c r="G7" s="28">
+        <f>(E7-D7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="28">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="J7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>KHARIS HERITAGE</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>482</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>46310.04166666666</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>46310.29166666666</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>46311.29166666666</v>
+      </c>
+      <c r="G8" s="28">
+        <f>(E8-D8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="28">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 277</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>46307.875</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>46308.25</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>46309.66666666666</v>
+      </c>
+      <c r="G9" s="28">
+        <f>(E9-D9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="28">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 173</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>46309.04166666666</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>46309.66666666666</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>46310.29166666666</v>
+      </c>
+      <c r="G10" s="28">
+        <f>(E10-D10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="28">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 175</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>46309.95833333334</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>46310.29166666666</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>46311.625</v>
+      </c>
+      <c r="G11" s="28">
+        <f>(E11-D11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="28">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J11" s="23" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>KHUNA BHUM</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>46308.45833333334</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>46309.20833333334</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>46309.91666666666</v>
+      </c>
+      <c r="G12" s="28">
+        <f>(E12-D12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="28">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="J12" s="23" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>SITC DALIAN</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>470</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>46309.33333333334</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>46310.20833333334</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>46311.25</v>
+      </c>
+      <c r="G13" s="28">
+        <f>(E13-D13)*24</f>
+        <v/>
+      </c>
+      <c r="H13" s="28">
+        <f>(F13-E13)*24</f>
+        <v/>
+      </c>
+      <c r="I13" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J13" s="23" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 172</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>46311.04166666666</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>46311.29166666666</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>46312.625</v>
+      </c>
+      <c r="G14" s="28">
+        <f>(E14-D14)*24</f>
+        <v/>
+      </c>
+      <c r="H14" s="28">
+        <f>(F14-E14)*24</f>
+        <v/>
+      </c>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J14" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE INCHEON</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>46308.625</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>46309.25</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>46311.25</v>
+      </c>
+      <c r="G15" s="28">
+        <f>(E15-D15)*24</f>
+        <v/>
+      </c>
+      <c r="H15" s="28">
+        <f>(F15-E15)*24</f>
+        <v/>
+      </c>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J15" s="23" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="39" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n"/>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G19" s="40" t="n"/>
+      <c r="H19" s="40" t="n"/>
+      <c r="I19" s="40" t="n"/>
+      <c r="J19" s="41" t="n"/>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C20" s="43" t="n"/>
+      <c r="D20" s="18" t="n">
+        <v>46299</v>
+      </c>
+      <c r="E20" s="18" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F20" s="16" t="inlineStr">
+        <is>
+          <t>Close on 4–24 Oct 2026 to renovate electric channel (KHUNA BHUM is alongside at 20D; other vessels are booked from 15/05)  —  Unchanged – conflicts with vessel bookings, please confirm</t>
+        </is>
+      </c>
+      <c r="G20" s="43" t="n"/>
+      <c r="H20" s="43" t="n"/>
+      <c r="I20" s="43" t="n"/>
+      <c r="J20" s="43" t="n"/>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>20E / G.25</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="inlineStr">
+        <is>
+          <t>Gate stopped</t>
+        </is>
+      </c>
+      <c r="C21" s="42" t="n"/>
+      <c r="D21" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E21" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>G.25 stops working 5–18 Oct 2026 to change trolley rail (in progress)  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G21" s="42" t="n"/>
+      <c r="H21" s="42" t="n"/>
+      <c r="I21" s="42" t="n"/>
+      <c r="J21" s="42" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="F19:J19"/>
+    <mergeCell ref="F20:J20"/>
+    <mergeCell ref="F21:J21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11829,7 +12729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O57"/>
+  <dimension ref="A1:O59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11870,7 +12770,7 @@
         </is>
       </c>
       <c r="B3" s="27" t="n">
-        <v>46308.375</v>
+        <v>46309.375</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -12519,9 +13419,10 @@
         </is>
       </c>
       <c r="N15" s="23" t="inlineStr"/>
-      <c r="O15" s="23">
-        <f>IF(J15&lt;=$B$3,"Sailed",IF(I15&lt;=$B$3,"Alongside",IF(H15&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O15" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -12542,10 +13443,10 @@
         <v>46304</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="F16" s="23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
@@ -12559,7 +13460,7 @@
         <v>46309.20833333334</v>
       </c>
       <c r="J16" s="11" t="n">
-        <v>46310.625</v>
+        <v>46310.33333333334</v>
       </c>
       <c r="K16" s="28">
         <f>(I16-H16)*24</f>
@@ -12581,114 +13482,113 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="29" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>WAN HAI 176</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>46309</v>
+      </c>
+      <c r="F17" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20AB</t>
+        </is>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>46310.45833333334</v>
+      </c>
+      <c r="I17" s="11" t="n">
+        <v>46310.45833333334</v>
+      </c>
+      <c r="J17" s="11" t="n">
+        <v>46311.66666666666</v>
+      </c>
+      <c r="K17" s="28">
+        <f>(I17-H17)*24</f>
+        <v/>
+      </c>
+      <c r="L17" s="28">
+        <f>(J17-I17)*24</f>
+        <v/>
+      </c>
+      <c r="M17" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N17" s="23" t="inlineStr"/>
+      <c r="O17" s="23">
+        <f>IF(J17&lt;=$B$3,"Sailed",IF(I17&lt;=$B$3,"Alongside",IF(H17&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="inlineStr">
         <is>
           <t>20B</t>
         </is>
       </c>
-      <c r="B17" s="29" t="inlineStr">
+      <c r="B18" s="29" t="inlineStr">
         <is>
           <t>KMTC GWANGYANG</t>
         </is>
       </c>
-      <c r="C17" s="24" t="n">
+      <c r="C18" s="24" t="n">
         <v>564</v>
       </c>
-      <c r="D17" s="21" t="n">
+      <c r="D18" s="21" t="n">
         <v>46293</v>
       </c>
-      <c r="E17" s="21" t="n">
+      <c r="E18" s="21" t="n">
         <v>46293</v>
       </c>
-      <c r="F17" s="24" t="n">
+      <c r="F18" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="G17" s="30" t="inlineStr">
+      <c r="G18" s="30" t="inlineStr">
         <is>
           <t>20B</t>
         </is>
       </c>
-      <c r="H17" s="31" t="n">
+      <c r="H18" s="31" t="n">
         <v>46292.79166666666</v>
       </c>
-      <c r="I17" s="31" t="n">
+      <c r="I18" s="31" t="n">
         <v>46292.79166666666</v>
       </c>
-      <c r="J17" s="31" t="n">
+      <c r="J18" s="31" t="n">
         <v>46294.20833333334</v>
       </c>
-      <c r="K17" s="32">
-        <f>(I17-H17)*24</f>
-        <v/>
-      </c>
-      <c r="L17" s="32">
-        <f>(J17-I17)*24</f>
-        <v/>
-      </c>
-      <c r="M17" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N17" s="24" t="inlineStr"/>
-      <c r="O17" s="24" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>20B</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>MILLENNIUM BRIGHT</t>
-        </is>
-      </c>
-      <c r="C18" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D18" s="10" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E18" s="10" t="n">
-        <v>46294</v>
-      </c>
-      <c r="F18" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
-        </is>
-      </c>
-      <c r="H18" s="11" t="n">
-        <v>46293.45833333334</v>
-      </c>
-      <c r="I18" s="11" t="n">
-        <v>46294.20833333334</v>
-      </c>
-      <c r="J18" s="11" t="n">
-        <v>46295.16666666666</v>
-      </c>
-      <c r="K18" s="28">
+      <c r="K18" s="32">
         <f>(I18-H18)*24</f>
         <v/>
       </c>
-      <c r="L18" s="28">
+      <c r="L18" s="32">
         <f>(J18-I18)*24</f>
         <v/>
       </c>
-      <c r="M18" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N18" s="23" t="inlineStr"/>
-      <c r="O18" s="23" t="inlineStr">
+      <c r="M18" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N18" s="24" t="inlineStr"/>
+      <c r="O18" s="24" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -12702,34 +13602,34 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>YM IMPROVEMENT</t>
+          <t>MILLENNIUM BRIGHT</t>
         </is>
       </c>
       <c r="C19" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>46296</v>
+        <v>46293</v>
       </c>
       <c r="E19" s="10" t="n">
-        <v>46300</v>
+        <v>46294</v>
       </c>
       <c r="F19" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>20C → 20B</t>
+        <v>2</v>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H19" s="11" t="n">
-        <v>46298.95833333334</v>
+        <v>46293.45833333334</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>46299.41666666666</v>
+        <v>46294.20833333334</v>
       </c>
       <c r="J19" s="11" t="n">
-        <v>46300.5</v>
+        <v>46295.16666666666</v>
       </c>
       <c r="K19" s="28">
         <f>(I19-H19)*24</f>
@@ -12759,34 +13659,34 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE SPICA</t>
+          <t>YM IMPROVEMENT</t>
         </is>
       </c>
       <c r="C20" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>46299</v>
+        <v>46296</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>46303</v>
+        <v>46300</v>
       </c>
       <c r="F20" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>20C → 20B</t>
         </is>
       </c>
       <c r="H20" s="11" t="n">
-        <v>46300.875</v>
+        <v>46298.95833333334</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>46301.54166666666</v>
+        <v>46299.41666666666</v>
       </c>
       <c r="J20" s="11" t="n">
-        <v>46303.54166666666</v>
+        <v>46300.5</v>
       </c>
       <c r="K20" s="28">
         <f>(I20-H20)*24</f>
@@ -12816,34 +13716,34 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>SITC HOCHIMINH</t>
+          <t>SAWASDEE SPICA</t>
         </is>
       </c>
       <c r="C21" s="23" t="n">
-        <v>470</v>
+        <v>564</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>46301</v>
+        <v>46299</v>
       </c>
       <c r="E21" s="10" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="F21" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20B</t>
+        <v>5</v>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H21" s="11" t="n">
-        <v>46302.625</v>
+        <v>46300.875</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>46303.58333333334</v>
+        <v>46301.54166666666</v>
       </c>
       <c r="J21" s="11" t="n">
-        <v>46304.70833333334</v>
+        <v>46303.54166666666</v>
       </c>
       <c r="K21" s="28">
         <f>(I21-H21)*24</f>
@@ -12873,34 +13773,34 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>INDURO</t>
+          <t>SITC HOCHIMINH</t>
         </is>
       </c>
       <c r="C22" s="23" t="n">
-        <v>565</v>
+        <v>470</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="F22" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20B</t>
         </is>
       </c>
       <c r="H22" s="11" t="n">
-        <v>46304.25</v>
+        <v>46302.625</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>46304.66666666666</v>
+        <v>46303.58333333334</v>
       </c>
       <c r="J22" s="11" t="n">
-        <v>46306.16666666666</v>
+        <v>46304.70833333334</v>
       </c>
       <c r="K22" s="28">
         <f>(I22-H22)*24</f>
@@ -12930,34 +13830,34 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 102</t>
+          <t>INDURO</t>
         </is>
       </c>
       <c r="C23" s="23" t="n">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D23" s="10" t="n">
         <v>46302</v>
       </c>
       <c r="E23" s="10" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="F23" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G23" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20B</t>
+        <v>4</v>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H23" s="11" t="n">
-        <v>46305.875</v>
+        <v>46304.25</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>46306.20833333334</v>
+        <v>46304.66666666666</v>
       </c>
       <c r="J23" s="11" t="n">
-        <v>46307.08333333334</v>
+        <v>46306.16666666666</v>
       </c>
       <c r="K23" s="28">
         <f>(I23-H23)*24</f>
@@ -12987,34 +13887,34 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>CEBU</t>
+          <t>XIN MING ZHOU 102</t>
         </is>
       </c>
       <c r="C24" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D24" s="10" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E24" s="10" t="n">
         <v>46306</v>
       </c>
-      <c r="E24" s="10" t="n">
-        <v>46308</v>
-      </c>
       <c r="F24" s="23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20B</t>
+          <t>20F → 20B</t>
         </is>
       </c>
       <c r="H24" s="11" t="n">
-        <v>46307.91666666666</v>
+        <v>46305.875</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>46308.25</v>
+        <v>46306.20833333334</v>
       </c>
       <c r="J24" s="11" t="n">
-        <v>46309.66666666666</v>
+        <v>46307.08333333334</v>
       </c>
       <c r="K24" s="28">
         <f>(I24-H24)*24</f>
@@ -13030,9 +13930,10 @@
         </is>
       </c>
       <c r="N24" s="23" t="inlineStr"/>
-      <c r="O24" s="23">
-        <f>IF(J24&lt;=$B$3,"Sailed",IF(I24&lt;=$B$3,"Alongside",IF(H24&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O24" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -13043,34 +13944,34 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 173</t>
+          <t>CEBU</t>
         </is>
       </c>
       <c r="C25" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="E25" s="10" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="F25" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G25" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>4</v>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20B</t>
         </is>
       </c>
       <c r="H25" s="11" t="n">
-        <v>46309.04166666666</v>
+        <v>46307.91666666666</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>46309.66666666666</v>
+        <v>46308.25</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>46310.29166666666</v>
+        <v>46309.54166666666</v>
       </c>
       <c r="K25" s="28">
         <f>(I25-H25)*24</f>
@@ -13099,34 +14000,34 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 176</t>
+          <t>M ODYSSEY</t>
         </is>
       </c>
       <c r="C26" s="23" t="n">
-        <v>564</v>
+        <v>449</v>
       </c>
       <c r="D26" s="10" t="n">
-        <v>46308</v>
+        <v>46293</v>
       </c>
       <c r="E26" s="10" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="F26" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>6</v>
+      </c>
+      <c r="G26" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20C → 20B</t>
         </is>
       </c>
       <c r="H26" s="11" t="n">
-        <v>46310.45833333334</v>
+        <v>46309.04166666666</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>46310.45833333334</v>
+        <v>46309.625</v>
       </c>
       <c r="J26" s="11" t="n">
-        <v>46311.66666666666</v>
+        <v>46310.20833333334</v>
       </c>
       <c r="K26" s="28">
         <f>(I26-H26)*24</f>
@@ -13138,7 +14039,7 @@
       </c>
       <c r="M26" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="N26" s="23" t="inlineStr"/>
@@ -13148,114 +14049,113 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="29" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>KHARIS HERITAGE</t>
+        </is>
+      </c>
+      <c r="C27" s="23" t="n">
+        <v>482</v>
+      </c>
+      <c r="D27" s="10" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E27" s="10" t="n">
+        <v>46309</v>
+      </c>
+      <c r="F27" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20B → 20C → 20B</t>
+        </is>
+      </c>
+      <c r="H27" s="11" t="n">
+        <v>46310.04166666666</v>
+      </c>
+      <c r="I27" s="11" t="n">
+        <v>46310.29166666666</v>
+      </c>
+      <c r="J27" s="11" t="n">
+        <v>46311.29166666666</v>
+      </c>
+      <c r="K27" s="28">
+        <f>(I27-H27)*24</f>
+        <v/>
+      </c>
+      <c r="L27" s="28">
+        <f>(J27-I27)*24</f>
+        <v/>
+      </c>
+      <c r="M27" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N27" s="23" t="inlineStr"/>
+      <c r="O27" s="23">
+        <f>IF(J27&lt;=$B$3,"Sailed",IF(I27&lt;=$B$3,"Alongside",IF(H27&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="29" t="inlineStr">
         <is>
           <t>20C</t>
         </is>
       </c>
-      <c r="B27" s="29" t="inlineStr">
+      <c r="B28" s="29" t="inlineStr">
         <is>
           <t>SAWASDEE DENEB</t>
         </is>
       </c>
-      <c r="C27" s="24" t="n">
+      <c r="C28" s="24" t="n">
         <v>564</v>
       </c>
-      <c r="D27" s="21" t="n">
+      <c r="D28" s="21" t="n">
         <v>46297</v>
       </c>
-      <c r="E27" s="21" t="n">
+      <c r="E28" s="21" t="n">
         <v>46302</v>
       </c>
-      <c r="F27" s="24" t="n">
+      <c r="F28" s="24" t="n">
         <v>6</v>
       </c>
-      <c r="G27" s="30" t="inlineStr">
+      <c r="G28" s="30" t="inlineStr">
         <is>
           <t>20C</t>
         </is>
       </c>
-      <c r="H27" s="31" t="n">
+      <c r="H28" s="31" t="n">
         <v>46300</v>
       </c>
-      <c r="I27" s="31" t="n">
+      <c r="I28" s="31" t="n">
         <v>46300.5</v>
       </c>
-      <c r="J27" s="31" t="n">
+      <c r="J28" s="31" t="n">
         <v>46302.45833333334</v>
       </c>
-      <c r="K27" s="32">
-        <f>(I27-H27)*24</f>
-        <v/>
-      </c>
-      <c r="L27" s="32">
-        <f>(J27-I27)*24</f>
-        <v/>
-      </c>
-      <c r="M27" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N27" s="24" t="inlineStr"/>
-      <c r="O27" s="24" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>20C</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>JOSCO LUCKY</t>
-        </is>
-      </c>
-      <c r="C28" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D28" s="10" t="n">
-        <v>46297</v>
-      </c>
-      <c r="E28" s="10" t="n">
-        <v>46303</v>
-      </c>
-      <c r="F28" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="G28" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 20D → 20C</t>
-        </is>
-      </c>
-      <c r="H28" s="11" t="n">
-        <v>46301.875</v>
-      </c>
-      <c r="I28" s="11" t="n">
-        <v>46302.54166666666</v>
-      </c>
-      <c r="J28" s="11" t="n">
-        <v>46303.54166666666</v>
-      </c>
-      <c r="K28" s="28">
+      <c r="K28" s="32">
         <f>(I28-H28)*24</f>
         <v/>
       </c>
-      <c r="L28" s="28">
+      <c r="L28" s="32">
         <f>(J28-I28)*24</f>
         <v/>
       </c>
-      <c r="M28" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N28" s="23" t="inlineStr"/>
-      <c r="O28" s="23" t="inlineStr">
+      <c r="M28" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N28" s="24" t="inlineStr"/>
+      <c r="O28" s="24" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -13269,34 +14169,34 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>ZHONG GU DONG HAI</t>
+          <t>JOSCO LUCKY</t>
         </is>
       </c>
       <c r="C29" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D29" s="10" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="E29" s="10" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="F29" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>20C</t>
+        <v>7</v>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20AB → 20D → 20C</t>
         </is>
       </c>
       <c r="H29" s="11" t="n">
-        <v>46302.58333333334</v>
+        <v>46301.875</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>46303.58333333334</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="J29" s="11" t="n">
-        <v>46304.58333333334</v>
+        <v>46303.54166666666</v>
       </c>
       <c r="K29" s="28">
         <f>(I29-H29)*24</f>
@@ -13319,118 +14219,118 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="33" t="inlineStr">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>20C</t>
         </is>
       </c>
-      <c r="B30" s="33" t="inlineStr">
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>ZHONG GU DONG HAI</t>
+        </is>
+      </c>
+      <c r="C30" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E30" s="10" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F30" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="H30" s="11" t="n">
+        <v>46302.58333333334</v>
+      </c>
+      <c r="I30" s="11" t="n">
+        <v>46303.58333333334</v>
+      </c>
+      <c r="J30" s="11" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="K30" s="28">
+        <f>(I30-H30)*24</f>
+        <v/>
+      </c>
+      <c r="L30" s="28">
+        <f>(J30-I30)*24</f>
+        <v/>
+      </c>
+      <c r="M30" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N30" s="23" t="inlineStr"/>
+      <c r="O30" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="33" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B31" s="33" t="inlineStr">
         <is>
           <t>YM INCEPTION</t>
         </is>
       </c>
-      <c r="C30" s="17" t="n">
+      <c r="C31" s="17" t="n">
         <v>564</v>
       </c>
-      <c r="D30" s="18" t="n">
+      <c r="D31" s="18" t="n">
         <v>46301</v>
       </c>
-      <c r="E30" s="18" t="n">
+      <c r="E31" s="18" t="n">
         <v>46305</v>
       </c>
-      <c r="F30" s="17" t="n">
+      <c r="F31" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="G30" s="6" t="inlineStr">
+      <c r="G31" s="6" t="inlineStr">
         <is>
           <t>20AB → 20C</t>
         </is>
       </c>
-      <c r="H30" s="25" t="n">
+      <c r="H31" s="25" t="n">
         <v>46303.54166666666</v>
       </c>
-      <c r="I30" s="25" t="n">
+      <c r="I31" s="25" t="n">
         <v>46304.54166666666</v>
       </c>
-      <c r="J30" s="25" t="n">
+      <c r="J31" s="25" t="n">
         <v>46305.58333333334</v>
       </c>
-      <c r="K30" s="34">
-        <f>(I30-H30)*24</f>
-        <v/>
-      </c>
-      <c r="L30" s="34">
-        <f>(J30-I30)*24</f>
-        <v/>
-      </c>
-      <c r="M30" s="17" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N30" s="17" t="inlineStr">
+      <c r="K31" s="34">
+        <f>(I31-H31)*24</f>
+        <v/>
+      </c>
+      <c r="L31" s="34">
+        <f>(J31-I31)*24</f>
+        <v/>
+      </c>
+      <c r="M31" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N31" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O30" s="17" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>20C</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>STARSHIP AQUILA</t>
-        </is>
-      </c>
-      <c r="C31" s="23" t="n">
-        <v>565</v>
-      </c>
-      <c r="D31" s="10" t="n">
-        <v>46303</v>
-      </c>
-      <c r="E31" s="10" t="n">
-        <v>46306</v>
-      </c>
-      <c r="F31" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>20C</t>
-        </is>
-      </c>
-      <c r="H31" s="11" t="n">
-        <v>46304.91666666666</v>
-      </c>
-      <c r="I31" s="11" t="n">
-        <v>46305.58333333334</v>
-      </c>
-      <c r="J31" s="11" t="n">
-        <v>46307.08333333334</v>
-      </c>
-      <c r="K31" s="28">
-        <f>(I31-H31)*24</f>
-        <v/>
-      </c>
-      <c r="L31" s="28">
-        <f>(J31-I31)*24</f>
-        <v/>
-      </c>
-      <c r="M31" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N31" s="23" t="inlineStr"/>
-      <c r="O31" s="23" t="inlineStr">
+      <c r="O31" s="17" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -13444,34 +14344,34 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 277</t>
+          <t>STARSHIP AQUILA</t>
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D32" s="10" t="n">
-        <v>46305</v>
+        <v>46303</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>46308</v>
+        <v>46306</v>
       </c>
       <c r="F32" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20B → 20C</t>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
         </is>
       </c>
       <c r="H32" s="11" t="n">
-        <v>46307.875</v>
+        <v>46304.91666666666</v>
       </c>
       <c r="I32" s="11" t="n">
-        <v>46308.25</v>
+        <v>46305.58333333334</v>
       </c>
       <c r="J32" s="11" t="n">
-        <v>46309.625</v>
+        <v>46307.08333333334</v>
       </c>
       <c r="K32" s="28">
         <f>(I32-H32)*24</f>
@@ -13487,9 +14387,10 @@
         </is>
       </c>
       <c r="N32" s="23" t="inlineStr"/>
-      <c r="O32" s="23">
-        <f>IF(J32&lt;=$B$3,"Sailed",IF(I32&lt;=$B$3,"Alongside",IF(H32&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O32" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -13500,34 +14401,34 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>M ODYSSEY</t>
+          <t>WAN HAI 277</t>
         </is>
       </c>
       <c r="C33" s="23" t="n">
-        <v>449</v>
+        <v>564</v>
       </c>
       <c r="D33" s="10" t="n">
-        <v>46293</v>
+        <v>46305</v>
       </c>
       <c r="E33" s="10" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="F33" s="23" t="n">
         <v>5</v>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>20B → 20C</t>
+          <t>20F → 20B → 20C</t>
         </is>
       </c>
       <c r="H33" s="11" t="n">
-        <v>46309.125</v>
+        <v>46307.875</v>
       </c>
       <c r="I33" s="11" t="n">
-        <v>46309.58333333334</v>
+        <v>46308.25</v>
       </c>
       <c r="J33" s="11" t="n">
-        <v>46310.20833333334</v>
+        <v>46309.66666666666</v>
       </c>
       <c r="K33" s="28">
         <f>(I33-H33)*24</f>
@@ -13556,34 +14457,34 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>KHARIS HERITAGE</t>
+          <t>WAN HAI 173</t>
         </is>
       </c>
       <c r="C34" s="23" t="n">
-        <v>482</v>
+        <v>565</v>
       </c>
       <c r="D34" s="10" t="n">
-        <v>46294</v>
+        <v>46307</v>
       </c>
       <c r="E34" s="10" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="F34" s="23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G34" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20B → 20C</t>
+          <t>20B → 20C</t>
         </is>
       </c>
       <c r="H34" s="11" t="n">
-        <v>46310.04166666666</v>
+        <v>46309.04166666666</v>
       </c>
       <c r="I34" s="11" t="n">
+        <v>46309.66666666666</v>
+      </c>
+      <c r="J34" s="11" t="n">
         <v>46310.29166666666</v>
-      </c>
-      <c r="J34" s="11" t="n">
-        <v>46311.29166666666</v>
       </c>
       <c r="K34" s="28">
         <f>(I34-H34)*24</f>
@@ -13605,114 +14506,113 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="29" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>WAN HAI 175</t>
+        </is>
+      </c>
+      <c r="C35" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D35" s="10" t="n">
+        <v>46308</v>
+      </c>
+      <c r="E35" s="10" t="n">
+        <v>46309</v>
+      </c>
+      <c r="F35" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>20D → 20C</t>
+        </is>
+      </c>
+      <c r="H35" s="11" t="n">
+        <v>46309.95833333334</v>
+      </c>
+      <c r="I35" s="11" t="n">
+        <v>46310.29166666666</v>
+      </c>
+      <c r="J35" s="11" t="n">
+        <v>46311.625</v>
+      </c>
+      <c r="K35" s="28">
+        <f>(I35-H35)*24</f>
+        <v/>
+      </c>
+      <c r="L35" s="28">
+        <f>(J35-I35)*24</f>
+        <v/>
+      </c>
+      <c r="M35" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N35" s="23" t="inlineStr"/>
+      <c r="O35" s="23">
+        <f>IF(J35&lt;=$B$3,"Sailed",IF(I35&lt;=$B$3,"Alongside",IF(H35&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="29" t="inlineStr">
         <is>
           <t>20D</t>
         </is>
       </c>
-      <c r="B35" s="29" t="inlineStr">
+      <c r="B36" s="29" t="inlineStr">
         <is>
           <t>BANGKOK</t>
         </is>
       </c>
-      <c r="C35" s="24" t="n">
+      <c r="C36" s="24" t="n">
         <v>551</v>
       </c>
-      <c r="D35" s="21" t="n">
+      <c r="D36" s="21" t="n">
         <v>46293</v>
       </c>
-      <c r="E35" s="21" t="n">
+      <c r="E36" s="21" t="n">
         <v>46294</v>
       </c>
-      <c r="F35" s="24" t="n">
+      <c r="F36" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="G35" s="30" t="inlineStr">
+      <c r="G36" s="30" t="inlineStr">
         <is>
           <t>20D</t>
         </is>
       </c>
-      <c r="H35" s="31" t="n">
+      <c r="H36" s="31" t="n">
         <v>46292.54166666666</v>
       </c>
-      <c r="I35" s="31" t="n">
+      <c r="I36" s="31" t="n">
         <v>46292.625</v>
       </c>
-      <c r="J35" s="31" t="n">
+      <c r="J36" s="31" t="n">
         <v>46294.58333333334</v>
       </c>
-      <c r="K35" s="32">
-        <f>(I35-H35)*24</f>
-        <v/>
-      </c>
-      <c r="L35" s="32">
-        <f>(J35-I35)*24</f>
-        <v/>
-      </c>
-      <c r="M35" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N35" s="24" t="inlineStr"/>
-      <c r="O35" s="24" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>HARI BHUM (Barge)</t>
-        </is>
-      </c>
-      <c r="C36" s="23" t="n">
-        <v>259</v>
-      </c>
-      <c r="D36" s="10" t="n">
-        <v>46297</v>
-      </c>
-      <c r="E36" s="10" t="n">
-        <v>46298</v>
-      </c>
-      <c r="F36" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="H36" s="11" t="n">
-        <v>46298.20833333334</v>
-      </c>
-      <c r="I36" s="11" t="n">
-        <v>46298.29166666666</v>
-      </c>
-      <c r="J36" s="11" t="n">
-        <v>46298.66666666666</v>
-      </c>
-      <c r="K36" s="28">
+      <c r="K36" s="32">
         <f>(I36-H36)*24</f>
         <v/>
       </c>
-      <c r="L36" s="28">
+      <c r="L36" s="32">
         <f>(J36-I36)*24</f>
         <v/>
       </c>
-      <c r="M36" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N36" s="23" t="inlineStr"/>
-      <c r="O36" s="23" t="inlineStr">
+      <c r="M36" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N36" s="24" t="inlineStr"/>
+      <c r="O36" s="24" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -13726,20 +14626,20 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>MTT BANGKOK</t>
+          <t>HARI BHUM (Barge)</t>
         </is>
       </c>
       <c r="C37" s="23" t="n">
-        <v>564</v>
+        <v>259</v>
       </c>
       <c r="D37" s="10" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="E37" s="10" t="n">
-        <v>46303</v>
+        <v>46298</v>
       </c>
       <c r="F37" s="23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
@@ -13747,13 +14647,13 @@
         </is>
       </c>
       <c r="H37" s="11" t="n">
-        <v>46302.54166666666</v>
+        <v>46298.20833333334</v>
       </c>
       <c r="I37" s="11" t="n">
-        <v>46302.58333333334</v>
+        <v>46298.29166666666</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>46304.08333333334</v>
+        <v>46298.66666666666</v>
       </c>
       <c r="K37" s="28">
         <f>(I37-H37)*24</f>
@@ -13783,34 +14683,34 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>HE JIN</t>
+          <t>MTT BANGKOK</t>
         </is>
       </c>
       <c r="C38" s="23" t="n">
-        <v>552</v>
+        <v>564</v>
       </c>
       <c r="D38" s="10" t="n">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="E38" s="10" t="n">
-        <v>46305</v>
+        <v>46303</v>
       </c>
       <c r="F38" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G38" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 22A → 20D</t>
+        <v>4</v>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H38" s="11" t="n">
-        <v>46304</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="I38" s="11" t="n">
-        <v>46304</v>
+        <v>46302.58333333334</v>
       </c>
       <c r="J38" s="11" t="n">
-        <v>46305.54166666666</v>
+        <v>46304.08333333334</v>
       </c>
       <c r="K38" s="28">
         <f>(I38-H38)*24</f>
@@ -13840,34 +14740,34 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>CUL HAIPHONG</t>
+          <t>HE JIN</t>
         </is>
       </c>
       <c r="C39" s="23" t="n">
-        <v>458</v>
+        <v>552</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E39" s="10" t="n">
         <v>46305</v>
       </c>
       <c r="F39" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>20B → 20D</t>
+          <t>20B → 20AB → 22A → 20D</t>
         </is>
       </c>
       <c r="H39" s="11" t="n">
-        <v>46304.83333333334</v>
+        <v>46304</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>46305.66666666666</v>
+        <v>46304</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>46306.25</v>
+        <v>46305.54166666666</v>
       </c>
       <c r="K39" s="28">
         <f>(I39-H39)*24</f>
@@ -13879,7 +14779,7 @@
       </c>
       <c r="M39" s="23" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N39" s="23" t="inlineStr"/>
@@ -13897,34 +14797,34 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>INCEDA</t>
+          <t>CUL HAIPHONG</t>
         </is>
       </c>
       <c r="C40" s="23" t="n">
-        <v>564</v>
+        <v>458</v>
       </c>
       <c r="D40" s="10" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E40" s="10" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="F40" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
+        <v>4</v>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20D</t>
         </is>
       </c>
       <c r="H40" s="11" t="n">
-        <v>46305.70833333334</v>
+        <v>46304.83333333334</v>
       </c>
       <c r="I40" s="11" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="J40" s="11" t="n">
         <v>46306.25</v>
-      </c>
-      <c r="J40" s="11" t="n">
-        <v>46307.58333333334</v>
       </c>
       <c r="K40" s="28">
         <f>(I40-H40)*24</f>
@@ -13936,7 +14836,7 @@
       </c>
       <c r="M40" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="N40" s="23" t="inlineStr"/>
@@ -13954,34 +14854,34 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE SUNRISE</t>
+          <t>INCEDA</t>
         </is>
       </c>
       <c r="C41" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D41" s="10" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="E41" s="10" t="n">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="F41" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="G41" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20D</t>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H41" s="11" t="n">
-        <v>46307.16666666666</v>
+        <v>46305.70833333334</v>
       </c>
       <c r="I41" s="11" t="n">
-        <v>46307.66666666666</v>
+        <v>46306.25</v>
       </c>
       <c r="J41" s="11" t="n">
-        <v>46309.20833333334</v>
+        <v>46307.58333333334</v>
       </c>
       <c r="K41" s="28">
         <f>(I41-H41)*24</f>
@@ -13997,9 +14897,10 @@
         </is>
       </c>
       <c r="N41" s="23" t="inlineStr"/>
-      <c r="O41" s="23">
-        <f>IF(J41&lt;=$B$3,"Sailed",IF(I41&lt;=$B$3,"Alongside",IF(H41&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O41" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -14010,34 +14911,34 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>KHUNA BHUM</t>
+          <t>SAWASDEE SUNRISE</t>
         </is>
       </c>
       <c r="C42" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D42" s="10" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="E42" s="10" t="n">
         <v>46308</v>
       </c>
       <c r="F42" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20D</t>
+          <t>20F → 20D</t>
         </is>
       </c>
       <c r="H42" s="11" t="n">
-        <v>46308.45833333334</v>
+        <v>46307.16666666666</v>
       </c>
       <c r="I42" s="11" t="n">
+        <v>46307.66666666666</v>
+      </c>
+      <c r="J42" s="11" t="n">
         <v>46309.20833333334</v>
-      </c>
-      <c r="J42" s="11" t="n">
-        <v>46309.91666666666</v>
       </c>
       <c r="K42" s="28">
         <f>(I42-H42)*24</f>
@@ -14049,13 +14950,14 @@
       </c>
       <c r="M42" s="23" t="inlineStr">
         <is>
-          <t>7B</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N42" s="23" t="inlineStr"/>
-      <c r="O42" s="23">
-        <f>IF(J42&lt;=$B$3,"Sailed",IF(I42&lt;=$B$3,"Alongside",IF(H42&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O42" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="43">
@@ -14066,34 +14968,34 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 175</t>
+          <t>KHUNA BHUM</t>
         </is>
       </c>
       <c r="C43" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="E43" s="10" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="F43" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G43" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
+        <v>5</v>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20D</t>
         </is>
       </c>
       <c r="H43" s="11" t="n">
-        <v>46310.04166666666</v>
+        <v>46308.45833333334</v>
       </c>
       <c r="I43" s="11" t="n">
-        <v>46310.29166666666</v>
+        <v>46309.20833333334</v>
       </c>
       <c r="J43" s="11" t="n">
-        <v>46311.70833333334</v>
+        <v>46309.91666666666</v>
       </c>
       <c r="K43" s="28">
         <f>(I43-H43)*24</f>
@@ -14105,7 +15007,7 @@
       </c>
       <c r="M43" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="N43" s="23" t="inlineStr"/>
@@ -14115,98 +15017,97 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="29" t="inlineStr">
-        <is>
-          <t>20E</t>
-        </is>
-      </c>
-      <c r="B44" s="29" t="inlineStr">
-        <is>
-          <t>TS CHIBA</t>
-        </is>
-      </c>
-      <c r="C44" s="24" t="n">
-        <v>485</v>
-      </c>
-      <c r="D44" s="21" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E44" s="21" t="n">
-        <v>46293</v>
-      </c>
-      <c r="F44" s="24" t="n">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>SITC DALIAN</t>
+        </is>
+      </c>
+      <c r="C44" s="23" t="n">
+        <v>470</v>
+      </c>
+      <c r="D44" s="10" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E44" s="10" t="n">
+        <v>46309</v>
+      </c>
+      <c r="F44" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="G44" s="30" t="inlineStr">
-        <is>
-          <t>20E</t>
-        </is>
-      </c>
-      <c r="H44" s="31" t="n">
-        <v>46293.29166666666</v>
-      </c>
-      <c r="I44" s="31" t="n">
-        <v>46293.29166666666</v>
-      </c>
-      <c r="J44" s="31" t="n">
-        <v>46294.16666666666</v>
-      </c>
-      <c r="K44" s="32">
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="H44" s="11" t="n">
+        <v>46309.33333333334</v>
+      </c>
+      <c r="I44" s="11" t="n">
+        <v>46310.20833333334</v>
+      </c>
+      <c r="J44" s="11" t="n">
+        <v>46311.25</v>
+      </c>
+      <c r="K44" s="28">
         <f>(I44-H44)*24</f>
         <v/>
       </c>
-      <c r="L44" s="32">
+      <c r="L44" s="28">
         <f>(J44-I44)*24</f>
         <v/>
       </c>
-      <c r="M44" s="24" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N44" s="24" t="inlineStr"/>
-      <c r="O44" s="24" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="M44" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N44" s="23" t="inlineStr"/>
+      <c r="O44" s="23">
+        <f>IF(J44&lt;=$B$3,"Sailed",IF(I44&lt;=$B$3,"Alongside",IF(H44&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>20E</t>
+          <t>20D</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>MITRA BHUM</t>
+          <t>WAN HAI 172</t>
         </is>
       </c>
       <c r="C45" s="23" t="n">
-        <v>485</v>
+        <v>565</v>
       </c>
       <c r="D45" s="10" t="n">
-        <v>46293</v>
+        <v>46309</v>
       </c>
       <c r="E45" s="10" t="n">
-        <v>46295</v>
+        <v>46309</v>
       </c>
       <c r="F45" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20E</t>
+        <v>1</v>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H45" s="11" t="n">
-        <v>46295.125</v>
+        <v>46311.04166666666</v>
       </c>
       <c r="I45" s="11" t="n">
-        <v>46295.20833333334</v>
+        <v>46311.29166666666</v>
       </c>
       <c r="J45" s="11" t="n">
-        <v>46295.75</v>
+        <v>46312.625</v>
       </c>
       <c r="K45" s="28">
         <f>(I45-H45)*24</f>
@@ -14222,125 +15123,120 @@
         </is>
       </c>
       <c r="N45" s="23" t="inlineStr"/>
-      <c r="O45" s="23" t="inlineStr">
+      <c r="O45" s="23">
+        <f>IF(J45&lt;=$B$3,"Sailed",IF(I45&lt;=$B$3,"Alongside",IF(H45&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="29" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B46" s="29" t="inlineStr">
+        <is>
+          <t>TS CHIBA</t>
+        </is>
+      </c>
+      <c r="C46" s="24" t="n">
+        <v>485</v>
+      </c>
+      <c r="D46" s="21" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E46" s="21" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F46" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="30" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="H46" s="31" t="n">
+        <v>46293.29166666666</v>
+      </c>
+      <c r="I46" s="31" t="n">
+        <v>46293.29166666666</v>
+      </c>
+      <c r="J46" s="31" t="n">
+        <v>46294.16666666666</v>
+      </c>
+      <c r="K46" s="32">
+        <f>(I46-H46)*24</f>
+        <v/>
+      </c>
+      <c r="L46" s="32">
+        <f>(J46-I46)*24</f>
+        <v/>
+      </c>
+      <c r="M46" s="24" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N46" s="24" t="inlineStr"/>
+      <c r="O46" s="24" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>20E</t>
         </is>
       </c>
-      <c r="B46" s="4" t="inlineStr">
-        <is>
-          <t>WAN HAI 278</t>
-        </is>
-      </c>
-      <c r="C46" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D46" s="10" t="n">
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>MITRA BHUM</t>
+        </is>
+      </c>
+      <c r="C47" s="23" t="n">
+        <v>485</v>
+      </c>
+      <c r="D47" s="10" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E47" s="10" t="n">
         <v>46295</v>
       </c>
-      <c r="E46" s="10" t="n">
-        <v>46300</v>
-      </c>
-      <c r="F46" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="G46" s="6" t="inlineStr">
+      <c r="F47" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
         <is>
           <t>20F → 20E</t>
         </is>
       </c>
-      <c r="H46" s="11" t="n">
-        <v>46297.75</v>
-      </c>
-      <c r="I46" s="11" t="n">
-        <v>46298.41666666666</v>
-      </c>
-      <c r="J46" s="11" t="n">
-        <v>46300.45833333334</v>
-      </c>
-      <c r="K46" s="28">
-        <f>(I46-H46)*24</f>
-        <v/>
-      </c>
-      <c r="L46" s="28">
-        <f>(J46-I46)*24</f>
-        <v/>
-      </c>
-      <c r="M46" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N46" s="23" t="inlineStr"/>
-      <c r="O46" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="35" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="B47" s="35" t="inlineStr">
-        <is>
-          <t>JARU BHUM</t>
-        </is>
-      </c>
-      <c r="C47" s="22" t="n">
-        <v>564</v>
-      </c>
-      <c r="D47" s="14" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E47" s="14" t="n">
-        <v>46293</v>
-      </c>
-      <c r="F47" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="G47" s="36" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="H47" s="37" t="n">
-        <v>46293.33333333334</v>
-      </c>
-      <c r="I47" s="37" t="n">
-        <v>46293.33333333334</v>
-      </c>
-      <c r="J47" s="37" t="n">
-        <v>46294.16666666666</v>
-      </c>
-      <c r="K47" s="38">
+      <c r="H47" s="11" t="n">
+        <v>46295.125</v>
+      </c>
+      <c r="I47" s="11" t="n">
+        <v>46295.20833333334</v>
+      </c>
+      <c r="J47" s="11" t="n">
+        <v>46295.75</v>
+      </c>
+      <c r="K47" s="28">
         <f>(I47-H47)*24</f>
         <v/>
       </c>
-      <c r="L47" s="38">
+      <c r="L47" s="28">
         <f>(J47-I47)*24</f>
         <v/>
       </c>
-      <c r="M47" s="22" t="inlineStr">
-        <is>
-          <t>7B</t>
-        </is>
-      </c>
-      <c r="N47" s="22" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O47" s="22" t="inlineStr">
+      <c r="M47" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N47" s="23" t="inlineStr"/>
+      <c r="O47" s="23" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -14349,39 +15245,39 @@
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>20F</t>
+          <t>20E</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>HOPE C</t>
+          <t>WAN HAI 278</t>
         </is>
       </c>
       <c r="C48" s="23" t="n">
-        <v>481</v>
+        <v>564</v>
       </c>
       <c r="D48" s="10" t="n">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="E48" s="10" t="n">
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="F48" s="23" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>20E → 20F</t>
+          <t>20F → 20E</t>
         </is>
       </c>
       <c r="H48" s="11" t="n">
-        <v>46294.70833333334</v>
+        <v>46297.75</v>
       </c>
       <c r="I48" s="11" t="n">
-        <v>46294.70833333334</v>
+        <v>46298.41666666666</v>
       </c>
       <c r="J48" s="11" t="n">
-        <v>46295.66666666666</v>
+        <v>46300.45833333334</v>
       </c>
       <c r="K48" s="28">
         <f>(I48-H48)*24</f>
@@ -14404,57 +15300,61 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="A49" s="35" t="inlineStr">
         <is>
           <t>20F</t>
         </is>
       </c>
-      <c r="B49" s="4" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="C49" s="23" t="n">
+      <c r="B49" s="35" t="inlineStr">
+        <is>
+          <t>JARU BHUM</t>
+        </is>
+      </c>
+      <c r="C49" s="22" t="n">
         <v>564</v>
       </c>
-      <c r="D49" s="10" t="n">
-        <v>46295</v>
-      </c>
-      <c r="E49" s="10" t="n">
-        <v>46298</v>
-      </c>
-      <c r="F49" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20F</t>
-        </is>
-      </c>
-      <c r="H49" s="11" t="n">
-        <v>46297.29166666666</v>
-      </c>
-      <c r="I49" s="11" t="n">
-        <v>46297.45833333334</v>
-      </c>
-      <c r="J49" s="11" t="n">
-        <v>46298.70833333334</v>
-      </c>
-      <c r="K49" s="28">
+      <c r="D49" s="14" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E49" s="14" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F49" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="36" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="H49" s="37" t="n">
+        <v>46293.33333333334</v>
+      </c>
+      <c r="I49" s="37" t="n">
+        <v>46293.33333333334</v>
+      </c>
+      <c r="J49" s="37" t="n">
+        <v>46294.16666666666</v>
+      </c>
+      <c r="K49" s="38">
         <f>(I49-H49)*24</f>
         <v/>
       </c>
-      <c r="L49" s="28">
+      <c r="L49" s="38">
         <f>(J49-I49)*24</f>
         <v/>
       </c>
-      <c r="M49" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N49" s="23" t="inlineStr"/>
-      <c r="O49" s="23" t="inlineStr">
+      <c r="M49" s="22" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="N49" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O49" s="22" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -14468,34 +15368,34 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 98</t>
+          <t>HOPE C</t>
         </is>
       </c>
       <c r="C50" s="23" t="n">
-        <v>564</v>
+        <v>481</v>
       </c>
       <c r="D50" s="10" t="n">
-        <v>46297</v>
+        <v>46293</v>
       </c>
       <c r="E50" s="10" t="n">
-        <v>46299</v>
+        <v>46295</v>
       </c>
       <c r="F50" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>20E → 20F</t>
         </is>
       </c>
       <c r="H50" s="11" t="n">
-        <v>46299.375</v>
+        <v>46294.70833333334</v>
       </c>
       <c r="I50" s="11" t="n">
-        <v>46299.375</v>
+        <v>46294.70833333334</v>
       </c>
       <c r="J50" s="11" t="n">
-        <v>46300.375</v>
+        <v>46295.66666666666</v>
       </c>
       <c r="K50" s="28">
         <f>(I50-H50)*24</f>
@@ -14525,34 +15425,34 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>XIN AN</t>
+          <t>KMTC BANGKOK</t>
         </is>
       </c>
       <c r="C51" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D51" s="10" t="n">
-        <v>46300</v>
+        <v>46295</v>
       </c>
       <c r="E51" s="10" t="n">
-        <v>46304</v>
+        <v>46298</v>
       </c>
       <c r="F51" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+        <v>4</v>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20F</t>
         </is>
       </c>
       <c r="H51" s="11" t="n">
-        <v>46302.54166666666</v>
+        <v>46297.29166666666</v>
       </c>
       <c r="I51" s="11" t="n">
-        <v>46302.58333333334</v>
+        <v>46297.45833333334</v>
       </c>
       <c r="J51" s="11" t="n">
-        <v>46304.54166666666</v>
+        <v>46298.70833333334</v>
       </c>
       <c r="K51" s="28">
         <f>(I51-H51)*24</f>
@@ -14582,34 +15482,34 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE ATLANTIC</t>
+          <t>XIN MING ZHOU 98</t>
         </is>
       </c>
       <c r="C52" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D52" s="10" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>46306</v>
+        <v>46299</v>
       </c>
       <c r="F52" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>20C → 20D → 20F</t>
+        <v>3</v>
+      </c>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
         </is>
       </c>
       <c r="H52" s="11" t="n">
-        <v>46302.83333333334</v>
+        <v>46299.375</v>
       </c>
       <c r="I52" s="11" t="n">
-        <v>46304.625</v>
+        <v>46299.375</v>
       </c>
       <c r="J52" s="11" t="n">
-        <v>46306.5</v>
+        <v>46300.375</v>
       </c>
       <c r="K52" s="28">
         <f>(I52-H52)*24</f>
@@ -14639,34 +15539,34 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>JOSCO SHINE</t>
+          <t>XIN AN</t>
         </is>
       </c>
       <c r="C53" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D53" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E53" s="10" t="n">
         <v>46304</v>
       </c>
-      <c r="E53" s="10" t="n">
-        <v>46307</v>
-      </c>
       <c r="F53" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 20F</t>
+        <v>5</v>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
         </is>
       </c>
       <c r="H53" s="11" t="n">
-        <v>46307.45833333334</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>46307.625</v>
+        <v>46302.58333333334</v>
       </c>
       <c r="J53" s="11" t="n">
-        <v>46308.25</v>
+        <v>46304.54166666666</v>
       </c>
       <c r="K53" s="28">
         <f>(I53-H53)*24</f>
@@ -14696,34 +15596,34 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>ALS SUMIRE</t>
+          <t>SAWASDEE ATLANTIC</t>
         </is>
       </c>
       <c r="C54" s="23" t="n">
-        <v>537</v>
+        <v>564</v>
       </c>
       <c r="D54" s="10" t="n">
-        <v>46294</v>
+        <v>46300</v>
       </c>
       <c r="E54" s="10" t="n">
-        <v>46308</v>
+        <v>46306</v>
       </c>
       <c r="F54" s="23" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G54" s="6" t="inlineStr">
         <is>
-          <t>20F → 20D → 20C → 20B → 20F</t>
+          <t>20C → 20D → 20F</t>
         </is>
       </c>
       <c r="H54" s="11" t="n">
-        <v>46307.91666666666</v>
+        <v>46302.83333333334</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>46308.25</v>
+        <v>46304.625</v>
       </c>
       <c r="J54" s="11" t="n">
-        <v>46309.25</v>
+        <v>46306.5</v>
       </c>
       <c r="K54" s="28">
         <f>(I54-H54)*24</f>
@@ -14735,13 +15635,14 @@
       </c>
       <c r="M54" s="23" t="inlineStr">
         <is>
-          <t>1C</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N54" s="23" t="inlineStr"/>
-      <c r="O54" s="23">
-        <f>IF(J54&lt;=$B$3,"Sailed",IF(I54&lt;=$B$3,"Alongside",IF(H54&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O54" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -14752,34 +15653,34 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE INCHEON</t>
+          <t>JOSCO SHINE</t>
         </is>
       </c>
       <c r="C55" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D55" s="10" t="n">
+        <v>46304</v>
+      </c>
+      <c r="E55" s="10" t="n">
         <v>46307</v>
       </c>
-      <c r="E55" s="10" t="n">
-        <v>46308</v>
-      </c>
       <c r="F55" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G55" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+        <v>4</v>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20AB → 20F</t>
         </is>
       </c>
       <c r="H55" s="11" t="n">
-        <v>46308.625</v>
+        <v>46307.45833333334</v>
       </c>
       <c r="I55" s="11" t="n">
-        <v>46309.25</v>
+        <v>46307.625</v>
       </c>
       <c r="J55" s="11" t="n">
-        <v>46310.625</v>
+        <v>46308.25</v>
       </c>
       <c r="K55" s="28">
         <f>(I55-H55)*24</f>
@@ -14795,20 +15696,134 @@
         </is>
       </c>
       <c r="N55" s="23" t="inlineStr"/>
-      <c r="O55" s="23">
-        <f>IF(J55&lt;=$B$3,"Sailed",IF(I55&lt;=$B$3,"Alongside",IF(H55&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O55" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>ALS SUMIRE</t>
+        </is>
+      </c>
+      <c r="C56" s="23" t="n">
+        <v>537</v>
+      </c>
+      <c r="D56" s="10" t="n">
+        <v>46294</v>
+      </c>
+      <c r="E56" s="10" t="n">
+        <v>46308</v>
+      </c>
+      <c r="F56" s="23" t="n">
+        <v>9</v>
+      </c>
+      <c r="G56" s="6" t="inlineStr">
+        <is>
+          <t>20F → 20D → 20C → 20B → 20F</t>
+        </is>
+      </c>
+      <c r="H56" s="11" t="n">
+        <v>46307.91666666666</v>
+      </c>
+      <c r="I56" s="11" t="n">
+        <v>46308.25</v>
+      </c>
+      <c r="J56" s="11" t="n">
+        <v>46309.25</v>
+      </c>
+      <c r="K56" s="28">
+        <f>(I56-H56)*24</f>
+        <v/>
+      </c>
+      <c r="L56" s="28">
+        <f>(J56-I56)*24</f>
+        <v/>
+      </c>
+      <c r="M56" s="23" t="inlineStr">
+        <is>
+          <t>1C</t>
+        </is>
+      </c>
+      <c r="N56" s="23" t="inlineStr"/>
+      <c r="O56" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>50 vessels in total. Orange cells: marked on sheet, or the vessel changed berth.</t>
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>SAWASDEE INCHEON</t>
+        </is>
+      </c>
+      <c r="C57" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D57" s="10" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E57" s="10" t="n">
+        <v>46309</v>
+      </c>
+      <c r="F57" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="H57" s="11" t="n">
+        <v>46308.625</v>
+      </c>
+      <c r="I57" s="11" t="n">
+        <v>46309.25</v>
+      </c>
+      <c r="J57" s="11" t="n">
+        <v>46311.25</v>
+      </c>
+      <c r="K57" s="28">
+        <f>(I57-H57)*24</f>
+        <v/>
+      </c>
+      <c r="L57" s="28">
+        <f>(J57-I57)*24</f>
+        <v/>
+      </c>
+      <c r="M57" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N57" s="23" t="inlineStr"/>
+      <c r="O57" s="23">
+        <f>IF(J57&lt;=$B$3,"Sailed",IF(I57&lt;=$B$3,"Alongside",IF(H57&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>52 vessels in total. Orange cells: marked on sheet, or the vessel changed berth.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:O55"/>
+  <autoFilter ref="A5:O57"/>
   <mergeCells count="1">
     <mergeCell ref="A2:O2"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add 16 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -28,10 +28,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Oct 2026" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 Oct 2026" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Oct 2026" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 Oct 2026" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$52</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$O$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$O$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -660,7 +661,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S60"/>
+  <dimension ref="A1:T61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -682,6 +683,7 @@
     <col width="44" customWidth="1" min="17" max="17"/>
     <col width="44" customWidth="1" min="18" max="18"/>
     <col width="44" customWidth="1" min="19" max="19"/>
+    <col width="44" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -792,6 +794,11 @@
       <c r="S4" s="3" t="inlineStr">
         <is>
           <t>15 Oct 2026</t>
+        </is>
+      </c>
+      <c r="T4" s="3" t="inlineStr">
+        <is>
+          <t>16 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -835,6 +842,11 @@
           <t>expected → 20C (returns for a new call, ETA 18/06)</t>
         </is>
       </c>
+      <c r="T5" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20D (was 20C)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -876,6 +888,7 @@
       <c r="Q6" s="5" t="inlineStr"/>
       <c r="R6" s="5" t="inlineStr"/>
       <c r="S6" s="5" t="inlineStr"/>
+      <c r="T6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -909,6 +922,7 @@
       <c r="Q7" s="5" t="inlineStr"/>
       <c r="R7" s="5" t="inlineStr"/>
       <c r="S7" s="5" t="inlineStr"/>
+      <c r="T7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -946,6 +960,7 @@
       <c r="Q8" s="5" t="inlineStr"/>
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr"/>
+      <c r="T8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -989,6 +1004,11 @@
       <c r="S9" s="6" t="inlineStr">
         <is>
           <t>expected → 20AB (times now announced: ETA 16/21, P.B 17/09, ETD 18/16)</t>
+        </is>
+      </c>
+      <c r="T9" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20AB</t>
         </is>
       </c>
     </row>
@@ -1028,6 +1048,11 @@
           <t>expected → 20C (returns for a new call, ETA 17/02)</t>
         </is>
       </c>
+      <c r="T10" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20B (ETA 17/02→16/14, P.B 17/08→16/14, ETD 18/07→17/12)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1069,6 +1094,7 @@
       <c r="Q11" s="5" t="inlineStr"/>
       <c r="R11" s="5" t="inlineStr"/>
       <c r="S11" s="5" t="inlineStr"/>
+      <c r="T11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1106,6 +1132,11 @@
           <t>expected → 20D (returns for a new call, shift 7B, ETA 17/18)</t>
         </is>
       </c>
+      <c r="T12" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20B (shift 7B, ETA/P.B 17/18→17/16)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1151,6 +1182,11 @@
           <t>expected → 20D (returns for a new call, ETA 19/23)</t>
         </is>
       </c>
+      <c r="T13" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20AB (was 20D)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1204,6 +1240,11 @@
           <t>expected → 20AB (returns for a new call, ETA 19/18)</t>
         </is>
       </c>
+      <c r="T14" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20C (was 20AB)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1261,6 +1302,7 @@
           <t>sailed (15/05)</t>
         </is>
       </c>
+      <c r="T15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1318,6 +1360,11 @@
           <t>alongside · 20B (P.B 15/07→15/06)</t>
         </is>
       </c>
+      <c r="T16" s="5" t="inlineStr">
+        <is>
+          <t>sailed (16/07)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1387,6 +1434,7 @@
         </is>
       </c>
       <c r="S17" s="5" t="inlineStr"/>
+      <c r="T17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1432,6 +1480,7 @@
       <c r="Q18" s="5" t="inlineStr"/>
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr"/>
+      <c r="T18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1485,6 +1534,7 @@
       <c r="Q19" s="5" t="inlineStr"/>
       <c r="R19" s="5" t="inlineStr"/>
       <c r="S19" s="5" t="inlineStr"/>
+      <c r="T19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1538,6 +1588,7 @@
       <c r="Q20" s="5" t="inlineStr"/>
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr"/>
+      <c r="T20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1587,6 +1638,7 @@
       <c r="Q21" s="5" t="inlineStr"/>
       <c r="R21" s="5" t="inlineStr"/>
       <c r="S21" s="5" t="inlineStr"/>
+      <c r="T21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1632,6 +1684,7 @@
       <c r="Q22" s="5" t="inlineStr"/>
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr"/>
+      <c r="T22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1689,6 +1742,7 @@
       <c r="Q23" s="5" t="inlineStr"/>
       <c r="R23" s="5" t="inlineStr"/>
       <c r="S23" s="5" t="inlineStr"/>
+      <c r="T23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1742,6 +1796,7 @@
       <c r="Q24" s="5" t="inlineStr"/>
       <c r="R24" s="5" t="inlineStr"/>
       <c r="S24" s="5" t="inlineStr"/>
+      <c r="T24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1779,6 +1834,7 @@
       <c r="Q25" s="5" t="inlineStr"/>
       <c r="R25" s="5" t="inlineStr"/>
       <c r="S25" s="5" t="inlineStr"/>
+      <c r="T25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1820,6 +1876,7 @@
       <c r="Q26" s="5" t="inlineStr"/>
       <c r="R26" s="5" t="inlineStr"/>
       <c r="S26" s="5" t="inlineStr"/>
+      <c r="T26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1873,6 +1930,7 @@
       <c r="Q27" s="5" t="inlineStr"/>
       <c r="R27" s="5" t="inlineStr"/>
       <c r="S27" s="5" t="inlineStr"/>
+      <c r="T27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1922,6 +1980,7 @@
       <c r="Q28" s="5" t="inlineStr"/>
       <c r="R28" s="5" t="inlineStr"/>
       <c r="S28" s="5" t="inlineStr"/>
+      <c r="T28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1971,6 +2030,7 @@
       <c r="Q29" s="5" t="inlineStr"/>
       <c r="R29" s="5" t="inlineStr"/>
       <c r="S29" s="5" t="inlineStr"/>
+      <c r="T29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -2028,6 +2088,7 @@
       <c r="Q30" s="5" t="inlineStr"/>
       <c r="R30" s="5" t="inlineStr"/>
       <c r="S30" s="5" t="inlineStr"/>
+      <c r="T30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2073,6 +2134,7 @@
       <c r="Q31" s="5" t="inlineStr"/>
       <c r="R31" s="5" t="inlineStr"/>
       <c r="S31" s="5" t="inlineStr"/>
+      <c r="T31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2122,6 +2184,7 @@
       <c r="Q32" s="5" t="inlineStr"/>
       <c r="R32" s="5" t="inlineStr"/>
       <c r="S32" s="5" t="inlineStr"/>
+      <c r="T32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2167,6 +2230,7 @@
       <c r="Q33" s="5" t="inlineStr"/>
       <c r="R33" s="5" t="inlineStr"/>
       <c r="S33" s="5" t="inlineStr"/>
+      <c r="T33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2216,6 +2280,7 @@
       <c r="Q34" s="5" t="inlineStr"/>
       <c r="R34" s="5" t="inlineStr"/>
       <c r="S34" s="5" t="inlineStr"/>
+      <c r="T34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2265,6 +2330,7 @@
       <c r="Q35" s="5" t="inlineStr"/>
       <c r="R35" s="5" t="inlineStr"/>
       <c r="S35" s="5" t="inlineStr"/>
+      <c r="T35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2310,6 +2376,7 @@
       <c r="Q36" s="5" t="inlineStr"/>
       <c r="R36" s="5" t="inlineStr"/>
       <c r="S36" s="5" t="inlineStr"/>
+      <c r="T36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2359,6 +2426,7 @@
       <c r="Q37" s="5" t="inlineStr"/>
       <c r="R37" s="5" t="inlineStr"/>
       <c r="S37" s="5" t="inlineStr"/>
+      <c r="T37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2408,6 +2476,7 @@
       <c r="Q38" s="5" t="inlineStr"/>
       <c r="R38" s="5" t="inlineStr"/>
       <c r="S38" s="5" t="inlineStr"/>
+      <c r="T38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2453,6 +2522,7 @@
       <c r="Q39" s="5" t="inlineStr"/>
       <c r="R39" s="5" t="inlineStr"/>
       <c r="S39" s="5" t="inlineStr"/>
+      <c r="T39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -2498,6 +2568,7 @@
       <c r="Q40" s="5" t="inlineStr"/>
       <c r="R40" s="5" t="inlineStr"/>
       <c r="S40" s="5" t="inlineStr"/>
+      <c r="T40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2547,6 +2618,7 @@
       <c r="Q41" s="5" t="inlineStr"/>
       <c r="R41" s="5" t="inlineStr"/>
       <c r="S41" s="5" t="inlineStr"/>
+      <c r="T41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -2592,6 +2664,7 @@
       <c r="Q42" s="5" t="inlineStr"/>
       <c r="R42" s="5" t="inlineStr"/>
       <c r="S42" s="5" t="inlineStr"/>
+      <c r="T42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2641,6 +2714,7 @@
       </c>
       <c r="R43" s="5" t="inlineStr"/>
       <c r="S43" s="5" t="inlineStr"/>
+      <c r="T43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -2690,6 +2764,7 @@
         </is>
       </c>
       <c r="S44" s="5" t="inlineStr"/>
+      <c r="T44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -2735,6 +2810,7 @@
       </c>
       <c r="R45" s="5" t="inlineStr"/>
       <c r="S45" s="5" t="inlineStr"/>
+      <c r="T45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -2788,6 +2864,7 @@
           <t>sailed (15/08)</t>
         </is>
       </c>
+      <c r="T46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -2837,6 +2914,7 @@
         </is>
       </c>
       <c r="S47" s="5" t="inlineStr"/>
+      <c r="T47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -2886,6 +2964,7 @@
           <t>sailed (14/22)</t>
         </is>
       </c>
+      <c r="T48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -2935,6 +3014,7 @@
           <t>sailed (14/16)</t>
         </is>
       </c>
+      <c r="T49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -2980,6 +3060,7 @@
           <t>sailed (14/13)</t>
         </is>
       </c>
+      <c r="T50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -3021,6 +3102,7 @@
           <t>sailed (15/07)</t>
         </is>
       </c>
+      <c r="T51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -3060,6 +3142,11 @@
       <c r="S52" s="5" t="inlineStr">
         <is>
           <t>alongside · 20F (ETD 16/06)</t>
+        </is>
+      </c>
+      <c r="T52" s="5" t="inlineStr">
+        <is>
+          <t>sailed (16/06)</t>
         </is>
       </c>
     </row>
@@ -3099,6 +3186,11 @@
           <t>alongside · 20AB (ETA 15/11→15/08, P.B 15/11→15/09)</t>
         </is>
       </c>
+      <c r="T53" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20AB (ETD 16/16)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -3134,6 +3226,11 @@
       <c r="S54" s="6" t="inlineStr">
         <is>
           <t>alongside · 20C (ETA 14/23→14/21)</t>
+        </is>
+      </c>
+      <c r="T54" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20C (ETD 16/15)</t>
         </is>
       </c>
     </row>
@@ -3169,6 +3266,11 @@
           <t>alongside · 20D (P.B 15/05)</t>
         </is>
       </c>
+      <c r="T55" s="5" t="inlineStr">
+        <is>
+          <t>sailed (16/06)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -3202,6 +3304,11 @@
           <t>expected · 20D</t>
         </is>
       </c>
+      <c r="T56" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20D (ETD 17/15→17/08)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -3233,6 +3340,11 @@
       <c r="S57" s="6" t="inlineStr">
         <is>
           <t>expected → 20B (times announced: ETA 16/17, ETD 18/07; was 20F)</t>
+        </is>
+      </c>
+      <c r="T57" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20C (ETA 16/17→16/19, P.B 16/17→17/08, ETD 18/07→18/16)</t>
         </is>
       </c>
     </row>
@@ -3264,6 +3376,11 @@
           <t>expected · 20B (new)</t>
         </is>
       </c>
+      <c r="T58" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20F (ETA 17/22→17/10)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -3293,6 +3410,11 @@
           <t>expected · 20F (new)</t>
         </is>
       </c>
+      <c r="T59" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -3320,6 +3442,41 @@
       <c r="S60" s="5" t="inlineStr">
         <is>
           <t>expected · 20F (new)</t>
+        </is>
+      </c>
+      <c r="T60" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20F (ETA 18/20→19/07, P.B 18/20→19/09, ETD 20/08→20/17)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>PUNNYA NAVEE</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr"/>
+      <c r="C61" s="5" t="inlineStr"/>
+      <c r="D61" s="5" t="inlineStr"/>
+      <c r="E61" s="5" t="inlineStr"/>
+      <c r="F61" s="5" t="inlineStr"/>
+      <c r="G61" s="5" t="inlineStr"/>
+      <c r="H61" s="5" t="inlineStr"/>
+      <c r="I61" s="5" t="inlineStr"/>
+      <c r="J61" s="5" t="inlineStr"/>
+      <c r="K61" s="5" t="inlineStr"/>
+      <c r="L61" s="5" t="inlineStr"/>
+      <c r="M61" s="5" t="inlineStr"/>
+      <c r="N61" s="5" t="inlineStr"/>
+      <c r="O61" s="5" t="inlineStr"/>
+      <c r="P61" s="5" t="inlineStr"/>
+      <c r="Q61" s="5" t="inlineStr"/>
+      <c r="R61" s="5" t="inlineStr"/>
+      <c r="S61" s="5" t="inlineStr"/>
+      <c r="T61" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F (new, LOA 304 m)</t>
         </is>
       </c>
     </row>
@@ -10772,7 +10929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12347,8 +12504,39 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="12" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B53" s="13" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="C53" s="13" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D53" s="14" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E53" s="14" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F53" s="13" t="inlineStr">
+        <is>
+          <t>CLOSE (Oct 5–20 2026) printed under 20E</t>
+        </is>
+      </c>
+      <c r="G53" s="13" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G52"/>
+  <autoFilter ref="A4:G53"/>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
@@ -13794,13 +13982,701 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 16 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Waiting for Berth (h)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 176</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>46310.33333333334</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>46310.375</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>46311.66666666666</v>
+      </c>
+      <c r="G4" s="24">
+        <f>(E4-D4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="24">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>BANGKOK</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>551</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46311.875</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46312.375</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46313.66666666666</v>
+      </c>
+      <c r="G5" s="24">
+        <f>(E5-D5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="24">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>MITRA BHUM</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>485</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46314.95833333334</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46315.375</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46316.33333333334</v>
+      </c>
+      <c r="G6" s="24">
+        <f>(E6-D6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="24">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>TS CHIBA</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>485</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46311.58333333334</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46311.58333333334</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46312.5</v>
+      </c>
+      <c r="G7" s="24">
+        <f>(E7-D7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="24">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>JARU BHUM</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>46312.66666666666</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>46312.66666666666</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>46313.45833333334</v>
+      </c>
+      <c r="G8" s="24">
+        <f>(E8-D8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="24">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 175</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>46309.875</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>46310.29166666666</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>46311.625</v>
+      </c>
+      <c r="G9" s="24">
+        <f>(E9-D9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="24">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>LITTLE DOLPHIN</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>46311.79166666666</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>46312.33333333334</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>46313.66666666666</v>
+      </c>
+      <c r="G10" s="24">
+        <f>(E10-D10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="24">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>CAPE FAWLEY</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>558</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>46314.75</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>46314.75</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>46316.45833333334</v>
+      </c>
+      <c r="G11" s="24">
+        <f>(E11-D11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="24">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J11" s="23" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 172</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>46311.04166666666</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>46311.29166666666</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>46312.33333333334</v>
+      </c>
+      <c r="G12" s="24">
+        <f>(E12-D12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="24">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J12" s="23" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>INFINITY</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>46313.25</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>46313.29166666666</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>46314.41666666666</v>
+      </c>
+      <c r="G13" s="24">
+        <f>(E13-D13)*24</f>
+        <v/>
+      </c>
+      <c r="H13" s="24">
+        <f>(F13-E13)*24</f>
+        <v/>
+      </c>
+      <c r="I13" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J13" s="23" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>PUNNYA NAVEE</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>304</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>46311.625</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>46311.625</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>46312.25</v>
+      </c>
+      <c r="G14" s="24">
+        <f>(E14-D14)*24</f>
+        <v/>
+      </c>
+      <c r="H14" s="24">
+        <f>(F14-E14)*24</f>
+        <v/>
+      </c>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J14" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>INGENUITY</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>46311.95833333334</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>46312.33333333334</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>46313.29166666666</v>
+      </c>
+      <c r="G15" s="24">
+        <f>(E15-D15)*24</f>
+        <v/>
+      </c>
+      <c r="H15" s="24">
+        <f>(F15-E15)*24</f>
+        <v/>
+      </c>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J15" s="23" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 108</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>46312.41666666666</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>46313.33333333334</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>46314.29166666666</v>
+      </c>
+      <c r="G16" s="24">
+        <f>(E16-D16)*24</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>(F16-E16)*24</f>
+        <v/>
+      </c>
+      <c r="I16" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J16" s="23" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>KMTC JAKARTA</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>46314.29166666666</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>46314.375</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>46315.70833333334</v>
+      </c>
+      <c r="G17" s="24">
+        <f>(E17-D17)*24</f>
+        <v/>
+      </c>
+      <c r="H17" s="24">
+        <f>(F17-E17)*24</f>
+        <v/>
+      </c>
+      <c r="I17" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J17" s="23" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="34" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G21" s="35" t="n"/>
+      <c r="H21" s="35" t="n"/>
+      <c r="I21" s="35" t="n"/>
+      <c r="J21" s="36" t="n"/>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C22" s="38" t="n"/>
+      <c r="D22" s="18" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E22" s="18" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F22" s="16" t="inlineStr">
+        <is>
+          <t>CLOSE (Oct 5–20 2026) printed under 20E  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G22" s="38" t="n"/>
+      <c r="H22" s="38" t="n"/>
+      <c r="I22" s="38" t="n"/>
+      <c r="J22" s="38" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="F22:J22"/>
+    <mergeCell ref="F21:J21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O63"/>
+  <dimension ref="A1:O64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -13841,7 +14717,7 @@
         </is>
       </c>
       <c r="B3" s="22" t="n">
-        <v>46310.375</v>
+        <v>46311.375</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -14457,10 +15333,10 @@
         <v>46308</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="F15" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
@@ -14513,10 +15389,10 @@
         <v>46293</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="F16" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
@@ -14559,34 +15435,34 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>CAPE FAWLEY</t>
+          <t>MITRA BHUM</t>
         </is>
       </c>
       <c r="C17" s="23" t="n">
-        <v>558</v>
+        <v>485</v>
       </c>
       <c r="D17" s="10" t="n">
         <v>46293</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="F17" s="23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20C → 20AB</t>
+          <t>20F → 20E → 20D → 20AB</t>
         </is>
       </c>
       <c r="H17" s="11" t="n">
-        <v>46314.75</v>
+        <v>46314.95833333334</v>
       </c>
       <c r="I17" s="11" t="n">
-        <v>46314.75</v>
+        <v>46315.375</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>46316.45833333334</v>
+        <v>46316.33333333334</v>
       </c>
       <c r="K17" s="24">
         <f>(I17-H17)*24</f>
@@ -15171,9 +16047,10 @@
         </is>
       </c>
       <c r="N27" s="23" t="inlineStr"/>
-      <c r="O27" s="23">
-        <f>IF(J27&lt;=$B$3,"Sailed",IF(I27&lt;=$B$3,"Alongside",IF(H27&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O27" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -15184,34 +16061,34 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>LITTLE DOLPHIN</t>
+          <t>TS CHIBA</t>
         </is>
       </c>
       <c r="C28" s="23" t="n">
-        <v>564</v>
+        <v>485</v>
       </c>
       <c r="D28" s="10" t="n">
-        <v>46310</v>
+        <v>46293</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="F28" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>3</v>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>20E → 20C → 20B</t>
         </is>
       </c>
       <c r="H28" s="11" t="n">
-        <v>46311.70833333334</v>
+        <v>46311.58333333334</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>46311.70833333334</v>
+        <v>46311.58333333334</v>
       </c>
       <c r="J28" s="11" t="n">
-        <v>46313.29166666666</v>
+        <v>46312.5</v>
       </c>
       <c r="K28" s="24">
         <f>(I28-H28)*24</f>
@@ -15240,34 +16117,34 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 108</t>
+          <t>JARU BHUM</t>
         </is>
       </c>
       <c r="C29" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D29" s="10" t="n">
-        <v>46310</v>
+        <v>46293</v>
       </c>
       <c r="E29" s="10" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="F29" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>3</v>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>20F → 20D → 20B</t>
         </is>
       </c>
       <c r="H29" s="11" t="n">
-        <v>46312.91666666666</v>
+        <v>46312.66666666666</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>46313.33333333334</v>
+        <v>46312.66666666666</v>
       </c>
       <c r="J29" s="11" t="n">
-        <v>46314.29166666666</v>
+        <v>46313.45833333334</v>
       </c>
       <c r="K29" s="24">
         <f>(I29-H29)*24</f>
@@ -15279,7 +16156,7 @@
       </c>
       <c r="M29" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="N29" s="23" t="inlineStr"/>
@@ -15709,10 +16586,10 @@
         <v>46308</v>
       </c>
       <c r="E37" s="10" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="F37" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
@@ -15755,34 +16632,34 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>TS CHIBA</t>
+          <t>LITTLE DOLPHIN</t>
         </is>
       </c>
       <c r="C38" s="23" t="n">
-        <v>485</v>
+        <v>564</v>
       </c>
       <c r="D38" s="10" t="n">
-        <v>46293</v>
+        <v>46310</v>
       </c>
       <c r="E38" s="10" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="F38" s="23" t="n">
         <v>2</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
-          <t>20E → 20C</t>
+          <t>20B → 20C</t>
         </is>
       </c>
       <c r="H38" s="11" t="n">
-        <v>46312.08333333334</v>
+        <v>46311.79166666666</v>
       </c>
       <c r="I38" s="11" t="n">
         <v>46312.33333333334</v>
       </c>
       <c r="J38" s="11" t="n">
-        <v>46313.29166666666</v>
+        <v>46313.66666666666</v>
       </c>
       <c r="K38" s="24">
         <f>(I38-H38)*24</f>
@@ -15811,34 +16688,34 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>INFINITY</t>
+          <t>CAPE FAWLEY</t>
         </is>
       </c>
       <c r="C39" s="23" t="n">
-        <v>565</v>
+        <v>558</v>
       </c>
       <c r="D39" s="10" t="n">
         <v>46293</v>
       </c>
       <c r="E39" s="10" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="F39" s="23" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20C</t>
+          <t>20AB → 20C → 20AB → 20C</t>
         </is>
       </c>
       <c r="H39" s="11" t="n">
-        <v>46313.25</v>
+        <v>46314.75</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>46313.29166666666</v>
+        <v>46314.75</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>46314.41666666666</v>
+        <v>46316.45833333334</v>
       </c>
       <c r="K39" s="24">
         <f>(I39-H39)*24</f>
@@ -16309,9 +17186,10 @@
         </is>
       </c>
       <c r="N47" s="23" t="inlineStr"/>
-      <c r="O47" s="23">
-        <f>IF(J47&lt;=$B$3,"Sailed",IF(I47&lt;=$B$3,"Alongside",IF(H47&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O47" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -16332,10 +17210,10 @@
         <v>46309</v>
       </c>
       <c r="E48" s="10" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="F48" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
@@ -16349,7 +17227,7 @@
         <v>46311.29166666666</v>
       </c>
       <c r="J48" s="11" t="n">
-        <v>46312.625</v>
+        <v>46312.33333333334</v>
       </c>
       <c r="K48" s="24">
         <f>(I48-H48)*24</f>
@@ -16378,34 +17256,34 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>JARU BHUM</t>
+          <t>INFINITY</t>
         </is>
       </c>
       <c r="C49" s="23" t="n">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D49" s="10" t="n">
         <v>46293</v>
       </c>
       <c r="E49" s="10" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="F49" s="23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>20F → 20D</t>
+          <t>20AB → 20C → 20D</t>
         </is>
       </c>
       <c r="H49" s="11" t="n">
-        <v>46312.75</v>
+        <v>46313.25</v>
       </c>
       <c r="I49" s="11" t="n">
-        <v>46312.75</v>
+        <v>46313.29166666666</v>
       </c>
       <c r="J49" s="11" t="n">
-        <v>46313.45833333334</v>
+        <v>46314.41666666666</v>
       </c>
       <c r="K49" s="24">
         <f>(I49-H49)*24</f>
@@ -16417,7 +17295,7 @@
       </c>
       <c r="M49" s="23" t="inlineStr">
         <is>
-          <t>7B</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N49" s="23" t="inlineStr"/>
@@ -16427,97 +17305,98 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="B50" s="4" t="inlineStr">
-        <is>
-          <t>MITRA BHUM</t>
-        </is>
-      </c>
-      <c r="C50" s="23" t="n">
-        <v>485</v>
-      </c>
-      <c r="D50" s="10" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E50" s="10" t="n">
-        <v>46310</v>
-      </c>
-      <c r="F50" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G50" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20E → 20D</t>
-        </is>
-      </c>
-      <c r="H50" s="11" t="n">
-        <v>46314.95833333334</v>
-      </c>
-      <c r="I50" s="11" t="n">
-        <v>46315.375</v>
-      </c>
-      <c r="J50" s="11" t="n">
-        <v>46316.33333333334</v>
-      </c>
-      <c r="K50" s="24">
+      <c r="A50" s="25" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B50" s="25" t="inlineStr">
+        <is>
+          <t>WAN HAI 278</t>
+        </is>
+      </c>
+      <c r="C50" s="26" t="n">
+        <v>564</v>
+      </c>
+      <c r="D50" s="27" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E50" s="27" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F50" s="26" t="n">
+        <v>6</v>
+      </c>
+      <c r="G50" s="33" t="inlineStr">
+        <is>
+          <t>20F → 20E</t>
+        </is>
+      </c>
+      <c r="H50" s="29" t="n">
+        <v>46297.75</v>
+      </c>
+      <c r="I50" s="29" t="n">
+        <v>46298.41666666666</v>
+      </c>
+      <c r="J50" s="29" t="n">
+        <v>46300.45833333334</v>
+      </c>
+      <c r="K50" s="30">
         <f>(I50-H50)*24</f>
         <v/>
       </c>
-      <c r="L50" s="24">
+      <c r="L50" s="30">
         <f>(J50-I50)*24</f>
         <v/>
       </c>
-      <c r="M50" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N50" s="23" t="inlineStr"/>
-      <c r="O50" s="23">
-        <f>IF(J50&lt;=$B$3,"Sailed",IF(I50&lt;=$B$3,"Alongside",IF(H50&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="M50" s="26" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N50" s="26" t="inlineStr"/>
+      <c r="O50" s="26" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>20E</t>
+          <t>20F</t>
         </is>
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>WAN HAI 278</t>
+          <t>HOPE C</t>
         </is>
       </c>
       <c r="C51" s="26" t="n">
-        <v>564</v>
+        <v>481</v>
       </c>
       <c r="D51" s="27" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E51" s="27" t="n">
         <v>46295</v>
       </c>
-      <c r="E51" s="27" t="n">
-        <v>46300</v>
-      </c>
       <c r="F51" s="26" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G51" s="33" t="inlineStr">
         <is>
-          <t>20F → 20E</t>
+          <t>20E → 20F</t>
         </is>
       </c>
       <c r="H51" s="29" t="n">
-        <v>46297.75</v>
+        <v>46294.70833333334</v>
       </c>
       <c r="I51" s="29" t="n">
-        <v>46298.41666666666</v>
+        <v>46294.70833333334</v>
       </c>
       <c r="J51" s="29" t="n">
-        <v>46300.45833333334</v>
+        <v>46295.66666666666</v>
       </c>
       <c r="K51" s="30">
         <f>(I51-H51)*24</f>
@@ -16540,57 +17419,57 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="25" t="inlineStr">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>20F</t>
         </is>
       </c>
-      <c r="B52" s="25" t="inlineStr">
-        <is>
-          <t>HOPE C</t>
-        </is>
-      </c>
-      <c r="C52" s="26" t="n">
-        <v>481</v>
-      </c>
-      <c r="D52" s="27" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E52" s="27" t="n">
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>KMTC BANGKOK</t>
+        </is>
+      </c>
+      <c r="C52" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D52" s="10" t="n">
         <v>46295</v>
       </c>
-      <c r="F52" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="G52" s="33" t="inlineStr">
-        <is>
-          <t>20E → 20F</t>
-        </is>
-      </c>
-      <c r="H52" s="29" t="n">
-        <v>46294.70833333334</v>
-      </c>
-      <c r="I52" s="29" t="n">
-        <v>46294.70833333334</v>
-      </c>
-      <c r="J52" s="29" t="n">
-        <v>46295.66666666666</v>
-      </c>
-      <c r="K52" s="30">
+      <c r="E52" s="10" t="n">
+        <v>46298</v>
+      </c>
+      <c r="F52" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20F</t>
+        </is>
+      </c>
+      <c r="H52" s="11" t="n">
+        <v>46297.29166666666</v>
+      </c>
+      <c r="I52" s="11" t="n">
+        <v>46297.45833333334</v>
+      </c>
+      <c r="J52" s="11" t="n">
+        <v>46298.70833333334</v>
+      </c>
+      <c r="K52" s="24">
         <f>(I52-H52)*24</f>
         <v/>
       </c>
-      <c r="L52" s="30">
+      <c r="L52" s="24">
         <f>(J52-I52)*24</f>
         <v/>
       </c>
-      <c r="M52" s="26" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N52" s="26" t="inlineStr"/>
-      <c r="O52" s="26" t="inlineStr">
+      <c r="M52" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N52" s="23" t="inlineStr"/>
+      <c r="O52" s="23" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -16604,34 +17483,34 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>KMTC BANGKOK</t>
+          <t>XIN MING ZHOU 98</t>
         </is>
       </c>
       <c r="C53" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D53" s="10" t="n">
-        <v>46295</v>
+        <v>46297</v>
       </c>
       <c r="E53" s="10" t="n">
-        <v>46298</v>
+        <v>46299</v>
       </c>
       <c r="F53" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G53" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20F</t>
+        <v>3</v>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
         </is>
       </c>
       <c r="H53" s="11" t="n">
-        <v>46297.29166666666</v>
+        <v>46299.375</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>46297.45833333334</v>
+        <v>46299.375</v>
       </c>
       <c r="J53" s="11" t="n">
-        <v>46298.70833333334</v>
+        <v>46300.375</v>
       </c>
       <c r="K53" s="24">
         <f>(I53-H53)*24</f>
@@ -16661,20 +17540,20 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 98</t>
+          <t>XIN AN</t>
         </is>
       </c>
       <c r="C54" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D54" s="10" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="E54" s="10" t="n">
-        <v>46299</v>
+        <v>46304</v>
       </c>
       <c r="F54" s="23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
@@ -16682,13 +17561,13 @@
         </is>
       </c>
       <c r="H54" s="11" t="n">
-        <v>46299.375</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>46299.375</v>
+        <v>46302.58333333334</v>
       </c>
       <c r="J54" s="11" t="n">
-        <v>46300.375</v>
+        <v>46304.54166666666</v>
       </c>
       <c r="K54" s="24">
         <f>(I54-H54)*24</f>
@@ -16718,7 +17597,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>XIN AN</t>
+          <t>SAWASDEE ATLANTIC</t>
         </is>
       </c>
       <c r="C55" s="23" t="n">
@@ -16728,24 +17607,24 @@
         <v>46300</v>
       </c>
       <c r="E55" s="10" t="n">
-        <v>46304</v>
+        <v>46306</v>
       </c>
       <c r="F55" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G55" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+        <v>7</v>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>20C → 20D → 20F</t>
         </is>
       </c>
       <c r="H55" s="11" t="n">
-        <v>46302.54166666666</v>
+        <v>46302.83333333334</v>
       </c>
       <c r="I55" s="11" t="n">
-        <v>46302.58333333334</v>
+        <v>46304.625</v>
       </c>
       <c r="J55" s="11" t="n">
-        <v>46304.54166666666</v>
+        <v>46306.5</v>
       </c>
       <c r="K55" s="24">
         <f>(I55-H55)*24</f>
@@ -16775,34 +17654,34 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE ATLANTIC</t>
+          <t>JOSCO SHINE</t>
         </is>
       </c>
       <c r="C56" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D56" s="10" t="n">
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="E56" s="10" t="n">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="F56" s="23" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>20C → 20D → 20F</t>
+          <t>20B → 20AB → 20F</t>
         </is>
       </c>
       <c r="H56" s="11" t="n">
-        <v>46302.83333333334</v>
+        <v>46307.45833333334</v>
       </c>
       <c r="I56" s="11" t="n">
-        <v>46304.625</v>
+        <v>46307.625</v>
       </c>
       <c r="J56" s="11" t="n">
-        <v>46306.5</v>
+        <v>46308.25</v>
       </c>
       <c r="K56" s="24">
         <f>(I56-H56)*24</f>
@@ -16832,34 +17711,34 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>JOSCO SHINE</t>
+          <t>ALS SUMIRE</t>
         </is>
       </c>
       <c r="C57" s="23" t="n">
-        <v>564</v>
+        <v>537</v>
       </c>
       <c r="D57" s="10" t="n">
-        <v>46304</v>
+        <v>46294</v>
       </c>
       <c r="E57" s="10" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="F57" s="23" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>20B → 20AB → 20F</t>
+          <t>20F → 20D → 20C → 20B → 20F</t>
         </is>
       </c>
       <c r="H57" s="11" t="n">
-        <v>46307.45833333334</v>
+        <v>46307.91666666666</v>
       </c>
       <c r="I57" s="11" t="n">
-        <v>46307.625</v>
+        <v>46308.25</v>
       </c>
       <c r="J57" s="11" t="n">
-        <v>46308.25</v>
+        <v>46309.25</v>
       </c>
       <c r="K57" s="24">
         <f>(I57-H57)*24</f>
@@ -16871,7 +17750,7 @@
       </c>
       <c r="M57" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>1C</t>
         </is>
       </c>
       <c r="N57" s="23" t="inlineStr"/>
@@ -16889,34 +17768,34 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>ALS SUMIRE</t>
+          <t>SAWASDEE INCHEON</t>
         </is>
       </c>
       <c r="C58" s="23" t="n">
-        <v>537</v>
+        <v>564</v>
       </c>
       <c r="D58" s="10" t="n">
-        <v>46294</v>
+        <v>46307</v>
       </c>
       <c r="E58" s="10" t="n">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="F58" s="23" t="n">
-        <v>9</v>
-      </c>
-      <c r="G58" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20D → 20C → 20B → 20F</t>
+        <v>4</v>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
         </is>
       </c>
       <c r="H58" s="11" t="n">
-        <v>46307.91666666666</v>
+        <v>46308.625</v>
       </c>
       <c r="I58" s="11" t="n">
-        <v>46308.25</v>
+        <v>46309.25</v>
       </c>
       <c r="J58" s="11" t="n">
-        <v>46309.25</v>
+        <v>46311.25</v>
       </c>
       <c r="K58" s="24">
         <f>(I58-H58)*24</f>
@@ -16928,7 +17807,7 @@
       </c>
       <c r="M58" s="23" t="inlineStr">
         <is>
-          <t>1C</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N58" s="23" t="inlineStr"/>
@@ -16946,20 +17825,20 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE INCHEON</t>
+          <t>PUNNYA NAVEE</t>
         </is>
       </c>
       <c r="C59" s="23" t="n">
-        <v>564</v>
+        <v>304</v>
       </c>
       <c r="D59" s="10" t="n">
-        <v>46307</v>
+        <v>46311</v>
       </c>
       <c r="E59" s="10" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="F59" s="23" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
@@ -16967,13 +17846,13 @@
         </is>
       </c>
       <c r="H59" s="11" t="n">
-        <v>46308.625</v>
+        <v>46311.625</v>
       </c>
       <c r="I59" s="11" t="n">
-        <v>46309.25</v>
+        <v>46311.625</v>
       </c>
       <c r="J59" s="11" t="n">
-        <v>46311.25</v>
+        <v>46312.25</v>
       </c>
       <c r="K59" s="24">
         <f>(I59-H59)*24</f>
@@ -17012,10 +17891,10 @@
         <v>46310</v>
       </c>
       <c r="E60" s="10" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="F60" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
@@ -17058,7 +17937,7 @@
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>KMTC JAKARTA</t>
+          <t>XIN MING ZHOU 108</t>
         </is>
       </c>
       <c r="C61" s="23" t="n">
@@ -17068,24 +17947,24 @@
         <v>46310</v>
       </c>
       <c r="E61" s="10" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="F61" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G61" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+        <v>2</v>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20F</t>
         </is>
       </c>
       <c r="H61" s="11" t="n">
-        <v>46313.83333333334</v>
+        <v>46312.41666666666</v>
       </c>
       <c r="I61" s="11" t="n">
-        <v>46313.83333333334</v>
+        <v>46313.33333333334</v>
       </c>
       <c r="J61" s="11" t="n">
-        <v>46315.33333333334</v>
+        <v>46314.29166666666</v>
       </c>
       <c r="K61" s="24">
         <f>(I61-H61)*24</f>
@@ -17106,15 +17985,71 @@
         <v/>
       </c>
     </row>
-    <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>56 vessels in total. Orange cells: marked on sheet, or the vessel changed berth.</t>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>KMTC JAKARTA</t>
+        </is>
+      </c>
+      <c r="C62" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D62" s="10" t="n">
+        <v>46310</v>
+      </c>
+      <c r="E62" s="10" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F62" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="H62" s="11" t="n">
+        <v>46314.29166666666</v>
+      </c>
+      <c r="I62" s="11" t="n">
+        <v>46314.375</v>
+      </c>
+      <c r="J62" s="11" t="n">
+        <v>46315.70833333334</v>
+      </c>
+      <c r="K62" s="24">
+        <f>(I62-H62)*24</f>
+        <v/>
+      </c>
+      <c r="L62" s="24">
+        <f>(J62-I62)*24</f>
+        <v/>
+      </c>
+      <c r="M62" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N62" s="23" t="inlineStr"/>
+      <c r="O62" s="23">
+        <f>IF(J62&lt;=$B$3,"Sailed",IF(I62&lt;=$B$3,"Alongside",IF(H62&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>57 vessels in total. Orange cells: marked on sheet, or the vessel changed berth.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:O61"/>
+  <autoFilter ref="A5:O62"/>
   <mergeCells count="1">
     <mergeCell ref="A2:O2"/>
   </mergeCells>

</xml_diff>

<commit_message>
Add 17 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -29,9 +29,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 Oct 2026" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Oct 2026" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 Oct 2026" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 Oct 2026" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$O$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -661,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T61"/>
+  <dimension ref="A1:U61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -684,6 +685,7 @@
     <col width="44" customWidth="1" min="18" max="18"/>
     <col width="44" customWidth="1" min="19" max="19"/>
     <col width="44" customWidth="1" min="20" max="20"/>
+    <col width="44" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -799,6 +801,11 @@
       <c r="T4" s="3" t="inlineStr">
         <is>
           <t>16 Oct 2026</t>
+        </is>
+      </c>
+      <c r="U4" s="3" t="inlineStr">
+        <is>
+          <t>17 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -847,6 +854,11 @@
           <t>expected → 20D (was 20C)</t>
         </is>
       </c>
+      <c r="U5" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20D (ETA 18/06→17/24)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -889,6 +901,7 @@
       <c r="R6" s="5" t="inlineStr"/>
       <c r="S6" s="5" t="inlineStr"/>
       <c r="T6" s="5" t="inlineStr"/>
+      <c r="U6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -923,6 +936,7 @@
       <c r="R7" s="5" t="inlineStr"/>
       <c r="S7" s="5" t="inlineStr"/>
       <c r="T7" s="5" t="inlineStr"/>
+      <c r="U7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -961,6 +975,7 @@
       <c r="R8" s="5" t="inlineStr"/>
       <c r="S8" s="5" t="inlineStr"/>
       <c r="T8" s="5" t="inlineStr"/>
+      <c r="U8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1009,6 +1024,11 @@
       <c r="T9" s="5" t="inlineStr">
         <is>
           <t>expected · 20AB</t>
+        </is>
+      </c>
+      <c r="U9" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20AB (actual ETA 16/15, P.B 17/09)</t>
         </is>
       </c>
     </row>
@@ -1053,6 +1073,11 @@
           <t>expected → 20B (ETA 17/02→16/14, P.B 17/08→16/14, ETD 18/07→17/12)</t>
         </is>
       </c>
+      <c r="U10" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20B (ETD 17/12→17/11)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1095,6 +1120,7 @@
       <c r="R11" s="5" t="inlineStr"/>
       <c r="S11" s="5" t="inlineStr"/>
       <c r="T11" s="5" t="inlineStr"/>
+      <c r="U11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1137,6 +1163,11 @@
           <t>expected → 20B (shift 7B, ETA/P.B 17/18→17/16)</t>
         </is>
       </c>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B (shift 7B)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1187,6 +1218,11 @@
           <t>expected → 20AB (was 20D)</t>
         </is>
       </c>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>no longer listed (dropped from the sheet)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1245,6 +1281,11 @@
           <t>expected → 20C (was 20AB)</t>
         </is>
       </c>
+      <c r="U14" s="5" t="inlineStr">
+        <is>
+          <t>20C row with only LOA 558 m printed (no name or times)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1303,6 +1344,7 @@
         </is>
       </c>
       <c r="T15" s="5" t="inlineStr"/>
+      <c r="U15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1365,6 +1407,7 @@
           <t>sailed (16/07)</t>
         </is>
       </c>
+      <c r="U16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1435,6 +1478,7 @@
       </c>
       <c r="S17" s="5" t="inlineStr"/>
       <c r="T17" s="5" t="inlineStr"/>
+      <c r="U17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1481,6 +1525,7 @@
       <c r="R18" s="5" t="inlineStr"/>
       <c r="S18" s="5" t="inlineStr"/>
       <c r="T18" s="5" t="inlineStr"/>
+      <c r="U18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1535,6 +1580,7 @@
       <c r="R19" s="5" t="inlineStr"/>
       <c r="S19" s="5" t="inlineStr"/>
       <c r="T19" s="5" t="inlineStr"/>
+      <c r="U19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1589,6 +1635,7 @@
       <c r="R20" s="5" t="inlineStr"/>
       <c r="S20" s="5" t="inlineStr"/>
       <c r="T20" s="5" t="inlineStr"/>
+      <c r="U20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1639,6 +1686,7 @@
       <c r="R21" s="5" t="inlineStr"/>
       <c r="S21" s="5" t="inlineStr"/>
       <c r="T21" s="5" t="inlineStr"/>
+      <c r="U21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1685,6 +1733,7 @@
       <c r="R22" s="5" t="inlineStr"/>
       <c r="S22" s="5" t="inlineStr"/>
       <c r="T22" s="5" t="inlineStr"/>
+      <c r="U22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1743,6 +1792,7 @@
       <c r="R23" s="5" t="inlineStr"/>
       <c r="S23" s="5" t="inlineStr"/>
       <c r="T23" s="5" t="inlineStr"/>
+      <c r="U23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1797,6 +1847,7 @@
       <c r="R24" s="5" t="inlineStr"/>
       <c r="S24" s="5" t="inlineStr"/>
       <c r="T24" s="5" t="inlineStr"/>
+      <c r="U24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1835,6 +1886,7 @@
       <c r="R25" s="5" t="inlineStr"/>
       <c r="S25" s="5" t="inlineStr"/>
       <c r="T25" s="5" t="inlineStr"/>
+      <c r="U25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1877,6 +1929,7 @@
       <c r="R26" s="5" t="inlineStr"/>
       <c r="S26" s="5" t="inlineStr"/>
       <c r="T26" s="5" t="inlineStr"/>
+      <c r="U26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1931,6 +1984,7 @@
       <c r="R27" s="5" t="inlineStr"/>
       <c r="S27" s="5" t="inlineStr"/>
       <c r="T27" s="5" t="inlineStr"/>
+      <c r="U27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -1981,6 +2035,7 @@
       <c r="R28" s="5" t="inlineStr"/>
       <c r="S28" s="5" t="inlineStr"/>
       <c r="T28" s="5" t="inlineStr"/>
+      <c r="U28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2031,6 +2086,7 @@
       <c r="R29" s="5" t="inlineStr"/>
       <c r="S29" s="5" t="inlineStr"/>
       <c r="T29" s="5" t="inlineStr"/>
+      <c r="U29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -2089,6 +2145,7 @@
       <c r="R30" s="5" t="inlineStr"/>
       <c r="S30" s="5" t="inlineStr"/>
       <c r="T30" s="5" t="inlineStr"/>
+      <c r="U30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2135,6 +2192,7 @@
       <c r="R31" s="5" t="inlineStr"/>
       <c r="S31" s="5" t="inlineStr"/>
       <c r="T31" s="5" t="inlineStr"/>
+      <c r="U31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2185,6 +2243,7 @@
       <c r="R32" s="5" t="inlineStr"/>
       <c r="S32" s="5" t="inlineStr"/>
       <c r="T32" s="5" t="inlineStr"/>
+      <c r="U32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2231,6 +2290,7 @@
       <c r="R33" s="5" t="inlineStr"/>
       <c r="S33" s="5" t="inlineStr"/>
       <c r="T33" s="5" t="inlineStr"/>
+      <c r="U33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2281,6 +2341,7 @@
       <c r="R34" s="5" t="inlineStr"/>
       <c r="S34" s="5" t="inlineStr"/>
       <c r="T34" s="5" t="inlineStr"/>
+      <c r="U34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2331,6 +2392,7 @@
       <c r="R35" s="5" t="inlineStr"/>
       <c r="S35" s="5" t="inlineStr"/>
       <c r="T35" s="5" t="inlineStr"/>
+      <c r="U35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2377,6 +2439,7 @@
       <c r="R36" s="5" t="inlineStr"/>
       <c r="S36" s="5" t="inlineStr"/>
       <c r="T36" s="5" t="inlineStr"/>
+      <c r="U36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2427,6 +2490,7 @@
       <c r="R37" s="5" t="inlineStr"/>
       <c r="S37" s="5" t="inlineStr"/>
       <c r="T37" s="5" t="inlineStr"/>
+      <c r="U37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2477,6 +2541,7 @@
       <c r="R38" s="5" t="inlineStr"/>
       <c r="S38" s="5" t="inlineStr"/>
       <c r="T38" s="5" t="inlineStr"/>
+      <c r="U38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2523,6 +2588,7 @@
       <c r="R39" s="5" t="inlineStr"/>
       <c r="S39" s="5" t="inlineStr"/>
       <c r="T39" s="5" t="inlineStr"/>
+      <c r="U39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -2569,6 +2635,7 @@
       <c r="R40" s="5" t="inlineStr"/>
       <c r="S40" s="5" t="inlineStr"/>
       <c r="T40" s="5" t="inlineStr"/>
+      <c r="U40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2619,6 +2686,7 @@
       <c r="R41" s="5" t="inlineStr"/>
       <c r="S41" s="5" t="inlineStr"/>
       <c r="T41" s="5" t="inlineStr"/>
+      <c r="U41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -2665,6 +2733,7 @@
       <c r="R42" s="5" t="inlineStr"/>
       <c r="S42" s="5" t="inlineStr"/>
       <c r="T42" s="5" t="inlineStr"/>
+      <c r="U42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2715,6 +2784,7 @@
       <c r="R43" s="5" t="inlineStr"/>
       <c r="S43" s="5" t="inlineStr"/>
       <c r="T43" s="5" t="inlineStr"/>
+      <c r="U43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -2765,6 +2835,7 @@
       </c>
       <c r="S44" s="5" t="inlineStr"/>
       <c r="T44" s="5" t="inlineStr"/>
+      <c r="U44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -2811,6 +2882,7 @@
       <c r="R45" s="5" t="inlineStr"/>
       <c r="S45" s="5" t="inlineStr"/>
       <c r="T45" s="5" t="inlineStr"/>
+      <c r="U45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -2865,6 +2937,7 @@
         </is>
       </c>
       <c r="T46" s="5" t="inlineStr"/>
+      <c r="U46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -2915,6 +2988,7 @@
       </c>
       <c r="S47" s="5" t="inlineStr"/>
       <c r="T47" s="5" t="inlineStr"/>
+      <c r="U47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -2965,6 +3039,7 @@
         </is>
       </c>
       <c r="T48" s="5" t="inlineStr"/>
+      <c r="U48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -3015,6 +3090,7 @@
         </is>
       </c>
       <c r="T49" s="5" t="inlineStr"/>
+      <c r="U49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -3061,6 +3137,7 @@
         </is>
       </c>
       <c r="T50" s="5" t="inlineStr"/>
+      <c r="U50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -3103,6 +3180,7 @@
         </is>
       </c>
       <c r="T51" s="5" t="inlineStr"/>
+      <c r="U51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -3149,6 +3227,7 @@
           <t>sailed (16/06)</t>
         </is>
       </c>
+      <c r="U52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -3191,6 +3270,11 @@
           <t>alongside · 20AB (ETD 16/16)</t>
         </is>
       </c>
+      <c r="U53" s="5" t="inlineStr">
+        <is>
+          <t>sailed (16/16)</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -3231,6 +3315,11 @@
       <c r="T54" s="5" t="inlineStr">
         <is>
           <t>alongside · 20C (ETD 16/15)</t>
+        </is>
+      </c>
+      <c r="U54" s="5" t="inlineStr">
+        <is>
+          <t>sailed (16/15)</t>
         </is>
       </c>
     </row>
@@ -3271,6 +3360,7 @@
           <t>sailed (16/06)</t>
         </is>
       </c>
+      <c r="U55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -3309,6 +3399,11 @@
           <t>alongside · 20D (ETD 17/15→17/08)</t>
         </is>
       </c>
+      <c r="U56" s="5" t="inlineStr">
+        <is>
+          <t>sailed (17/08)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -3345,6 +3440,11 @@
       <c r="T57" s="6" t="inlineStr">
         <is>
           <t>expected → 20C (ETA 16/17→16/19, P.B 16/17→17/08, ETD 18/07→18/16)</t>
+        </is>
+      </c>
+      <c r="U57" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20C (actual ETA 17/01)</t>
         </is>
       </c>
     </row>
@@ -3381,6 +3481,11 @@
           <t>expected → 20F (ETA 17/22→17/10)</t>
         </is>
       </c>
+      <c r="U58" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -3415,6 +3520,11 @@
           <t>expected · 20F</t>
         </is>
       </c>
+      <c r="U59" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20F (actual ETA 16/23)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -3447,6 +3557,11 @@
       <c r="T60" s="6" t="inlineStr">
         <is>
           <t>expected · 20F (ETA 18/20→19/07, P.B 18/20→19/09, ETD 20/08→20/17)</t>
+        </is>
+      </c>
+      <c r="U60" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20F (ETA 19/07→19/08)</t>
         </is>
       </c>
     </row>
@@ -3477,6 +3592,11 @@
       <c r="T61" s="5" t="inlineStr">
         <is>
           <t>expected · 20F (new, LOA 304 m)</t>
+        </is>
+      </c>
+      <c r="U61" s="6" t="inlineStr">
+        <is>
+          <t>alongside → 20D (ETA 16/15→16/18, P.B 16/15→17/03, ETD 17/06→17/15)</t>
         </is>
       </c>
     </row>
@@ -10929,7 +11049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12535,8 +12655,39 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" s="12" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B54" s="13" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="C54" s="13" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D54" s="14" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E54" s="14" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F54" s="13" t="inlineStr">
+        <is>
+          <t>CLOSE (Oct 5–20 2026) printed under 20E</t>
+        </is>
+      </c>
+      <c r="G54" s="13" t="inlineStr">
+        <is>
+          <t>Unchanged</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G53"/>
+  <autoFilter ref="A4:G54"/>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
@@ -14670,6 +14821,504 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 17 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Waiting for Berth (h)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>BANGKOK</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>551</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>46311.625</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>46312.375</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>46313.66666666666</v>
+      </c>
+      <c r="G4" s="24">
+        <f>(E4-D4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="24">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>TS CHIBA</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>485</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46311.58333333334</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46311.58333333334</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46312.45833333334</v>
+      </c>
+      <c r="G5" s="24">
+        <f>(E5-D5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="24">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>JARU BHUM</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46312.66666666666</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46312.66666666666</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46313.45833333334</v>
+      </c>
+      <c r="G6" s="24">
+        <f>(E6-D6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="24">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="J6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>LITTLE DOLPHIN</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46312.04166666666</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46312.33333333334</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46313.66666666666</v>
+      </c>
+      <c r="G7" s="24">
+        <f>(E7-D7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="24">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>PUNNYA NAVEE</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>304</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>46311.75</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>46312.125</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>46312.625</v>
+      </c>
+      <c r="G8" s="24">
+        <f>(E8-D8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="24">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>INFINITY</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>46313</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>46313.29166666666</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>46314.41666666666</v>
+      </c>
+      <c r="G9" s="24">
+        <f>(E9-D9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="24">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>INGENUITY</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>46311.95833333334</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>46312.33333333334</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>46313.29166666666</v>
+      </c>
+      <c r="G10" s="24">
+        <f>(E10-D10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="24">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 108</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>46312.41666666666</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>46313.33333333334</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>46314.29166666666</v>
+      </c>
+      <c r="G11" s="24">
+        <f>(E11-D11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="24">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J11" s="23" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>KMTC JAKARTA</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>46314.33333333334</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>46314.375</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>46315.70833333334</v>
+      </c>
+      <c r="G12" s="24">
+        <f>(E12-D12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="24">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J12" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="34" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G16" s="35" t="n"/>
+      <c r="H16" s="35" t="n"/>
+      <c r="I16" s="35" t="n"/>
+      <c r="J16" s="36" t="n"/>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C17" s="38" t="n"/>
+      <c r="D17" s="18" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E17" s="18" t="n">
+        <v>46315</v>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>CLOSE (Oct 5–20 2026) printed under 20E  —  Unchanged</t>
+        </is>
+      </c>
+      <c r="G17" s="38" t="n"/>
+      <c r="H17" s="38" t="n"/>
+      <c r="I17" s="38" t="n"/>
+      <c r="J17" s="38" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="F17:J17"/>
+    <mergeCell ref="F16:J16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -14717,7 +15366,7 @@
         </is>
       </c>
       <c r="B3" s="22" t="n">
-        <v>46311.375</v>
+        <v>46312.375</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -15366,9 +16015,10 @@
         </is>
       </c>
       <c r="N15" s="23" t="inlineStr"/>
-      <c r="O15" s="23">
-        <f>IF(J15&lt;=$B$3,"Sailed",IF(I15&lt;=$B$3,"Alongside",IF(H15&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O15" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -15389,10 +16039,10 @@
         <v>46293</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="F16" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
@@ -15400,7 +16050,7 @@
         </is>
       </c>
       <c r="H16" s="11" t="n">
-        <v>46311.875</v>
+        <v>46311.625</v>
       </c>
       <c r="I16" s="11" t="n">
         <v>46312.375</v>
@@ -15478,9 +16128,10 @@
         </is>
       </c>
       <c r="N17" s="23" t="inlineStr"/>
-      <c r="O17" s="23">
-        <f>IF(J17&lt;=$B$3,"Sailed",IF(I17&lt;=$B$3,"Alongside",IF(H17&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O17" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -16071,10 +16722,10 @@
         <v>46293</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="F28" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
@@ -16088,7 +16739,7 @@
         <v>46311.58333333334</v>
       </c>
       <c r="J28" s="11" t="n">
-        <v>46312.5</v>
+        <v>46312.45833333334</v>
       </c>
       <c r="K28" s="24">
         <f>(I28-H28)*24</f>
@@ -16127,10 +16778,10 @@
         <v>46293</v>
       </c>
       <c r="E29" s="10" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="F29" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
@@ -16619,9 +17270,10 @@
         </is>
       </c>
       <c r="N37" s="23" t="inlineStr"/>
-      <c r="O37" s="23">
-        <f>IF(J37&lt;=$B$3,"Sailed",IF(I37&lt;=$B$3,"Alongside",IF(H37&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O37" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -16642,10 +17294,10 @@
         <v>46310</v>
       </c>
       <c r="E38" s="10" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="F38" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -16653,7 +17305,7 @@
         </is>
       </c>
       <c r="H38" s="11" t="n">
-        <v>46311.79166666666</v>
+        <v>46312.04166666666</v>
       </c>
       <c r="I38" s="11" t="n">
         <v>46312.33333333334</v>
@@ -16731,9 +17383,10 @@
         </is>
       </c>
       <c r="N39" s="23" t="inlineStr"/>
-      <c r="O39" s="23">
-        <f>IF(J39&lt;=$B$3,"Sailed",IF(I39&lt;=$B$3,"Alongside",IF(H39&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O39" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="40">
@@ -17243,9 +17896,10 @@
         </is>
       </c>
       <c r="N48" s="23" t="inlineStr"/>
-      <c r="O48" s="23">
-        <f>IF(J48&lt;=$B$3,"Sailed",IF(I48&lt;=$B$3,"Alongside",IF(H48&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O48" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -17256,34 +17910,34 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>INFINITY</t>
+          <t>PUNNYA NAVEE</t>
         </is>
       </c>
       <c r="C49" s="23" t="n">
-        <v>565</v>
+        <v>304</v>
       </c>
       <c r="D49" s="10" t="n">
-        <v>46293</v>
+        <v>46311</v>
       </c>
       <c r="E49" s="10" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="F49" s="23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20C → 20D</t>
+          <t>20F → 20D</t>
         </is>
       </c>
       <c r="H49" s="11" t="n">
-        <v>46313.25</v>
+        <v>46311.75</v>
       </c>
       <c r="I49" s="11" t="n">
-        <v>46313.29166666666</v>
+        <v>46312.125</v>
       </c>
       <c r="J49" s="11" t="n">
-        <v>46314.41666666666</v>
+        <v>46312.625</v>
       </c>
       <c r="K49" s="24">
         <f>(I49-H49)*24</f>
@@ -17305,98 +17959,97 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="25" t="inlineStr">
-        <is>
-          <t>20E</t>
-        </is>
-      </c>
-      <c r="B50" s="25" t="inlineStr">
-        <is>
-          <t>WAN HAI 278</t>
-        </is>
-      </c>
-      <c r="C50" s="26" t="n">
-        <v>564</v>
-      </c>
-      <c r="D50" s="27" t="n">
-        <v>46295</v>
-      </c>
-      <c r="E50" s="27" t="n">
-        <v>46300</v>
-      </c>
-      <c r="F50" s="26" t="n">
-        <v>6</v>
-      </c>
-      <c r="G50" s="33" t="inlineStr">
-        <is>
-          <t>20F → 20E</t>
-        </is>
-      </c>
-      <c r="H50" s="29" t="n">
-        <v>46297.75</v>
-      </c>
-      <c r="I50" s="29" t="n">
-        <v>46298.41666666666</v>
-      </c>
-      <c r="J50" s="29" t="n">
-        <v>46300.45833333334</v>
-      </c>
-      <c r="K50" s="30">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>INFINITY</t>
+        </is>
+      </c>
+      <c r="C50" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D50" s="10" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E50" s="10" t="n">
+        <v>46312</v>
+      </c>
+      <c r="F50" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20C → 20D</t>
+        </is>
+      </c>
+      <c r="H50" s="11" t="n">
+        <v>46313</v>
+      </c>
+      <c r="I50" s="11" t="n">
+        <v>46313.29166666666</v>
+      </c>
+      <c r="J50" s="11" t="n">
+        <v>46314.41666666666</v>
+      </c>
+      <c r="K50" s="24">
         <f>(I50-H50)*24</f>
         <v/>
       </c>
-      <c r="L50" s="30">
+      <c r="L50" s="24">
         <f>(J50-I50)*24</f>
         <v/>
       </c>
-      <c r="M50" s="26" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N50" s="26" t="inlineStr"/>
-      <c r="O50" s="26" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="M50" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N50" s="23" t="inlineStr"/>
+      <c r="O50" s="23">
+        <f>IF(J50&lt;=$B$3,"Sailed",IF(I50&lt;=$B$3,"Alongside",IF(H50&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>20F</t>
+          <t>20E</t>
         </is>
       </c>
       <c r="B51" s="25" t="inlineStr">
         <is>
-          <t>HOPE C</t>
+          <t>WAN HAI 278</t>
         </is>
       </c>
       <c r="C51" s="26" t="n">
-        <v>481</v>
+        <v>564</v>
       </c>
       <c r="D51" s="27" t="n">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="E51" s="27" t="n">
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="F51" s="26" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G51" s="33" t="inlineStr">
         <is>
-          <t>20E → 20F</t>
+          <t>20F → 20E</t>
         </is>
       </c>
       <c r="H51" s="29" t="n">
-        <v>46294.70833333334</v>
+        <v>46297.75</v>
       </c>
       <c r="I51" s="29" t="n">
-        <v>46294.70833333334</v>
+        <v>46298.41666666666</v>
       </c>
       <c r="J51" s="29" t="n">
-        <v>46295.66666666666</v>
+        <v>46300.45833333334</v>
       </c>
       <c r="K51" s="30">
         <f>(I51-H51)*24</f>
@@ -17419,57 +18072,57 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+      <c r="A52" s="25" t="inlineStr">
         <is>
           <t>20F</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
-        <is>
-          <t>KMTC BANGKOK</t>
-        </is>
-      </c>
-      <c r="C52" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D52" s="10" t="n">
+      <c r="B52" s="25" t="inlineStr">
+        <is>
+          <t>HOPE C</t>
+        </is>
+      </c>
+      <c r="C52" s="26" t="n">
+        <v>481</v>
+      </c>
+      <c r="D52" s="27" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E52" s="27" t="n">
         <v>46295</v>
       </c>
-      <c r="E52" s="10" t="n">
-        <v>46298</v>
-      </c>
-      <c r="F52" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20F</t>
-        </is>
-      </c>
-      <c r="H52" s="11" t="n">
-        <v>46297.29166666666</v>
-      </c>
-      <c r="I52" s="11" t="n">
-        <v>46297.45833333334</v>
-      </c>
-      <c r="J52" s="11" t="n">
-        <v>46298.70833333334</v>
-      </c>
-      <c r="K52" s="24">
+      <c r="F52" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="G52" s="33" t="inlineStr">
+        <is>
+          <t>20E → 20F</t>
+        </is>
+      </c>
+      <c r="H52" s="29" t="n">
+        <v>46294.70833333334</v>
+      </c>
+      <c r="I52" s="29" t="n">
+        <v>46294.70833333334</v>
+      </c>
+      <c r="J52" s="29" t="n">
+        <v>46295.66666666666</v>
+      </c>
+      <c r="K52" s="30">
         <f>(I52-H52)*24</f>
         <v/>
       </c>
-      <c r="L52" s="24">
+      <c r="L52" s="30">
         <f>(J52-I52)*24</f>
         <v/>
       </c>
-      <c r="M52" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N52" s="23" t="inlineStr"/>
-      <c r="O52" s="23" t="inlineStr">
+      <c r="M52" s="26" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N52" s="26" t="inlineStr"/>
+      <c r="O52" s="26" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -17483,34 +18136,34 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 98</t>
+          <t>KMTC BANGKOK</t>
         </is>
       </c>
       <c r="C53" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D53" s="10" t="n">
-        <v>46297</v>
+        <v>46295</v>
       </c>
       <c r="E53" s="10" t="n">
-        <v>46299</v>
+        <v>46298</v>
       </c>
       <c r="F53" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G53" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+        <v>4</v>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20F</t>
         </is>
       </c>
       <c r="H53" s="11" t="n">
-        <v>46299.375</v>
+        <v>46297.29166666666</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>46299.375</v>
+        <v>46297.45833333334</v>
       </c>
       <c r="J53" s="11" t="n">
-        <v>46300.375</v>
+        <v>46298.70833333334</v>
       </c>
       <c r="K53" s="24">
         <f>(I53-H53)*24</f>
@@ -17540,20 +18193,20 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>XIN AN</t>
+          <t>XIN MING ZHOU 98</t>
         </is>
       </c>
       <c r="C54" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D54" s="10" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="E54" s="10" t="n">
-        <v>46304</v>
+        <v>46299</v>
       </c>
       <c r="F54" s="23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
@@ -17561,13 +18214,13 @@
         </is>
       </c>
       <c r="H54" s="11" t="n">
-        <v>46302.54166666666</v>
+        <v>46299.375</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>46302.58333333334</v>
+        <v>46299.375</v>
       </c>
       <c r="J54" s="11" t="n">
-        <v>46304.54166666666</v>
+        <v>46300.375</v>
       </c>
       <c r="K54" s="24">
         <f>(I54-H54)*24</f>
@@ -17597,7 +18250,7 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE ATLANTIC</t>
+          <t>XIN AN</t>
         </is>
       </c>
       <c r="C55" s="23" t="n">
@@ -17607,24 +18260,24 @@
         <v>46300</v>
       </c>
       <c r="E55" s="10" t="n">
-        <v>46306</v>
+        <v>46304</v>
       </c>
       <c r="F55" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="G55" s="6" t="inlineStr">
-        <is>
-          <t>20C → 20D → 20F</t>
+        <v>5</v>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
         </is>
       </c>
       <c r="H55" s="11" t="n">
-        <v>46302.83333333334</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="I55" s="11" t="n">
-        <v>46304.625</v>
+        <v>46302.58333333334</v>
       </c>
       <c r="J55" s="11" t="n">
-        <v>46306.5</v>
+        <v>46304.54166666666</v>
       </c>
       <c r="K55" s="24">
         <f>(I55-H55)*24</f>
@@ -17654,34 +18307,34 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>JOSCO SHINE</t>
+          <t>SAWASDEE ATLANTIC</t>
         </is>
       </c>
       <c r="C56" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D56" s="10" t="n">
-        <v>46304</v>
+        <v>46300</v>
       </c>
       <c r="E56" s="10" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="F56" s="23" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>20B → 20AB → 20F</t>
+          <t>20C → 20D → 20F</t>
         </is>
       </c>
       <c r="H56" s="11" t="n">
-        <v>46307.45833333334</v>
+        <v>46302.83333333334</v>
       </c>
       <c r="I56" s="11" t="n">
-        <v>46307.625</v>
+        <v>46304.625</v>
       </c>
       <c r="J56" s="11" t="n">
-        <v>46308.25</v>
+        <v>46306.5</v>
       </c>
       <c r="K56" s="24">
         <f>(I56-H56)*24</f>
@@ -17711,34 +18364,34 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>ALS SUMIRE</t>
+          <t>JOSCO SHINE</t>
         </is>
       </c>
       <c r="C57" s="23" t="n">
-        <v>537</v>
+        <v>564</v>
       </c>
       <c r="D57" s="10" t="n">
-        <v>46294</v>
+        <v>46304</v>
       </c>
       <c r="E57" s="10" t="n">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="F57" s="23" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>20F → 20D → 20C → 20B → 20F</t>
+          <t>20B → 20AB → 20F</t>
         </is>
       </c>
       <c r="H57" s="11" t="n">
-        <v>46307.91666666666</v>
+        <v>46307.45833333334</v>
       </c>
       <c r="I57" s="11" t="n">
+        <v>46307.625</v>
+      </c>
+      <c r="J57" s="11" t="n">
         <v>46308.25</v>
-      </c>
-      <c r="J57" s="11" t="n">
-        <v>46309.25</v>
       </c>
       <c r="K57" s="24">
         <f>(I57-H57)*24</f>
@@ -17750,7 +18403,7 @@
       </c>
       <c r="M57" s="23" t="inlineStr">
         <is>
-          <t>1C</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N57" s="23" t="inlineStr"/>
@@ -17768,34 +18421,34 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE INCHEON</t>
+          <t>ALS SUMIRE</t>
         </is>
       </c>
       <c r="C58" s="23" t="n">
-        <v>564</v>
+        <v>537</v>
       </c>
       <c r="D58" s="10" t="n">
-        <v>46307</v>
+        <v>46294</v>
       </c>
       <c r="E58" s="10" t="n">
-        <v>46310</v>
+        <v>46308</v>
       </c>
       <c r="F58" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G58" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+        <v>9</v>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>20F → 20D → 20C → 20B → 20F</t>
         </is>
       </c>
       <c r="H58" s="11" t="n">
-        <v>46308.625</v>
+        <v>46307.91666666666</v>
       </c>
       <c r="I58" s="11" t="n">
+        <v>46308.25</v>
+      </c>
+      <c r="J58" s="11" t="n">
         <v>46309.25</v>
-      </c>
-      <c r="J58" s="11" t="n">
-        <v>46311.25</v>
       </c>
       <c r="K58" s="24">
         <f>(I58-H58)*24</f>
@@ -17807,7 +18460,7 @@
       </c>
       <c r="M58" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>1C</t>
         </is>
       </c>
       <c r="N58" s="23" t="inlineStr"/>
@@ -17825,20 +18478,20 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>PUNNYA NAVEE</t>
+          <t>SAWASDEE INCHEON</t>
         </is>
       </c>
       <c r="C59" s="23" t="n">
-        <v>304</v>
+        <v>564</v>
       </c>
       <c r="D59" s="10" t="n">
-        <v>46311</v>
+        <v>46307</v>
       </c>
       <c r="E59" s="10" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="F59" s="23" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
@@ -17846,13 +18499,13 @@
         </is>
       </c>
       <c r="H59" s="11" t="n">
-        <v>46311.625</v>
+        <v>46308.625</v>
       </c>
       <c r="I59" s="11" t="n">
-        <v>46311.625</v>
+        <v>46309.25</v>
       </c>
       <c r="J59" s="11" t="n">
-        <v>46312.25</v>
+        <v>46311.25</v>
       </c>
       <c r="K59" s="24">
         <f>(I59-H59)*24</f>
@@ -17868,9 +18521,10 @@
         </is>
       </c>
       <c r="N59" s="23" t="inlineStr"/>
-      <c r="O59" s="23">
-        <f>IF(J59&lt;=$B$3,"Sailed",IF(I59&lt;=$B$3,"Alongside",IF(H59&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O59" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -17891,10 +18545,10 @@
         <v>46310</v>
       </c>
       <c r="E60" s="10" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="F60" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
@@ -17947,10 +18601,10 @@
         <v>46310</v>
       </c>
       <c r="E61" s="10" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="F61" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
@@ -18003,10 +18657,10 @@
         <v>46310</v>
       </c>
       <c r="E62" s="10" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="F62" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
@@ -18014,7 +18668,7 @@
         </is>
       </c>
       <c r="H62" s="11" t="n">
-        <v>46314.29166666666</v>
+        <v>46314.33333333334</v>
       </c>
       <c r="I62" s="11" t="n">
         <v>46314.375</v>

</xml_diff>

<commit_message>
Add 18 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -30,9 +30,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Oct 2026" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 Oct 2026" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 Oct 2026" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 Oct 2026" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$O$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -662,7 +663,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U61"/>
+  <dimension ref="A1:V61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -686,6 +687,7 @@
     <col width="44" customWidth="1" min="19" max="19"/>
     <col width="44" customWidth="1" min="20" max="20"/>
     <col width="44" customWidth="1" min="21" max="21"/>
+    <col width="44" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -806,6 +808,11 @@
       <c r="U4" s="3" t="inlineStr">
         <is>
           <t>17 Oct 2026</t>
+        </is>
+      </c>
+      <c r="V4" s="3" t="inlineStr">
+        <is>
+          <t>18 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -857,6 +864,11 @@
       <c r="U5" s="6" t="inlineStr">
         <is>
           <t>expected · 20D (ETA 18/06→17/24)</t>
+        </is>
+      </c>
+      <c r="V5" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20D (ETD 19/10→19/09)</t>
         </is>
       </c>
     </row>
@@ -902,6 +914,7 @@
       <c r="S6" s="5" t="inlineStr"/>
       <c r="T6" s="5" t="inlineStr"/>
       <c r="U6" s="5" t="inlineStr"/>
+      <c r="V6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -937,6 +950,7 @@
       <c r="S7" s="5" t="inlineStr"/>
       <c r="T7" s="5" t="inlineStr"/>
       <c r="U7" s="5" t="inlineStr"/>
+      <c r="V7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -976,6 +990,7 @@
       <c r="S8" s="5" t="inlineStr"/>
       <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr"/>
+      <c r="V8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1029,6 +1044,11 @@
       <c r="U9" s="5" t="inlineStr">
         <is>
           <t>alongside · 20AB (actual ETA 16/15, P.B 17/09)</t>
+        </is>
+      </c>
+      <c r="V9" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20AB (ETD 18/16→19/08)</t>
         </is>
       </c>
     </row>
@@ -1078,6 +1098,11 @@
           <t>alongside · 20B (ETD 17/12→17/11)</t>
         </is>
       </c>
+      <c r="V10" s="5" t="inlineStr">
+        <is>
+          <t>sailed (17/11)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1121,6 +1146,7 @@
       <c r="S11" s="5" t="inlineStr"/>
       <c r="T11" s="5" t="inlineStr"/>
       <c r="U11" s="5" t="inlineStr"/>
+      <c r="V11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1168,6 +1194,11 @@
           <t>expected · 20B (shift 7B)</t>
         </is>
       </c>
+      <c r="V12" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20B (ETD 18/11→18/10, 7B)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1223,6 +1254,11 @@
           <t>no longer listed (dropped from the sheet)</t>
         </is>
       </c>
+      <c r="V13" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20C (listed again; ETA 19/23→20/17, P.B 20/09→20/17, ETD 21/08→21/13)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1286,6 +1322,11 @@
           <t>20C row with only LOA 558 m printed (no name or times)</t>
         </is>
       </c>
+      <c r="V14" s="5" t="inlineStr">
+        <is>
+          <t>no longer listed (the unnamed LOA 558 m row is gone)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1345,6 +1386,7 @@
       </c>
       <c r="T15" s="5" t="inlineStr"/>
       <c r="U15" s="5" t="inlineStr"/>
+      <c r="V15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1408,6 +1450,7 @@
         </is>
       </c>
       <c r="U16" s="5" t="inlineStr"/>
+      <c r="V16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1479,6 +1522,7 @@
       <c r="S17" s="5" t="inlineStr"/>
       <c r="T17" s="5" t="inlineStr"/>
       <c r="U17" s="5" t="inlineStr"/>
+      <c r="V17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1526,6 +1570,7 @@
       <c r="S18" s="5" t="inlineStr"/>
       <c r="T18" s="5" t="inlineStr"/>
       <c r="U18" s="5" t="inlineStr"/>
+      <c r="V18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1581,6 +1626,7 @@
       <c r="S19" s="5" t="inlineStr"/>
       <c r="T19" s="5" t="inlineStr"/>
       <c r="U19" s="5" t="inlineStr"/>
+      <c r="V19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1636,6 +1682,7 @@
       <c r="S20" s="5" t="inlineStr"/>
       <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr"/>
+      <c r="V20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1687,6 +1734,7 @@
       <c r="S21" s="5" t="inlineStr"/>
       <c r="T21" s="5" t="inlineStr"/>
       <c r="U21" s="5" t="inlineStr"/>
+      <c r="V21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1734,6 +1782,7 @@
       <c r="S22" s="5" t="inlineStr"/>
       <c r="T22" s="5" t="inlineStr"/>
       <c r="U22" s="5" t="inlineStr"/>
+      <c r="V22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1793,6 +1842,7 @@
       <c r="S23" s="5" t="inlineStr"/>
       <c r="T23" s="5" t="inlineStr"/>
       <c r="U23" s="5" t="inlineStr"/>
+      <c r="V23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1848,6 +1898,7 @@
       <c r="S24" s="5" t="inlineStr"/>
       <c r="T24" s="5" t="inlineStr"/>
       <c r="U24" s="5" t="inlineStr"/>
+      <c r="V24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1887,6 +1938,7 @@
       <c r="S25" s="5" t="inlineStr"/>
       <c r="T25" s="5" t="inlineStr"/>
       <c r="U25" s="5" t="inlineStr"/>
+      <c r="V25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1930,6 +1982,7 @@
       <c r="S26" s="5" t="inlineStr"/>
       <c r="T26" s="5" t="inlineStr"/>
       <c r="U26" s="5" t="inlineStr"/>
+      <c r="V26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1985,6 +2038,7 @@
       <c r="S27" s="5" t="inlineStr"/>
       <c r="T27" s="5" t="inlineStr"/>
       <c r="U27" s="5" t="inlineStr"/>
+      <c r="V27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2036,6 +2090,7 @@
       <c r="S28" s="5" t="inlineStr"/>
       <c r="T28" s="5" t="inlineStr"/>
       <c r="U28" s="5" t="inlineStr"/>
+      <c r="V28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2087,6 +2142,7 @@
       <c r="S29" s="5" t="inlineStr"/>
       <c r="T29" s="5" t="inlineStr"/>
       <c r="U29" s="5" t="inlineStr"/>
+      <c r="V29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -2146,6 +2202,7 @@
       <c r="S30" s="5" t="inlineStr"/>
       <c r="T30" s="5" t="inlineStr"/>
       <c r="U30" s="5" t="inlineStr"/>
+      <c r="V30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2193,6 +2250,11 @@
       <c r="S31" s="5" t="inlineStr"/>
       <c r="T31" s="5" t="inlineStr"/>
       <c r="U31" s="5" t="inlineStr"/>
+      <c r="V31" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20B (returns for a new call, ETA 20/15)</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2244,6 +2306,7 @@
       <c r="S32" s="5" t="inlineStr"/>
       <c r="T32" s="5" t="inlineStr"/>
       <c r="U32" s="5" t="inlineStr"/>
+      <c r="V32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2291,6 +2354,7 @@
       <c r="S33" s="5" t="inlineStr"/>
       <c r="T33" s="5" t="inlineStr"/>
       <c r="U33" s="5" t="inlineStr"/>
+      <c r="V33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2342,6 +2406,7 @@
       <c r="S34" s="5" t="inlineStr"/>
       <c r="T34" s="5" t="inlineStr"/>
       <c r="U34" s="5" t="inlineStr"/>
+      <c r="V34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2393,6 +2458,7 @@
       <c r="S35" s="5" t="inlineStr"/>
       <c r="T35" s="5" t="inlineStr"/>
       <c r="U35" s="5" t="inlineStr"/>
+      <c r="V35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2440,6 +2506,7 @@
       <c r="S36" s="5" t="inlineStr"/>
       <c r="T36" s="5" t="inlineStr"/>
       <c r="U36" s="5" t="inlineStr"/>
+      <c r="V36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2491,6 +2558,7 @@
       <c r="S37" s="5" t="inlineStr"/>
       <c r="T37" s="5" t="inlineStr"/>
       <c r="U37" s="5" t="inlineStr"/>
+      <c r="V37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2542,6 +2610,7 @@
       <c r="S38" s="5" t="inlineStr"/>
       <c r="T38" s="5" t="inlineStr"/>
       <c r="U38" s="5" t="inlineStr"/>
+      <c r="V38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2589,6 +2658,7 @@
       <c r="S39" s="5" t="inlineStr"/>
       <c r="T39" s="5" t="inlineStr"/>
       <c r="U39" s="5" t="inlineStr"/>
+      <c r="V39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -2636,6 +2706,7 @@
       <c r="S40" s="5" t="inlineStr"/>
       <c r="T40" s="5" t="inlineStr"/>
       <c r="U40" s="5" t="inlineStr"/>
+      <c r="V40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2687,6 +2758,7 @@
       <c r="S41" s="5" t="inlineStr"/>
       <c r="T41" s="5" t="inlineStr"/>
       <c r="U41" s="5" t="inlineStr"/>
+      <c r="V41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -2734,6 +2806,7 @@
       <c r="S42" s="5" t="inlineStr"/>
       <c r="T42" s="5" t="inlineStr"/>
       <c r="U42" s="5" t="inlineStr"/>
+      <c r="V42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2785,6 +2858,7 @@
       <c r="S43" s="5" t="inlineStr"/>
       <c r="T43" s="5" t="inlineStr"/>
       <c r="U43" s="5" t="inlineStr"/>
+      <c r="V43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -2836,6 +2910,7 @@
       <c r="S44" s="5" t="inlineStr"/>
       <c r="T44" s="5" t="inlineStr"/>
       <c r="U44" s="5" t="inlineStr"/>
+      <c r="V44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -2883,6 +2958,7 @@
       <c r="S45" s="5" t="inlineStr"/>
       <c r="T45" s="5" t="inlineStr"/>
       <c r="U45" s="5" t="inlineStr"/>
+      <c r="V45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -2938,6 +3014,7 @@
       </c>
       <c r="T46" s="5" t="inlineStr"/>
       <c r="U46" s="5" t="inlineStr"/>
+      <c r="V46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -2989,6 +3066,7 @@
       <c r="S47" s="5" t="inlineStr"/>
       <c r="T47" s="5" t="inlineStr"/>
       <c r="U47" s="5" t="inlineStr"/>
+      <c r="V47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -3040,6 +3118,7 @@
       </c>
       <c r="T48" s="5" t="inlineStr"/>
       <c r="U48" s="5" t="inlineStr"/>
+      <c r="V48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -3091,6 +3170,7 @@
       </c>
       <c r="T49" s="5" t="inlineStr"/>
       <c r="U49" s="5" t="inlineStr"/>
+      <c r="V49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -3138,6 +3218,7 @@
       </c>
       <c r="T50" s="5" t="inlineStr"/>
       <c r="U50" s="5" t="inlineStr"/>
+      <c r="V50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -3181,6 +3262,7 @@
       </c>
       <c r="T51" s="5" t="inlineStr"/>
       <c r="U51" s="5" t="inlineStr"/>
+      <c r="V51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -3228,6 +3310,7 @@
         </is>
       </c>
       <c r="U52" s="5" t="inlineStr"/>
+      <c r="V52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -3275,6 +3358,7 @@
           <t>sailed (16/16)</t>
         </is>
       </c>
+      <c r="V53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -3322,6 +3406,7 @@
           <t>sailed (16/15)</t>
         </is>
       </c>
+      <c r="V54" s="5" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -3361,6 +3446,7 @@
         </is>
       </c>
       <c r="U55" s="5" t="inlineStr"/>
+      <c r="V55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -3404,6 +3490,7 @@
           <t>sailed (17/08)</t>
         </is>
       </c>
+      <c r="V56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -3445,6 +3532,11 @@
       <c r="U57" s="5" t="inlineStr">
         <is>
           <t>alongside · 20C (actual ETA 17/01)</t>
+        </is>
+      </c>
+      <c r="V57" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20C (ETD 18/16)</t>
         </is>
       </c>
     </row>
@@ -3486,6 +3578,11 @@
           <t>expected · 20F</t>
         </is>
       </c>
+      <c r="V58" s="5" t="inlineStr">
+        <is>
+          <t>alongside · 20F (ETD 19/07)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -3525,6 +3622,11 @@
           <t>alongside · 20F (actual ETA 16/23)</t>
         </is>
       </c>
+      <c r="V59" s="5" t="inlineStr">
+        <is>
+          <t>sailed (18/07)</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -3562,6 +3664,11 @@
       <c r="U60" s="6" t="inlineStr">
         <is>
           <t>expected · 20F (ETA 19/07→19/08)</t>
+        </is>
+      </c>
+      <c r="V60" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20F (marked, ETA 19/08→19/12, P.B 19/09→19/12, ETD 20/17)</t>
         </is>
       </c>
     </row>
@@ -3597,6 +3704,11 @@
       <c r="U61" s="6" t="inlineStr">
         <is>
           <t>alongside → 20D (ETA 16/15→16/18, P.B 16/15→17/03, ETD 17/06→17/15)</t>
+        </is>
+      </c>
+      <c r="V61" s="5" t="inlineStr">
+        <is>
+          <t>sailed (17/15)</t>
         </is>
       </c>
     </row>
@@ -11049,7 +11161,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12686,8 +12798,76 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" s="12" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B55" s="13" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C55" s="13" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D55" s="14" t="n">
+        <v>46314</v>
+      </c>
+      <c r="E55" s="19" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F55" s="13" t="inlineStr">
+        <is>
+          <t>20D CLOSE from Oct 19 2026 (end date not printed on the sheet)</t>
+        </is>
+      </c>
+      <c r="G55" s="13" t="inlineStr">
+        <is>
+          <t>New</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="15" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="C56" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E56" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F56" s="16" t="inlineStr">
+        <is>
+          <t>(no notice – the CLOSE (Oct 5–20 2026) line under 20E is gone)</t>
+        </is>
+      </c>
+      <c r="G56" s="16" t="inlineStr">
+        <is>
+          <t>Dropped from sheet: 20E closure no longer printed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G54"/>
+  <autoFilter ref="A4:G56"/>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
@@ -15313,6 +15493,505 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="F17:J17"/>
+    <mergeCell ref="F16:J16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 18 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Waiting for Berth (h)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>BANGKOK</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>551</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>46311.625</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>46312.375</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>46314.33333333334</v>
+      </c>
+      <c r="G4" s="24">
+        <f>(E4-D4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="24">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>JARU BHUM</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46312.66666666666</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46312.66666666666</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46313.41666666666</v>
+      </c>
+      <c r="G5" s="24">
+        <f>(E5-D5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="24">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>7B</t>
+        </is>
+      </c>
+      <c r="J5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>MTT BANGKOK</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46315.625</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46315.625</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46316.54166666666</v>
+      </c>
+      <c r="G6" s="24">
+        <f>(E6-D6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="24">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>LITTLE DOLPHIN</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46312.04166666666</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46312.33333333334</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46313.66666666666</v>
+      </c>
+      <c r="G7" s="24">
+        <f>(E7-D7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="24">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>MITRA BHUM</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>485</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>46315.70833333334</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>46315.70833333334</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>46316.54166666666</v>
+      </c>
+      <c r="G8" s="24">
+        <f>(E8-D8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="24">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>INFINITY</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>46313</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>46313.29166666666</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>46314.375</v>
+      </c>
+      <c r="G9" s="24">
+        <f>(E9-D9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="24">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 108</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>46312.41666666666</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>46313.33333333334</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>46314.29166666666</v>
+      </c>
+      <c r="G10" s="24">
+        <f>(E10-D10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="24">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>KMTC JAKARTA</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="n">
+        <v>564</v>
+      </c>
+      <c r="D11" s="20" t="n">
+        <v>46314.5</v>
+      </c>
+      <c r="E11" s="20" t="n">
+        <v>46314.5</v>
+      </c>
+      <c r="F11" s="20" t="n">
+        <v>46315.70833333334</v>
+      </c>
+      <c r="G11" s="32">
+        <f>(E11-D11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="32">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J11" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="34" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G15" s="35" t="n"/>
+      <c r="H15" s="35" t="n"/>
+      <c r="I15" s="35" t="n"/>
+      <c r="J15" s="36" t="n"/>
+    </row>
+    <row r="16" ht="42" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C16" s="38" t="n"/>
+      <c r="D16" s="18" t="n">
+        <v>46314</v>
+      </c>
+      <c r="E16" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>20D CLOSE from Oct 19 2026 (end date not printed on the sheet)  —  New</t>
+        </is>
+      </c>
+      <c r="G16" s="38" t="n"/>
+      <c r="H16" s="38" t="n"/>
+      <c r="I16" s="38" t="n"/>
+      <c r="J16" s="38" t="n"/>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C17" s="38" t="n"/>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>(no notice – the CLOSE (Oct 5–20 2026) line under 20E is gone)  —  Dropped from sheet: 20E closure no longer printed</t>
+        </is>
+      </c>
+      <c r="G17" s="38" t="n"/>
+      <c r="H17" s="38" t="n"/>
+      <c r="I17" s="38" t="n"/>
+      <c r="J17" s="38" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="F17:J17"/>
+    <mergeCell ref="F15:J15"/>
     <mergeCell ref="F16:J16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15366,7 +16045,7 @@
         </is>
       </c>
       <c r="B3" s="22" t="n">
-        <v>46312.375</v>
+        <v>46313.375</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -16039,10 +16718,10 @@
         <v>46293</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="F16" s="23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
@@ -16056,7 +16735,7 @@
         <v>46312.375</v>
       </c>
       <c r="J16" s="11" t="n">
-        <v>46313.66666666666</v>
+        <v>46314.33333333334</v>
       </c>
       <c r="K16" s="24">
         <f>(I16-H16)*24</f>
@@ -16078,114 +16757,114 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>20AB</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>MITRA BHUM</t>
-        </is>
-      </c>
-      <c r="C17" s="23" t="n">
-        <v>485</v>
-      </c>
-      <c r="D17" s="10" t="n">
+      <c r="A17" s="25" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B17" s="25" t="inlineStr">
+        <is>
+          <t>KMTC GWANGYANG</t>
+        </is>
+      </c>
+      <c r="C17" s="26" t="n">
+        <v>564</v>
+      </c>
+      <c r="D17" s="27" t="n">
         <v>46293</v>
       </c>
-      <c r="E17" s="10" t="n">
-        <v>46311</v>
-      </c>
-      <c r="F17" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20E → 20D → 20AB</t>
-        </is>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>46314.95833333334</v>
-      </c>
-      <c r="I17" s="11" t="n">
-        <v>46315.375</v>
-      </c>
-      <c r="J17" s="11" t="n">
-        <v>46316.33333333334</v>
-      </c>
-      <c r="K17" s="24">
+      <c r="E17" s="27" t="n">
+        <v>46293</v>
+      </c>
+      <c r="F17" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="28" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="H17" s="29" t="n">
+        <v>46292.79166666666</v>
+      </c>
+      <c r="I17" s="29" t="n">
+        <v>46292.79166666666</v>
+      </c>
+      <c r="J17" s="29" t="n">
+        <v>46294.20833333334</v>
+      </c>
+      <c r="K17" s="30">
         <f>(I17-H17)*24</f>
         <v/>
       </c>
-      <c r="L17" s="24">
+      <c r="L17" s="30">
         <f>(J17-I17)*24</f>
         <v/>
       </c>
-      <c r="M17" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N17" s="23" t="inlineStr"/>
-      <c r="O17" s="23" t="inlineStr">
+      <c r="M17" s="26" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N17" s="26" t="inlineStr"/>
+      <c r="O17" s="26" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>20B</t>
         </is>
       </c>
-      <c r="B18" s="25" t="inlineStr">
-        <is>
-          <t>KMTC GWANGYANG</t>
-        </is>
-      </c>
-      <c r="C18" s="26" t="n">
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>MILLENNIUM BRIGHT</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D18" s="27" t="n">
+      <c r="D18" s="10" t="n">
         <v>46293</v>
       </c>
-      <c r="E18" s="27" t="n">
-        <v>46293</v>
-      </c>
-      <c r="F18" s="26" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="28" t="inlineStr">
+      <c r="E18" s="10" t="n">
+        <v>46294</v>
+      </c>
+      <c r="F18" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="5" t="inlineStr">
         <is>
           <t>20B</t>
         </is>
       </c>
-      <c r="H18" s="29" t="n">
-        <v>46292.79166666666</v>
-      </c>
-      <c r="I18" s="29" t="n">
-        <v>46292.79166666666</v>
-      </c>
-      <c r="J18" s="29" t="n">
+      <c r="H18" s="11" t="n">
+        <v>46293.45833333334</v>
+      </c>
+      <c r="I18" s="11" t="n">
         <v>46294.20833333334</v>
       </c>
-      <c r="K18" s="30">
+      <c r="J18" s="11" t="n">
+        <v>46295.16666666666</v>
+      </c>
+      <c r="K18" s="24">
         <f>(I18-H18)*24</f>
         <v/>
       </c>
-      <c r="L18" s="30">
+      <c r="L18" s="24">
         <f>(J18-I18)*24</f>
         <v/>
       </c>
-      <c r="M18" s="26" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N18" s="26" t="inlineStr"/>
-      <c r="O18" s="26" t="inlineStr">
+      <c r="M18" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N18" s="23" t="inlineStr"/>
+      <c r="O18" s="23" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -16199,34 +16878,34 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>MILLENNIUM BRIGHT</t>
+          <t>YM IMPROVEMENT</t>
         </is>
       </c>
       <c r="C19" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="E19" s="10" t="n">
-        <v>46294</v>
+        <v>46300</v>
       </c>
       <c r="F19" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>5</v>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>20C → 20B</t>
         </is>
       </c>
       <c r="H19" s="11" t="n">
-        <v>46293.45833333334</v>
+        <v>46298.95833333334</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>46294.20833333334</v>
+        <v>46299.41666666666</v>
       </c>
       <c r="J19" s="11" t="n">
-        <v>46295.16666666666</v>
+        <v>46300.5</v>
       </c>
       <c r="K19" s="24">
         <f>(I19-H19)*24</f>
@@ -16256,34 +16935,34 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>YM IMPROVEMENT</t>
+          <t>SAWASDEE SPICA</t>
         </is>
       </c>
       <c r="C20" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>46296</v>
+        <v>46299</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="F20" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>20C → 20B</t>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H20" s="11" t="n">
-        <v>46298.95833333334</v>
+        <v>46300.875</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>46299.41666666666</v>
+        <v>46301.54166666666</v>
       </c>
       <c r="J20" s="11" t="n">
-        <v>46300.5</v>
+        <v>46303.54166666666</v>
       </c>
       <c r="K20" s="24">
         <f>(I20-H20)*24</f>
@@ -16313,34 +16992,34 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE SPICA</t>
+          <t>SITC HOCHIMINH</t>
         </is>
       </c>
       <c r="C21" s="23" t="n">
-        <v>564</v>
+        <v>470</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>46299</v>
+        <v>46301</v>
       </c>
       <c r="E21" s="10" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="F21" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>4</v>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20B</t>
         </is>
       </c>
       <c r="H21" s="11" t="n">
-        <v>46300.875</v>
+        <v>46302.625</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>46301.54166666666</v>
+        <v>46303.58333333334</v>
       </c>
       <c r="J21" s="11" t="n">
-        <v>46303.54166666666</v>
+        <v>46304.70833333334</v>
       </c>
       <c r="K21" s="24">
         <f>(I21-H21)*24</f>
@@ -16370,34 +17049,34 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>SITC HOCHIMINH</t>
+          <t>INDURO</t>
         </is>
       </c>
       <c r="C22" s="23" t="n">
-        <v>470</v>
+        <v>565</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="F22" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20B</t>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H22" s="11" t="n">
-        <v>46302.625</v>
+        <v>46304.25</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>46303.58333333334</v>
+        <v>46304.66666666666</v>
       </c>
       <c r="J22" s="11" t="n">
-        <v>46304.70833333334</v>
+        <v>46306.16666666666</v>
       </c>
       <c r="K22" s="24">
         <f>(I22-H22)*24</f>
@@ -16427,34 +17106,34 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>INDURO</t>
+          <t>XIN MING ZHOU 102</t>
         </is>
       </c>
       <c r="C23" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D23" s="10" t="n">
         <v>46302</v>
       </c>
       <c r="E23" s="10" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="F23" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>5</v>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>20F → 20B</t>
         </is>
       </c>
       <c r="H23" s="11" t="n">
-        <v>46304.25</v>
+        <v>46305.875</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>46304.66666666666</v>
+        <v>46306.20833333334</v>
       </c>
       <c r="J23" s="11" t="n">
-        <v>46306.16666666666</v>
+        <v>46307.08333333334</v>
       </c>
       <c r="K23" s="24">
         <f>(I23-H23)*24</f>
@@ -16484,34 +17163,34 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 102</t>
+          <t>CEBU</t>
         </is>
       </c>
       <c r="C24" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="E24" s="10" t="n">
-        <v>46306</v>
+        <v>46309</v>
       </c>
       <c r="F24" s="23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>20F → 20B</t>
+          <t>20AB → 20B</t>
         </is>
       </c>
       <c r="H24" s="11" t="n">
-        <v>46305.875</v>
+        <v>46307.91666666666</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>46306.20833333334</v>
+        <v>46308.25</v>
       </c>
       <c r="J24" s="11" t="n">
-        <v>46307.08333333334</v>
+        <v>46309.54166666666</v>
       </c>
       <c r="K24" s="24">
         <f>(I24-H24)*24</f>
@@ -16541,34 +17220,34 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>CEBU</t>
+          <t>M ODYSSEY</t>
         </is>
       </c>
       <c r="C25" s="23" t="n">
-        <v>564</v>
+        <v>449</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>46306</v>
+        <v>46293</v>
       </c>
       <c r="E25" s="10" t="n">
         <v>46309</v>
       </c>
       <c r="F25" s="23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20B</t>
+          <t>20B → 20C → 20B</t>
         </is>
       </c>
       <c r="H25" s="11" t="n">
-        <v>46307.91666666666</v>
+        <v>46309.04166666666</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>46308.25</v>
+        <v>46309.625</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>46309.54166666666</v>
+        <v>46310.20833333334</v>
       </c>
       <c r="K25" s="24">
         <f>(I25-H25)*24</f>
@@ -16580,7 +17259,7 @@
       </c>
       <c r="M25" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="N25" s="23" t="inlineStr"/>
@@ -16598,34 +17277,34 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>M ODYSSEY</t>
+          <t>KHARIS HERITAGE</t>
         </is>
       </c>
       <c r="C26" s="23" t="n">
-        <v>449</v>
+        <v>482</v>
       </c>
       <c r="D26" s="10" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="E26" s="10" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="F26" s="23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>20B → 20C → 20B</t>
+          <t>20AB → 20B → 20C → 20B</t>
         </is>
       </c>
       <c r="H26" s="11" t="n">
-        <v>46309.04166666666</v>
+        <v>46310.04166666666</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>46309.625</v>
+        <v>46310.25</v>
       </c>
       <c r="J26" s="11" t="n">
-        <v>46310.20833333334</v>
+        <v>46311.29166666666</v>
       </c>
       <c r="K26" s="24">
         <f>(I26-H26)*24</f>
@@ -16637,7 +17316,7 @@
       </c>
       <c r="M26" s="23" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N26" s="23" t="inlineStr"/>
@@ -16655,34 +17334,34 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>KHARIS HERITAGE</t>
+          <t>TS CHIBA</t>
         </is>
       </c>
       <c r="C27" s="23" t="n">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="D27" s="10" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="E27" s="10" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="F27" s="23" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20B → 20C → 20B</t>
+          <t>20E → 20C → 20B</t>
         </is>
       </c>
       <c r="H27" s="11" t="n">
-        <v>46310.04166666666</v>
+        <v>46311.58333333334</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>46310.25</v>
+        <v>46311.58333333334</v>
       </c>
       <c r="J27" s="11" t="n">
-        <v>46311.29166666666</v>
+        <v>46312.45833333334</v>
       </c>
       <c r="K27" s="24">
         <f>(I27-H27)*24</f>
@@ -16712,34 +17391,34 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>TS CHIBA</t>
+          <t>JARU BHUM</t>
         </is>
       </c>
       <c r="C28" s="23" t="n">
-        <v>485</v>
+        <v>564</v>
       </c>
       <c r="D28" s="10" t="n">
         <v>46293</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="F28" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>20E → 20C → 20B</t>
+          <t>20F → 20D → 20B</t>
         </is>
       </c>
       <c r="H28" s="11" t="n">
-        <v>46311.58333333334</v>
+        <v>46312.66666666666</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>46311.58333333334</v>
+        <v>46312.66666666666</v>
       </c>
       <c r="J28" s="11" t="n">
-        <v>46312.45833333334</v>
+        <v>46313.41666666666</v>
       </c>
       <c r="K28" s="24">
         <f>(I28-H28)*24</f>
@@ -16751,7 +17430,7 @@
       </c>
       <c r="M28" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="N28" s="23" t="inlineStr"/>
@@ -16768,34 +17447,34 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>JARU BHUM</t>
+          <t>MTT BANGKOK</t>
         </is>
       </c>
       <c r="C29" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D29" s="10" t="n">
-        <v>46293</v>
+        <v>46300</v>
       </c>
       <c r="E29" s="10" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="F29" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>20F → 20D → 20B</t>
+          <t>20D → 20B</t>
         </is>
       </c>
       <c r="H29" s="11" t="n">
-        <v>46312.66666666666</v>
+        <v>46315.625</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>46312.66666666666</v>
+        <v>46315.625</v>
       </c>
       <c r="J29" s="11" t="n">
-        <v>46313.45833333334</v>
+        <v>46316.54166666666</v>
       </c>
       <c r="K29" s="24">
         <f>(I29-H29)*24</f>
@@ -16807,7 +17486,7 @@
       </c>
       <c r="M29" s="23" t="inlineStr">
         <is>
-          <t>7B</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N29" s="23" t="inlineStr"/>
@@ -17294,10 +17973,10 @@
         <v>46310</v>
       </c>
       <c r="E38" s="10" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="F38" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -17390,114 +18069,113 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="25" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>MITRA BHUM</t>
+        </is>
+      </c>
+      <c r="C40" s="23" t="n">
+        <v>485</v>
+      </c>
+      <c r="D40" s="10" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E40" s="10" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F40" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="G40" s="6" t="inlineStr">
+        <is>
+          <t>20F → 20E → 20D → 20AB → 20C</t>
+        </is>
+      </c>
+      <c r="H40" s="11" t="n">
+        <v>46315.70833333334</v>
+      </c>
+      <c r="I40" s="11" t="n">
+        <v>46315.70833333334</v>
+      </c>
+      <c r="J40" s="11" t="n">
+        <v>46316.54166666666</v>
+      </c>
+      <c r="K40" s="24">
+        <f>(I40-H40)*24</f>
+        <v/>
+      </c>
+      <c r="L40" s="24">
+        <f>(J40-I40)*24</f>
+        <v/>
+      </c>
+      <c r="M40" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N40" s="23" t="inlineStr"/>
+      <c r="O40" s="23">
+        <f>IF(J40&lt;=$B$3,"Sailed",IF(I40&lt;=$B$3,"Alongside",IF(H40&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="25" t="inlineStr">
         <is>
           <t>20D</t>
         </is>
       </c>
-      <c r="B40" s="25" t="inlineStr">
+      <c r="B41" s="25" t="inlineStr">
         <is>
           <t>HARI BHUM (Barge)</t>
         </is>
       </c>
-      <c r="C40" s="26" t="n">
+      <c r="C41" s="26" t="n">
         <v>259</v>
       </c>
-      <c r="D40" s="27" t="n">
+      <c r="D41" s="27" t="n">
         <v>46297</v>
       </c>
-      <c r="E40" s="27" t="n">
+      <c r="E41" s="27" t="n">
         <v>46298</v>
       </c>
-      <c r="F40" s="26" t="n">
+      <c r="F41" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="G40" s="28" t="inlineStr">
+      <c r="G41" s="28" t="inlineStr">
         <is>
           <t>20D</t>
         </is>
       </c>
-      <c r="H40" s="29" t="n">
+      <c r="H41" s="29" t="n">
         <v>46298.20833333334</v>
       </c>
-      <c r="I40" s="29" t="n">
+      <c r="I41" s="29" t="n">
         <v>46298.29166666666</v>
       </c>
-      <c r="J40" s="29" t="n">
+      <c r="J41" s="29" t="n">
         <v>46298.66666666666</v>
       </c>
-      <c r="K40" s="30">
-        <f>(I40-H40)*24</f>
-        <v/>
-      </c>
-      <c r="L40" s="30">
-        <f>(J40-I40)*24</f>
-        <v/>
-      </c>
-      <c r="M40" s="26" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N40" s="26" t="inlineStr"/>
-      <c r="O40" s="26" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="B41" s="4" t="inlineStr">
-        <is>
-          <t>MTT BANGKOK</t>
-        </is>
-      </c>
-      <c r="C41" s="23" t="n">
-        <v>564</v>
-      </c>
-      <c r="D41" s="10" t="n">
-        <v>46300</v>
-      </c>
-      <c r="E41" s="10" t="n">
-        <v>46303</v>
-      </c>
-      <c r="F41" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="H41" s="11" t="n">
-        <v>46302.54166666666</v>
-      </c>
-      <c r="I41" s="11" t="n">
-        <v>46302.58333333334</v>
-      </c>
-      <c r="J41" s="11" t="n">
-        <v>46304.08333333334</v>
-      </c>
-      <c r="K41" s="24">
+      <c r="K41" s="30">
         <f>(I41-H41)*24</f>
         <v/>
       </c>
-      <c r="L41" s="24">
+      <c r="L41" s="30">
         <f>(J41-I41)*24</f>
         <v/>
       </c>
-      <c r="M41" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N41" s="23" t="inlineStr"/>
-      <c r="O41" s="23" t="inlineStr">
+      <c r="M41" s="26" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N41" s="26" t="inlineStr"/>
+      <c r="O41" s="26" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -17953,9 +18631,10 @@
         </is>
       </c>
       <c r="N49" s="23" t="inlineStr"/>
-      <c r="O49" s="23">
-        <f>IF(J49&lt;=$B$3,"Sailed",IF(I49&lt;=$B$3,"Alongside",IF(H49&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O49" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -17976,10 +18655,10 @@
         <v>46293</v>
       </c>
       <c r="E50" s="10" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="F50" s="23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
@@ -17993,7 +18672,7 @@
         <v>46313.29166666666</v>
       </c>
       <c r="J50" s="11" t="n">
-        <v>46314.41666666666</v>
+        <v>46314.375</v>
       </c>
       <c r="K50" s="24">
         <f>(I50-H50)*24</f>
@@ -18578,9 +19257,10 @@
         </is>
       </c>
       <c r="N60" s="23" t="inlineStr"/>
-      <c r="O60" s="23">
-        <f>IF(J60&lt;=$B$3,"Sailed",IF(I60&lt;=$B$3,"Alongside",IF(H60&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O60" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="61">
@@ -18601,10 +19281,10 @@
         <v>46310</v>
       </c>
       <c r="E61" s="10" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="F61" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
@@ -18640,57 +19320,61 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="4" t="inlineStr">
+      <c r="A62" s="31" t="inlineStr">
         <is>
           <t>20F</t>
         </is>
       </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="B62" s="31" t="inlineStr">
         <is>
           <t>KMTC JAKARTA</t>
         </is>
       </c>
-      <c r="C62" s="23" t="n">
+      <c r="C62" s="17" t="n">
         <v>564</v>
       </c>
-      <c r="D62" s="10" t="n">
+      <c r="D62" s="18" t="n">
         <v>46310</v>
       </c>
-      <c r="E62" s="10" t="n">
-        <v>46312</v>
-      </c>
-      <c r="F62" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G62" s="5" t="inlineStr">
+      <c r="E62" s="18" t="n">
+        <v>46313</v>
+      </c>
+      <c r="F62" s="17" t="n">
+        <v>4</v>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
         <is>
           <t>20F</t>
         </is>
       </c>
-      <c r="H62" s="11" t="n">
-        <v>46314.33333333334</v>
-      </c>
-      <c r="I62" s="11" t="n">
-        <v>46314.375</v>
-      </c>
-      <c r="J62" s="11" t="n">
+      <c r="H62" s="20" t="n">
+        <v>46314.5</v>
+      </c>
+      <c r="I62" s="20" t="n">
+        <v>46314.5</v>
+      </c>
+      <c r="J62" s="20" t="n">
         <v>46315.70833333334</v>
       </c>
-      <c r="K62" s="24">
+      <c r="K62" s="32">
         <f>(I62-H62)*24</f>
         <v/>
       </c>
-      <c r="L62" s="24">
+      <c r="L62" s="32">
         <f>(J62-I62)*24</f>
         <v/>
       </c>
-      <c r="M62" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N62" s="23" t="inlineStr"/>
-      <c r="O62" s="23">
+      <c r="M62" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N62" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O62" s="17">
         <f>IF(J62&lt;=$B$3,"Sailed",IF(I62&lt;=$B$3,"Alongside",IF(H62&lt;=$B$3,"At anchorage","Expected")))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add 19 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -31,9 +31,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 Oct 2026" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 Oct 2026" sheetId="23" state="visible" r:id="rId23"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 Oct 2026" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 Oct 2026" sheetId="25" state="visible" r:id="rId25"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$57</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$O$62</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -663,7 +664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V61"/>
+  <dimension ref="A1:W63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -688,6 +689,7 @@
     <col width="44" customWidth="1" min="20" max="20"/>
     <col width="44" customWidth="1" min="21" max="21"/>
     <col width="44" customWidth="1" min="22" max="22"/>
+    <col width="44" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -813,6 +815,11 @@
       <c r="V4" s="3" t="inlineStr">
         <is>
           <t>18 Oct 2026</t>
+        </is>
+      </c>
+      <c r="W4" s="3" t="inlineStr">
+        <is>
+          <t>19 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -869,6 +876,11 @@
       <c r="V5" s="6" t="inlineStr">
         <is>
           <t>alongside · 20D (ETD 19/10→19/09)</t>
+        </is>
+      </c>
+      <c r="W5" s="5" t="inlineStr">
+        <is>
+          <t>sailed (19/09)</t>
         </is>
       </c>
     </row>
@@ -915,6 +927,7 @@
       <c r="T6" s="5" t="inlineStr"/>
       <c r="U6" s="5" t="inlineStr"/>
       <c r="V6" s="5" t="inlineStr"/>
+      <c r="W6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -951,6 +964,7 @@
       <c r="T7" s="5" t="inlineStr"/>
       <c r="U7" s="5" t="inlineStr"/>
       <c r="V7" s="5" t="inlineStr"/>
+      <c r="W7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -991,6 +1005,11 @@
       <c r="T8" s="5" t="inlineStr"/>
       <c r="U8" s="5" t="inlineStr"/>
       <c r="V8" s="5" t="inlineStr"/>
+      <c r="W8" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20C (returns for a new call, ETA 19/14)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1049,6 +1068,11 @@
       <c r="V9" s="6" t="inlineStr">
         <is>
           <t>alongside · 20AB (ETD 18/16→19/08)</t>
+        </is>
+      </c>
+      <c r="W9" s="5" t="inlineStr">
+        <is>
+          <t>sailed (19/08)</t>
         </is>
       </c>
     </row>
@@ -1103,6 +1127,7 @@
           <t>sailed (17/11)</t>
         </is>
       </c>
+      <c r="W10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1147,6 +1172,11 @@
       <c r="T11" s="5" t="inlineStr"/>
       <c r="U11" s="5" t="inlineStr"/>
       <c r="V11" s="5" t="inlineStr"/>
+      <c r="W11" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20AB (returns for a new call, shift 4A, ETA 20/24)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1199,6 +1229,11 @@
           <t>alongside · 20B (ETD 18/11→18/10, 7B)</t>
         </is>
       </c>
+      <c r="W12" s="5" t="inlineStr">
+        <is>
+          <t>sailed (18/10)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1259,6 +1294,11 @@
           <t>expected → 20C (listed again; ETA 19/23→20/17, P.B 20/09→20/17, ETD 21/08→21/13)</t>
         </is>
       </c>
+      <c r="W13" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20B (ETA/P.B 20/17→21/13, ETD 21/13→22/05)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1327,6 +1367,11 @@
           <t>no longer listed (the unnamed LOA 558 m row is gone)</t>
         </is>
       </c>
+      <c r="W14" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20C (listed again with times: ETA 21/11, P.B 21/12, ETD 23/12)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1387,6 +1432,7 @@
       <c r="T15" s="5" t="inlineStr"/>
       <c r="U15" s="5" t="inlineStr"/>
       <c r="V15" s="5" t="inlineStr"/>
+      <c r="W15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1451,6 +1497,7 @@
       </c>
       <c r="U16" s="5" t="inlineStr"/>
       <c r="V16" s="5" t="inlineStr"/>
+      <c r="W16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1523,6 +1570,11 @@
       <c r="T17" s="5" t="inlineStr"/>
       <c r="U17" s="5" t="inlineStr"/>
       <c r="V17" s="5" t="inlineStr"/>
+      <c r="W17" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20E (returns for another call, 1C, ETA 21/17)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1571,6 +1623,7 @@
       <c r="T18" s="5" t="inlineStr"/>
       <c r="U18" s="5" t="inlineStr"/>
       <c r="V18" s="5" t="inlineStr"/>
+      <c r="W18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1627,6 +1680,7 @@
       <c r="T19" s="5" t="inlineStr"/>
       <c r="U19" s="5" t="inlineStr"/>
       <c r="V19" s="5" t="inlineStr"/>
+      <c r="W19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1683,6 +1737,7 @@
       <c r="T20" s="5" t="inlineStr"/>
       <c r="U20" s="5" t="inlineStr"/>
       <c r="V20" s="5" t="inlineStr"/>
+      <c r="W20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1735,6 +1790,7 @@
       <c r="T21" s="5" t="inlineStr"/>
       <c r="U21" s="5" t="inlineStr"/>
       <c r="V21" s="5" t="inlineStr"/>
+      <c r="W21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1783,6 +1839,7 @@
       <c r="T22" s="5" t="inlineStr"/>
       <c r="U22" s="5" t="inlineStr"/>
       <c r="V22" s="5" t="inlineStr"/>
+      <c r="W22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1843,6 +1900,7 @@
       <c r="T23" s="5" t="inlineStr"/>
       <c r="U23" s="5" t="inlineStr"/>
       <c r="V23" s="5" t="inlineStr"/>
+      <c r="W23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1899,6 +1957,7 @@
       <c r="T24" s="5" t="inlineStr"/>
       <c r="U24" s="5" t="inlineStr"/>
       <c r="V24" s="5" t="inlineStr"/>
+      <c r="W24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1939,6 +1998,7 @@
       <c r="T25" s="5" t="inlineStr"/>
       <c r="U25" s="5" t="inlineStr"/>
       <c r="V25" s="5" t="inlineStr"/>
+      <c r="W25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1983,6 +2043,7 @@
       <c r="T26" s="5" t="inlineStr"/>
       <c r="U26" s="5" t="inlineStr"/>
       <c r="V26" s="5" t="inlineStr"/>
+      <c r="W26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -2039,6 +2100,7 @@
       <c r="T27" s="5" t="inlineStr"/>
       <c r="U27" s="5" t="inlineStr"/>
       <c r="V27" s="5" t="inlineStr"/>
+      <c r="W27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2091,6 +2153,7 @@
       <c r="T28" s="5" t="inlineStr"/>
       <c r="U28" s="5" t="inlineStr"/>
       <c r="V28" s="5" t="inlineStr"/>
+      <c r="W28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2143,6 +2206,11 @@
       <c r="T29" s="5" t="inlineStr"/>
       <c r="U29" s="5" t="inlineStr"/>
       <c r="V29" s="5" t="inlineStr"/>
+      <c r="W29" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20F (returns for a new call, ETA 21/17)</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -2203,6 +2271,7 @@
       <c r="T30" s="5" t="inlineStr"/>
       <c r="U30" s="5" t="inlineStr"/>
       <c r="V30" s="5" t="inlineStr"/>
+      <c r="W30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2255,6 +2324,11 @@
           <t>expected → 20B (returns for a new call, ETA 20/15)</t>
         </is>
       </c>
+      <c r="W31" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20E</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2307,6 +2381,7 @@
       <c r="T32" s="5" t="inlineStr"/>
       <c r="U32" s="5" t="inlineStr"/>
       <c r="V32" s="5" t="inlineStr"/>
+      <c r="W32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2355,6 +2430,7 @@
       <c r="T33" s="5" t="inlineStr"/>
       <c r="U33" s="5" t="inlineStr"/>
       <c r="V33" s="5" t="inlineStr"/>
+      <c r="W33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2407,6 +2483,7 @@
       <c r="T34" s="5" t="inlineStr"/>
       <c r="U34" s="5" t="inlineStr"/>
       <c r="V34" s="5" t="inlineStr"/>
+      <c r="W34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2459,6 +2536,7 @@
       <c r="T35" s="5" t="inlineStr"/>
       <c r="U35" s="5" t="inlineStr"/>
       <c r="V35" s="5" t="inlineStr"/>
+      <c r="W35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2507,6 +2585,7 @@
       <c r="T36" s="5" t="inlineStr"/>
       <c r="U36" s="5" t="inlineStr"/>
       <c r="V36" s="5" t="inlineStr"/>
+      <c r="W36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2559,6 +2638,7 @@
       <c r="T37" s="5" t="inlineStr"/>
       <c r="U37" s="5" t="inlineStr"/>
       <c r="V37" s="5" t="inlineStr"/>
+      <c r="W37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2611,6 +2691,7 @@
       <c r="T38" s="5" t="inlineStr"/>
       <c r="U38" s="5" t="inlineStr"/>
       <c r="V38" s="5" t="inlineStr"/>
+      <c r="W38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2659,6 +2740,7 @@
       <c r="T39" s="5" t="inlineStr"/>
       <c r="U39" s="5" t="inlineStr"/>
       <c r="V39" s="5" t="inlineStr"/>
+      <c r="W39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -2707,6 +2789,7 @@
       <c r="T40" s="5" t="inlineStr"/>
       <c r="U40" s="5" t="inlineStr"/>
       <c r="V40" s="5" t="inlineStr"/>
+      <c r="W40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2759,6 +2842,7 @@
       <c r="T41" s="5" t="inlineStr"/>
       <c r="U41" s="5" t="inlineStr"/>
       <c r="V41" s="5" t="inlineStr"/>
+      <c r="W41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -2807,6 +2891,7 @@
       <c r="T42" s="5" t="inlineStr"/>
       <c r="U42" s="5" t="inlineStr"/>
       <c r="V42" s="5" t="inlineStr"/>
+      <c r="W42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2859,6 +2944,7 @@
       <c r="T43" s="5" t="inlineStr"/>
       <c r="U43" s="5" t="inlineStr"/>
       <c r="V43" s="5" t="inlineStr"/>
+      <c r="W43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -2911,6 +2997,7 @@
       <c r="T44" s="5" t="inlineStr"/>
       <c r="U44" s="5" t="inlineStr"/>
       <c r="V44" s="5" t="inlineStr"/>
+      <c r="W44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -2959,6 +3046,7 @@
       <c r="T45" s="5" t="inlineStr"/>
       <c r="U45" s="5" t="inlineStr"/>
       <c r="V45" s="5" t="inlineStr"/>
+      <c r="W45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -3015,6 +3103,7 @@
       <c r="T46" s="5" t="inlineStr"/>
       <c r="U46" s="5" t="inlineStr"/>
       <c r="V46" s="5" t="inlineStr"/>
+      <c r="W46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -3067,6 +3156,7 @@
       <c r="T47" s="5" t="inlineStr"/>
       <c r="U47" s="5" t="inlineStr"/>
       <c r="V47" s="5" t="inlineStr"/>
+      <c r="W47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -3119,6 +3209,7 @@
       <c r="T48" s="5" t="inlineStr"/>
       <c r="U48" s="5" t="inlineStr"/>
       <c r="V48" s="5" t="inlineStr"/>
+      <c r="W48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -3171,6 +3262,7 @@
       <c r="T49" s="5" t="inlineStr"/>
       <c r="U49" s="5" t="inlineStr"/>
       <c r="V49" s="5" t="inlineStr"/>
+      <c r="W49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -3219,6 +3311,7 @@
       <c r="T50" s="5" t="inlineStr"/>
       <c r="U50" s="5" t="inlineStr"/>
       <c r="V50" s="5" t="inlineStr"/>
+      <c r="W50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -3263,6 +3356,7 @@
       <c r="T51" s="5" t="inlineStr"/>
       <c r="U51" s="5" t="inlineStr"/>
       <c r="V51" s="5" t="inlineStr"/>
+      <c r="W51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -3311,6 +3405,7 @@
       </c>
       <c r="U52" s="5" t="inlineStr"/>
       <c r="V52" s="5" t="inlineStr"/>
+      <c r="W52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -3359,6 +3454,7 @@
         </is>
       </c>
       <c r="V53" s="5" t="inlineStr"/>
+      <c r="W53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -3407,6 +3503,7 @@
         </is>
       </c>
       <c r="V54" s="5" t="inlineStr"/>
+      <c r="W54" s="5" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -3447,6 +3544,7 @@
       </c>
       <c r="U55" s="5" t="inlineStr"/>
       <c r="V55" s="5" t="inlineStr"/>
+      <c r="W55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -3491,6 +3589,7 @@
         </is>
       </c>
       <c r="V56" s="5" t="inlineStr"/>
+      <c r="W56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -3537,6 +3636,11 @@
       <c r="V57" s="5" t="inlineStr">
         <is>
           <t>alongside · 20C (ETD 18/16)</t>
+        </is>
+      </c>
+      <c r="W57" s="5" t="inlineStr">
+        <is>
+          <t>sailed (18/16)</t>
         </is>
       </c>
     </row>
@@ -3583,6 +3687,11 @@
           <t>alongside · 20F (ETD 19/07)</t>
         </is>
       </c>
+      <c r="W58" s="6" t="inlineStr">
+        <is>
+          <t>alongside · 20F (ETD 19/07→19/12)</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -3627,6 +3736,7 @@
           <t>sailed (18/07)</t>
         </is>
       </c>
+      <c r="W59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -3669,6 +3779,11 @@
       <c r="V60" s="6" t="inlineStr">
         <is>
           <t>expected · 20F (marked, ETA 19/08→19/12, P.B 19/09→19/12, ETD 20/17)</t>
+        </is>
+      </c>
+      <c r="W60" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20B (ETA/P.B 19/12→19/10)</t>
         </is>
       </c>
     </row>
@@ -3709,6 +3824,73 @@
       <c r="V61" s="5" t="inlineStr">
         <is>
           <t>sailed (17/15)</t>
+        </is>
+      </c>
+      <c r="W61" s="5" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>SKY ORION</t>
+        </is>
+      </c>
+      <c r="B62" s="5" t="inlineStr"/>
+      <c r="C62" s="5" t="inlineStr"/>
+      <c r="D62" s="5" t="inlineStr"/>
+      <c r="E62" s="5" t="inlineStr"/>
+      <c r="F62" s="5" t="inlineStr"/>
+      <c r="G62" s="5" t="inlineStr"/>
+      <c r="H62" s="5" t="inlineStr"/>
+      <c r="I62" s="5" t="inlineStr"/>
+      <c r="J62" s="5" t="inlineStr"/>
+      <c r="K62" s="5" t="inlineStr"/>
+      <c r="L62" s="5" t="inlineStr"/>
+      <c r="M62" s="5" t="inlineStr"/>
+      <c r="N62" s="5" t="inlineStr"/>
+      <c r="O62" s="5" t="inlineStr"/>
+      <c r="P62" s="5" t="inlineStr"/>
+      <c r="Q62" s="5" t="inlineStr"/>
+      <c r="R62" s="5" t="inlineStr"/>
+      <c r="S62" s="5" t="inlineStr"/>
+      <c r="T62" s="5" t="inlineStr"/>
+      <c r="U62" s="5" t="inlineStr"/>
+      <c r="V62" s="5" t="inlineStr"/>
+      <c r="W62" s="5" t="inlineStr">
+        <is>
+          <t>listed at 20AB without times (new, schedule TBA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>SAWASDEE MIMOSA</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr"/>
+      <c r="C63" s="5" t="inlineStr"/>
+      <c r="D63" s="5" t="inlineStr"/>
+      <c r="E63" s="5" t="inlineStr"/>
+      <c r="F63" s="5" t="inlineStr"/>
+      <c r="G63" s="5" t="inlineStr"/>
+      <c r="H63" s="5" t="inlineStr"/>
+      <c r="I63" s="5" t="inlineStr"/>
+      <c r="J63" s="5" t="inlineStr"/>
+      <c r="K63" s="5" t="inlineStr"/>
+      <c r="L63" s="5" t="inlineStr"/>
+      <c r="M63" s="5" t="inlineStr"/>
+      <c r="N63" s="5" t="inlineStr"/>
+      <c r="O63" s="5" t="inlineStr"/>
+      <c r="P63" s="5" t="inlineStr"/>
+      <c r="Q63" s="5" t="inlineStr"/>
+      <c r="R63" s="5" t="inlineStr"/>
+      <c r="S63" s="5" t="inlineStr"/>
+      <c r="T63" s="5" t="inlineStr"/>
+      <c r="U63" s="5" t="inlineStr"/>
+      <c r="V63" s="5" t="inlineStr"/>
+      <c r="W63" s="5" t="inlineStr">
+        <is>
+          <t>listed at 20B without times (new, schedule TBA)</t>
         </is>
       </c>
     </row>
@@ -11161,7 +11343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12866,8 +13048,43 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="12" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B57" s="13" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="C57" s="13" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="D57" s="19" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E57" s="19" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F57" s="13" t="inlineStr">
+        <is>
+          <t>(no notice – the CLOSE from Oct 19 line is no longer printed; 20D has no vessels on this sheet)</t>
+        </is>
+      </c>
+      <c r="G57" s="13" t="inlineStr">
+        <is>
+          <t>Dropped from sheet: 20D closure no longer printed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:G56"/>
+  <autoFilter ref="A4:G57"/>
   <mergeCells count="1">
     <mergeCell ref="A2:G2"/>
   </mergeCells>
@@ -15992,6 +16209,508 @@
   <mergeCells count="3">
     <mergeCell ref="F17:J17"/>
     <mergeCell ref="F15:J15"/>
+    <mergeCell ref="F16:J16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 19 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Waiting for Berth (h)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>HOPE C</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>481</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>46316</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>46316.375</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>46316.91666666666</v>
+      </c>
+      <c r="G4" s="24">
+        <f>(E4-D4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="24">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>4A</t>
+        </is>
+      </c>
+      <c r="J4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>KMTC JAKARTA</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46314.41666666666</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46314.41666666666</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46315.70833333334</v>
+      </c>
+      <c r="G5" s="24">
+        <f>(E5-D5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="24">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>MITRA BHUM</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>485</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46316.54166666666</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46316.54166666666</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46317.20833333334</v>
+      </c>
+      <c r="G6" s="24">
+        <f>(E6-D6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="24">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>MILLENNIUM BRIGHT</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46314.58333333334</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46314.58333333334</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46315.5</v>
+      </c>
+      <c r="G7" s="24">
+        <f>(E7-D7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="24">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>CAPE FAWLEY</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>558</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>46316.45833333334</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>46316.5</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>46318.5</v>
+      </c>
+      <c r="G8" s="24">
+        <f>(E8-D8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="24">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>MTT BANGKOK</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>46315.625</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>46315.625</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>46316.54166666666</v>
+      </c>
+      <c r="G9" s="24">
+        <f>(E9-D9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="24">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>ALS SUMIRE</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>537</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>46316.70833333334</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>46316.70833333334</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>46317.70833333334</v>
+      </c>
+      <c r="G10" s="24">
+        <f>(E10-D10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="24">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>1C</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 108</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>46312.41666666666</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>46313.33333333334</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>46314.5</v>
+      </c>
+      <c r="G11" s="24">
+        <f>(E11-D11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="24">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J11" s="23" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>GREEN PARK</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>482</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>46316.70833333334</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>46317.58333333334</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>46318.54166666666</v>
+      </c>
+      <c r="G12" s="24">
+        <f>(E12-D12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="24">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J12" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="34" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G16" s="35" t="n"/>
+      <c r="H16" s="35" t="n"/>
+      <c r="I16" s="35" t="n"/>
+      <c r="J16" s="36" t="n"/>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>Berth closed</t>
+        </is>
+      </c>
+      <c r="C17" s="38" t="n"/>
+      <c r="D17" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>(no notice – the CLOSE from Oct 19 line is no longer printed; 20D has no vessels on this sheet)  —  Dropped from sheet: 20D closure no longer printed</t>
+        </is>
+      </c>
+      <c r="G17" s="38" t="n"/>
+      <c r="H17" s="38" t="n"/>
+      <c r="I17" s="38" t="n"/>
+      <c r="J17" s="38" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="F17:J17"/>
     <mergeCell ref="F16:J16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16045,7 +16764,7 @@
         </is>
       </c>
       <c r="B3" s="22" t="n">
-        <v>46313.375</v>
+        <v>46314.375</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -16366,34 +17085,34 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>GREEN PARK</t>
+          <t>KANWAY FORTUNE</t>
         </is>
       </c>
       <c r="C10" s="23" t="n">
-        <v>482</v>
+        <v>564</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>46300</v>
+        <v>46301</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="F10" s="23" t="n">
         <v>5</v>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20B → 20AB</t>
+          <t>20D → 20F → 20AB</t>
         </is>
       </c>
       <c r="H10" s="11" t="n">
-        <v>46302.41666666666</v>
+        <v>46303.66666666666</v>
       </c>
       <c r="I10" s="11" t="n">
-        <v>46303.58333333334</v>
+        <v>46304.58333333334</v>
       </c>
       <c r="J10" s="11" t="n">
-        <v>46304.66666666666</v>
+        <v>46305.625</v>
       </c>
       <c r="K10" s="24">
         <f>(I10-H10)*24</f>
@@ -16423,34 +17142,34 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>KANWAY FORTUNE</t>
+          <t>CNC MARS</t>
         </is>
       </c>
       <c r="C11" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="F11" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>20D → 20F → 20AB</t>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
         </is>
       </c>
       <c r="H11" s="11" t="n">
-        <v>46303.66666666666</v>
+        <v>46304.91666666666</v>
       </c>
       <c r="I11" s="11" t="n">
-        <v>46304.58333333334</v>
+        <v>46305.625</v>
       </c>
       <c r="J11" s="11" t="n">
-        <v>46305.625</v>
+        <v>46306.625</v>
       </c>
       <c r="K11" s="24">
         <f>(I11-H11)*24</f>
@@ -16480,34 +17199,34 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>CNC MARS</t>
+          <t>SAMAL</t>
         </is>
       </c>
       <c r="C12" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>46302</v>
+        <v>46304</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="F12" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>20AB</t>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20F → 20AB</t>
         </is>
       </c>
       <c r="H12" s="11" t="n">
-        <v>46304.91666666666</v>
+        <v>46307.375</v>
       </c>
       <c r="I12" s="11" t="n">
-        <v>46305.625</v>
+        <v>46307.66666666666</v>
       </c>
       <c r="J12" s="11" t="n">
-        <v>46306.625</v>
+        <v>46309.20833333334</v>
       </c>
       <c r="K12" s="24">
         <f>(I12-H12)*24</f>
@@ -16537,34 +17256,34 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>SAMAL</t>
+          <t>KMTC TAIPEIS</t>
         </is>
       </c>
       <c r="C13" s="23" t="n">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D13" s="10" t="n">
         <v>46304</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="F13" s="23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20F → 20AB</t>
+          <t>20D → 20C → 20AB</t>
         </is>
       </c>
       <c r="H13" s="11" t="n">
-        <v>46307.375</v>
+        <v>46308.08333333334</v>
       </c>
       <c r="I13" s="11" t="n">
-        <v>46307.66666666666</v>
+        <v>46309.20833333334</v>
       </c>
       <c r="J13" s="11" t="n">
-        <v>46309.20833333334</v>
+        <v>46310.33333333334</v>
       </c>
       <c r="K13" s="24">
         <f>(I13-H13)*24</f>
@@ -16594,34 +17313,34 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>KMTC TAIPEIS</t>
+          <t>WAN HAI 176</t>
         </is>
       </c>
       <c r="C14" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D14" s="10" t="n">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="F14" s="23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>20D → 20C → 20AB</t>
+          <t>20B → 20AB</t>
         </is>
       </c>
       <c r="H14" s="11" t="n">
-        <v>46308.08333333334</v>
+        <v>46310.33333333334</v>
       </c>
       <c r="I14" s="11" t="n">
-        <v>46309.20833333334</v>
+        <v>46310.375</v>
       </c>
       <c r="J14" s="11" t="n">
-        <v>46310.33333333334</v>
+        <v>46311.66666666666</v>
       </c>
       <c r="K14" s="24">
         <f>(I14-H14)*24</f>
@@ -16651,34 +17370,34 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 176</t>
+          <t>BANGKOK</t>
         </is>
       </c>
       <c r="C15" s="23" t="n">
-        <v>564</v>
+        <v>551</v>
       </c>
       <c r="D15" s="10" t="n">
-        <v>46308</v>
+        <v>46293</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>46311</v>
+        <v>46313</v>
       </c>
       <c r="F15" s="23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>20B → 20AB</t>
+          <t>20D → 20AB</t>
         </is>
       </c>
       <c r="H15" s="11" t="n">
-        <v>46310.33333333334</v>
+        <v>46311.625</v>
       </c>
       <c r="I15" s="11" t="n">
-        <v>46310.375</v>
+        <v>46312.375</v>
       </c>
       <c r="J15" s="11" t="n">
-        <v>46311.66666666666</v>
+        <v>46314.33333333334</v>
       </c>
       <c r="K15" s="24">
         <f>(I15-H15)*24</f>
@@ -16708,34 +17427,34 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>BANGKOK</t>
+          <t>HOPE C</t>
         </is>
       </c>
       <c r="C16" s="23" t="n">
-        <v>551</v>
+        <v>481</v>
       </c>
       <c r="D16" s="10" t="n">
         <v>46293</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="F16" s="23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
-          <t>20D → 20AB</t>
+          <t>20E → 20F → 20AB</t>
         </is>
       </c>
       <c r="H16" s="11" t="n">
-        <v>46311.625</v>
+        <v>46316</v>
       </c>
       <c r="I16" s="11" t="n">
-        <v>46312.375</v>
+        <v>46316.375</v>
       </c>
       <c r="J16" s="11" t="n">
-        <v>46314.33333333334</v>
+        <v>46316.91666666666</v>
       </c>
       <c r="K16" s="24">
         <f>(I16-H16)*24</f>
@@ -16747,7 +17466,7 @@
       </c>
       <c r="M16" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="N16" s="23" t="inlineStr"/>
@@ -16821,34 +17540,34 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>MILLENNIUM BRIGHT</t>
+          <t>YM IMPROVEMENT</t>
         </is>
       </c>
       <c r="C18" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D18" s="10" t="n">
-        <v>46293</v>
+        <v>46296</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>46294</v>
+        <v>46300</v>
       </c>
       <c r="F18" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G18" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>5</v>
+      </c>
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>20C → 20B</t>
         </is>
       </c>
       <c r="H18" s="11" t="n">
-        <v>46293.45833333334</v>
+        <v>46298.95833333334</v>
       </c>
       <c r="I18" s="11" t="n">
-        <v>46294.20833333334</v>
+        <v>46299.41666666666</v>
       </c>
       <c r="J18" s="11" t="n">
-        <v>46295.16666666666</v>
+        <v>46300.5</v>
       </c>
       <c r="K18" s="24">
         <f>(I18-H18)*24</f>
@@ -16878,34 +17597,34 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>YM IMPROVEMENT</t>
+          <t>SAWASDEE SPICA</t>
         </is>
       </c>
       <c r="C19" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>46296</v>
+        <v>46299</v>
       </c>
       <c r="E19" s="10" t="n">
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="F19" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>20C → 20B</t>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H19" s="11" t="n">
-        <v>46298.95833333334</v>
+        <v>46300.875</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>46299.41666666666</v>
+        <v>46301.54166666666</v>
       </c>
       <c r="J19" s="11" t="n">
-        <v>46300.5</v>
+        <v>46303.54166666666</v>
       </c>
       <c r="K19" s="24">
         <f>(I19-H19)*24</f>
@@ -16935,34 +17654,34 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE SPICA</t>
+          <t>SITC HOCHIMINH</t>
         </is>
       </c>
       <c r="C20" s="23" t="n">
-        <v>564</v>
+        <v>470</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>46299</v>
+        <v>46301</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="F20" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>4</v>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20B</t>
         </is>
       </c>
       <c r="H20" s="11" t="n">
-        <v>46300.875</v>
+        <v>46302.625</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>46301.54166666666</v>
+        <v>46303.58333333334</v>
       </c>
       <c r="J20" s="11" t="n">
-        <v>46303.54166666666</v>
+        <v>46304.70833333334</v>
       </c>
       <c r="K20" s="24">
         <f>(I20-H20)*24</f>
@@ -16992,34 +17711,34 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>SITC HOCHIMINH</t>
+          <t>INDURO</t>
         </is>
       </c>
       <c r="C21" s="23" t="n">
-        <v>470</v>
+        <v>565</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="E21" s="10" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="F21" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20B</t>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H21" s="11" t="n">
-        <v>46302.625</v>
+        <v>46304.25</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>46303.58333333334</v>
+        <v>46304.66666666666</v>
       </c>
       <c r="J21" s="11" t="n">
-        <v>46304.70833333334</v>
+        <v>46306.16666666666</v>
       </c>
       <c r="K21" s="24">
         <f>(I21-H21)*24</f>
@@ -17049,34 +17768,34 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>INDURO</t>
+          <t>XIN MING ZHOU 102</t>
         </is>
       </c>
       <c r="C22" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D22" s="10" t="n">
         <v>46302</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="F22" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G22" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>5</v>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>20F → 20B</t>
         </is>
       </c>
       <c r="H22" s="11" t="n">
-        <v>46304.25</v>
+        <v>46305.875</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>46304.66666666666</v>
+        <v>46306.20833333334</v>
       </c>
       <c r="J22" s="11" t="n">
-        <v>46306.16666666666</v>
+        <v>46307.08333333334</v>
       </c>
       <c r="K22" s="24">
         <f>(I22-H22)*24</f>
@@ -17106,34 +17825,34 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 102</t>
+          <t>CEBU</t>
         </is>
       </c>
       <c r="C23" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D23" s="10" t="n">
-        <v>46302</v>
+        <v>46306</v>
       </c>
       <c r="E23" s="10" t="n">
-        <v>46306</v>
+        <v>46309</v>
       </c>
       <c r="F23" s="23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>20F → 20B</t>
+          <t>20AB → 20B</t>
         </is>
       </c>
       <c r="H23" s="11" t="n">
-        <v>46305.875</v>
+        <v>46307.91666666666</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>46306.20833333334</v>
+        <v>46308.25</v>
       </c>
       <c r="J23" s="11" t="n">
-        <v>46307.08333333334</v>
+        <v>46309.54166666666</v>
       </c>
       <c r="K23" s="24">
         <f>(I23-H23)*24</f>
@@ -17163,34 +17882,34 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>CEBU</t>
+          <t>M ODYSSEY</t>
         </is>
       </c>
       <c r="C24" s="23" t="n">
-        <v>564</v>
+        <v>449</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>46306</v>
+        <v>46293</v>
       </c>
       <c r="E24" s="10" t="n">
         <v>46309</v>
       </c>
       <c r="F24" s="23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20B</t>
+          <t>20B → 20C → 20B</t>
         </is>
       </c>
       <c r="H24" s="11" t="n">
-        <v>46307.91666666666</v>
+        <v>46309.04166666666</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>46308.25</v>
+        <v>46309.625</v>
       </c>
       <c r="J24" s="11" t="n">
-        <v>46309.54166666666</v>
+        <v>46310.20833333334</v>
       </c>
       <c r="K24" s="24">
         <f>(I24-H24)*24</f>
@@ -17202,7 +17921,7 @@
       </c>
       <c r="M24" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="N24" s="23" t="inlineStr"/>
@@ -17220,34 +17939,34 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>M ODYSSEY</t>
+          <t>KHARIS HERITAGE</t>
         </is>
       </c>
       <c r="C25" s="23" t="n">
-        <v>449</v>
+        <v>482</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="E25" s="10" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="F25" s="23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>20B → 20C → 20B</t>
+          <t>20AB → 20B → 20C → 20B</t>
         </is>
       </c>
       <c r="H25" s="11" t="n">
-        <v>46309.04166666666</v>
+        <v>46310.04166666666</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>46309.625</v>
+        <v>46310.25</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>46310.20833333334</v>
+        <v>46311.29166666666</v>
       </c>
       <c r="K25" s="24">
         <f>(I25-H25)*24</f>
@@ -17259,7 +17978,7 @@
       </c>
       <c r="M25" s="23" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N25" s="23" t="inlineStr"/>
@@ -17277,34 +17996,34 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>KHARIS HERITAGE</t>
+          <t>TS CHIBA</t>
         </is>
       </c>
       <c r="C26" s="23" t="n">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="D26" s="10" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="E26" s="10" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="F26" s="23" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20B → 20C → 20B</t>
+          <t>20E → 20C → 20B</t>
         </is>
       </c>
       <c r="H26" s="11" t="n">
-        <v>46310.04166666666</v>
+        <v>46311.58333333334</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>46310.25</v>
+        <v>46311.58333333334</v>
       </c>
       <c r="J26" s="11" t="n">
-        <v>46311.29166666666</v>
+        <v>46312.45833333334</v>
       </c>
       <c r="K26" s="24">
         <f>(I26-H26)*24</f>
@@ -17334,34 +18053,34 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>TS CHIBA</t>
+          <t>JARU BHUM</t>
         </is>
       </c>
       <c r="C27" s="23" t="n">
-        <v>485</v>
+        <v>564</v>
       </c>
       <c r="D27" s="10" t="n">
         <v>46293</v>
       </c>
       <c r="E27" s="10" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="F27" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>20E → 20C → 20B</t>
+          <t>20F → 20D → 20B</t>
         </is>
       </c>
       <c r="H27" s="11" t="n">
-        <v>46311.58333333334</v>
+        <v>46312.66666666666</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>46311.58333333334</v>
+        <v>46312.66666666666</v>
       </c>
       <c r="J27" s="11" t="n">
-        <v>46312.45833333334</v>
+        <v>46313.41666666666</v>
       </c>
       <c r="K27" s="24">
         <f>(I27-H27)*24</f>
@@ -17373,7 +18092,7 @@
       </c>
       <c r="M27" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="N27" s="23" t="inlineStr"/>
@@ -17391,34 +18110,34 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>JARU BHUM</t>
+          <t>KMTC JAKARTA</t>
         </is>
       </c>
       <c r="C28" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D28" s="10" t="n">
-        <v>46293</v>
+        <v>46310</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="F28" s="23" t="n">
         <v>5</v>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>20F → 20D → 20B</t>
+          <t>20F → 20B</t>
         </is>
       </c>
       <c r="H28" s="11" t="n">
-        <v>46312.66666666666</v>
+        <v>46314.41666666666</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>46312.66666666666</v>
+        <v>46314.41666666666</v>
       </c>
       <c r="J28" s="11" t="n">
-        <v>46313.41666666666</v>
+        <v>46315.70833333334</v>
       </c>
       <c r="K28" s="24">
         <f>(I28-H28)*24</f>
@@ -17430,7 +18149,7 @@
       </c>
       <c r="M28" s="23" t="inlineStr">
         <is>
-          <t>7B</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N28" s="23" t="inlineStr"/>
@@ -17447,34 +18166,34 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>MTT BANGKOK</t>
+          <t>MITRA BHUM</t>
         </is>
       </c>
       <c r="C29" s="23" t="n">
-        <v>564</v>
+        <v>485</v>
       </c>
       <c r="D29" s="10" t="n">
-        <v>46300</v>
+        <v>46293</v>
       </c>
       <c r="E29" s="10" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="F29" s="23" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>20D → 20B</t>
+          <t>20F → 20E → 20D → 20AB → 20C → 20B</t>
         </is>
       </c>
       <c r="H29" s="11" t="n">
-        <v>46315.625</v>
+        <v>46316.54166666666</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>46315.625</v>
+        <v>46316.54166666666</v>
       </c>
       <c r="J29" s="11" t="n">
-        <v>46316.54166666666</v>
+        <v>46317.20833333334</v>
       </c>
       <c r="K29" s="24">
         <f>(I29-H29)*24</f>
@@ -18006,9 +18725,10 @@
         </is>
       </c>
       <c r="N38" s="23" t="inlineStr"/>
-      <c r="O38" s="23">
-        <f>IF(J38&lt;=$B$3,"Sailed",IF(I38&lt;=$B$3,"Alongside",IF(H38&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O38" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="39">
@@ -18019,34 +18739,34 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>CAPE FAWLEY</t>
+          <t>MILLENNIUM BRIGHT</t>
         </is>
       </c>
       <c r="C39" s="23" t="n">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="D39" s="10" t="n">
         <v>46293</v>
       </c>
       <c r="E39" s="10" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="F39" s="23" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20C → 20AB → 20C</t>
+          <t>20B → 20C</t>
         </is>
       </c>
       <c r="H39" s="11" t="n">
-        <v>46314.75</v>
+        <v>46314.58333333334</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>46314.75</v>
+        <v>46314.58333333334</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>46316.45833333334</v>
+        <v>46315.5</v>
       </c>
       <c r="K39" s="24">
         <f>(I39-H39)*24</f>
@@ -18062,10 +18782,9 @@
         </is>
       </c>
       <c r="N39" s="23" t="inlineStr"/>
-      <c r="O39" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="O39" s="23">
+        <f>IF(J39&lt;=$B$3,"Sailed",IF(I39&lt;=$B$3,"Alongside",IF(H39&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -18076,34 +18795,34 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>MITRA BHUM</t>
+          <t>CAPE FAWLEY</t>
         </is>
       </c>
       <c r="C40" s="23" t="n">
-        <v>485</v>
+        <v>558</v>
       </c>
       <c r="D40" s="10" t="n">
         <v>46293</v>
       </c>
       <c r="E40" s="10" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="F40" s="23" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>20F → 20E → 20D → 20AB → 20C</t>
+          <t>20AB → 20C → 20AB → 20C</t>
         </is>
       </c>
       <c r="H40" s="11" t="n">
-        <v>46315.70833333334</v>
+        <v>46316.45833333334</v>
       </c>
       <c r="I40" s="11" t="n">
-        <v>46315.70833333334</v>
+        <v>46316.5</v>
       </c>
       <c r="J40" s="11" t="n">
-        <v>46316.54166666666</v>
+        <v>46318.5</v>
       </c>
       <c r="K40" s="24">
         <f>(I40-H40)*24</f>
@@ -18688,9 +19407,10 @@
         </is>
       </c>
       <c r="N50" s="23" t="inlineStr"/>
-      <c r="O50" s="23">
-        <f>IF(J50&lt;=$B$3,"Sailed",IF(I50&lt;=$B$3,"Alongside",IF(H50&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O50" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="51">
@@ -18751,98 +19471,97 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="25" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="B52" s="25" t="inlineStr">
-        <is>
-          <t>HOPE C</t>
-        </is>
-      </c>
-      <c r="C52" s="26" t="n">
-        <v>481</v>
-      </c>
-      <c r="D52" s="27" t="n">
-        <v>46293</v>
-      </c>
-      <c r="E52" s="27" t="n">
-        <v>46295</v>
-      </c>
-      <c r="F52" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="G52" s="33" t="inlineStr">
-        <is>
-          <t>20E → 20F</t>
-        </is>
-      </c>
-      <c r="H52" s="29" t="n">
-        <v>46294.70833333334</v>
-      </c>
-      <c r="I52" s="29" t="n">
-        <v>46294.70833333334</v>
-      </c>
-      <c r="J52" s="29" t="n">
-        <v>46295.66666666666</v>
-      </c>
-      <c r="K52" s="30">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>MTT BANGKOK</t>
+        </is>
+      </c>
+      <c r="C52" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D52" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E52" s="10" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F52" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="G52" s="6" t="inlineStr">
+        <is>
+          <t>20D → 20B → 20E</t>
+        </is>
+      </c>
+      <c r="H52" s="11" t="n">
+        <v>46315.625</v>
+      </c>
+      <c r="I52" s="11" t="n">
+        <v>46315.625</v>
+      </c>
+      <c r="J52" s="11" t="n">
+        <v>46316.54166666666</v>
+      </c>
+      <c r="K52" s="24">
         <f>(I52-H52)*24</f>
         <v/>
       </c>
-      <c r="L52" s="30">
+      <c r="L52" s="24">
         <f>(J52-I52)*24</f>
         <v/>
       </c>
-      <c r="M52" s="26" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N52" s="26" t="inlineStr"/>
-      <c r="O52" s="26" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="M52" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N52" s="23" t="inlineStr"/>
+      <c r="O52" s="23">
+        <f>IF(J52&lt;=$B$3,"Sailed",IF(I52&lt;=$B$3,"Alongside",IF(H52&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>20F</t>
+          <t>20E</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>KMTC BANGKOK</t>
+          <t>ALS SUMIRE</t>
         </is>
       </c>
       <c r="C53" s="23" t="n">
-        <v>564</v>
+        <v>537</v>
       </c>
       <c r="D53" s="10" t="n">
-        <v>46295</v>
+        <v>46294</v>
       </c>
       <c r="E53" s="10" t="n">
-        <v>46298</v>
+        <v>46314</v>
       </c>
       <c r="F53" s="23" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20F</t>
+          <t>20F → 20D → 20C → 20B → 20F → 20E</t>
         </is>
       </c>
       <c r="H53" s="11" t="n">
-        <v>46297.29166666666</v>
+        <v>46316.70833333334</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>46297.45833333334</v>
+        <v>46316.70833333334</v>
       </c>
       <c r="J53" s="11" t="n">
-        <v>46298.70833333334</v>
+        <v>46317.70833333334</v>
       </c>
       <c r="K53" s="24">
         <f>(I53-H53)*24</f>
@@ -18854,68 +19573,67 @@
       </c>
       <c r="M53" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>1C</t>
         </is>
       </c>
       <c r="N53" s="23" t="inlineStr"/>
-      <c r="O53" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="O53" s="23">
+        <f>IF(J53&lt;=$B$3,"Sailed",IF(I53&lt;=$B$3,"Alongside",IF(H53&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
+      <c r="A54" s="25" t="inlineStr">
         <is>
           <t>20F</t>
         </is>
       </c>
-      <c r="B54" s="4" t="inlineStr">
-        <is>
-          <t>XIN MING ZHOU 98</t>
-        </is>
-      </c>
-      <c r="C54" s="23" t="n">
+      <c r="B54" s="25" t="inlineStr">
+        <is>
+          <t>KMTC BANGKOK</t>
+        </is>
+      </c>
+      <c r="C54" s="26" t="n">
         <v>564</v>
       </c>
-      <c r="D54" s="10" t="n">
-        <v>46297</v>
-      </c>
-      <c r="E54" s="10" t="n">
-        <v>46299</v>
-      </c>
-      <c r="F54" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G54" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="H54" s="11" t="n">
-        <v>46299.375</v>
-      </c>
-      <c r="I54" s="11" t="n">
-        <v>46299.375</v>
-      </c>
-      <c r="J54" s="11" t="n">
-        <v>46300.375</v>
-      </c>
-      <c r="K54" s="24">
+      <c r="D54" s="27" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E54" s="27" t="n">
+        <v>46298</v>
+      </c>
+      <c r="F54" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="G54" s="33" t="inlineStr">
+        <is>
+          <t>20AB → 20F</t>
+        </is>
+      </c>
+      <c r="H54" s="29" t="n">
+        <v>46297.29166666666</v>
+      </c>
+      <c r="I54" s="29" t="n">
+        <v>46297.45833333334</v>
+      </c>
+      <c r="J54" s="29" t="n">
+        <v>46298.70833333334</v>
+      </c>
+      <c r="K54" s="30">
         <f>(I54-H54)*24</f>
         <v/>
       </c>
-      <c r="L54" s="24">
+      <c r="L54" s="30">
         <f>(J54-I54)*24</f>
         <v/>
       </c>
-      <c r="M54" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N54" s="23" t="inlineStr"/>
-      <c r="O54" s="23" t="inlineStr">
+      <c r="M54" s="26" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N54" s="26" t="inlineStr"/>
+      <c r="O54" s="26" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -18929,20 +19647,20 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>XIN AN</t>
+          <t>XIN MING ZHOU 98</t>
         </is>
       </c>
       <c r="C55" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D55" s="10" t="n">
-        <v>46300</v>
+        <v>46297</v>
       </c>
       <c r="E55" s="10" t="n">
-        <v>46304</v>
+        <v>46299</v>
       </c>
       <c r="F55" s="23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
@@ -18950,13 +19668,13 @@
         </is>
       </c>
       <c r="H55" s="11" t="n">
-        <v>46302.54166666666</v>
+        <v>46299.375</v>
       </c>
       <c r="I55" s="11" t="n">
-        <v>46302.58333333334</v>
+        <v>46299.375</v>
       </c>
       <c r="J55" s="11" t="n">
-        <v>46304.54166666666</v>
+        <v>46300.375</v>
       </c>
       <c r="K55" s="24">
         <f>(I55-H55)*24</f>
@@ -18986,7 +19704,7 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE ATLANTIC</t>
+          <t>XIN AN</t>
         </is>
       </c>
       <c r="C56" s="23" t="n">
@@ -18996,24 +19714,24 @@
         <v>46300</v>
       </c>
       <c r="E56" s="10" t="n">
-        <v>46306</v>
+        <v>46304</v>
       </c>
       <c r="F56" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="G56" s="6" t="inlineStr">
-        <is>
-          <t>20C → 20D → 20F</t>
+        <v>5</v>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
         </is>
       </c>
       <c r="H56" s="11" t="n">
-        <v>46302.83333333334</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="I56" s="11" t="n">
-        <v>46304.625</v>
+        <v>46302.58333333334</v>
       </c>
       <c r="J56" s="11" t="n">
-        <v>46306.5</v>
+        <v>46304.54166666666</v>
       </c>
       <c r="K56" s="24">
         <f>(I56-H56)*24</f>
@@ -19043,34 +19761,34 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>JOSCO SHINE</t>
+          <t>SAWASDEE ATLANTIC</t>
         </is>
       </c>
       <c r="C57" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D57" s="10" t="n">
-        <v>46304</v>
+        <v>46300</v>
       </c>
       <c r="E57" s="10" t="n">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="F57" s="23" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>20B → 20AB → 20F</t>
+          <t>20C → 20D → 20F</t>
         </is>
       </c>
       <c r="H57" s="11" t="n">
-        <v>46307.45833333334</v>
+        <v>46302.83333333334</v>
       </c>
       <c r="I57" s="11" t="n">
-        <v>46307.625</v>
+        <v>46304.625</v>
       </c>
       <c r="J57" s="11" t="n">
-        <v>46308.25</v>
+        <v>46306.5</v>
       </c>
       <c r="K57" s="24">
         <f>(I57-H57)*24</f>
@@ -19100,34 +19818,34 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>ALS SUMIRE</t>
+          <t>JOSCO SHINE</t>
         </is>
       </c>
       <c r="C58" s="23" t="n">
-        <v>537</v>
+        <v>564</v>
       </c>
       <c r="D58" s="10" t="n">
-        <v>46294</v>
+        <v>46304</v>
       </c>
       <c r="E58" s="10" t="n">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="F58" s="23" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>20F → 20D → 20C → 20B → 20F</t>
+          <t>20B → 20AB → 20F</t>
         </is>
       </c>
       <c r="H58" s="11" t="n">
-        <v>46307.91666666666</v>
+        <v>46307.45833333334</v>
       </c>
       <c r="I58" s="11" t="n">
+        <v>46307.625</v>
+      </c>
+      <c r="J58" s="11" t="n">
         <v>46308.25</v>
-      </c>
-      <c r="J58" s="11" t="n">
-        <v>46309.25</v>
       </c>
       <c r="K58" s="24">
         <f>(I58-H58)*24</f>
@@ -19139,7 +19857,7 @@
       </c>
       <c r="M58" s="23" t="inlineStr">
         <is>
-          <t>1C</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N58" s="23" t="inlineStr"/>
@@ -19281,10 +19999,10 @@
         <v>46310</v>
       </c>
       <c r="E61" s="10" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="F61" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
@@ -19298,7 +20016,7 @@
         <v>46313.33333333334</v>
       </c>
       <c r="J61" s="11" t="n">
-        <v>46314.29166666666</v>
+        <v>46314.5</v>
       </c>
       <c r="K61" s="24">
         <f>(I61-H61)*24</f>
@@ -19320,61 +20038,57 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="31" t="inlineStr">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>20F</t>
         </is>
       </c>
-      <c r="B62" s="31" t="inlineStr">
-        <is>
-          <t>KMTC JAKARTA</t>
-        </is>
-      </c>
-      <c r="C62" s="17" t="n">
-        <v>564</v>
-      </c>
-      <c r="D62" s="18" t="n">
-        <v>46310</v>
-      </c>
-      <c r="E62" s="18" t="n">
-        <v>46313</v>
-      </c>
-      <c r="F62" s="17" t="n">
-        <v>4</v>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>GREEN PARK</t>
+        </is>
+      </c>
+      <c r="C62" s="23" t="n">
+        <v>482</v>
+      </c>
+      <c r="D62" s="10" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E62" s="10" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F62" s="23" t="n">
+        <v>6</v>
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="H62" s="20" t="n">
-        <v>46314.5</v>
-      </c>
-      <c r="I62" s="20" t="n">
-        <v>46314.5</v>
-      </c>
-      <c r="J62" s="20" t="n">
-        <v>46315.70833333334</v>
-      </c>
-      <c r="K62" s="32">
+          <t>20AB → 20B → 20AB → 20F</t>
+        </is>
+      </c>
+      <c r="H62" s="11" t="n">
+        <v>46316.70833333334</v>
+      </c>
+      <c r="I62" s="11" t="n">
+        <v>46317.58333333334</v>
+      </c>
+      <c r="J62" s="11" t="n">
+        <v>46318.54166666666</v>
+      </c>
+      <c r="K62" s="24">
         <f>(I62-H62)*24</f>
         <v/>
       </c>
-      <c r="L62" s="32">
+      <c r="L62" s="24">
         <f>(J62-I62)*24</f>
         <v/>
       </c>
-      <c r="M62" s="17" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N62" s="17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O62" s="17">
+      <c r="M62" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N62" s="23" t="inlineStr"/>
+      <c r="O62" s="23">
         <f>IF(J62&lt;=$B$3,"Sailed",IF(I62&lt;=$B$3,"Alongside",IF(H62&lt;=$B$3,"At anchorage","Expected")))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Add 23 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -35,6 +35,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 Oct 2026" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 Oct 2026" sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22 Oct 2026" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23 Oct 2026" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$57</definedName>
@@ -673,7 +674,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z74"/>
+  <dimension ref="A1:AA74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -702,6 +703,7 @@
     <col width="44" customWidth="1" min="24" max="24"/>
     <col width="44" customWidth="1" min="25" max="25"/>
     <col width="44" customWidth="1" min="26" max="26"/>
+    <col width="44" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -847,6 +849,11 @@
       <c r="Z4" s="3" t="inlineStr">
         <is>
           <t>22 Oct 2026</t>
+        </is>
+      </c>
+      <c r="AA4" s="3" t="inlineStr">
+        <is>
+          <t>23 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -913,6 +920,7 @@
       <c r="X5" s="5" t="inlineStr"/>
       <c r="Y5" s="5" t="inlineStr"/>
       <c r="Z5" s="5" t="inlineStr"/>
+      <c r="AA5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -961,6 +969,7 @@
       <c r="X6" s="5" t="inlineStr"/>
       <c r="Y6" s="5" t="inlineStr"/>
       <c r="Z6" s="5" t="inlineStr"/>
+      <c r="AA6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1013,6 +1022,11 @@
           <t>expected · 20AB (ETA 22/14→22/13)</t>
         </is>
       </c>
+      <c r="AA7" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20AB</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1069,6 +1083,7 @@
         </is>
       </c>
       <c r="Z8" s="5" t="inlineStr"/>
+      <c r="AA8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1137,6 +1152,7 @@
       <c r="X9" s="5" t="inlineStr"/>
       <c r="Y9" s="5" t="inlineStr"/>
       <c r="Z9" s="5" t="inlineStr"/>
+      <c r="AA9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1193,6 +1209,7 @@
       <c r="X10" s="5" t="inlineStr"/>
       <c r="Y10" s="5" t="inlineStr"/>
       <c r="Z10" s="5" t="inlineStr"/>
+      <c r="AA10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1257,6 +1274,7 @@
           <t>sailed (21/22)</t>
         </is>
       </c>
+      <c r="AA11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1317,6 +1335,7 @@
       <c r="X12" s="5" t="inlineStr"/>
       <c r="Y12" s="5" t="inlineStr"/>
       <c r="Z12" s="5" t="inlineStr"/>
+      <c r="AA12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1397,6 +1416,7 @@
           <t>sailed (22/05)</t>
         </is>
       </c>
+      <c r="AA13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1485,6 +1505,11 @@
           <t>expected · 20C</t>
         </is>
       </c>
+      <c r="AA14" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1549,6 +1574,7 @@
       <c r="X15" s="5" t="inlineStr"/>
       <c r="Y15" s="5" t="inlineStr"/>
       <c r="Z15" s="5" t="inlineStr"/>
+      <c r="AA15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1617,6 +1643,7 @@
       <c r="X16" s="5" t="inlineStr"/>
       <c r="Y16" s="5" t="inlineStr"/>
       <c r="Z16" s="5" t="inlineStr"/>
+      <c r="AA16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1705,6 +1732,11 @@
         </is>
       </c>
       <c r="Z17" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20AB (1C)</t>
+        </is>
+      </c>
+      <c r="AA17" s="5" t="inlineStr">
         <is>
           <t>expected · 20AB (1C)</t>
         </is>
@@ -1761,6 +1793,11 @@
       <c r="X18" s="5" t="inlineStr"/>
       <c r="Y18" s="5" t="inlineStr"/>
       <c r="Z18" s="5" t="inlineStr"/>
+      <c r="AA18" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20D (ETA 25/02→25/06, P.B 25/04→25/06)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1821,6 +1858,7 @@
       <c r="X19" s="5" t="inlineStr"/>
       <c r="Y19" s="5" t="inlineStr"/>
       <c r="Z19" s="5" t="inlineStr"/>
+      <c r="AA19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1881,6 +1919,11 @@
       <c r="X20" s="5" t="inlineStr"/>
       <c r="Y20" s="5" t="inlineStr"/>
       <c r="Z20" s="5" t="inlineStr"/>
+      <c r="AA20" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1937,6 +1980,7 @@
       <c r="X21" s="5" t="inlineStr"/>
       <c r="Y21" s="5" t="inlineStr"/>
       <c r="Z21" s="5" t="inlineStr"/>
+      <c r="AA21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1989,6 +2033,7 @@
       <c r="X22" s="5" t="inlineStr"/>
       <c r="Y22" s="5" t="inlineStr"/>
       <c r="Z22" s="5" t="inlineStr"/>
+      <c r="AA22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2053,6 +2098,7 @@
       <c r="X23" s="5" t="inlineStr"/>
       <c r="Y23" s="5" t="inlineStr"/>
       <c r="Z23" s="5" t="inlineStr"/>
+      <c r="AA23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -2113,6 +2159,7 @@
       <c r="X24" s="5" t="inlineStr"/>
       <c r="Y24" s="5" t="inlineStr"/>
       <c r="Z24" s="5" t="inlineStr"/>
+      <c r="AA24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2157,6 +2204,7 @@
       <c r="X25" s="5" t="inlineStr"/>
       <c r="Y25" s="5" t="inlineStr"/>
       <c r="Z25" s="5" t="inlineStr"/>
+      <c r="AA25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -2205,6 +2253,7 @@
       <c r="X26" s="5" t="inlineStr"/>
       <c r="Y26" s="5" t="inlineStr"/>
       <c r="Z26" s="5" t="inlineStr"/>
+      <c r="AA26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -2265,6 +2314,7 @@
       <c r="X27" s="5" t="inlineStr"/>
       <c r="Y27" s="5" t="inlineStr"/>
       <c r="Z27" s="5" t="inlineStr"/>
+      <c r="AA27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2321,6 +2371,7 @@
       <c r="X28" s="5" t="inlineStr"/>
       <c r="Y28" s="5" t="inlineStr"/>
       <c r="Z28" s="5" t="inlineStr"/>
+      <c r="AA28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2391,6 +2442,11 @@
       <c r="Z29" s="6" t="inlineStr">
         <is>
           <t>expected · 20B (ETA 21/14→21/16)</t>
+        </is>
+      </c>
+      <c r="AA29" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B</t>
         </is>
       </c>
     </row>
@@ -2457,6 +2513,7 @@
       <c r="X30" s="5" t="inlineStr"/>
       <c r="Y30" s="5" t="inlineStr"/>
       <c r="Z30" s="5" t="inlineStr"/>
+      <c r="AA30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2529,6 +2586,7 @@
           <t>sailed (21/20)</t>
         </is>
       </c>
+      <c r="AA31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2585,6 +2643,7 @@
       <c r="X32" s="5" t="inlineStr"/>
       <c r="Y32" s="5" t="inlineStr"/>
       <c r="Z32" s="5" t="inlineStr"/>
+      <c r="AA32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2637,6 +2696,7 @@
       <c r="X33" s="5" t="inlineStr"/>
       <c r="Y33" s="5" t="inlineStr"/>
       <c r="Z33" s="5" t="inlineStr"/>
+      <c r="AA33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2693,6 +2753,7 @@
       <c r="X34" s="5" t="inlineStr"/>
       <c r="Y34" s="5" t="inlineStr"/>
       <c r="Z34" s="5" t="inlineStr"/>
+      <c r="AA34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2749,6 +2810,7 @@
       <c r="X35" s="5" t="inlineStr"/>
       <c r="Y35" s="5" t="inlineStr"/>
       <c r="Z35" s="5" t="inlineStr"/>
+      <c r="AA35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2801,6 +2863,7 @@
       <c r="X36" s="5" t="inlineStr"/>
       <c r="Y36" s="5" t="inlineStr"/>
       <c r="Z36" s="5" t="inlineStr"/>
+      <c r="AA36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2857,6 +2920,11 @@
       <c r="X37" s="5" t="inlineStr"/>
       <c r="Y37" s="5" t="inlineStr"/>
       <c r="Z37" s="5" t="inlineStr"/>
+      <c r="AA37" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20AB</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2913,6 +2981,7 @@
       <c r="X38" s="5" t="inlineStr"/>
       <c r="Y38" s="5" t="inlineStr"/>
       <c r="Z38" s="5" t="inlineStr"/>
+      <c r="AA38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2965,6 +3034,7 @@
       <c r="X39" s="5" t="inlineStr"/>
       <c r="Y39" s="5" t="inlineStr"/>
       <c r="Z39" s="5" t="inlineStr"/>
+      <c r="AA39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -3017,6 +3087,7 @@
       <c r="X40" s="5" t="inlineStr"/>
       <c r="Y40" s="5" t="inlineStr"/>
       <c r="Z40" s="5" t="inlineStr"/>
+      <c r="AA40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -3073,6 +3144,7 @@
       <c r="X41" s="5" t="inlineStr"/>
       <c r="Y41" s="5" t="inlineStr"/>
       <c r="Z41" s="5" t="inlineStr"/>
+      <c r="AA41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -3125,6 +3197,7 @@
       <c r="X42" s="5" t="inlineStr"/>
       <c r="Y42" s="5" t="inlineStr"/>
       <c r="Z42" s="5" t="inlineStr"/>
+      <c r="AA42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -3181,6 +3254,7 @@
       <c r="X43" s="5" t="inlineStr"/>
       <c r="Y43" s="5" t="inlineStr"/>
       <c r="Z43" s="5" t="inlineStr"/>
+      <c r="AA43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -3237,6 +3311,7 @@
       <c r="X44" s="5" t="inlineStr"/>
       <c r="Y44" s="5" t="inlineStr"/>
       <c r="Z44" s="5" t="inlineStr"/>
+      <c r="AA44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -3289,6 +3364,7 @@
       <c r="X45" s="5" t="inlineStr"/>
       <c r="Y45" s="5" t="inlineStr"/>
       <c r="Z45" s="5" t="inlineStr"/>
+      <c r="AA45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -3349,6 +3425,7 @@
       <c r="X46" s="5" t="inlineStr"/>
       <c r="Y46" s="5" t="inlineStr"/>
       <c r="Z46" s="5" t="inlineStr"/>
+      <c r="AA46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -3405,6 +3482,7 @@
       <c r="X47" s="5" t="inlineStr"/>
       <c r="Y47" s="5" t="inlineStr"/>
       <c r="Z47" s="5" t="inlineStr"/>
+      <c r="AA47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -3461,6 +3539,7 @@
       <c r="X48" s="5" t="inlineStr"/>
       <c r="Y48" s="5" t="inlineStr"/>
       <c r="Z48" s="5" t="inlineStr"/>
+      <c r="AA48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -3517,6 +3596,7 @@
       <c r="X49" s="5" t="inlineStr"/>
       <c r="Y49" s="5" t="inlineStr"/>
       <c r="Z49" s="5" t="inlineStr"/>
+      <c r="AA49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -3569,6 +3649,7 @@
       <c r="X50" s="5" t="inlineStr"/>
       <c r="Y50" s="5" t="inlineStr"/>
       <c r="Z50" s="5" t="inlineStr"/>
+      <c r="AA50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -3617,6 +3698,7 @@
       <c r="X51" s="5" t="inlineStr"/>
       <c r="Y51" s="5" t="inlineStr"/>
       <c r="Z51" s="5" t="inlineStr"/>
+      <c r="AA51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -3669,6 +3751,7 @@
       <c r="X52" s="5" t="inlineStr"/>
       <c r="Y52" s="5" t="inlineStr"/>
       <c r="Z52" s="5" t="inlineStr"/>
+      <c r="AA52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -3721,6 +3804,7 @@
       <c r="X53" s="5" t="inlineStr"/>
       <c r="Y53" s="5" t="inlineStr"/>
       <c r="Z53" s="5" t="inlineStr"/>
+      <c r="AA53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -3773,6 +3857,7 @@
       <c r="X54" s="5" t="inlineStr"/>
       <c r="Y54" s="5" t="inlineStr"/>
       <c r="Z54" s="5" t="inlineStr"/>
+      <c r="AA54" s="5" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -3817,6 +3902,7 @@
       <c r="X55" s="5" t="inlineStr"/>
       <c r="Y55" s="5" t="inlineStr"/>
       <c r="Z55" s="5" t="inlineStr"/>
+      <c r="AA55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -3865,6 +3951,7 @@
       <c r="X56" s="5" t="inlineStr"/>
       <c r="Y56" s="5" t="inlineStr"/>
       <c r="Z56" s="5" t="inlineStr"/>
+      <c r="AA56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -3921,6 +4008,7 @@
       <c r="X57" s="5" t="inlineStr"/>
       <c r="Y57" s="5" t="inlineStr"/>
       <c r="Z57" s="5" t="inlineStr"/>
+      <c r="AA57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -3977,6 +4065,7 @@
       </c>
       <c r="Y58" s="5" t="inlineStr"/>
       <c r="Z58" s="5" t="inlineStr"/>
+      <c r="AA58" s="5" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -4025,6 +4114,7 @@
       <c r="X59" s="5" t="inlineStr"/>
       <c r="Y59" s="5" t="inlineStr"/>
       <c r="Z59" s="5" t="inlineStr"/>
+      <c r="AA59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -4085,6 +4175,7 @@
         </is>
       </c>
       <c r="Z60" s="5" t="inlineStr"/>
+      <c r="AA60" s="5" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -4129,6 +4220,7 @@
       <c r="X61" s="5" t="inlineStr"/>
       <c r="Y61" s="5" t="inlineStr"/>
       <c r="Z61" s="5" t="inlineStr"/>
+      <c r="AA61" s="5" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -4177,6 +4269,11 @@
           <t>expected · 20E</t>
         </is>
       </c>
+      <c r="AA62" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20E</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -4223,6 +4320,11 @@
       <c r="Z63" s="6" t="inlineStr">
         <is>
           <t>expected → 20C (full schedule now listed: P.B 24/15, ETD 26/03)</t>
+        </is>
+      </c>
+      <c r="AA63" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20C (ETA 23/22→23/17)</t>
         </is>
       </c>
     </row>
@@ -4269,6 +4371,11 @@
           <t>expected · 20B</t>
         </is>
       </c>
+      <c r="AA64" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20B (ETA 22/17→22/18)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -4313,6 +4420,11 @@
           <t>at anchorage · 20F (ETD 23/10→23/09)</t>
         </is>
       </c>
+      <c r="AA65" s="5" t="inlineStr">
+        <is>
+          <t>sailed (23/09)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -4355,6 +4467,11 @@
       <c r="Z66" s="6" t="inlineStr">
         <is>
           <t>expected · 22A, then shifts to 20F (ETD 23/10→23/09)</t>
+        </is>
+      </c>
+      <c r="AA66" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20F only (no longer listed at 22A; P.B 23/09)</t>
         </is>
       </c>
     </row>
@@ -4397,6 +4514,11 @@
           <t>expected · 20C</t>
         </is>
       </c>
+      <c r="AA67" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -4435,6 +4557,11 @@
       <c r="Z68" s="6" t="inlineStr">
         <is>
           <t>expected → 20E (schedule now listed: ETA 23/06, P.B 24/03, ETD 25/01)</t>
+        </is>
+      </c>
+      <c r="AA68" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20E (ETA 23/06→23/10)</t>
         </is>
       </c>
     </row>
@@ -4473,6 +4600,11 @@
           <t>expected · 20AB (new call)</t>
         </is>
       </c>
+      <c r="AA69" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20AB</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -4509,6 +4641,11 @@
           <t>expected · 20B (new)</t>
         </is>
       </c>
+      <c r="AA70" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -4545,6 +4682,11 @@
           <t>expected · 20B (new)</t>
         </is>
       </c>
+      <c r="AA71" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -4581,6 +4723,11 @@
           <t>expected · 20D (new)</t>
         </is>
       </c>
+      <c r="AA72" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20D (ETA 25/02→25/06, P.B 25/04→25/06)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -4617,6 +4764,11 @@
           <t>expected · 20E (new)</t>
         </is>
       </c>
+      <c r="AA73" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20E</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -4651,6 +4803,11 @@
       <c r="Z74" s="5" t="inlineStr">
         <is>
           <t>expected · 20F (new)</t>
+        </is>
+      </c>
+      <c r="AA74" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F</t>
         </is>
       </c>
     </row>
@@ -19597,6 +19754,748 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 23 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Waiting for Berth (h)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>ALS SUMIRE</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>537</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>46316.83333333334</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>46317.54166666666</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>46318.66666666666</v>
+      </c>
+      <c r="G4" s="24">
+        <f>(E4-D4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="24">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>1C</t>
+        </is>
+      </c>
+      <c r="J4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>KMTC GWANGYANG</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46317.54166666666</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46318.58333333334</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46320.08333333334</v>
+      </c>
+      <c r="G5" s="24">
+        <f>(E5-D5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="24">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>KANWAY FORTUNE</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46320.20833333334</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46320.625</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46292.125</v>
+      </c>
+      <c r="G6" s="24">
+        <f>(E6-D6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="24">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>GREEN PARK</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>482</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46316.66666666666</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46317.58333333334</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46318.54166666666</v>
+      </c>
+      <c r="G7" s="24">
+        <f>(E7-D7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="24">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>CA MANILA</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>548</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>46317.75</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>46318.54166666666</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>46320</v>
+      </c>
+      <c r="G8" s="24">
+        <f>(E8-D8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="24">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>ASL TAIPEIS</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>46320</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>46320.16666666666</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>46321.125</v>
+      </c>
+      <c r="G9" s="24">
+        <f>(E9-D9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="24">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>ZHONG GU BEI HAI</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>561</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>46321.58333333334</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>46321.58333333334</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>46293.125</v>
+      </c>
+      <c r="G10" s="24">
+        <f>(E10-D10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="24">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>CAPE FAWLEY</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>558</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>46316.45833333334</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>46316.5</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>46318.5</v>
+      </c>
+      <c r="G11" s="24">
+        <f>(E11-D11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="24">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J11" s="23" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>HORAI BRIDGE</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>46318.04166666666</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>46318.5</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>46319.625</v>
+      </c>
+      <c r="G12" s="24">
+        <f>(E12-D12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="24">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J12" s="23" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE MIMOSA</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>46318.70833333334</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>46319.625</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>46321.125</v>
+      </c>
+      <c r="G13" s="24">
+        <f>(E13-D13)*24</f>
+        <v/>
+      </c>
+      <c r="H13" s="24">
+        <f>(F13-E13)*24</f>
+        <v/>
+      </c>
+      <c r="I13" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J13" s="23" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>KMTC BANGKOK</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>46320.25</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>46320.25</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>46321.5</v>
+      </c>
+      <c r="G14" s="24">
+        <f>(E14-D14)*24</f>
+        <v/>
+      </c>
+      <c r="H14" s="24">
+        <f>(F14-E14)*24</f>
+        <v/>
+      </c>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J14" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>SKY ORION</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>46317.04166666666</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>46317.54166666666</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>46319.04166666666</v>
+      </c>
+      <c r="G15" s="24">
+        <f>(E15-D15)*24</f>
+        <v/>
+      </c>
+      <c r="H15" s="24">
+        <f>(F15-E15)*24</f>
+        <v/>
+      </c>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J15" s="23" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>YM IMAGE</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>46318.41666666666</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>46319.125</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>46320.04166666666</v>
+      </c>
+      <c r="G16" s="24">
+        <f>(E16-D16)*24</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>(F16-E16)*24</f>
+        <v/>
+      </c>
+      <c r="I16" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J16" s="23" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>HEUNG A HOCHIMINH</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>46320.91666666666</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>46321.25</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>46292.58333333334</v>
+      </c>
+      <c r="G17" s="24">
+        <f>(E17-D17)*24</f>
+        <v/>
+      </c>
+      <c r="H17" s="24">
+        <f>(F17-E17)*24</f>
+        <v/>
+      </c>
+      <c r="I17" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J17" s="23" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 272</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>46318.375</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>46318.375</v>
+      </c>
+      <c r="F18" s="11" t="n">
+        <v>46319.58333333334</v>
+      </c>
+      <c r="G18" s="24">
+        <f>(E18-D18)*24</f>
+        <v/>
+      </c>
+      <c r="H18" s="24">
+        <f>(F18-E18)*24</f>
+        <v/>
+      </c>
+      <c r="I18" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J18" s="23" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 106</t>
+        </is>
+      </c>
+      <c r="C19" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>46320.41666666666</v>
+      </c>
+      <c r="E19" s="11" t="n">
+        <v>46320.54166666666</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>46321.5</v>
+      </c>
+      <c r="G19" s="24">
+        <f>(E19-D19)*24</f>
+        <v/>
+      </c>
+      <c r="H19" s="24">
+        <f>(F19-E19)*24</f>
+        <v/>
+      </c>
+      <c r="I19" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J19" s="23" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="34" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G23" s="35" t="n"/>
+      <c r="H23" s="35" t="n"/>
+      <c r="I23" s="35" t="n"/>
+      <c r="J23" s="36" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="39" t="inlineStr">
+        <is>
+          <t>No notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F23:J23"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -19644,7 +20543,7 @@
         </is>
       </c>
       <c r="B3" s="22" t="n">
-        <v>46317.375</v>
+        <v>46318.375</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -20264,10 +21163,10 @@
         <v>46294</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F15" s="23" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
@@ -20320,10 +21219,10 @@
         <v>46293</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F16" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
@@ -20376,10 +21275,10 @@
         <v>46301</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F17" s="23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
@@ -21116,10 +22015,10 @@
         <v>46300</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F30" s="23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
@@ -21172,10 +22071,10 @@
         <v>46315</v>
       </c>
       <c r="E31" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F31" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
@@ -21183,7 +22082,7 @@
         </is>
       </c>
       <c r="H31" s="11" t="n">
-        <v>46317.66666666666</v>
+        <v>46317.75</v>
       </c>
       <c r="I31" s="11" t="n">
         <v>46318.54166666666</v>
@@ -21228,10 +22127,10 @@
         <v>46317</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F32" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
@@ -21284,10 +22183,10 @@
         <v>46296</v>
       </c>
       <c r="E33" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F33" s="23" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
@@ -21914,10 +22813,10 @@
         <v>46293</v>
       </c>
       <c r="E44" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F44" s="23" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
@@ -21970,10 +22869,10 @@
         <v>46316</v>
       </c>
       <c r="E45" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F45" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
@@ -22026,10 +22925,10 @@
         <v>46317</v>
       </c>
       <c r="E46" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F46" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
@@ -22037,7 +22936,7 @@
         </is>
       </c>
       <c r="H46" s="11" t="n">
-        <v>46318.91666666666</v>
+        <v>46318.70833333334</v>
       </c>
       <c r="I46" s="11" t="n">
         <v>46319.625</v>
@@ -22652,10 +23551,10 @@
         <v>46295</v>
       </c>
       <c r="E57" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F57" s="23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
@@ -22663,10 +23562,10 @@
         </is>
       </c>
       <c r="H57" s="11" t="n">
-        <v>46320.08333333334</v>
+        <v>46320.25</v>
       </c>
       <c r="I57" s="11" t="n">
-        <v>46320.16666666666</v>
+        <v>46320.25</v>
       </c>
       <c r="J57" s="11" t="n">
         <v>46321.5</v>
@@ -22826,10 +23725,10 @@
         <v>46315</v>
       </c>
       <c r="E60" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F60" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
@@ -22882,10 +23781,10 @@
         <v>46317</v>
       </c>
       <c r="E61" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F61" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
@@ -22893,7 +23792,7 @@
         </is>
       </c>
       <c r="H61" s="11" t="n">
-        <v>46318.25</v>
+        <v>46318.41666666666</v>
       </c>
       <c r="I61" s="11" t="n">
         <v>46319.125</v>
@@ -22938,10 +23837,10 @@
         <v>46317</v>
       </c>
       <c r="E62" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F62" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
@@ -23426,9 +24325,10 @@
         </is>
       </c>
       <c r="N70" s="23" t="inlineStr"/>
-      <c r="O70" s="23">
-        <f>IF(J70&lt;=$B$3,"Sailed",IF(I70&lt;=$B$3,"Alongside",IF(H70&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O70" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -23449,10 +24349,10 @@
         <v>46315</v>
       </c>
       <c r="E71" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F71" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G71" s="6" t="inlineStr">
         <is>
@@ -23505,10 +24405,10 @@
         <v>46317</v>
       </c>
       <c r="E72" s="10" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="F72" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add 24 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -36,10 +36,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 Oct 2026" sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22 Oct 2026" sheetId="28" state="visible" r:id="rId28"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23 Oct 2026" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24 Oct 2026" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$57</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$O$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$O$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -674,7 +675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA74"/>
+  <dimension ref="A1:AB77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -704,6 +705,7 @@
     <col width="44" customWidth="1" min="25" max="25"/>
     <col width="44" customWidth="1" min="26" max="26"/>
     <col width="44" customWidth="1" min="27" max="27"/>
+    <col width="44" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -854,6 +856,11 @@
       <c r="AA4" s="3" t="inlineStr">
         <is>
           <t>23 Oct 2026</t>
+        </is>
+      </c>
+      <c r="AB4" s="3" t="inlineStr">
+        <is>
+          <t>24 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -921,6 +928,7 @@
       <c r="Y5" s="5" t="inlineStr"/>
       <c r="Z5" s="5" t="inlineStr"/>
       <c r="AA5" s="5" t="inlineStr"/>
+      <c r="AB5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -970,6 +978,7 @@
       <c r="Y6" s="5" t="inlineStr"/>
       <c r="Z6" s="5" t="inlineStr"/>
       <c r="AA6" s="5" t="inlineStr"/>
+      <c r="AB6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1027,6 +1036,11 @@
           <t>expected · 20AB</t>
         </is>
       </c>
+      <c r="AB7" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20AB (ETD 25/02→25/01)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1084,6 +1098,7 @@
       </c>
       <c r="Z8" s="5" t="inlineStr"/>
       <c r="AA8" s="5" t="inlineStr"/>
+      <c r="AB8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1153,6 +1168,7 @@
       <c r="Y9" s="5" t="inlineStr"/>
       <c r="Z9" s="5" t="inlineStr"/>
       <c r="AA9" s="5" t="inlineStr"/>
+      <c r="AB9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1210,6 +1226,7 @@
       <c r="Y10" s="5" t="inlineStr"/>
       <c r="Z10" s="5" t="inlineStr"/>
       <c r="AA10" s="5" t="inlineStr"/>
+      <c r="AB10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1275,6 +1292,7 @@
         </is>
       </c>
       <c r="AA11" s="5" t="inlineStr"/>
+      <c r="AB11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1336,6 +1354,7 @@
       <c r="Y12" s="5" t="inlineStr"/>
       <c r="Z12" s="5" t="inlineStr"/>
       <c r="AA12" s="5" t="inlineStr"/>
+      <c r="AB12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1417,6 +1436,7 @@
         </is>
       </c>
       <c r="AA13" s="5" t="inlineStr"/>
+      <c r="AB13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1510,6 +1530,11 @@
           <t>expected · 20C</t>
         </is>
       </c>
+      <c r="AB14" s="5" t="inlineStr">
+        <is>
+          <t>sailed (23/12)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1575,6 +1600,7 @@
       <c r="Y15" s="5" t="inlineStr"/>
       <c r="Z15" s="5" t="inlineStr"/>
       <c r="AA15" s="5" t="inlineStr"/>
+      <c r="AB15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1644,6 +1670,7 @@
       <c r="Y16" s="5" t="inlineStr"/>
       <c r="Z16" s="5" t="inlineStr"/>
       <c r="AA16" s="5" t="inlineStr"/>
+      <c r="AB16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1739,6 +1766,11 @@
       <c r="AA17" s="5" t="inlineStr">
         <is>
           <t>expected · 20AB (1C)</t>
+        </is>
+      </c>
+      <c r="AB17" s="5" t="inlineStr">
+        <is>
+          <t>sailed (23/16)</t>
         </is>
       </c>
     </row>
@@ -1798,6 +1830,11 @@
           <t>expected · 20D (ETA 25/02→25/06, P.B 25/04→25/06)</t>
         </is>
       </c>
+      <c r="AB18" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1859,6 +1896,7 @@
       <c r="Y19" s="5" t="inlineStr"/>
       <c r="Z19" s="5" t="inlineStr"/>
       <c r="AA19" s="5" t="inlineStr"/>
+      <c r="AB19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1922,6 +1960,11 @@
       <c r="AA20" s="5" t="inlineStr">
         <is>
           <t>expected · 20B</t>
+        </is>
+      </c>
+      <c r="AB20" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20B (ETA 26/14→26/20, P.B 26/14→27/05, ETD 28/03→28/14)</t>
         </is>
       </c>
     </row>
@@ -1981,6 +2024,7 @@
       <c r="Y21" s="5" t="inlineStr"/>
       <c r="Z21" s="5" t="inlineStr"/>
       <c r="AA21" s="5" t="inlineStr"/>
+      <c r="AB21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -2034,6 +2078,7 @@
       <c r="Y22" s="5" t="inlineStr"/>
       <c r="Z22" s="5" t="inlineStr"/>
       <c r="AA22" s="5" t="inlineStr"/>
+      <c r="AB22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2099,6 +2144,7 @@
       <c r="Y23" s="5" t="inlineStr"/>
       <c r="Z23" s="5" t="inlineStr"/>
       <c r="AA23" s="5" t="inlineStr"/>
+      <c r="AB23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -2160,6 +2206,7 @@
       <c r="Y24" s="5" t="inlineStr"/>
       <c r="Z24" s="5" t="inlineStr"/>
       <c r="AA24" s="5" t="inlineStr"/>
+      <c r="AB24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2205,6 +2252,7 @@
       <c r="Y25" s="5" t="inlineStr"/>
       <c r="Z25" s="5" t="inlineStr"/>
       <c r="AA25" s="5" t="inlineStr"/>
+      <c r="AB25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -2254,6 +2302,7 @@
       <c r="Y26" s="5" t="inlineStr"/>
       <c r="Z26" s="5" t="inlineStr"/>
       <c r="AA26" s="5" t="inlineStr"/>
+      <c r="AB26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -2315,6 +2364,7 @@
       <c r="Y27" s="5" t="inlineStr"/>
       <c r="Z27" s="5" t="inlineStr"/>
       <c r="AA27" s="5" t="inlineStr"/>
+      <c r="AB27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2372,6 +2422,7 @@
       <c r="Y28" s="5" t="inlineStr"/>
       <c r="Z28" s="5" t="inlineStr"/>
       <c r="AA28" s="5" t="inlineStr"/>
+      <c r="AB28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2447,6 +2498,11 @@
       <c r="AA29" s="5" t="inlineStr">
         <is>
           <t>expected · 20B</t>
+        </is>
+      </c>
+      <c r="AB29" s="5" t="inlineStr">
+        <is>
+          <t>sailed (23/13)</t>
         </is>
       </c>
     </row>
@@ -2514,6 +2570,7 @@
       <c r="Y30" s="5" t="inlineStr"/>
       <c r="Z30" s="5" t="inlineStr"/>
       <c r="AA30" s="5" t="inlineStr"/>
+      <c r="AB30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2587,6 +2644,7 @@
         </is>
       </c>
       <c r="AA31" s="5" t="inlineStr"/>
+      <c r="AB31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2644,6 +2702,7 @@
       <c r="Y32" s="5" t="inlineStr"/>
       <c r="Z32" s="5" t="inlineStr"/>
       <c r="AA32" s="5" t="inlineStr"/>
+      <c r="AB32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2697,6 +2756,7 @@
       <c r="Y33" s="5" t="inlineStr"/>
       <c r="Z33" s="5" t="inlineStr"/>
       <c r="AA33" s="5" t="inlineStr"/>
+      <c r="AB33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2754,6 +2814,7 @@
       <c r="Y34" s="5" t="inlineStr"/>
       <c r="Z34" s="5" t="inlineStr"/>
       <c r="AA34" s="5" t="inlineStr"/>
+      <c r="AB34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2811,6 +2872,7 @@
       <c r="Y35" s="5" t="inlineStr"/>
       <c r="Z35" s="5" t="inlineStr"/>
       <c r="AA35" s="5" t="inlineStr"/>
+      <c r="AB35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2864,6 +2926,7 @@
       <c r="Y36" s="5" t="inlineStr"/>
       <c r="Z36" s="5" t="inlineStr"/>
       <c r="AA36" s="5" t="inlineStr"/>
+      <c r="AB36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2925,6 +2988,11 @@
           <t>expected · 20AB</t>
         </is>
       </c>
+      <c r="AB37" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20AB (ETD 27/03→26/16)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2982,6 +3050,7 @@
       <c r="Y38" s="5" t="inlineStr"/>
       <c r="Z38" s="5" t="inlineStr"/>
       <c r="AA38" s="5" t="inlineStr"/>
+      <c r="AB38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -3035,6 +3104,7 @@
       <c r="Y39" s="5" t="inlineStr"/>
       <c r="Z39" s="5" t="inlineStr"/>
       <c r="AA39" s="5" t="inlineStr"/>
+      <c r="AB39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -3088,6 +3158,7 @@
       <c r="Y40" s="5" t="inlineStr"/>
       <c r="Z40" s="5" t="inlineStr"/>
       <c r="AA40" s="5" t="inlineStr"/>
+      <c r="AB40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -3145,6 +3216,7 @@
       <c r="Y41" s="5" t="inlineStr"/>
       <c r="Z41" s="5" t="inlineStr"/>
       <c r="AA41" s="5" t="inlineStr"/>
+      <c r="AB41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -3198,6 +3270,7 @@
       <c r="Y42" s="5" t="inlineStr"/>
       <c r="Z42" s="5" t="inlineStr"/>
       <c r="AA42" s="5" t="inlineStr"/>
+      <c r="AB42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -3255,6 +3328,7 @@
       <c r="Y43" s="5" t="inlineStr"/>
       <c r="Z43" s="5" t="inlineStr"/>
       <c r="AA43" s="5" t="inlineStr"/>
+      <c r="AB43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -3312,6 +3386,7 @@
       <c r="Y44" s="5" t="inlineStr"/>
       <c r="Z44" s="5" t="inlineStr"/>
       <c r="AA44" s="5" t="inlineStr"/>
+      <c r="AB44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -3365,6 +3440,7 @@
       <c r="Y45" s="5" t="inlineStr"/>
       <c r="Z45" s="5" t="inlineStr"/>
       <c r="AA45" s="5" t="inlineStr"/>
+      <c r="AB45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -3426,6 +3502,7 @@
       <c r="Y46" s="5" t="inlineStr"/>
       <c r="Z46" s="5" t="inlineStr"/>
       <c r="AA46" s="5" t="inlineStr"/>
+      <c r="AB46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -3483,6 +3560,7 @@
       <c r="Y47" s="5" t="inlineStr"/>
       <c r="Z47" s="5" t="inlineStr"/>
       <c r="AA47" s="5" t="inlineStr"/>
+      <c r="AB47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -3540,6 +3618,7 @@
       <c r="Y48" s="5" t="inlineStr"/>
       <c r="Z48" s="5" t="inlineStr"/>
       <c r="AA48" s="5" t="inlineStr"/>
+      <c r="AB48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -3597,6 +3676,7 @@
       <c r="Y49" s="5" t="inlineStr"/>
       <c r="Z49" s="5" t="inlineStr"/>
       <c r="AA49" s="5" t="inlineStr"/>
+      <c r="AB49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -3650,6 +3730,7 @@
       <c r="Y50" s="5" t="inlineStr"/>
       <c r="Z50" s="5" t="inlineStr"/>
       <c r="AA50" s="5" t="inlineStr"/>
+      <c r="AB50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -3699,6 +3780,7 @@
       <c r="Y51" s="5" t="inlineStr"/>
       <c r="Z51" s="5" t="inlineStr"/>
       <c r="AA51" s="5" t="inlineStr"/>
+      <c r="AB51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -3752,6 +3834,7 @@
       <c r="Y52" s="5" t="inlineStr"/>
       <c r="Z52" s="5" t="inlineStr"/>
       <c r="AA52" s="5" t="inlineStr"/>
+      <c r="AB52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -3805,6 +3888,7 @@
       <c r="Y53" s="5" t="inlineStr"/>
       <c r="Z53" s="5" t="inlineStr"/>
       <c r="AA53" s="5" t="inlineStr"/>
+      <c r="AB53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -3858,6 +3942,7 @@
       <c r="Y54" s="5" t="inlineStr"/>
       <c r="Z54" s="5" t="inlineStr"/>
       <c r="AA54" s="5" t="inlineStr"/>
+      <c r="AB54" s="5" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -3903,6 +3988,7 @@
       <c r="Y55" s="5" t="inlineStr"/>
       <c r="Z55" s="5" t="inlineStr"/>
       <c r="AA55" s="5" t="inlineStr"/>
+      <c r="AB55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -3952,6 +4038,7 @@
       <c r="Y56" s="5" t="inlineStr"/>
       <c r="Z56" s="5" t="inlineStr"/>
       <c r="AA56" s="5" t="inlineStr"/>
+      <c r="AB56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -4009,6 +4096,7 @@
       <c r="Y57" s="5" t="inlineStr"/>
       <c r="Z57" s="5" t="inlineStr"/>
       <c r="AA57" s="5" t="inlineStr"/>
+      <c r="AB57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -4066,6 +4154,7 @@
       <c r="Y58" s="5" t="inlineStr"/>
       <c r="Z58" s="5" t="inlineStr"/>
       <c r="AA58" s="5" t="inlineStr"/>
+      <c r="AB58" s="5" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -4115,6 +4204,7 @@
       <c r="Y59" s="5" t="inlineStr"/>
       <c r="Z59" s="5" t="inlineStr"/>
       <c r="AA59" s="5" t="inlineStr"/>
+      <c r="AB59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -4176,6 +4266,7 @@
       </c>
       <c r="Z60" s="5" t="inlineStr"/>
       <c r="AA60" s="5" t="inlineStr"/>
+      <c r="AB60" s="5" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -4221,6 +4312,7 @@
       <c r="Y61" s="5" t="inlineStr"/>
       <c r="Z61" s="5" t="inlineStr"/>
       <c r="AA61" s="5" t="inlineStr"/>
+      <c r="AB61" s="5" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -4274,6 +4366,11 @@
           <t>expected · 20E</t>
         </is>
       </c>
+      <c r="AB62" s="5" t="inlineStr">
+        <is>
+          <t>sailed (24/01)</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -4325,6 +4422,11 @@
       <c r="AA63" s="6" t="inlineStr">
         <is>
           <t>expected · 20C (ETA 23/22→23/17)</t>
+        </is>
+      </c>
+      <c r="AB63" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C</t>
         </is>
       </c>
     </row>
@@ -4376,6 +4478,11 @@
           <t>expected · 20B (ETA 22/17→22/18)</t>
         </is>
       </c>
+      <c r="AB64" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -4425,6 +4532,7 @@
           <t>sailed (23/09)</t>
         </is>
       </c>
+      <c r="AB65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -4472,6 +4580,11 @@
       <c r="AA66" s="6" t="inlineStr">
         <is>
           <t>expected → 20F only (no longer listed at 22A; P.B 23/09)</t>
+        </is>
+      </c>
+      <c r="AB66" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F (shows ETA “22A”, P.B 23/09)</t>
         </is>
       </c>
     </row>
@@ -4519,6 +4632,11 @@
           <t>expected · 20C</t>
         </is>
       </c>
+      <c r="AB67" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -4562,6 +4680,11 @@
       <c r="AA68" s="6" t="inlineStr">
         <is>
           <t>expected · 20E (ETA 23/06→23/10)</t>
+        </is>
+      </c>
+      <c r="AB68" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20E (ETA 23/10→23/06)</t>
         </is>
       </c>
     </row>
@@ -4605,6 +4728,11 @@
           <t>expected · 20AB</t>
         </is>
       </c>
+      <c r="AB69" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20AB (ETD 27/03→26/16)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -4646,6 +4774,11 @@
           <t>expected · 20B</t>
         </is>
       </c>
+      <c r="AB70" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20B</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -4687,6 +4820,11 @@
           <t>expected · 20B</t>
         </is>
       </c>
+      <c r="AB71" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20B (ETA 26/14→26/20, P.B 26/14→27/05, ETD 28/03→28/14)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -4728,6 +4866,11 @@
           <t>expected · 20D (ETA 25/02→25/06, P.B 25/04→25/06)</t>
         </is>
       </c>
+      <c r="AB72" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -4769,6 +4912,11 @@
           <t>expected · 20E</t>
         </is>
       </c>
+      <c r="AB73" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20F (moved from 20E; ETA 25/22→25/14, P.B 26/06→25/15, ETD 27/14→27/04)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -4808,6 +4956,125 @@
       <c r="AA74" s="5" t="inlineStr">
         <is>
           <t>expected · 20F</t>
+        </is>
+      </c>
+      <c r="AB74" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20E (moved from 20F)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>XIN AN</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr"/>
+      <c r="C75" s="5" t="inlineStr"/>
+      <c r="D75" s="5" t="inlineStr"/>
+      <c r="E75" s="5" t="inlineStr"/>
+      <c r="F75" s="5" t="inlineStr"/>
+      <c r="G75" s="5" t="inlineStr"/>
+      <c r="H75" s="5" t="inlineStr"/>
+      <c r="I75" s="5" t="inlineStr"/>
+      <c r="J75" s="5" t="inlineStr"/>
+      <c r="K75" s="5" t="inlineStr"/>
+      <c r="L75" s="5" t="inlineStr"/>
+      <c r="M75" s="5" t="inlineStr"/>
+      <c r="N75" s="5" t="inlineStr"/>
+      <c r="O75" s="5" t="inlineStr"/>
+      <c r="P75" s="5" t="inlineStr"/>
+      <c r="Q75" s="5" t="inlineStr"/>
+      <c r="R75" s="5" t="inlineStr"/>
+      <c r="S75" s="5" t="inlineStr"/>
+      <c r="T75" s="5" t="inlineStr"/>
+      <c r="U75" s="5" t="inlineStr"/>
+      <c r="V75" s="5" t="inlineStr"/>
+      <c r="W75" s="5" t="inlineStr"/>
+      <c r="X75" s="5" t="inlineStr"/>
+      <c r="Y75" s="5" t="inlineStr"/>
+      <c r="Z75" s="5" t="inlineStr"/>
+      <c r="AA75" s="5" t="inlineStr"/>
+      <c r="AB75" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>PUNNYA NAVEE (barge)</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr"/>
+      <c r="C76" s="5" t="inlineStr"/>
+      <c r="D76" s="5" t="inlineStr"/>
+      <c r="E76" s="5" t="inlineStr"/>
+      <c r="F76" s="5" t="inlineStr"/>
+      <c r="G76" s="5" t="inlineStr"/>
+      <c r="H76" s="5" t="inlineStr"/>
+      <c r="I76" s="5" t="inlineStr"/>
+      <c r="J76" s="5" t="inlineStr"/>
+      <c r="K76" s="5" t="inlineStr"/>
+      <c r="L76" s="5" t="inlineStr"/>
+      <c r="M76" s="5" t="inlineStr"/>
+      <c r="N76" s="5" t="inlineStr"/>
+      <c r="O76" s="5" t="inlineStr"/>
+      <c r="P76" s="5" t="inlineStr"/>
+      <c r="Q76" s="5" t="inlineStr"/>
+      <c r="R76" s="5" t="inlineStr"/>
+      <c r="S76" s="5" t="inlineStr"/>
+      <c r="T76" s="5" t="inlineStr"/>
+      <c r="U76" s="5" t="inlineStr"/>
+      <c r="V76" s="5" t="inlineStr"/>
+      <c r="W76" s="5" t="inlineStr"/>
+      <c r="X76" s="5" t="inlineStr"/>
+      <c r="Y76" s="5" t="inlineStr"/>
+      <c r="Z76" s="5" t="inlineStr"/>
+      <c r="AA76" s="5" t="inlineStr"/>
+      <c r="AB76" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D (new, barge)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>HARI BHUM (barge)</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr"/>
+      <c r="C77" s="5" t="inlineStr"/>
+      <c r="D77" s="5" t="inlineStr"/>
+      <c r="E77" s="5" t="inlineStr"/>
+      <c r="F77" s="5" t="inlineStr"/>
+      <c r="G77" s="5" t="inlineStr"/>
+      <c r="H77" s="5" t="inlineStr"/>
+      <c r="I77" s="5" t="inlineStr"/>
+      <c r="J77" s="5" t="inlineStr"/>
+      <c r="K77" s="5" t="inlineStr"/>
+      <c r="L77" s="5" t="inlineStr"/>
+      <c r="M77" s="5" t="inlineStr"/>
+      <c r="N77" s="5" t="inlineStr"/>
+      <c r="O77" s="5" t="inlineStr"/>
+      <c r="P77" s="5" t="inlineStr"/>
+      <c r="Q77" s="5" t="inlineStr"/>
+      <c r="R77" s="5" t="inlineStr"/>
+      <c r="S77" s="5" t="inlineStr"/>
+      <c r="T77" s="5" t="inlineStr"/>
+      <c r="U77" s="5" t="inlineStr"/>
+      <c r="V77" s="5" t="inlineStr"/>
+      <c r="W77" s="5" t="inlineStr"/>
+      <c r="X77" s="5" t="inlineStr"/>
+      <c r="Y77" s="5" t="inlineStr"/>
+      <c r="Z77" s="5" t="inlineStr"/>
+      <c r="AA77" s="5" t="inlineStr"/>
+      <c r="AB77" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D (new, barge)</t>
         </is>
       </c>
     </row>
@@ -20502,7 +20769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O74"/>
+  <dimension ref="A1:O76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20543,7 +20810,7 @@
         </is>
       </c>
       <c r="B3" s="22" t="n">
-        <v>46318.375</v>
+        <v>46319.375</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -21196,9 +21463,10 @@
         </is>
       </c>
       <c r="N15" s="23" t="inlineStr"/>
-      <c r="O15" s="23">
-        <f>IF(J15&lt;=$B$3,"Sailed",IF(I15&lt;=$B$3,"Alongside",IF(H15&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O15" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -21219,10 +21487,10 @@
         <v>46293</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="F16" s="23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G16" s="6" t="inlineStr">
         <is>
@@ -21236,7 +21504,7 @@
         <v>46318.58333333334</v>
       </c>
       <c r="J16" s="11" t="n">
-        <v>46320.08333333334</v>
+        <v>46320.04166666666</v>
       </c>
       <c r="K16" s="24">
         <f>(I16-H16)*24</f>
@@ -21275,10 +21543,10 @@
         <v>46301</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="F17" s="23" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
@@ -21292,7 +21560,7 @@
         <v>46320.625</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>46292.125</v>
+        <v>46321.66666666666</v>
       </c>
       <c r="K17" s="24">
         <f>(I17-H17)*24</f>
@@ -21321,34 +21589,34 @@
       </c>
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>YM IMPROVEMENT</t>
+          <t>ZHONG GU BEI HAI</t>
         </is>
       </c>
       <c r="C18" s="28" t="n">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="D18" s="29" t="n">
         <v>46296</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>46300</v>
+        <v>46319</v>
       </c>
       <c r="F18" s="28" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="G18" s="30" t="inlineStr">
         <is>
-          <t>20C → 20B</t>
+          <t>20B → 20AB → 20B</t>
         </is>
       </c>
       <c r="H18" s="31" t="n">
-        <v>46298.95833333334</v>
+        <v>46321.83333333334</v>
       </c>
       <c r="I18" s="31" t="n">
-        <v>46299.41666666666</v>
+        <v>46292.20833333334</v>
       </c>
       <c r="J18" s="31" t="n">
-        <v>46300.5</v>
+        <v>46293.58333333334</v>
       </c>
       <c r="K18" s="32">
         <f>(I18-H18)*24</f>
@@ -21364,10 +21632,9 @@
         </is>
       </c>
       <c r="N18" s="28" t="inlineStr"/>
-      <c r="O18" s="28" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="O18" s="28">
+        <f>IF(J18&lt;=$B$3,"Sailed",IF(I18&lt;=$B$3,"Alongside",IF(H18&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="19">
@@ -21378,34 +21645,34 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE SPICA</t>
+          <t>YM IMPROVEMENT</t>
         </is>
       </c>
       <c r="C19" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>46299</v>
+        <v>46296</v>
       </c>
       <c r="E19" s="10" t="n">
-        <v>46303</v>
+        <v>46300</v>
       </c>
       <c r="F19" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>20C → 20B</t>
         </is>
       </c>
       <c r="H19" s="11" t="n">
-        <v>46300.875</v>
+        <v>46298.95833333334</v>
       </c>
       <c r="I19" s="11" t="n">
-        <v>46301.54166666666</v>
+        <v>46299.41666666666</v>
       </c>
       <c r="J19" s="11" t="n">
-        <v>46303.54166666666</v>
+        <v>46300.5</v>
       </c>
       <c r="K19" s="24">
         <f>(I19-H19)*24</f>
@@ -21435,34 +21702,34 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>SITC HOCHIMINH</t>
+          <t>SAWASDEE SPICA</t>
         </is>
       </c>
       <c r="C20" s="23" t="n">
-        <v>470</v>
+        <v>564</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>46301</v>
+        <v>46299</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="F20" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20B</t>
+        <v>5</v>
+      </c>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H20" s="11" t="n">
-        <v>46302.625</v>
+        <v>46300.875</v>
       </c>
       <c r="I20" s="11" t="n">
-        <v>46303.58333333334</v>
+        <v>46301.54166666666</v>
       </c>
       <c r="J20" s="11" t="n">
-        <v>46304.70833333334</v>
+        <v>46303.54166666666</v>
       </c>
       <c r="K20" s="24">
         <f>(I20-H20)*24</f>
@@ -21492,34 +21759,34 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>INDURO</t>
+          <t>SITC HOCHIMINH</t>
         </is>
       </c>
       <c r="C21" s="23" t="n">
-        <v>565</v>
+        <v>470</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E21" s="10" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="F21" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="G21" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20B</t>
         </is>
       </c>
       <c r="H21" s="11" t="n">
-        <v>46304.25</v>
+        <v>46302.625</v>
       </c>
       <c r="I21" s="11" t="n">
-        <v>46304.66666666666</v>
+        <v>46303.58333333334</v>
       </c>
       <c r="J21" s="11" t="n">
-        <v>46306.16666666666</v>
+        <v>46304.70833333334</v>
       </c>
       <c r="K21" s="24">
         <f>(I21-H21)*24</f>
@@ -21549,34 +21816,34 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 102</t>
+          <t>INDURO</t>
         </is>
       </c>
       <c r="C22" s="23" t="n">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D22" s="10" t="n">
         <v>46302</v>
       </c>
       <c r="E22" s="10" t="n">
-        <v>46306</v>
+        <v>46305</v>
       </c>
       <c r="F22" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G22" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20B</t>
+        <v>4</v>
+      </c>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H22" s="11" t="n">
-        <v>46305.875</v>
+        <v>46304.25</v>
       </c>
       <c r="I22" s="11" t="n">
-        <v>46306.20833333334</v>
+        <v>46304.66666666666</v>
       </c>
       <c r="J22" s="11" t="n">
-        <v>46307.08333333334</v>
+        <v>46306.16666666666</v>
       </c>
       <c r="K22" s="24">
         <f>(I22-H22)*24</f>
@@ -21606,34 +21873,34 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>CEBU</t>
+          <t>XIN MING ZHOU 102</t>
         </is>
       </c>
       <c r="C23" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D23" s="10" t="n">
+        <v>46302</v>
+      </c>
+      <c r="E23" s="10" t="n">
         <v>46306</v>
       </c>
-      <c r="E23" s="10" t="n">
-        <v>46309</v>
-      </c>
       <c r="F23" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20B</t>
+          <t>20F → 20B</t>
         </is>
       </c>
       <c r="H23" s="11" t="n">
-        <v>46307.91666666666</v>
+        <v>46305.875</v>
       </c>
       <c r="I23" s="11" t="n">
-        <v>46308.25</v>
+        <v>46306.20833333334</v>
       </c>
       <c r="J23" s="11" t="n">
-        <v>46309.54166666666</v>
+        <v>46307.08333333334</v>
       </c>
       <c r="K23" s="24">
         <f>(I23-H23)*24</f>
@@ -21663,34 +21930,34 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>M ODYSSEY</t>
+          <t>CEBU</t>
         </is>
       </c>
       <c r="C24" s="23" t="n">
-        <v>449</v>
+        <v>564</v>
       </c>
       <c r="D24" s="10" t="n">
-        <v>46293</v>
+        <v>46306</v>
       </c>
       <c r="E24" s="10" t="n">
         <v>46309</v>
       </c>
       <c r="F24" s="23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G24" s="6" t="inlineStr">
         <is>
-          <t>20B → 20C → 20B</t>
+          <t>20AB → 20B</t>
         </is>
       </c>
       <c r="H24" s="11" t="n">
-        <v>46309.04166666666</v>
+        <v>46307.91666666666</v>
       </c>
       <c r="I24" s="11" t="n">
-        <v>46309.625</v>
+        <v>46308.25</v>
       </c>
       <c r="J24" s="11" t="n">
-        <v>46310.20833333334</v>
+        <v>46309.54166666666</v>
       </c>
       <c r="K24" s="24">
         <f>(I24-H24)*24</f>
@@ -21702,7 +21969,7 @@
       </c>
       <c r="M24" s="23" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N24" s="23" t="inlineStr"/>
@@ -21720,34 +21987,34 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>KHARIS HERITAGE</t>
+          <t>M ODYSSEY</t>
         </is>
       </c>
       <c r="C25" s="23" t="n">
-        <v>482</v>
+        <v>449</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="E25" s="10" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="F25" s="23" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20B → 20C → 20B</t>
+          <t>20B → 20C → 20B</t>
         </is>
       </c>
       <c r="H25" s="11" t="n">
-        <v>46310.04166666666</v>
+        <v>46309.04166666666</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>46310.25</v>
+        <v>46309.625</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>46311.29166666666</v>
+        <v>46310.20833333334</v>
       </c>
       <c r="K25" s="24">
         <f>(I25-H25)*24</f>
@@ -21759,7 +22026,7 @@
       </c>
       <c r="M25" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="N25" s="23" t="inlineStr"/>
@@ -21777,34 +22044,34 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>TS CHIBA</t>
+          <t>KHARIS HERITAGE</t>
         </is>
       </c>
       <c r="C26" s="23" t="n">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="D26" s="10" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="E26" s="10" t="n">
-        <v>46312</v>
+        <v>46310</v>
       </c>
       <c r="F26" s="23" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>20E → 20C → 20B</t>
+          <t>20AB → 20B → 20C → 20B</t>
         </is>
       </c>
       <c r="H26" s="11" t="n">
-        <v>46311.58333333334</v>
+        <v>46310.04166666666</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>46311.58333333334</v>
+        <v>46310.25</v>
       </c>
       <c r="J26" s="11" t="n">
-        <v>46312.45833333334</v>
+        <v>46311.29166666666</v>
       </c>
       <c r="K26" s="24">
         <f>(I26-H26)*24</f>
@@ -21834,34 +22101,34 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>JARU BHUM</t>
+          <t>TS CHIBA</t>
         </is>
       </c>
       <c r="C27" s="23" t="n">
-        <v>564</v>
+        <v>485</v>
       </c>
       <c r="D27" s="10" t="n">
         <v>46293</v>
       </c>
       <c r="E27" s="10" t="n">
-        <v>46313</v>
+        <v>46312</v>
       </c>
       <c r="F27" s="23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>20F → 20D → 20B</t>
+          <t>20E → 20C → 20B</t>
         </is>
       </c>
       <c r="H27" s="11" t="n">
-        <v>46312.66666666666</v>
+        <v>46311.58333333334</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>46312.66666666666</v>
+        <v>46311.58333333334</v>
       </c>
       <c r="J27" s="11" t="n">
-        <v>46313.41666666666</v>
+        <v>46312.45833333334</v>
       </c>
       <c r="K27" s="24">
         <f>(I27-H27)*24</f>
@@ -21873,7 +22140,7 @@
       </c>
       <c r="M27" s="23" t="inlineStr">
         <is>
-          <t>7B</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N27" s="23" t="inlineStr"/>
@@ -21891,34 +22158,34 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>KMTC JAKARTA</t>
+          <t>JARU BHUM</t>
         </is>
       </c>
       <c r="C28" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D28" s="10" t="n">
-        <v>46310</v>
+        <v>46293</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>46315</v>
+        <v>46313</v>
       </c>
       <c r="F28" s="23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>20F → 20B</t>
+          <t>20F → 20D → 20B</t>
         </is>
       </c>
       <c r="H28" s="11" t="n">
-        <v>46314.41666666666</v>
+        <v>46312.66666666666</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>46314.41666666666</v>
+        <v>46312.66666666666</v>
       </c>
       <c r="J28" s="11" t="n">
-        <v>46315.70833333334</v>
+        <v>46313.41666666666</v>
       </c>
       <c r="K28" s="24">
         <f>(I28-H28)*24</f>
@@ -21930,7 +22197,7 @@
       </c>
       <c r="M28" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="N28" s="23" t="inlineStr"/>
@@ -21948,34 +22215,34 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>MITRA BHUM</t>
+          <t>KMTC JAKARTA</t>
         </is>
       </c>
       <c r="C29" s="23" t="n">
-        <v>485</v>
+        <v>564</v>
       </c>
       <c r="D29" s="10" t="n">
-        <v>46293</v>
+        <v>46310</v>
       </c>
       <c r="E29" s="10" t="n">
-        <v>46316</v>
+        <v>46315</v>
       </c>
       <c r="F29" s="23" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>20F → 20E → 20D → 20AB → 20C → 20B</t>
+          <t>20F → 20B</t>
         </is>
       </c>
       <c r="H29" s="11" t="n">
-        <v>46316.54166666666</v>
+        <v>46314.41666666666</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>46316.54166666666</v>
+        <v>46314.41666666666</v>
       </c>
       <c r="J29" s="11" t="n">
-        <v>46317.20833333334</v>
+        <v>46315.70833333334</v>
       </c>
       <c r="K29" s="24">
         <f>(I29-H29)*24</f>
@@ -22005,34 +22272,34 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>GREEN PARK</t>
+          <t>MITRA BHUM</t>
         </is>
       </c>
       <c r="C30" s="23" t="n">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="D30" s="10" t="n">
-        <v>46300</v>
+        <v>46293</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>46318</v>
+        <v>46316</v>
       </c>
       <c r="F30" s="23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20B → 20AB → 20F → 20B</t>
+          <t>20F → 20E → 20D → 20AB → 20C → 20B</t>
         </is>
       </c>
       <c r="H30" s="11" t="n">
-        <v>46316.66666666666</v>
+        <v>46316.54166666666</v>
       </c>
       <c r="I30" s="11" t="n">
-        <v>46317.58333333334</v>
+        <v>46316.54166666666</v>
       </c>
       <c r="J30" s="11" t="n">
-        <v>46318.54166666666</v>
+        <v>46317.20833333334</v>
       </c>
       <c r="K30" s="24">
         <f>(I30-H30)*24</f>
@@ -22048,9 +22315,10 @@
         </is>
       </c>
       <c r="N30" s="23" t="inlineStr"/>
-      <c r="O30" s="23">
-        <f>IF(J30&lt;=$B$3,"Sailed",IF(I30&lt;=$B$3,"Alongside",IF(H30&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O30" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="31">
@@ -22061,34 +22329,34 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>CA MANILA</t>
+          <t>GREEN PARK</t>
         </is>
       </c>
       <c r="C31" s="23" t="n">
-        <v>548</v>
+        <v>482</v>
       </c>
       <c r="D31" s="10" t="n">
-        <v>46315</v>
+        <v>46300</v>
       </c>
       <c r="E31" s="10" t="n">
         <v>46318</v>
       </c>
       <c r="F31" s="23" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>20C → 20B</t>
+          <t>20AB → 20B → 20AB → 20F → 20B</t>
         </is>
       </c>
       <c r="H31" s="11" t="n">
-        <v>46317.75</v>
+        <v>46316.66666666666</v>
       </c>
       <c r="I31" s="11" t="n">
+        <v>46317.58333333334</v>
+      </c>
+      <c r="J31" s="11" t="n">
         <v>46318.54166666666</v>
-      </c>
-      <c r="J31" s="11" t="n">
-        <v>46320</v>
       </c>
       <c r="K31" s="24">
         <f>(I31-H31)*24</f>
@@ -22104,9 +22372,10 @@
         </is>
       </c>
       <c r="N31" s="23" t="inlineStr"/>
-      <c r="O31" s="23">
-        <f>IF(J31&lt;=$B$3,"Sailed",IF(I31&lt;=$B$3,"Alongside",IF(H31&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O31" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="32">
@@ -22117,34 +22386,34 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>ASL TAIPEIS</t>
+          <t>CA MANILA</t>
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>564</v>
+        <v>548</v>
       </c>
       <c r="D32" s="10" t="n">
-        <v>46317</v>
+        <v>46315</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="F32" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G32" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
+        <v>5</v>
+      </c>
+      <c r="G32" s="6" t="inlineStr">
+        <is>
+          <t>20C → 20B</t>
         </is>
       </c>
       <c r="H32" s="11" t="n">
+        <v>46317.75</v>
+      </c>
+      <c r="I32" s="11" t="n">
+        <v>46318.54166666666</v>
+      </c>
+      <c r="J32" s="11" t="n">
         <v>46320</v>
-      </c>
-      <c r="I32" s="11" t="n">
-        <v>46320.16666666666</v>
-      </c>
-      <c r="J32" s="11" t="n">
-        <v>46321.125</v>
       </c>
       <c r="K32" s="24">
         <f>(I32-H32)*24</f>
@@ -22173,34 +22442,34 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>ZHONG GU BEI HAI</t>
+          <t>ASL TAIPEIS</t>
         </is>
       </c>
       <c r="C33" s="23" t="n">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="D33" s="10" t="n">
-        <v>46296</v>
+        <v>46317</v>
       </c>
       <c r="E33" s="10" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="F33" s="23" t="n">
-        <v>8</v>
-      </c>
-      <c r="G33" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 20B</t>
+        <v>3</v>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H33" s="11" t="n">
-        <v>46321.58333333334</v>
+        <v>46320</v>
       </c>
       <c r="I33" s="11" t="n">
-        <v>46321.58333333334</v>
+        <v>46320.16666666666</v>
       </c>
       <c r="J33" s="11" t="n">
-        <v>46293.125</v>
+        <v>46321.125</v>
       </c>
       <c r="K33" s="24">
         <f>(I33-H33)*24</f>
@@ -22229,34 +22498,34 @@
       </c>
       <c r="B34" s="27" t="inlineStr">
         <is>
-          <t>SAWASDEE DENEB</t>
+          <t>XIN AN</t>
         </is>
       </c>
       <c r="C34" s="28" t="n">
         <v>564</v>
       </c>
       <c r="D34" s="29" t="n">
-        <v>46297</v>
+        <v>46300</v>
       </c>
       <c r="E34" s="29" t="n">
-        <v>46302</v>
+        <v>46319</v>
       </c>
       <c r="F34" s="28" t="n">
         <v>6</v>
       </c>
-      <c r="G34" s="33" t="inlineStr">
-        <is>
-          <t>20C</t>
+      <c r="G34" s="30" t="inlineStr">
+        <is>
+          <t>20F → 20C</t>
         </is>
       </c>
       <c r="H34" s="31" t="n">
-        <v>46300</v>
+        <v>46321.75</v>
       </c>
       <c r="I34" s="31" t="n">
-        <v>46300.5</v>
+        <v>46292.16666666666</v>
       </c>
       <c r="J34" s="31" t="n">
-        <v>46302.45833333334</v>
+        <v>46293.20833333334</v>
       </c>
       <c r="K34" s="32">
         <f>(I34-H34)*24</f>
@@ -22272,10 +22541,9 @@
         </is>
       </c>
       <c r="N34" s="28" t="inlineStr"/>
-      <c r="O34" s="28" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="O34" s="28">
+        <f>IF(J34&lt;=$B$3,"Sailed",IF(I34&lt;=$B$3,"Alongside",IF(H34&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -22286,7 +22554,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>JOSCO LUCKY</t>
+          <t>SAWASDEE DENEB</t>
         </is>
       </c>
       <c r="C35" s="23" t="n">
@@ -22296,24 +22564,24 @@
         <v>46297</v>
       </c>
       <c r="E35" s="10" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="F35" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="G35" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 20D → 20C</t>
+        <v>6</v>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
         </is>
       </c>
       <c r="H35" s="11" t="n">
-        <v>46301.875</v>
+        <v>46300</v>
       </c>
       <c r="I35" s="11" t="n">
-        <v>46302.54166666666</v>
+        <v>46300.5</v>
       </c>
       <c r="J35" s="11" t="n">
-        <v>46303.54166666666</v>
+        <v>46302.45833333334</v>
       </c>
       <c r="K35" s="24">
         <f>(I35-H35)*24</f>
@@ -22343,34 +22611,34 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>ZHONG GU DONG HAI</t>
+          <t>JOSCO LUCKY</t>
         </is>
       </c>
       <c r="C36" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D36" s="10" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="E36" s="10" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="F36" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G36" s="5" t="inlineStr">
-        <is>
-          <t>20C</t>
+        <v>7</v>
+      </c>
+      <c r="G36" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20AB → 20D → 20C</t>
         </is>
       </c>
       <c r="H36" s="11" t="n">
-        <v>46302.58333333334</v>
+        <v>46301.875</v>
       </c>
       <c r="I36" s="11" t="n">
-        <v>46303.58333333334</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="J36" s="11" t="n">
-        <v>46304.58333333334</v>
+        <v>46303.54166666666</v>
       </c>
       <c r="K36" s="24">
         <f>(I36-H36)*24</f>
@@ -22393,118 +22661,118 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="25" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>20C</t>
         </is>
       </c>
-      <c r="B37" s="25" t="inlineStr">
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>ZHONG GU DONG HAI</t>
+        </is>
+      </c>
+      <c r="C37" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D37" s="10" t="n">
+        <v>46301</v>
+      </c>
+      <c r="E37" s="10" t="n">
+        <v>46304</v>
+      </c>
+      <c r="F37" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="H37" s="11" t="n">
+        <v>46302.58333333334</v>
+      </c>
+      <c r="I37" s="11" t="n">
+        <v>46303.58333333334</v>
+      </c>
+      <c r="J37" s="11" t="n">
+        <v>46304.58333333334</v>
+      </c>
+      <c r="K37" s="24">
+        <f>(I37-H37)*24</f>
+        <v/>
+      </c>
+      <c r="L37" s="24">
+        <f>(J37-I37)*24</f>
+        <v/>
+      </c>
+      <c r="M37" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N37" s="23" t="inlineStr"/>
+      <c r="O37" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="25" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B38" s="25" t="inlineStr">
         <is>
           <t>YM INCEPTION</t>
         </is>
       </c>
-      <c r="C37" s="17" t="n">
+      <c r="C38" s="17" t="n">
         <v>564</v>
       </c>
-      <c r="D37" s="18" t="n">
+      <c r="D38" s="18" t="n">
         <v>46301</v>
       </c>
-      <c r="E37" s="18" t="n">
+      <c r="E38" s="18" t="n">
         <v>46305</v>
       </c>
-      <c r="F37" s="17" t="n">
+      <c r="F38" s="17" t="n">
         <v>5</v>
       </c>
-      <c r="G37" s="6" t="inlineStr">
+      <c r="G38" s="6" t="inlineStr">
         <is>
           <t>20AB → 20C</t>
         </is>
       </c>
-      <c r="H37" s="20" t="n">
+      <c r="H38" s="20" t="n">
         <v>46303.54166666666</v>
       </c>
-      <c r="I37" s="20" t="n">
+      <c r="I38" s="20" t="n">
         <v>46304.54166666666</v>
       </c>
-      <c r="J37" s="20" t="n">
+      <c r="J38" s="20" t="n">
         <v>46305.58333333334</v>
       </c>
-      <c r="K37" s="26">
-        <f>(I37-H37)*24</f>
-        <v/>
-      </c>
-      <c r="L37" s="26">
-        <f>(J37-I37)*24</f>
-        <v/>
-      </c>
-      <c r="M37" s="17" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N37" s="17" t="inlineStr">
+      <c r="K38" s="26">
+        <f>(I38-H38)*24</f>
+        <v/>
+      </c>
+      <c r="L38" s="26">
+        <f>(J38-I38)*24</f>
+        <v/>
+      </c>
+      <c r="M38" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N38" s="17" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O37" s="17" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>20C</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>STARSHIP AQUILA</t>
-        </is>
-      </c>
-      <c r="C38" s="23" t="n">
-        <v>565</v>
-      </c>
-      <c r="D38" s="10" t="n">
-        <v>46303</v>
-      </c>
-      <c r="E38" s="10" t="n">
-        <v>46306</v>
-      </c>
-      <c r="F38" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G38" s="5" t="inlineStr">
-        <is>
-          <t>20C</t>
-        </is>
-      </c>
-      <c r="H38" s="11" t="n">
-        <v>46304.91666666666</v>
-      </c>
-      <c r="I38" s="11" t="n">
-        <v>46305.58333333334</v>
-      </c>
-      <c r="J38" s="11" t="n">
-        <v>46307.08333333334</v>
-      </c>
-      <c r="K38" s="24">
-        <f>(I38-H38)*24</f>
-        <v/>
-      </c>
-      <c r="L38" s="24">
-        <f>(J38-I38)*24</f>
-        <v/>
-      </c>
-      <c r="M38" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N38" s="23" t="inlineStr"/>
-      <c r="O38" s="23" t="inlineStr">
+      <c r="O38" s="17" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -22518,34 +22786,34 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 277</t>
+          <t>STARSHIP AQUILA</t>
         </is>
       </c>
       <c r="C39" s="23" t="n">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>46305</v>
+        <v>46303</v>
       </c>
       <c r="E39" s="10" t="n">
-        <v>46309</v>
+        <v>46306</v>
       </c>
       <c r="F39" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G39" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20B → 20C</t>
+        <v>4</v>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
         </is>
       </c>
       <c r="H39" s="11" t="n">
-        <v>46307.875</v>
+        <v>46304.91666666666</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>46308.25</v>
+        <v>46305.58333333334</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>46309.66666666666</v>
+        <v>46307.08333333334</v>
       </c>
       <c r="K39" s="24">
         <f>(I39-H39)*24</f>
@@ -22575,34 +22843,34 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 173</t>
+          <t>WAN HAI 277</t>
         </is>
       </c>
       <c r="C40" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D40" s="10" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="E40" s="10" t="n">
         <v>46309</v>
       </c>
       <c r="F40" s="23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>20B → 20C</t>
+          <t>20F → 20B → 20C</t>
         </is>
       </c>
       <c r="H40" s="11" t="n">
-        <v>46309.04166666666</v>
+        <v>46307.875</v>
       </c>
       <c r="I40" s="11" t="n">
+        <v>46308.25</v>
+      </c>
+      <c r="J40" s="11" t="n">
         <v>46309.66666666666</v>
-      </c>
-      <c r="J40" s="11" t="n">
-        <v>46310.29166666666</v>
       </c>
       <c r="K40" s="24">
         <f>(I40-H40)*24</f>
@@ -22632,34 +22900,34 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 175</t>
+          <t>WAN HAI 173</t>
         </is>
       </c>
       <c r="C41" s="23" t="n">
         <v>565</v>
       </c>
       <c r="D41" s="10" t="n">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="E41" s="10" t="n">
-        <v>46311</v>
+        <v>46309</v>
       </c>
       <c r="F41" s="23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>20D → 20C</t>
+          <t>20B → 20C</t>
         </is>
       </c>
       <c r="H41" s="11" t="n">
-        <v>46309.875</v>
+        <v>46309.04166666666</v>
       </c>
       <c r="I41" s="11" t="n">
+        <v>46309.66666666666</v>
+      </c>
+      <c r="J41" s="11" t="n">
         <v>46310.29166666666</v>
-      </c>
-      <c r="J41" s="11" t="n">
-        <v>46311.625</v>
       </c>
       <c r="K41" s="24">
         <f>(I41-H41)*24</f>
@@ -22689,34 +22957,34 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>LITTLE DOLPHIN</t>
+          <t>WAN HAI 175</t>
         </is>
       </c>
       <c r="C42" s="23" t="n">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D42" s="10" t="n">
-        <v>46310</v>
+        <v>46308</v>
       </c>
       <c r="E42" s="10" t="n">
-        <v>46313</v>
+        <v>46311</v>
       </c>
       <c r="F42" s="23" t="n">
         <v>4</v>
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>20B → 20C</t>
+          <t>20D → 20C</t>
         </is>
       </c>
       <c r="H42" s="11" t="n">
-        <v>46312.04166666666</v>
+        <v>46309.875</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>46312.33333333334</v>
+        <v>46310.29166666666</v>
       </c>
       <c r="J42" s="11" t="n">
-        <v>46313.66666666666</v>
+        <v>46311.625</v>
       </c>
       <c r="K42" s="24">
         <f>(I42-H42)*24</f>
@@ -22746,17 +23014,17 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>MILLENNIUM BRIGHT</t>
+          <t>LITTLE DOLPHIN</t>
         </is>
       </c>
       <c r="C43" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>46293</v>
+        <v>46310</v>
       </c>
       <c r="E43" s="10" t="n">
-        <v>46315</v>
+        <v>46313</v>
       </c>
       <c r="F43" s="23" t="n">
         <v>4</v>
@@ -22767,13 +23035,13 @@
         </is>
       </c>
       <c r="H43" s="11" t="n">
-        <v>46314.58333333334</v>
+        <v>46312.04166666666</v>
       </c>
       <c r="I43" s="11" t="n">
-        <v>46314.58333333334</v>
+        <v>46312.33333333334</v>
       </c>
       <c r="J43" s="11" t="n">
-        <v>46315.5</v>
+        <v>46313.66666666666</v>
       </c>
       <c r="K43" s="24">
         <f>(I43-H43)*24</f>
@@ -22803,34 +23071,34 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>CAPE FAWLEY</t>
+          <t>MILLENNIUM BRIGHT</t>
         </is>
       </c>
       <c r="C44" s="23" t="n">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="D44" s="10" t="n">
         <v>46293</v>
       </c>
       <c r="E44" s="10" t="n">
-        <v>46318</v>
+        <v>46315</v>
       </c>
       <c r="F44" s="23" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20C → 20AB → 20C</t>
+          <t>20B → 20C</t>
         </is>
       </c>
       <c r="H44" s="11" t="n">
-        <v>46316.45833333334</v>
+        <v>46314.58333333334</v>
       </c>
       <c r="I44" s="11" t="n">
-        <v>46316.5</v>
+        <v>46314.58333333334</v>
       </c>
       <c r="J44" s="11" t="n">
-        <v>46318.5</v>
+        <v>46315.5</v>
       </c>
       <c r="K44" s="24">
         <f>(I44-H44)*24</f>
@@ -22846,9 +23114,10 @@
         </is>
       </c>
       <c r="N44" s="23" t="inlineStr"/>
-      <c r="O44" s="23">
-        <f>IF(J44&lt;=$B$3,"Sailed",IF(I44&lt;=$B$3,"Alongside",IF(H44&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O44" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -22859,34 +23128,34 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>HORAI BRIDGE</t>
+          <t>CAPE FAWLEY</t>
         </is>
       </c>
       <c r="C45" s="23" t="n">
-        <v>564</v>
+        <v>558</v>
       </c>
       <c r="D45" s="10" t="n">
-        <v>46316</v>
+        <v>46293</v>
       </c>
       <c r="E45" s="10" t="n">
         <v>46318</v>
       </c>
       <c r="F45" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G45" s="5" t="inlineStr">
-        <is>
-          <t>20C</t>
+        <v>12</v>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20C → 20AB → 20C</t>
         </is>
       </c>
       <c r="H45" s="11" t="n">
-        <v>46318.04166666666</v>
+        <v>46316.45833333334</v>
       </c>
       <c r="I45" s="11" t="n">
+        <v>46316.5</v>
+      </c>
+      <c r="J45" s="11" t="n">
         <v>46318.5</v>
-      </c>
-      <c r="J45" s="11" t="n">
-        <v>46319.625</v>
       </c>
       <c r="K45" s="24">
         <f>(I45-H45)*24</f>
@@ -22902,9 +23171,10 @@
         </is>
       </c>
       <c r="N45" s="23" t="inlineStr"/>
-      <c r="O45" s="23">
-        <f>IF(J45&lt;=$B$3,"Sailed",IF(I45&lt;=$B$3,"Alongside",IF(H45&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O45" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -22915,20 +23185,20 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE MIMOSA</t>
+          <t>HORAI BRIDGE</t>
         </is>
       </c>
       <c r="C46" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D46" s="10" t="n">
-        <v>46317</v>
+        <v>46316</v>
       </c>
       <c r="E46" s="10" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="F46" s="23" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
@@ -22936,13 +23206,13 @@
         </is>
       </c>
       <c r="H46" s="11" t="n">
-        <v>46318.70833333334</v>
+        <v>46318.04166666666</v>
       </c>
       <c r="I46" s="11" t="n">
+        <v>46318.5</v>
+      </c>
+      <c r="J46" s="11" t="n">
         <v>46319.625</v>
-      </c>
-      <c r="J46" s="11" t="n">
-        <v>46321.125</v>
       </c>
       <c r="K46" s="24">
         <f>(I46-H46)*24</f>
@@ -22964,114 +23234,113 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="27" t="inlineStr">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>SAWASDEE MIMOSA</t>
+        </is>
+      </c>
+      <c r="C47" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D47" s="10" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E47" s="10" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F47" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="H47" s="11" t="n">
+        <v>46318.70833333334</v>
+      </c>
+      <c r="I47" s="11" t="n">
+        <v>46319.625</v>
+      </c>
+      <c r="J47" s="11" t="n">
+        <v>46321.125</v>
+      </c>
+      <c r="K47" s="24">
+        <f>(I47-H47)*24</f>
+        <v/>
+      </c>
+      <c r="L47" s="24">
+        <f>(J47-I47)*24</f>
+        <v/>
+      </c>
+      <c r="M47" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N47" s="23" t="inlineStr"/>
+      <c r="O47" s="23">
+        <f>IF(J47&lt;=$B$3,"Sailed",IF(I47&lt;=$B$3,"Alongside",IF(H47&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="27" t="inlineStr">
         <is>
           <t>20D</t>
         </is>
       </c>
-      <c r="B47" s="27" t="inlineStr">
+      <c r="B48" s="27" t="inlineStr">
         <is>
           <t>HARI BHUM (Barge)</t>
         </is>
       </c>
-      <c r="C47" s="28" t="n">
+      <c r="C48" s="28" t="n">
         <v>259</v>
       </c>
-      <c r="D47" s="29" t="n">
+      <c r="D48" s="29" t="n">
         <v>46297</v>
       </c>
-      <c r="E47" s="29" t="n">
+      <c r="E48" s="29" t="n">
         <v>46298</v>
       </c>
-      <c r="F47" s="28" t="n">
+      <c r="F48" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="G47" s="33" t="inlineStr">
+      <c r="G48" s="33" t="inlineStr">
         <is>
           <t>20D</t>
         </is>
       </c>
-      <c r="H47" s="31" t="n">
+      <c r="H48" s="31" t="n">
         <v>46298.20833333334</v>
       </c>
-      <c r="I47" s="31" t="n">
+      <c r="I48" s="31" t="n">
         <v>46298.29166666666</v>
       </c>
-      <c r="J47" s="31" t="n">
+      <c r="J48" s="31" t="n">
         <v>46298.66666666666</v>
       </c>
-      <c r="K47" s="32">
-        <f>(I47-H47)*24</f>
-        <v/>
-      </c>
-      <c r="L47" s="32">
-        <f>(J47-I47)*24</f>
-        <v/>
-      </c>
-      <c r="M47" s="28" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N47" s="28" t="inlineStr"/>
-      <c r="O47" s="28" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
-        <is>
-          <t>20D</t>
-        </is>
-      </c>
-      <c r="B48" s="4" t="inlineStr">
-        <is>
-          <t>HE JIN</t>
-        </is>
-      </c>
-      <c r="C48" s="23" t="n">
-        <v>552</v>
-      </c>
-      <c r="D48" s="10" t="n">
-        <v>46301</v>
-      </c>
-      <c r="E48" s="10" t="n">
-        <v>46305</v>
-      </c>
-      <c r="F48" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G48" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 22A → 20D</t>
-        </is>
-      </c>
-      <c r="H48" s="11" t="n">
-        <v>46304</v>
-      </c>
-      <c r="I48" s="11" t="n">
-        <v>46304</v>
-      </c>
-      <c r="J48" s="11" t="n">
-        <v>46305.54166666666</v>
-      </c>
-      <c r="K48" s="24">
+      <c r="K48" s="32">
         <f>(I48-H48)*24</f>
         <v/>
       </c>
-      <c r="L48" s="24">
+      <c r="L48" s="32">
         <f>(J48-I48)*24</f>
         <v/>
       </c>
-      <c r="M48" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N48" s="23" t="inlineStr"/>
-      <c r="O48" s="23" t="inlineStr">
+      <c r="M48" s="28" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N48" s="28" t="inlineStr"/>
+      <c r="O48" s="28" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -23085,34 +23354,34 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>CUL HAIPHONG</t>
+          <t>HE JIN</t>
         </is>
       </c>
       <c r="C49" s="23" t="n">
-        <v>458</v>
+        <v>552</v>
       </c>
       <c r="D49" s="10" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E49" s="10" t="n">
         <v>46305</v>
       </c>
       <c r="F49" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>20B → 20D</t>
+          <t>20B → 20AB → 22A → 20D</t>
         </is>
       </c>
       <c r="H49" s="11" t="n">
-        <v>46304.83333333334</v>
+        <v>46304</v>
       </c>
       <c r="I49" s="11" t="n">
-        <v>46305.66666666666</v>
+        <v>46304</v>
       </c>
       <c r="J49" s="11" t="n">
-        <v>46306.25</v>
+        <v>46305.54166666666</v>
       </c>
       <c r="K49" s="24">
         <f>(I49-H49)*24</f>
@@ -23124,7 +23393,7 @@
       </c>
       <c r="M49" s="23" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N49" s="23" t="inlineStr"/>
@@ -23142,34 +23411,34 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>INCEDA</t>
+          <t>CUL HAIPHONG</t>
         </is>
       </c>
       <c r="C50" s="23" t="n">
-        <v>564</v>
+        <v>458</v>
       </c>
       <c r="D50" s="10" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E50" s="10" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="F50" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G50" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
+        <v>4</v>
+      </c>
+      <c r="G50" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20D</t>
         </is>
       </c>
       <c r="H50" s="11" t="n">
-        <v>46305.70833333334</v>
+        <v>46304.83333333334</v>
       </c>
       <c r="I50" s="11" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="J50" s="11" t="n">
         <v>46306.25</v>
-      </c>
-      <c r="J50" s="11" t="n">
-        <v>46307.58333333334</v>
       </c>
       <c r="K50" s="24">
         <f>(I50-H50)*24</f>
@@ -23181,7 +23450,7 @@
       </c>
       <c r="M50" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="N50" s="23" t="inlineStr"/>
@@ -23199,34 +23468,34 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE SUNRISE</t>
+          <t>INCEDA</t>
         </is>
       </c>
       <c r="C51" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D51" s="10" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="E51" s="10" t="n">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="F51" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="G51" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20D</t>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H51" s="11" t="n">
-        <v>46307.16666666666</v>
+        <v>46305.70833333334</v>
       </c>
       <c r="I51" s="11" t="n">
-        <v>46307.66666666666</v>
+        <v>46306.25</v>
       </c>
       <c r="J51" s="11" t="n">
-        <v>46309.20833333334</v>
+        <v>46307.58333333334</v>
       </c>
       <c r="K51" s="24">
         <f>(I51-H51)*24</f>
@@ -23256,34 +23525,34 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>KHUNA BHUM</t>
+          <t>SAWASDEE SUNRISE</t>
         </is>
       </c>
       <c r="C52" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D52" s="10" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="F52" s="23" t="n">
         <v>5</v>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20D</t>
+          <t>20F → 20D</t>
         </is>
       </c>
       <c r="H52" s="11" t="n">
-        <v>46308.45833333334</v>
+        <v>46307.16666666666</v>
       </c>
       <c r="I52" s="11" t="n">
+        <v>46307.66666666666</v>
+      </c>
+      <c r="J52" s="11" t="n">
         <v>46309.20833333334</v>
-      </c>
-      <c r="J52" s="11" t="n">
-        <v>46309.91666666666</v>
       </c>
       <c r="K52" s="24">
         <f>(I52-H52)*24</f>
@@ -23295,7 +23564,7 @@
       </c>
       <c r="M52" s="23" t="inlineStr">
         <is>
-          <t>7B</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N52" s="23" t="inlineStr"/>
@@ -23313,34 +23582,34 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>SITC DALIAN</t>
+          <t>KHUNA BHUM</t>
         </is>
       </c>
       <c r="C53" s="23" t="n">
-        <v>470</v>
+        <v>564</v>
       </c>
       <c r="D53" s="10" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E53" s="10" t="n">
         <v>46309</v>
       </c>
-      <c r="E53" s="10" t="n">
-        <v>46310</v>
-      </c>
       <c r="F53" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G53" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
+        <v>5</v>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20D</t>
         </is>
       </c>
       <c r="H53" s="11" t="n">
-        <v>46309.33333333334</v>
+        <v>46308.45833333334</v>
       </c>
       <c r="I53" s="11" t="n">
-        <v>46310.20833333334</v>
+        <v>46309.20833333334</v>
       </c>
       <c r="J53" s="11" t="n">
-        <v>46311.25</v>
+        <v>46309.91666666666</v>
       </c>
       <c r="K53" s="24">
         <f>(I53-H53)*24</f>
@@ -23352,7 +23621,7 @@
       </c>
       <c r="M53" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="N53" s="23" t="inlineStr"/>
@@ -23370,20 +23639,20 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 172</t>
+          <t>SITC DALIAN</t>
         </is>
       </c>
       <c r="C54" s="23" t="n">
-        <v>565</v>
+        <v>470</v>
       </c>
       <c r="D54" s="10" t="n">
         <v>46309</v>
       </c>
       <c r="E54" s="10" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="F54" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
@@ -23391,13 +23660,13 @@
         </is>
       </c>
       <c r="H54" s="11" t="n">
-        <v>46311.04166666666</v>
+        <v>46309.33333333334</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>46311.29166666666</v>
+        <v>46310.20833333334</v>
       </c>
       <c r="J54" s="11" t="n">
-        <v>46312.33333333334</v>
+        <v>46311.25</v>
       </c>
       <c r="K54" s="24">
         <f>(I54-H54)*24</f>
@@ -23427,34 +23696,34 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>PUNNYA NAVEE</t>
+          <t>WAN HAI 172</t>
         </is>
       </c>
       <c r="C55" s="23" t="n">
-        <v>304</v>
+        <v>565</v>
       </c>
       <c r="D55" s="10" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E55" s="10" t="n">
         <v>46311</v>
       </c>
-      <c r="E55" s="10" t="n">
-        <v>46312</v>
-      </c>
       <c r="F55" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G55" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20D</t>
+        <v>3</v>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H55" s="11" t="n">
-        <v>46311.75</v>
+        <v>46311.04166666666</v>
       </c>
       <c r="I55" s="11" t="n">
-        <v>46312.125</v>
+        <v>46311.29166666666</v>
       </c>
       <c r="J55" s="11" t="n">
-        <v>46312.625</v>
+        <v>46312.33333333334</v>
       </c>
       <c r="K55" s="24">
         <f>(I55-H55)*24</f>
@@ -23484,34 +23753,34 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>INFINITY</t>
+          <t>PUNNYA NAVEE</t>
         </is>
       </c>
       <c r="C56" s="23" t="n">
-        <v>565</v>
+        <v>304</v>
       </c>
       <c r="D56" s="10" t="n">
-        <v>46293</v>
+        <v>46311</v>
       </c>
       <c r="E56" s="10" t="n">
-        <v>46313</v>
+        <v>46312</v>
       </c>
       <c r="F56" s="23" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20C → 20D</t>
+          <t>20F → 20D</t>
         </is>
       </c>
       <c r="H56" s="11" t="n">
-        <v>46313</v>
+        <v>46311.75</v>
       </c>
       <c r="I56" s="11" t="n">
-        <v>46313.29166666666</v>
+        <v>46312.125</v>
       </c>
       <c r="J56" s="11" t="n">
-        <v>46314.375</v>
+        <v>46312.625</v>
       </c>
       <c r="K56" s="24">
         <f>(I56-H56)*24</f>
@@ -23541,34 +23810,34 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>KMTC BANGKOK</t>
+          <t>INFINITY</t>
         </is>
       </c>
       <c r="C57" s="23" t="n">
         <v>565</v>
       </c>
       <c r="D57" s="10" t="n">
-        <v>46295</v>
+        <v>46293</v>
       </c>
       <c r="E57" s="10" t="n">
-        <v>46318</v>
+        <v>46313</v>
       </c>
       <c r="F57" s="23" t="n">
         <v>6</v>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20F → 20D</t>
+          <t>20AB → 20C → 20D</t>
         </is>
       </c>
       <c r="H57" s="11" t="n">
-        <v>46320.25</v>
+        <v>46313</v>
       </c>
       <c r="I57" s="11" t="n">
-        <v>46320.25</v>
+        <v>46313.29166666666</v>
       </c>
       <c r="J57" s="11" t="n">
-        <v>46321.5</v>
+        <v>46314.375</v>
       </c>
       <c r="K57" s="24">
         <f>(I57-H57)*24</f>
@@ -23584,165 +23853,160 @@
         </is>
       </c>
       <c r="N57" s="23" t="inlineStr"/>
-      <c r="O57" s="23">
-        <f>IF(J57&lt;=$B$3,"Sailed",IF(I57&lt;=$B$3,"Alongside",IF(H57&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O57" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="27" t="inlineStr">
-        <is>
-          <t>20E</t>
-        </is>
-      </c>
-      <c r="B58" s="27" t="inlineStr">
-        <is>
-          <t>WAN HAI 278</t>
-        </is>
-      </c>
-      <c r="C58" s="28" t="n">
-        <v>564</v>
-      </c>
-      <c r="D58" s="29" t="n">
-        <v>46295</v>
-      </c>
-      <c r="E58" s="29" t="n">
-        <v>46300</v>
-      </c>
-      <c r="F58" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="G58" s="30" t="inlineStr">
-        <is>
-          <t>20F → 20E</t>
-        </is>
-      </c>
-      <c r="H58" s="31" t="n">
-        <v>46297.75</v>
-      </c>
-      <c r="I58" s="31" t="n">
-        <v>46298.41666666666</v>
-      </c>
-      <c r="J58" s="31" t="n">
-        <v>46300.45833333334</v>
-      </c>
-      <c r="K58" s="32">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>PUNNYA NAVEE (barge)</t>
+        </is>
+      </c>
+      <c r="C58" s="23" t="n">
+        <v>304</v>
+      </c>
+      <c r="D58" s="10" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E58" s="10" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F58" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="H58" s="11" t="n">
+        <v>46319.5</v>
+      </c>
+      <c r="I58" s="11" t="n">
+        <v>46319.5</v>
+      </c>
+      <c r="J58" s="11" t="n">
+        <v>46319.95833333334</v>
+      </c>
+      <c r="K58" s="24">
         <f>(I58-H58)*24</f>
         <v/>
       </c>
-      <c r="L58" s="32">
+      <c r="L58" s="24">
         <f>(J58-I58)*24</f>
         <v/>
       </c>
-      <c r="M58" s="28" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N58" s="28" t="inlineStr"/>
-      <c r="O58" s="28" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="M58" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N58" s="23" t="inlineStr"/>
+      <c r="O58" s="23">
+        <f>IF(J58&lt;=$B$3,"Sailed",IF(I58&lt;=$B$3,"Alongside",IF(H58&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="25" t="inlineStr">
-        <is>
-          <t>20E</t>
-        </is>
-      </c>
-      <c r="B59" s="25" t="inlineStr">
-        <is>
-          <t>MTT BANGKOK</t>
-        </is>
-      </c>
-      <c r="C59" s="17" t="n">
-        <v>564</v>
-      </c>
-      <c r="D59" s="18" t="n">
-        <v>46300</v>
-      </c>
-      <c r="E59" s="18" t="n">
-        <v>46316</v>
-      </c>
-      <c r="F59" s="17" t="n">
-        <v>8</v>
-      </c>
-      <c r="G59" s="6" t="inlineStr">
-        <is>
-          <t>20D → 20B → 20E</t>
-        </is>
-      </c>
-      <c r="H59" s="20" t="n">
-        <v>46315.625</v>
-      </c>
-      <c r="I59" s="20" t="n">
-        <v>46315.75</v>
-      </c>
-      <c r="J59" s="20" t="n">
-        <v>46316.83333333334</v>
-      </c>
-      <c r="K59" s="26">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>HARI BHUM (barge)</t>
+        </is>
+      </c>
+      <c r="C59" s="23" t="n">
+        <v>259</v>
+      </c>
+      <c r="D59" s="10" t="n">
+        <v>46319</v>
+      </c>
+      <c r="E59" s="10" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F59" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="H59" s="11" t="n">
+        <v>46319.91666666666</v>
+      </c>
+      <c r="I59" s="11" t="n">
+        <v>46319.91666666666</v>
+      </c>
+      <c r="J59" s="11" t="n">
+        <v>46320.29166666666</v>
+      </c>
+      <c r="K59" s="24">
         <f>(I59-H59)*24</f>
         <v/>
       </c>
-      <c r="L59" s="26">
+      <c r="L59" s="24">
         <f>(J59-I59)*24</f>
         <v/>
       </c>
-      <c r="M59" s="17" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N59" s="17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O59" s="17" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="M59" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N59" s="23" t="inlineStr"/>
+      <c r="O59" s="23">
+        <f>IF(J59&lt;=$B$3,"Sailed",IF(I59&lt;=$B$3,"Alongside",IF(H59&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>20E</t>
+          <t>20D</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>SKY ORION</t>
+          <t>KMTC BANGKOK</t>
         </is>
       </c>
       <c r="C60" s="23" t="n">
         <v>565</v>
       </c>
       <c r="D60" s="10" t="n">
-        <v>46315</v>
+        <v>46295</v>
       </c>
       <c r="E60" s="10" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="F60" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G60" s="5" t="inlineStr">
-        <is>
-          <t>20E</t>
+        <v>7</v>
+      </c>
+      <c r="G60" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20F → 20D</t>
         </is>
       </c>
       <c r="H60" s="11" t="n">
-        <v>46317.04166666666</v>
+        <v>46320.25</v>
       </c>
       <c r="I60" s="11" t="n">
-        <v>46317.54166666666</v>
+        <v>46320.25</v>
       </c>
       <c r="J60" s="11" t="n">
-        <v>46319.04166666666</v>
+        <v>46321.5</v>
       </c>
       <c r="K60" s="24">
         <f>(I60-H60)*24</f>
@@ -23764,169 +24028,175 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="4" t="inlineStr">
+      <c r="A61" s="27" t="inlineStr">
         <is>
           <t>20E</t>
         </is>
       </c>
-      <c r="B61" s="4" t="inlineStr">
-        <is>
-          <t>YM IMAGE</t>
-        </is>
-      </c>
-      <c r="C61" s="23" t="n">
+      <c r="B61" s="27" t="inlineStr">
+        <is>
+          <t>WAN HAI 278</t>
+        </is>
+      </c>
+      <c r="C61" s="28" t="n">
+        <v>564</v>
+      </c>
+      <c r="D61" s="29" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E61" s="29" t="n">
+        <v>46300</v>
+      </c>
+      <c r="F61" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="G61" s="30" t="inlineStr">
+        <is>
+          <t>20F → 20E</t>
+        </is>
+      </c>
+      <c r="H61" s="31" t="n">
+        <v>46297.75</v>
+      </c>
+      <c r="I61" s="31" t="n">
+        <v>46298.41666666666</v>
+      </c>
+      <c r="J61" s="31" t="n">
+        <v>46300.45833333334</v>
+      </c>
+      <c r="K61" s="32">
+        <f>(I61-H61)*24</f>
+        <v/>
+      </c>
+      <c r="L61" s="32">
+        <f>(J61-I61)*24</f>
+        <v/>
+      </c>
+      <c r="M61" s="28" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N61" s="28" t="inlineStr"/>
+      <c r="O61" s="28" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="25" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B62" s="25" t="inlineStr">
+        <is>
+          <t>MTT BANGKOK</t>
+        </is>
+      </c>
+      <c r="C62" s="17" t="n">
+        <v>564</v>
+      </c>
+      <c r="D62" s="18" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E62" s="18" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F62" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="G62" s="6" t="inlineStr">
+        <is>
+          <t>20D → 20B → 20E</t>
+        </is>
+      </c>
+      <c r="H62" s="20" t="n">
+        <v>46315.625</v>
+      </c>
+      <c r="I62" s="20" t="n">
+        <v>46315.75</v>
+      </c>
+      <c r="J62" s="20" t="n">
+        <v>46316.83333333334</v>
+      </c>
+      <c r="K62" s="26">
+        <f>(I62-H62)*24</f>
+        <v/>
+      </c>
+      <c r="L62" s="26">
+        <f>(J62-I62)*24</f>
+        <v/>
+      </c>
+      <c r="M62" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N62" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O62" s="17" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>SKY ORION</t>
+        </is>
+      </c>
+      <c r="C63" s="23" t="n">
         <v>565</v>
       </c>
-      <c r="D61" s="10" t="n">
-        <v>46317</v>
-      </c>
-      <c r="E61" s="10" t="n">
+      <c r="D63" s="10" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E63" s="10" t="n">
         <v>46318</v>
       </c>
-      <c r="F61" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G61" s="5" t="inlineStr">
+      <c r="F63" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
         <is>
           <t>20E</t>
         </is>
       </c>
-      <c r="H61" s="11" t="n">
-        <v>46318.41666666666</v>
-      </c>
-      <c r="I61" s="11" t="n">
-        <v>46319.125</v>
-      </c>
-      <c r="J61" s="11" t="n">
-        <v>46320.04166666666</v>
-      </c>
-      <c r="K61" s="24">
-        <f>(I61-H61)*24</f>
-        <v/>
-      </c>
-      <c r="L61" s="24">
-        <f>(J61-I61)*24</f>
-        <v/>
-      </c>
-      <c r="M61" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N61" s="23" t="inlineStr"/>
-      <c r="O61" s="23">
-        <f>IF(J61&lt;=$B$3,"Sailed",IF(I61&lt;=$B$3,"Alongside",IF(H61&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="4" t="inlineStr">
-        <is>
-          <t>20E</t>
-        </is>
-      </c>
-      <c r="B62" s="4" t="inlineStr">
-        <is>
-          <t>HEUNG A HOCHIMINH</t>
-        </is>
-      </c>
-      <c r="C62" s="23" t="n">
-        <v>565</v>
-      </c>
-      <c r="D62" s="10" t="n">
-        <v>46317</v>
-      </c>
-      <c r="E62" s="10" t="n">
-        <v>46318</v>
-      </c>
-      <c r="F62" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G62" s="5" t="inlineStr">
-        <is>
-          <t>20E</t>
-        </is>
-      </c>
-      <c r="H62" s="11" t="n">
-        <v>46320.91666666666</v>
-      </c>
-      <c r="I62" s="11" t="n">
-        <v>46321.25</v>
-      </c>
-      <c r="J62" s="11" t="n">
-        <v>46292.58333333334</v>
-      </c>
-      <c r="K62" s="24">
-        <f>(I62-H62)*24</f>
-        <v/>
-      </c>
-      <c r="L62" s="24">
-        <f>(J62-I62)*24</f>
-        <v/>
-      </c>
-      <c r="M62" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N62" s="23" t="inlineStr"/>
-      <c r="O62" s="23">
-        <f>IF(J62&lt;=$B$3,"Sailed",IF(I62&lt;=$B$3,"Alongside",IF(H62&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="27" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="B63" s="27" t="inlineStr">
-        <is>
-          <t>XIN MING ZHOU 98</t>
-        </is>
-      </c>
-      <c r="C63" s="28" t="n">
-        <v>564</v>
-      </c>
-      <c r="D63" s="29" t="n">
-        <v>46297</v>
-      </c>
-      <c r="E63" s="29" t="n">
-        <v>46299</v>
-      </c>
-      <c r="F63" s="28" t="n">
-        <v>3</v>
-      </c>
-      <c r="G63" s="33" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="H63" s="31" t="n">
-        <v>46299.375</v>
-      </c>
-      <c r="I63" s="31" t="n">
-        <v>46299.375</v>
-      </c>
-      <c r="J63" s="31" t="n">
-        <v>46300.375</v>
-      </c>
-      <c r="K63" s="32">
+      <c r="H63" s="11" t="n">
+        <v>46317.04166666666</v>
+      </c>
+      <c r="I63" s="11" t="n">
+        <v>46317.54166666666</v>
+      </c>
+      <c r="J63" s="11" t="n">
+        <v>46319.04166666666</v>
+      </c>
+      <c r="K63" s="24">
         <f>(I63-H63)*24</f>
         <v/>
       </c>
-      <c r="L63" s="32">
+      <c r="L63" s="24">
         <f>(J63-I63)*24</f>
         <v/>
       </c>
-      <c r="M63" s="28" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N63" s="28" t="inlineStr"/>
-      <c r="O63" s="28" t="inlineStr">
+      <c r="M63" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N63" s="23" t="inlineStr"/>
+      <c r="O63" s="23" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -23935,39 +24205,39 @@
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>20F</t>
+          <t>20E</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>XIN AN</t>
+          <t>YM IMAGE</t>
         </is>
       </c>
       <c r="C64" s="23" t="n">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D64" s="10" t="n">
-        <v>46300</v>
+        <v>46317</v>
       </c>
       <c r="E64" s="10" t="n">
-        <v>46304</v>
+        <v>46319</v>
       </c>
       <c r="F64" s="23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>20F</t>
+          <t>20E</t>
         </is>
       </c>
       <c r="H64" s="11" t="n">
-        <v>46302.54166666666</v>
+        <v>46318.25</v>
       </c>
       <c r="I64" s="11" t="n">
-        <v>46302.58333333334</v>
+        <v>46319.125</v>
       </c>
       <c r="J64" s="11" t="n">
-        <v>46304.54166666666</v>
+        <v>46320.04166666666</v>
       </c>
       <c r="K64" s="24">
         <f>(I64-H64)*24</f>
@@ -23983,48 +24253,47 @@
         </is>
       </c>
       <c r="N64" s="23" t="inlineStr"/>
-      <c r="O64" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="O64" s="23">
+        <f>IF(J64&lt;=$B$3,"Sailed",IF(I64&lt;=$B$3,"Alongside",IF(H64&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>20F</t>
+          <t>20E</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE ATLANTIC</t>
+          <t>XIN MING ZHOU 106</t>
         </is>
       </c>
       <c r="C65" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D65" s="10" t="n">
-        <v>46300</v>
+        <v>46317</v>
       </c>
       <c r="E65" s="10" t="n">
-        <v>46306</v>
+        <v>46319</v>
       </c>
       <c r="F65" s="23" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G65" s="6" t="inlineStr">
         <is>
-          <t>20C → 20D → 20F</t>
+          <t>20F → 20E</t>
         </is>
       </c>
       <c r="H65" s="11" t="n">
-        <v>46302.83333333334</v>
+        <v>46320.41666666666</v>
       </c>
       <c r="I65" s="11" t="n">
-        <v>46304.625</v>
+        <v>46320.54166666666</v>
       </c>
       <c r="J65" s="11" t="n">
-        <v>46306.5</v>
+        <v>46321.5</v>
       </c>
       <c r="K65" s="24">
         <f>(I65-H65)*24</f>
@@ -24040,64 +24309,63 @@
         </is>
       </c>
       <c r="N65" s="23" t="inlineStr"/>
-      <c r="O65" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="O65" s="23">
+        <f>IF(J65&lt;=$B$3,"Sailed",IF(I65&lt;=$B$3,"Alongside",IF(H65&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="4" t="inlineStr">
+      <c r="A66" s="27" t="inlineStr">
         <is>
           <t>20F</t>
         </is>
       </c>
-      <c r="B66" s="4" t="inlineStr">
-        <is>
-          <t>JOSCO SHINE</t>
-        </is>
-      </c>
-      <c r="C66" s="23" t="n">
+      <c r="B66" s="27" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 98</t>
+        </is>
+      </c>
+      <c r="C66" s="28" t="n">
         <v>564</v>
       </c>
-      <c r="D66" s="10" t="n">
-        <v>46304</v>
-      </c>
-      <c r="E66" s="10" t="n">
-        <v>46307</v>
-      </c>
-      <c r="F66" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G66" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 20F</t>
-        </is>
-      </c>
-      <c r="H66" s="11" t="n">
-        <v>46307.45833333334</v>
-      </c>
-      <c r="I66" s="11" t="n">
-        <v>46307.625</v>
-      </c>
-      <c r="J66" s="11" t="n">
-        <v>46308.25</v>
-      </c>
-      <c r="K66" s="24">
+      <c r="D66" s="29" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E66" s="29" t="n">
+        <v>46299</v>
+      </c>
+      <c r="F66" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="G66" s="33" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="H66" s="31" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="I66" s="31" t="n">
+        <v>46299.375</v>
+      </c>
+      <c r="J66" s="31" t="n">
+        <v>46300.375</v>
+      </c>
+      <c r="K66" s="32">
         <f>(I66-H66)*24</f>
         <v/>
       </c>
-      <c r="L66" s="24">
+      <c r="L66" s="32">
         <f>(J66-I66)*24</f>
         <v/>
       </c>
-      <c r="M66" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N66" s="23" t="inlineStr"/>
-      <c r="O66" s="23" t="inlineStr">
+      <c r="M66" s="28" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N66" s="28" t="inlineStr"/>
+      <c r="O66" s="28" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -24111,34 +24379,34 @@
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE INCHEON</t>
+          <t>SAWASDEE ATLANTIC</t>
         </is>
       </c>
       <c r="C67" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D67" s="10" t="n">
-        <v>46307</v>
+        <v>46300</v>
       </c>
       <c r="E67" s="10" t="n">
-        <v>46310</v>
+        <v>46306</v>
       </c>
       <c r="F67" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G67" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+        <v>7</v>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>20C → 20D → 20F</t>
         </is>
       </c>
       <c r="H67" s="11" t="n">
-        <v>46308.625</v>
+        <v>46302.83333333334</v>
       </c>
       <c r="I67" s="11" t="n">
-        <v>46309.25</v>
+        <v>46304.625</v>
       </c>
       <c r="J67" s="11" t="n">
-        <v>46311.25</v>
+        <v>46306.5</v>
       </c>
       <c r="K67" s="24">
         <f>(I67-H67)*24</f>
@@ -24168,34 +24436,34 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>INGENUITY</t>
+          <t>JOSCO SHINE</t>
         </is>
       </c>
       <c r="C68" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D68" s="10" t="n">
-        <v>46310</v>
+        <v>46304</v>
       </c>
       <c r="E68" s="10" t="n">
-        <v>46312</v>
+        <v>46307</v>
       </c>
       <c r="F68" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G68" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+        <v>4</v>
+      </c>
+      <c r="G68" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20AB → 20F</t>
         </is>
       </c>
       <c r="H68" s="11" t="n">
-        <v>46311.95833333334</v>
+        <v>46307.45833333334</v>
       </c>
       <c r="I68" s="11" t="n">
-        <v>46312.33333333334</v>
+        <v>46307.625</v>
       </c>
       <c r="J68" s="11" t="n">
-        <v>46313.29166666666</v>
+        <v>46308.25</v>
       </c>
       <c r="K68" s="24">
         <f>(I68-H68)*24</f>
@@ -24225,34 +24493,34 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 108</t>
+          <t>SAWASDEE INCHEON</t>
         </is>
       </c>
       <c r="C69" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D69" s="10" t="n">
+        <v>46307</v>
+      </c>
+      <c r="E69" s="10" t="n">
         <v>46310</v>
       </c>
-      <c r="E69" s="10" t="n">
-        <v>46314</v>
-      </c>
       <c r="F69" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G69" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20F</t>
+        <v>4</v>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
         </is>
       </c>
       <c r="H69" s="11" t="n">
-        <v>46312.41666666666</v>
+        <v>46308.625</v>
       </c>
       <c r="I69" s="11" t="n">
-        <v>46313.33333333334</v>
+        <v>46309.25</v>
       </c>
       <c r="J69" s="11" t="n">
-        <v>46314.5</v>
+        <v>46311.25</v>
       </c>
       <c r="K69" s="24">
         <f>(I69-H69)*24</f>
@@ -24282,17 +24550,17 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>RENOWN</t>
+          <t>INGENUITY</t>
         </is>
       </c>
       <c r="C70" s="23" t="n">
-        <v>458</v>
+        <v>564</v>
       </c>
       <c r="D70" s="10" t="n">
-        <v>46315</v>
+        <v>46310</v>
       </c>
       <c r="E70" s="10" t="n">
-        <v>46317</v>
+        <v>46312</v>
       </c>
       <c r="F70" s="23" t="n">
         <v>3</v>
@@ -24303,13 +24571,13 @@
         </is>
       </c>
       <c r="H70" s="11" t="n">
-        <v>46315.75</v>
+        <v>46311.95833333334</v>
       </c>
       <c r="I70" s="11" t="n">
-        <v>46317.41666666666</v>
+        <v>46312.33333333334</v>
       </c>
       <c r="J70" s="11" t="n">
-        <v>46318.375</v>
+        <v>46313.29166666666</v>
       </c>
       <c r="K70" s="24">
         <f>(I70-H70)*24</f>
@@ -24339,34 +24607,34 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 272</t>
+          <t>XIN MING ZHOU 108</t>
         </is>
       </c>
       <c r="C71" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D71" s="10" t="n">
-        <v>46315</v>
+        <v>46310</v>
       </c>
       <c r="E71" s="10" t="n">
-        <v>46318</v>
+        <v>46314</v>
       </c>
       <c r="F71" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G71" s="6" t="inlineStr">
         <is>
-          <t>22A → 20F</t>
+          <t>20B → 20F</t>
         </is>
       </c>
       <c r="H71" s="11" t="n">
-        <v>46318.375</v>
+        <v>46312.41666666666</v>
       </c>
       <c r="I71" s="11" t="n">
-        <v>46318.375</v>
+        <v>46313.33333333334</v>
       </c>
       <c r="J71" s="11" t="n">
-        <v>46319.58333333334</v>
+        <v>46314.5</v>
       </c>
       <c r="K71" s="24">
         <f>(I71-H71)*24</f>
@@ -24382,9 +24650,10 @@
         </is>
       </c>
       <c r="N71" s="23" t="inlineStr"/>
-      <c r="O71" s="23">
-        <f>IF(J71&lt;=$B$3,"Sailed",IF(I71&lt;=$B$3,"Alongside",IF(H71&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O71" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -24395,20 +24664,20 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 106</t>
+          <t>RENOWN</t>
         </is>
       </c>
       <c r="C72" s="23" t="n">
-        <v>564</v>
+        <v>458</v>
       </c>
       <c r="D72" s="10" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E72" s="10" t="n">
         <v>46317</v>
       </c>
-      <c r="E72" s="10" t="n">
-        <v>46318</v>
-      </c>
       <c r="F72" s="23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
@@ -24416,13 +24685,13 @@
         </is>
       </c>
       <c r="H72" s="11" t="n">
-        <v>46320.41666666666</v>
+        <v>46315.75</v>
       </c>
       <c r="I72" s="11" t="n">
-        <v>46320.54166666666</v>
+        <v>46317.41666666666</v>
       </c>
       <c r="J72" s="11" t="n">
-        <v>46321.5</v>
+        <v>46318.375</v>
       </c>
       <c r="K72" s="24">
         <f>(I72-H72)*24</f>
@@ -24438,22 +24707,839 @@
         </is>
       </c>
       <c r="N72" s="23" t="inlineStr"/>
-      <c r="O72" s="23">
-        <f>IF(J72&lt;=$B$3,"Sailed",IF(I72&lt;=$B$3,"Alongside",IF(H72&lt;=$B$3,"At anchorage","Expected")))</f>
+      <c r="O72" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>WAN HAI 272</t>
+        </is>
+      </c>
+      <c r="C73" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D73" s="10" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E73" s="10" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F73" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
+          <t>22A → 20F</t>
+        </is>
+      </c>
+      <c r="H73" s="11" t="n">
+        <v>46318.375</v>
+      </c>
+      <c r="I73" s="11" t="n">
+        <v>46318.375</v>
+      </c>
+      <c r="J73" s="11" t="n">
+        <v>46319.58333333334</v>
+      </c>
+      <c r="K73" s="24">
+        <f>(I73-H73)*24</f>
+        <v/>
+      </c>
+      <c r="L73" s="24">
+        <f>(J73-I73)*24</f>
+        <v/>
+      </c>
+      <c r="M73" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N73" s="23" t="inlineStr"/>
+      <c r="O73" s="23">
+        <f>IF(J73&lt;=$B$3,"Sailed",IF(I73&lt;=$B$3,"Alongside",IF(H73&lt;=$B$3,"At anchorage","Expected")))</f>
         <v/>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>67 vessels in total. Orange cells: marked on sheet, or the vessel changed berth.</t>
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>HEUNG A HOCHIMINH</t>
+        </is>
+      </c>
+      <c r="C74" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D74" s="10" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E74" s="10" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F74" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G74" s="6" t="inlineStr">
+        <is>
+          <t>20E → 20F</t>
+        </is>
+      </c>
+      <c r="H74" s="11" t="n">
+        <v>46320.58333333334</v>
+      </c>
+      <c r="I74" s="11" t="n">
+        <v>46320.625</v>
+      </c>
+      <c r="J74" s="11" t="n">
+        <v>46292.16666666666</v>
+      </c>
+      <c r="K74" s="24">
+        <f>(I74-H74)*24</f>
+        <v/>
+      </c>
+      <c r="L74" s="24">
+        <f>(J74-I74)*24</f>
+        <v/>
+      </c>
+      <c r="M74" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N74" s="23" t="inlineStr"/>
+      <c r="O74" s="23">
+        <f>IF(J74&lt;=$B$3,"Sailed",IF(I74&lt;=$B$3,"Alongside",IF(H74&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>69 vessels in total. Orange cells: marked on sheet, or the vessel changed berth.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:O72"/>
+  <autoFilter ref="A5:O74"/>
   <mergeCells count="1">
     <mergeCell ref="A2:O2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 24 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Waiting for Berth (h)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>KMTC GWANGYANG</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>46317.54166666666</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>46318.58333333334</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>46320.04166666666</v>
+      </c>
+      <c r="G4" s="24">
+        <f>(E4-D4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="24">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>KANWAY FORTUNE</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46320.20833333334</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46320.625</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46321.66666666666</v>
+      </c>
+      <c r="G5" s="24">
+        <f>(E5-D5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="24">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>CA MANILA</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>548</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46317.75</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46318.54166666666</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46320</v>
+      </c>
+      <c r="G6" s="24">
+        <f>(E6-D6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="24">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>ASL TAIPEIS</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46320</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46320.16666666666</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46321.125</v>
+      </c>
+      <c r="G7" s="24">
+        <f>(E7-D7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="24">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>ZHONG GU BEI HAI</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>561</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>46321.83333333334</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>46292.20833333334</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>46293.58333333334</v>
+      </c>
+      <c r="G8" s="24">
+        <f>(E8-D8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="24">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>HORAI BRIDGE</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>46318.04166666666</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>46318.5</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>46319.625</v>
+      </c>
+      <c r="G9" s="24">
+        <f>(E9-D9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="24">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE MIMOSA</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>46318.70833333334</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>46319.625</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>46321.125</v>
+      </c>
+      <c r="G10" s="24">
+        <f>(E10-D10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="24">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>XIN AN</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>46321.75</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>46292.16666666666</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>46293.20833333334</v>
+      </c>
+      <c r="G11" s="24">
+        <f>(E11-D11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="24">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J11" s="23" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>PUNNYA NAVEE (barge)</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>304</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>46319.5</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>46319.5</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>46319.95833333334</v>
+      </c>
+      <c r="G12" s="24">
+        <f>(E12-D12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="24">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J12" s="23" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>HARI BHUM (barge)</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>259</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>46319.91666666666</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>46319.91666666666</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>46320.29166666666</v>
+      </c>
+      <c r="G13" s="24">
+        <f>(E13-D13)*24</f>
+        <v/>
+      </c>
+      <c r="H13" s="24">
+        <f>(F13-E13)*24</f>
+        <v/>
+      </c>
+      <c r="I13" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J13" s="23" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>KMTC BANGKOK</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>46320.25</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>46320.25</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>46321.5</v>
+      </c>
+      <c r="G14" s="24">
+        <f>(E14-D14)*24</f>
+        <v/>
+      </c>
+      <c r="H14" s="24">
+        <f>(F14-E14)*24</f>
+        <v/>
+      </c>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J14" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>YM IMAGE</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>46318.25</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>46319.125</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>46320.04166666666</v>
+      </c>
+      <c r="G15" s="24">
+        <f>(E15-D15)*24</f>
+        <v/>
+      </c>
+      <c r="H15" s="24">
+        <f>(F15-E15)*24</f>
+        <v/>
+      </c>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J15" s="23" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 106</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>46320.41666666666</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>46320.54166666666</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>46321.5</v>
+      </c>
+      <c r="G16" s="24">
+        <f>(E16-D16)*24</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>(F16-E16)*24</f>
+        <v/>
+      </c>
+      <c r="I16" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J16" s="23" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 272</t>
+        </is>
+      </c>
+      <c r="C17" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>46318.375</v>
+      </c>
+      <c r="E17" s="11" t="n">
+        <v>46318.375</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>46319.58333333334</v>
+      </c>
+      <c r="G17" s="24">
+        <f>(E17-D17)*24</f>
+        <v/>
+      </c>
+      <c r="H17" s="24">
+        <f>(F17-E17)*24</f>
+        <v/>
+      </c>
+      <c r="I17" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J17" s="23" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>HEUNG A HOCHIMINH</t>
+        </is>
+      </c>
+      <c r="C18" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>46320.58333333334</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>46320.625</v>
+      </c>
+      <c r="F18" s="11" t="n">
+        <v>46292.16666666666</v>
+      </c>
+      <c r="G18" s="24">
+        <f>(E18-D18)*24</f>
+        <v/>
+      </c>
+      <c r="H18" s="24">
+        <f>(F18-E18)*24</f>
+        <v/>
+      </c>
+      <c r="I18" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J18" s="23" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="34" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G22" s="35" t="n"/>
+      <c r="H22" s="35" t="n"/>
+      <c r="I22" s="35" t="n"/>
+      <c r="J22" s="36" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="39" t="inlineStr">
+        <is>
+          <t>No notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F22:J22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 25 Oct 2026 ship movement data, Excel files and history continuity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAT_Berth_Window.xlsx
+++ b/PAT_Berth_Window.xlsx
@@ -37,10 +37,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22 Oct 2026" sheetId="28" state="visible" r:id="rId28"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23 Oct 2026" sheetId="29" state="visible" r:id="rId29"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24 Oct 2026" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25 Oct 2026" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Berth Notices'!$A$4:$G$57</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$O$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Vessel List by Berth'!$A$5:$O$77</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -675,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB77"/>
+  <dimension ref="A1:AC80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -706,6 +707,7 @@
     <col width="44" customWidth="1" min="26" max="26"/>
     <col width="44" customWidth="1" min="27" max="27"/>
     <col width="44" customWidth="1" min="28" max="28"/>
+    <col width="44" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -861,6 +863,11 @@
       <c r="AB4" s="3" t="inlineStr">
         <is>
           <t>24 Oct 2026</t>
+        </is>
+      </c>
+      <c r="AC4" s="3" t="inlineStr">
+        <is>
+          <t>25 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -929,6 +936,7 @@
       <c r="Z5" s="5" t="inlineStr"/>
       <c r="AA5" s="5" t="inlineStr"/>
       <c r="AB5" s="5" t="inlineStr"/>
+      <c r="AC5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -979,6 +987,7 @@
       <c r="Z6" s="5" t="inlineStr"/>
       <c r="AA6" s="5" t="inlineStr"/>
       <c r="AB6" s="5" t="inlineStr"/>
+      <c r="AC6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1041,6 +1050,11 @@
           <t>expected · 20AB (ETD 25/02→25/01)</t>
         </is>
       </c>
+      <c r="AC7" s="5" t="inlineStr">
+        <is>
+          <t>sailed (25/01)</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -1099,6 +1113,7 @@
       <c r="Z8" s="5" t="inlineStr"/>
       <c r="AA8" s="5" t="inlineStr"/>
       <c r="AB8" s="5" t="inlineStr"/>
+      <c r="AC8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -1169,6 +1184,7 @@
       <c r="Z9" s="5" t="inlineStr"/>
       <c r="AA9" s="5" t="inlineStr"/>
       <c r="AB9" s="5" t="inlineStr"/>
+      <c r="AC9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -1227,6 +1243,7 @@
       <c r="Z10" s="5" t="inlineStr"/>
       <c r="AA10" s="5" t="inlineStr"/>
       <c r="AB10" s="5" t="inlineStr"/>
+      <c r="AC10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1293,6 +1310,7 @@
       </c>
       <c r="AA11" s="5" t="inlineStr"/>
       <c r="AB11" s="5" t="inlineStr"/>
+      <c r="AC11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1355,6 +1373,7 @@
       <c r="Z12" s="5" t="inlineStr"/>
       <c r="AA12" s="5" t="inlineStr"/>
       <c r="AB12" s="5" t="inlineStr"/>
+      <c r="AC12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1437,6 +1456,7 @@
       </c>
       <c r="AA13" s="5" t="inlineStr"/>
       <c r="AB13" s="5" t="inlineStr"/>
+      <c r="AC13" s="5" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1535,6 +1555,7 @@
           <t>sailed (23/12)</t>
         </is>
       </c>
+      <c r="AC14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1601,6 +1622,11 @@
       <c r="Z15" s="5" t="inlineStr"/>
       <c r="AA15" s="5" t="inlineStr"/>
       <c r="AB15" s="5" t="inlineStr"/>
+      <c r="AC15" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C (new call: ETA 28/03, ETD 29/06)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1671,6 +1697,7 @@
       <c r="Z16" s="5" t="inlineStr"/>
       <c r="AA16" s="5" t="inlineStr"/>
       <c r="AB16" s="5" t="inlineStr"/>
+      <c r="AC16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1773,6 +1800,7 @@
           <t>sailed (23/16)</t>
         </is>
       </c>
+      <c r="AC17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1835,6 +1863,11 @@
           <t>expected · 20D</t>
         </is>
       </c>
+      <c r="AC18" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20D (ETD 26/12→26/13)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1897,6 +1930,7 @@
       <c r="Z19" s="5" t="inlineStr"/>
       <c r="AA19" s="5" t="inlineStr"/>
       <c r="AB19" s="5" t="inlineStr"/>
+      <c r="AC19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1965,6 +1999,11 @@
       <c r="AB20" s="6" t="inlineStr">
         <is>
           <t>expected · 20B (ETA 26/14→26/20, P.B 26/14→27/05, ETD 28/03→28/14)</t>
+        </is>
+      </c>
+      <c r="AC20" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20C (moved from 20B; ETA 26/20→26/15, P.B 27/05→26/15, ETD 28/14→28/03)</t>
         </is>
       </c>
     </row>
@@ -2025,6 +2064,7 @@
       <c r="Z21" s="5" t="inlineStr"/>
       <c r="AA21" s="5" t="inlineStr"/>
       <c r="AB21" s="5" t="inlineStr"/>
+      <c r="AC21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -2079,6 +2119,7 @@
       <c r="Z22" s="5" t="inlineStr"/>
       <c r="AA22" s="5" t="inlineStr"/>
       <c r="AB22" s="5" t="inlineStr"/>
+      <c r="AC22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -2145,6 +2186,7 @@
       <c r="Z23" s="5" t="inlineStr"/>
       <c r="AA23" s="5" t="inlineStr"/>
       <c r="AB23" s="5" t="inlineStr"/>
+      <c r="AC23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -2207,6 +2249,7 @@
       <c r="Z24" s="5" t="inlineStr"/>
       <c r="AA24" s="5" t="inlineStr"/>
       <c r="AB24" s="5" t="inlineStr"/>
+      <c r="AC24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -2253,6 +2296,7 @@
       <c r="Z25" s="5" t="inlineStr"/>
       <c r="AA25" s="5" t="inlineStr"/>
       <c r="AB25" s="5" t="inlineStr"/>
+      <c r="AC25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -2303,6 +2347,7 @@
       <c r="Z26" s="5" t="inlineStr"/>
       <c r="AA26" s="5" t="inlineStr"/>
       <c r="AB26" s="5" t="inlineStr"/>
+      <c r="AC26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -2365,6 +2410,7 @@
       <c r="Z27" s="5" t="inlineStr"/>
       <c r="AA27" s="5" t="inlineStr"/>
       <c r="AB27" s="5" t="inlineStr"/>
+      <c r="AC27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2423,6 +2469,11 @@
       <c r="Z28" s="5" t="inlineStr"/>
       <c r="AA28" s="5" t="inlineStr"/>
       <c r="AB28" s="5" t="inlineStr"/>
+      <c r="AC28" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20AB (new call: ETA 27/05, ETD 28/13)</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2505,6 +2556,7 @@
           <t>sailed (23/13)</t>
         </is>
       </c>
+      <c r="AC29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -2571,6 +2623,7 @@
       <c r="Z30" s="5" t="inlineStr"/>
       <c r="AA30" s="5" t="inlineStr"/>
       <c r="AB30" s="5" t="inlineStr"/>
+      <c r="AC30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2645,6 +2698,7 @@
       </c>
       <c r="AA31" s="5" t="inlineStr"/>
       <c r="AB31" s="5" t="inlineStr"/>
+      <c r="AC31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2703,6 +2757,11 @@
       <c r="Z32" s="5" t="inlineStr"/>
       <c r="AA32" s="5" t="inlineStr"/>
       <c r="AB32" s="5" t="inlineStr"/>
+      <c r="AC32" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20B (moved from 20C)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2757,6 +2816,7 @@
       <c r="Z33" s="5" t="inlineStr"/>
       <c r="AA33" s="5" t="inlineStr"/>
       <c r="AB33" s="5" t="inlineStr"/>
+      <c r="AC33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2815,6 +2875,7 @@
       <c r="Z34" s="5" t="inlineStr"/>
       <c r="AA34" s="5" t="inlineStr"/>
       <c r="AB34" s="5" t="inlineStr"/>
+      <c r="AC34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2873,6 +2934,7 @@
       <c r="Z35" s="5" t="inlineStr"/>
       <c r="AA35" s="5" t="inlineStr"/>
       <c r="AB35" s="5" t="inlineStr"/>
+      <c r="AC35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2927,6 +2989,7 @@
       <c r="Z36" s="5" t="inlineStr"/>
       <c r="AA36" s="5" t="inlineStr"/>
       <c r="AB36" s="5" t="inlineStr"/>
+      <c r="AC36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2993,6 +3056,11 @@
           <t>expected · 20AB (ETD 27/03→26/16)</t>
         </is>
       </c>
+      <c r="AC37" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20AB (ETA 25/05→25/06)</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -3051,6 +3119,7 @@
       <c r="Z38" s="5" t="inlineStr"/>
       <c r="AA38" s="5" t="inlineStr"/>
       <c r="AB38" s="5" t="inlineStr"/>
+      <c r="AC38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -3105,6 +3174,7 @@
       <c r="Z39" s="5" t="inlineStr"/>
       <c r="AA39" s="5" t="inlineStr"/>
       <c r="AB39" s="5" t="inlineStr"/>
+      <c r="AC39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -3159,6 +3229,7 @@
       <c r="Z40" s="5" t="inlineStr"/>
       <c r="AA40" s="5" t="inlineStr"/>
       <c r="AB40" s="5" t="inlineStr"/>
+      <c r="AC40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -3217,6 +3288,7 @@
       <c r="Z41" s="5" t="inlineStr"/>
       <c r="AA41" s="5" t="inlineStr"/>
       <c r="AB41" s="5" t="inlineStr"/>
+      <c r="AC41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -3271,6 +3343,7 @@
       <c r="Z42" s="5" t="inlineStr"/>
       <c r="AA42" s="5" t="inlineStr"/>
       <c r="AB42" s="5" t="inlineStr"/>
+      <c r="AC42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -3329,6 +3402,7 @@
       <c r="Z43" s="5" t="inlineStr"/>
       <c r="AA43" s="5" t="inlineStr"/>
       <c r="AB43" s="5" t="inlineStr"/>
+      <c r="AC43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -3387,6 +3461,7 @@
       <c r="Z44" s="5" t="inlineStr"/>
       <c r="AA44" s="5" t="inlineStr"/>
       <c r="AB44" s="5" t="inlineStr"/>
+      <c r="AC44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -3441,6 +3516,7 @@
       <c r="Z45" s="5" t="inlineStr"/>
       <c r="AA45" s="5" t="inlineStr"/>
       <c r="AB45" s="5" t="inlineStr"/>
+      <c r="AC45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -3503,6 +3579,7 @@
       <c r="Z46" s="5" t="inlineStr"/>
       <c r="AA46" s="5" t="inlineStr"/>
       <c r="AB46" s="5" t="inlineStr"/>
+      <c r="AC46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -3561,6 +3638,7 @@
       <c r="Z47" s="5" t="inlineStr"/>
       <c r="AA47" s="5" t="inlineStr"/>
       <c r="AB47" s="5" t="inlineStr"/>
+      <c r="AC47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -3619,6 +3697,7 @@
       <c r="Z48" s="5" t="inlineStr"/>
       <c r="AA48" s="5" t="inlineStr"/>
       <c r="AB48" s="5" t="inlineStr"/>
+      <c r="AC48" s="5" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -3677,6 +3756,7 @@
       <c r="Z49" s="5" t="inlineStr"/>
       <c r="AA49" s="5" t="inlineStr"/>
       <c r="AB49" s="5" t="inlineStr"/>
+      <c r="AC49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -3731,6 +3811,7 @@
       <c r="Z50" s="5" t="inlineStr"/>
       <c r="AA50" s="5" t="inlineStr"/>
       <c r="AB50" s="5" t="inlineStr"/>
+      <c r="AC50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -3781,6 +3862,7 @@
       <c r="Z51" s="5" t="inlineStr"/>
       <c r="AA51" s="5" t="inlineStr"/>
       <c r="AB51" s="5" t="inlineStr"/>
+      <c r="AC51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -3835,6 +3917,7 @@
       <c r="Z52" s="5" t="inlineStr"/>
       <c r="AA52" s="5" t="inlineStr"/>
       <c r="AB52" s="5" t="inlineStr"/>
+      <c r="AC52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -3889,6 +3972,7 @@
       <c r="Z53" s="5" t="inlineStr"/>
       <c r="AA53" s="5" t="inlineStr"/>
       <c r="AB53" s="5" t="inlineStr"/>
+      <c r="AC53" s="5" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -3943,6 +4027,7 @@
       <c r="Z54" s="5" t="inlineStr"/>
       <c r="AA54" s="5" t="inlineStr"/>
       <c r="AB54" s="5" t="inlineStr"/>
+      <c r="AC54" s="5" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -3989,6 +4074,7 @@
       <c r="Z55" s="5" t="inlineStr"/>
       <c r="AA55" s="5" t="inlineStr"/>
       <c r="AB55" s="5" t="inlineStr"/>
+      <c r="AC55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -4039,6 +4125,7 @@
       <c r="Z56" s="5" t="inlineStr"/>
       <c r="AA56" s="5" t="inlineStr"/>
       <c r="AB56" s="5" t="inlineStr"/>
+      <c r="AC56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -4097,6 +4184,7 @@
       <c r="Z57" s="5" t="inlineStr"/>
       <c r="AA57" s="5" t="inlineStr"/>
       <c r="AB57" s="5" t="inlineStr"/>
+      <c r="AC57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -4155,6 +4243,7 @@
       <c r="Z58" s="5" t="inlineStr"/>
       <c r="AA58" s="5" t="inlineStr"/>
       <c r="AB58" s="5" t="inlineStr"/>
+      <c r="AC58" s="5" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -4205,6 +4294,7 @@
       <c r="Z59" s="5" t="inlineStr"/>
       <c r="AA59" s="5" t="inlineStr"/>
       <c r="AB59" s="5" t="inlineStr"/>
+      <c r="AC59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -4267,6 +4357,7 @@
       <c r="Z60" s="5" t="inlineStr"/>
       <c r="AA60" s="5" t="inlineStr"/>
       <c r="AB60" s="5" t="inlineStr"/>
+      <c r="AC60" s="5" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -4313,6 +4404,7 @@
       <c r="Z61" s="5" t="inlineStr"/>
       <c r="AA61" s="5" t="inlineStr"/>
       <c r="AB61" s="5" t="inlineStr"/>
+      <c r="AC61" s="5" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -4371,6 +4463,7 @@
           <t>sailed (24/01)</t>
         </is>
       </c>
+      <c r="AC62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -4425,6 +4518,11 @@
         </is>
       </c>
       <c r="AB63" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20C</t>
+        </is>
+      </c>
+      <c r="AC63" s="5" t="inlineStr">
         <is>
           <t>expected · 20C</t>
         </is>
@@ -4483,6 +4581,11 @@
           <t>expected · 20B</t>
         </is>
       </c>
+      <c r="AC64" s="5" t="inlineStr">
+        <is>
+          <t>sailed (24/24)</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -4533,6 +4636,7 @@
         </is>
       </c>
       <c r="AB65" s="5" t="inlineStr"/>
+      <c r="AC65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -4585,6 +4689,11 @@
       <c r="AB66" s="5" t="inlineStr">
         <is>
           <t>expected · 20F (shows ETA “22A”, P.B 23/09)</t>
+        </is>
+      </c>
+      <c r="AC66" s="5" t="inlineStr">
+        <is>
+          <t>sailed (24/14)</t>
         </is>
       </c>
     </row>
@@ -4637,6 +4746,11 @@
           <t>expected · 20C</t>
         </is>
       </c>
+      <c r="AC67" s="5" t="inlineStr">
+        <is>
+          <t>sailed (24/15)</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -4685,6 +4799,11 @@
       <c r="AB68" s="6" t="inlineStr">
         <is>
           <t>expected · 20E (ETA 23/10→23/06)</t>
+        </is>
+      </c>
+      <c r="AC68" s="5" t="inlineStr">
+        <is>
+          <t>sailed (25/01)</t>
         </is>
       </c>
     </row>
@@ -4733,6 +4852,11 @@
           <t>expected · 20AB (ETD 27/03→26/16)</t>
         </is>
       </c>
+      <c r="AC69" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20AB (ETA 25/05→25/06)</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -4779,6 +4903,11 @@
           <t>expected · 20B</t>
         </is>
       </c>
+      <c r="AC70" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20B (ETA 24/24→25/06, P.B 25/04→25/14, ETD 26/03→26/12)</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -4825,6 +4954,11 @@
           <t>expected · 20B (ETA 26/14→26/20, P.B 26/14→27/05, ETD 28/03→28/14)</t>
         </is>
       </c>
+      <c r="AC71" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20C (moved from 20B; ETA 26/20→26/15, P.B 27/05→26/15, ETD 28/14→28/03)</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -4871,6 +5005,11 @@
           <t>expected · 20D</t>
         </is>
       </c>
+      <c r="AC72" s="6" t="inlineStr">
+        <is>
+          <t>expected · 20D (ETD 26/12→26/13)</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -4917,6 +5056,11 @@
           <t>expected → 20F (moved from 20E; ETA 25/22→25/14, P.B 26/06→25/15, ETD 27/14→27/04)</t>
         </is>
       </c>
+      <c r="AC73" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -4961,6 +5105,11 @@
       <c r="AB74" s="6" t="inlineStr">
         <is>
           <t>expected → 20E (moved from 20F)</t>
+        </is>
+      </c>
+      <c r="AC74" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20E</t>
         </is>
       </c>
     </row>
@@ -5001,6 +5150,11 @@
           <t>expected · 20C (new)</t>
         </is>
       </c>
+      <c r="AC75" s="6" t="inlineStr">
+        <is>
+          <t>expected → 20B (moved from 20C)</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
@@ -5039,6 +5193,11 @@
           <t>expected · 20D (new, barge)</t>
         </is>
       </c>
+      <c r="AC76" s="5" t="inlineStr">
+        <is>
+          <t>sailed (24/23)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -5075,6 +5234,128 @@
       <c r="AB77" s="5" t="inlineStr">
         <is>
           <t>expected · 20D (new, barge)</t>
+        </is>
+      </c>
+      <c r="AC77" s="5" t="inlineStr">
+        <is>
+          <t>sailed (25/07)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>SAWASDEE VEGA</t>
+        </is>
+      </c>
+      <c r="B78" s="5" t="inlineStr"/>
+      <c r="C78" s="5" t="inlineStr"/>
+      <c r="D78" s="5" t="inlineStr"/>
+      <c r="E78" s="5" t="inlineStr"/>
+      <c r="F78" s="5" t="inlineStr"/>
+      <c r="G78" s="5" t="inlineStr"/>
+      <c r="H78" s="5" t="inlineStr"/>
+      <c r="I78" s="5" t="inlineStr"/>
+      <c r="J78" s="5" t="inlineStr"/>
+      <c r="K78" s="5" t="inlineStr"/>
+      <c r="L78" s="5" t="inlineStr"/>
+      <c r="M78" s="5" t="inlineStr"/>
+      <c r="N78" s="5" t="inlineStr"/>
+      <c r="O78" s="5" t="inlineStr"/>
+      <c r="P78" s="5" t="inlineStr"/>
+      <c r="Q78" s="5" t="inlineStr"/>
+      <c r="R78" s="5" t="inlineStr"/>
+      <c r="S78" s="5" t="inlineStr"/>
+      <c r="T78" s="5" t="inlineStr"/>
+      <c r="U78" s="5" t="inlineStr"/>
+      <c r="V78" s="5" t="inlineStr"/>
+      <c r="W78" s="5" t="inlineStr"/>
+      <c r="X78" s="5" t="inlineStr"/>
+      <c r="Y78" s="5" t="inlineStr"/>
+      <c r="Z78" s="5" t="inlineStr"/>
+      <c r="AA78" s="5" t="inlineStr"/>
+      <c r="AB78" s="5" t="inlineStr"/>
+      <c r="AC78" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20D (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>KUO LONG</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr"/>
+      <c r="C79" s="5" t="inlineStr"/>
+      <c r="D79" s="5" t="inlineStr"/>
+      <c r="E79" s="5" t="inlineStr"/>
+      <c r="F79" s="5" t="inlineStr"/>
+      <c r="G79" s="5" t="inlineStr"/>
+      <c r="H79" s="5" t="inlineStr"/>
+      <c r="I79" s="5" t="inlineStr"/>
+      <c r="J79" s="5" t="inlineStr"/>
+      <c r="K79" s="5" t="inlineStr"/>
+      <c r="L79" s="5" t="inlineStr"/>
+      <c r="M79" s="5" t="inlineStr"/>
+      <c r="N79" s="5" t="inlineStr"/>
+      <c r="O79" s="5" t="inlineStr"/>
+      <c r="P79" s="5" t="inlineStr"/>
+      <c r="Q79" s="5" t="inlineStr"/>
+      <c r="R79" s="5" t="inlineStr"/>
+      <c r="S79" s="5" t="inlineStr"/>
+      <c r="T79" s="5" t="inlineStr"/>
+      <c r="U79" s="5" t="inlineStr"/>
+      <c r="V79" s="5" t="inlineStr"/>
+      <c r="W79" s="5" t="inlineStr"/>
+      <c r="X79" s="5" t="inlineStr"/>
+      <c r="Y79" s="5" t="inlineStr"/>
+      <c r="Z79" s="5" t="inlineStr"/>
+      <c r="AA79" s="5" t="inlineStr"/>
+      <c r="AB79" s="5" t="inlineStr"/>
+      <c r="AC79" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20E (new)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>WAN HAI 276</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr"/>
+      <c r="C80" s="5" t="inlineStr"/>
+      <c r="D80" s="5" t="inlineStr"/>
+      <c r="E80" s="5" t="inlineStr"/>
+      <c r="F80" s="5" t="inlineStr"/>
+      <c r="G80" s="5" t="inlineStr"/>
+      <c r="H80" s="5" t="inlineStr"/>
+      <c r="I80" s="5" t="inlineStr"/>
+      <c r="J80" s="5" t="inlineStr"/>
+      <c r="K80" s="5" t="inlineStr"/>
+      <c r="L80" s="5" t="inlineStr"/>
+      <c r="M80" s="5" t="inlineStr"/>
+      <c r="N80" s="5" t="inlineStr"/>
+      <c r="O80" s="5" t="inlineStr"/>
+      <c r="P80" s="5" t="inlineStr"/>
+      <c r="Q80" s="5" t="inlineStr"/>
+      <c r="R80" s="5" t="inlineStr"/>
+      <c r="S80" s="5" t="inlineStr"/>
+      <c r="T80" s="5" t="inlineStr"/>
+      <c r="U80" s="5" t="inlineStr"/>
+      <c r="V80" s="5" t="inlineStr"/>
+      <c r="W80" s="5" t="inlineStr"/>
+      <c r="X80" s="5" t="inlineStr"/>
+      <c r="Y80" s="5" t="inlineStr"/>
+      <c r="Z80" s="5" t="inlineStr"/>
+      <c r="AA80" s="5" t="inlineStr"/>
+      <c r="AB80" s="5" t="inlineStr"/>
+      <c r="AC80" s="5" t="inlineStr">
+        <is>
+          <t>expected · 20F (new)</t>
         </is>
       </c>
     </row>
@@ -20769,7 +21050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O76"/>
+  <dimension ref="A1:O79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20810,7 +21091,7 @@
         </is>
       </c>
       <c r="B3" s="22" t="n">
-        <v>46319.375</v>
+        <v>46320.375</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
@@ -20903,34 +21184,34 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>SKY CHALLENGE</t>
+          <t>KMTC TOKYO</t>
         </is>
       </c>
       <c r="C6" s="23" t="n">
         <v>565</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>46293</v>
+        <v>46299</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>46295</v>
+        <v>46320</v>
       </c>
       <c r="F6" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>20AB</t>
+        <v>6</v>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>20F → 20AB</t>
         </is>
       </c>
       <c r="H6" s="11" t="n">
-        <v>46294.33333333334</v>
+        <v>46292.20833333334</v>
       </c>
       <c r="I6" s="11" t="n">
-        <v>46294.66666666666</v>
+        <v>46292.20833333334</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>46296.16666666666</v>
+        <v>46293.54166666666</v>
       </c>
       <c r="K6" s="24">
         <f>(I6-H6)*24</f>
@@ -20946,10 +21227,9 @@
         </is>
       </c>
       <c r="N6" s="23" t="inlineStr"/>
-      <c r="O6" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="O6" s="23">
+        <f>IF(J6&lt;=$B$3,"Sailed",IF(I6&lt;=$B$3,"Alongside",IF(H6&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -20960,34 +21240,34 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>RESURGENCE</t>
+          <t>SKY CHALLENGE</t>
         </is>
       </c>
       <c r="C7" s="23" t="n">
-        <v>458</v>
+        <v>565</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>46296</v>
+        <v>46293</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>46299</v>
+        <v>46295</v>
       </c>
       <c r="F7" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>20E → 20AB</t>
+        <v>3</v>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
         </is>
       </c>
       <c r="H7" s="11" t="n">
-        <v>46298.5</v>
+        <v>46294.33333333334</v>
       </c>
       <c r="I7" s="11" t="n">
-        <v>46298.5</v>
+        <v>46294.66666666666</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>46299.70833333334</v>
+        <v>46296.16666666666</v>
       </c>
       <c r="K7" s="24">
         <f>(I7-H7)*24</f>
@@ -21017,34 +21297,34 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>KMTC TOKYO</t>
+          <t>RESURGENCE</t>
         </is>
       </c>
       <c r="C8" s="23" t="n">
-        <v>565</v>
+        <v>458</v>
       </c>
       <c r="D8" s="10" t="n">
+        <v>46296</v>
+      </c>
+      <c r="E8" s="10" t="n">
         <v>46299</v>
       </c>
-      <c r="E8" s="10" t="n">
-        <v>46303</v>
-      </c>
       <c r="F8" s="23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G8" s="6" t="inlineStr">
         <is>
-          <t>20F → 20AB</t>
+          <t>20E → 20AB</t>
         </is>
       </c>
       <c r="H8" s="11" t="n">
-        <v>46301.54166666666</v>
+        <v>46298.5</v>
       </c>
       <c r="I8" s="11" t="n">
-        <v>46301.54166666666</v>
+        <v>46298.5</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>46303.5</v>
+        <v>46299.70833333334</v>
       </c>
       <c r="K8" s="24">
         <f>(I8-H8)*24</f>
@@ -21520,9 +21800,10 @@
         </is>
       </c>
       <c r="N16" s="23" t="inlineStr"/>
-      <c r="O16" s="23">
-        <f>IF(J16&lt;=$B$3,"Sailed",IF(I16&lt;=$B$3,"Alongside",IF(H16&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O16" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -21543,10 +21824,10 @@
         <v>46301</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="F17" s="23" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
@@ -21554,7 +21835,7 @@
         </is>
       </c>
       <c r="H17" s="11" t="n">
-        <v>46320.20833333334</v>
+        <v>46320.25</v>
       </c>
       <c r="I17" s="11" t="n">
         <v>46320.625</v>
@@ -21589,34 +21870,34 @@
       </c>
       <c r="B18" s="27" t="inlineStr">
         <is>
-          <t>ZHONG GU BEI HAI</t>
+          <t>XIN AN</t>
         </is>
       </c>
       <c r="C18" s="28" t="n">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="D18" s="29" t="n">
-        <v>46296</v>
+        <v>46300</v>
       </c>
       <c r="E18" s="29" t="n">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="F18" s="28" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G18" s="30" t="inlineStr">
         <is>
-          <t>20B → 20AB → 20B</t>
+          <t>20F → 20C → 20B</t>
         </is>
       </c>
       <c r="H18" s="31" t="n">
-        <v>46321.83333333334</v>
+        <v>46321.75</v>
       </c>
       <c r="I18" s="31" t="n">
-        <v>46292.20833333334</v>
+        <v>46292.16666666666</v>
       </c>
       <c r="J18" s="31" t="n">
-        <v>46293.58333333334</v>
+        <v>46293.20833333334</v>
       </c>
       <c r="K18" s="32">
         <f>(I18-H18)*24</f>
@@ -21987,34 +22268,34 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>M ODYSSEY</t>
+          <t>KHARIS HERITAGE</t>
         </is>
       </c>
       <c r="C25" s="23" t="n">
-        <v>449</v>
+        <v>482</v>
       </c>
       <c r="D25" s="10" t="n">
-        <v>46293</v>
+        <v>46294</v>
       </c>
       <c r="E25" s="10" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="F25" s="23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>20B → 20C → 20B</t>
+          <t>20AB → 20B → 20C → 20B</t>
         </is>
       </c>
       <c r="H25" s="11" t="n">
-        <v>46309.04166666666</v>
+        <v>46310.04166666666</v>
       </c>
       <c r="I25" s="11" t="n">
-        <v>46309.625</v>
+        <v>46310.25</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>46310.20833333334</v>
+        <v>46311.29166666666</v>
       </c>
       <c r="K25" s="24">
         <f>(I25-H25)*24</f>
@@ -22026,7 +22307,7 @@
       </c>
       <c r="M25" s="23" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N25" s="23" t="inlineStr"/>
@@ -22044,34 +22325,34 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>KHARIS HERITAGE</t>
+          <t>TS CHIBA</t>
         </is>
       </c>
       <c r="C26" s="23" t="n">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="D26" s="10" t="n">
-        <v>46294</v>
+        <v>46293</v>
       </c>
       <c r="E26" s="10" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="F26" s="23" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20B → 20C → 20B</t>
+          <t>20E → 20C → 20B</t>
         </is>
       </c>
       <c r="H26" s="11" t="n">
-        <v>46310.04166666666</v>
+        <v>46311.58333333334</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>46310.25</v>
+        <v>46311.58333333334</v>
       </c>
       <c r="J26" s="11" t="n">
-        <v>46311.29166666666</v>
+        <v>46312.45833333334</v>
       </c>
       <c r="K26" s="24">
         <f>(I26-H26)*24</f>
@@ -22101,34 +22382,34 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>TS CHIBA</t>
+          <t>JARU BHUM</t>
         </is>
       </c>
       <c r="C27" s="23" t="n">
-        <v>485</v>
+        <v>564</v>
       </c>
       <c r="D27" s="10" t="n">
         <v>46293</v>
       </c>
       <c r="E27" s="10" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
       <c r="F27" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>20E → 20C → 20B</t>
+          <t>20F → 20D → 20B</t>
         </is>
       </c>
       <c r="H27" s="11" t="n">
-        <v>46311.58333333334</v>
+        <v>46312.66666666666</v>
       </c>
       <c r="I27" s="11" t="n">
-        <v>46311.58333333334</v>
+        <v>46312.66666666666</v>
       </c>
       <c r="J27" s="11" t="n">
-        <v>46312.45833333334</v>
+        <v>46313.41666666666</v>
       </c>
       <c r="K27" s="24">
         <f>(I27-H27)*24</f>
@@ -22140,7 +22421,7 @@
       </c>
       <c r="M27" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="N27" s="23" t="inlineStr"/>
@@ -22158,34 +22439,34 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>JARU BHUM</t>
+          <t>KMTC JAKARTA</t>
         </is>
       </c>
       <c r="C28" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D28" s="10" t="n">
-        <v>46293</v>
+        <v>46310</v>
       </c>
       <c r="E28" s="10" t="n">
-        <v>46313</v>
+        <v>46315</v>
       </c>
       <c r="F28" s="23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>20F → 20D → 20B</t>
+          <t>20F → 20B</t>
         </is>
       </c>
       <c r="H28" s="11" t="n">
-        <v>46312.66666666666</v>
+        <v>46314.41666666666</v>
       </c>
       <c r="I28" s="11" t="n">
-        <v>46312.66666666666</v>
+        <v>46314.41666666666</v>
       </c>
       <c r="J28" s="11" t="n">
-        <v>46313.41666666666</v>
+        <v>46315.70833333334</v>
       </c>
       <c r="K28" s="24">
         <f>(I28-H28)*24</f>
@@ -22197,7 +22478,7 @@
       </c>
       <c r="M28" s="23" t="inlineStr">
         <is>
-          <t>7B</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N28" s="23" t="inlineStr"/>
@@ -22215,34 +22496,34 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>KMTC JAKARTA</t>
+          <t>MITRA BHUM</t>
         </is>
       </c>
       <c r="C29" s="23" t="n">
-        <v>564</v>
+        <v>485</v>
       </c>
       <c r="D29" s="10" t="n">
-        <v>46310</v>
+        <v>46293</v>
       </c>
       <c r="E29" s="10" t="n">
-        <v>46315</v>
+        <v>46316</v>
       </c>
       <c r="F29" s="23" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>20F → 20B</t>
+          <t>20F → 20E → 20D → 20AB → 20C → 20B</t>
         </is>
       </c>
       <c r="H29" s="11" t="n">
-        <v>46314.41666666666</v>
+        <v>46316.54166666666</v>
       </c>
       <c r="I29" s="11" t="n">
-        <v>46314.41666666666</v>
+        <v>46316.54166666666</v>
       </c>
       <c r="J29" s="11" t="n">
-        <v>46315.70833333334</v>
+        <v>46317.20833333334</v>
       </c>
       <c r="K29" s="24">
         <f>(I29-H29)*24</f>
@@ -22272,34 +22553,34 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>MITRA BHUM</t>
+          <t>GREEN PARK</t>
         </is>
       </c>
       <c r="C30" s="23" t="n">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="D30" s="10" t="n">
-        <v>46293</v>
+        <v>46300</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>46316</v>
+        <v>46318</v>
       </c>
       <c r="F30" s="23" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G30" s="6" t="inlineStr">
         <is>
-          <t>20F → 20E → 20D → 20AB → 20C → 20B</t>
+          <t>20AB → 20B → 20AB → 20F → 20B</t>
         </is>
       </c>
       <c r="H30" s="11" t="n">
-        <v>46316.54166666666</v>
+        <v>46316.66666666666</v>
       </c>
       <c r="I30" s="11" t="n">
-        <v>46316.54166666666</v>
+        <v>46317.58333333334</v>
       </c>
       <c r="J30" s="11" t="n">
-        <v>46317.20833333334</v>
+        <v>46318.54166666666</v>
       </c>
       <c r="K30" s="24">
         <f>(I30-H30)*24</f>
@@ -22329,34 +22610,34 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>GREEN PARK</t>
+          <t>CA MANILA</t>
         </is>
       </c>
       <c r="C31" s="23" t="n">
-        <v>482</v>
+        <v>548</v>
       </c>
       <c r="D31" s="10" t="n">
-        <v>46300</v>
+        <v>46315</v>
       </c>
       <c r="E31" s="10" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="F31" s="23" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20B → 20AB → 20F → 20B</t>
+          <t>20C → 20B</t>
         </is>
       </c>
       <c r="H31" s="11" t="n">
-        <v>46316.66666666666</v>
+        <v>46317.75</v>
       </c>
       <c r="I31" s="11" t="n">
-        <v>46317.58333333334</v>
+        <v>46318.54166666666</v>
       </c>
       <c r="J31" s="11" t="n">
-        <v>46318.54166666666</v>
+        <v>46320</v>
       </c>
       <c r="K31" s="24">
         <f>(I31-H31)*24</f>
@@ -22386,34 +22667,34 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>CA MANILA</t>
+          <t>ASL TAIPEIS</t>
         </is>
       </c>
       <c r="C32" s="23" t="n">
-        <v>548</v>
+        <v>564</v>
       </c>
       <c r="D32" s="10" t="n">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="E32" s="10" t="n">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="F32" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G32" s="6" t="inlineStr">
-        <is>
-          <t>20C → 20B</t>
+        <v>4</v>
+      </c>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
         </is>
       </c>
       <c r="H32" s="11" t="n">
-        <v>46317.75</v>
+        <v>46320.25</v>
       </c>
       <c r="I32" s="11" t="n">
-        <v>46318.54166666666</v>
+        <v>46320.58333333334</v>
       </c>
       <c r="J32" s="11" t="n">
-        <v>46320</v>
+        <v>46321.5</v>
       </c>
       <c r="K32" s="24">
         <f>(I32-H32)*24</f>
@@ -22435,115 +22716,116 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>20B</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>ASL TAIPEIS</t>
-        </is>
-      </c>
-      <c r="C33" s="23" t="n">
+      <c r="A33" s="27" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B33" s="27" t="inlineStr">
+        <is>
+          <t>M ODYSSEY</t>
+        </is>
+      </c>
+      <c r="C33" s="28" t="n">
+        <v>449</v>
+      </c>
+      <c r="D33" s="29" t="n">
+        <v>46293</v>
+      </c>
+      <c r="E33" s="29" t="n">
+        <v>46320</v>
+      </c>
+      <c r="F33" s="28" t="n">
+        <v>7</v>
+      </c>
+      <c r="G33" s="30" t="inlineStr">
+        <is>
+          <t>20B → 20C → 20B → 20C</t>
+        </is>
+      </c>
+      <c r="H33" s="31" t="n">
+        <v>46293.125</v>
+      </c>
+      <c r="I33" s="31" t="n">
+        <v>46293.20833333334</v>
+      </c>
+      <c r="J33" s="31" t="n">
+        <v>46294.25</v>
+      </c>
+      <c r="K33" s="32">
+        <f>(I33-H33)*24</f>
+        <v/>
+      </c>
+      <c r="L33" s="32">
+        <f>(J33-I33)*24</f>
+        <v/>
+      </c>
+      <c r="M33" s="28" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N33" s="28" t="inlineStr"/>
+      <c r="O33" s="28">
+        <f>IF(J33&lt;=$B$3,"Sailed",IF(I33&lt;=$B$3,"Alongside",IF(H33&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>SAWASDEE DENEB</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="n">
         <v>564</v>
       </c>
-      <c r="D33" s="10" t="n">
-        <v>46317</v>
-      </c>
-      <c r="E33" s="10" t="n">
-        <v>46319</v>
-      </c>
-      <c r="F33" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G33" s="5" t="inlineStr">
-        <is>
-          <t>20B</t>
-        </is>
-      </c>
-      <c r="H33" s="11" t="n">
-        <v>46320</v>
-      </c>
-      <c r="I33" s="11" t="n">
-        <v>46320.16666666666</v>
-      </c>
-      <c r="J33" s="11" t="n">
-        <v>46321.125</v>
-      </c>
-      <c r="K33" s="24">
-        <f>(I33-H33)*24</f>
-        <v/>
-      </c>
-      <c r="L33" s="24">
-        <f>(J33-I33)*24</f>
-        <v/>
-      </c>
-      <c r="M33" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N33" s="23" t="inlineStr"/>
-      <c r="O33" s="23">
-        <f>IF(J33&lt;=$B$3,"Sailed",IF(I33&lt;=$B$3,"Alongside",IF(H33&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="27" t="inlineStr">
+      <c r="D34" s="10" t="n">
+        <v>46297</v>
+      </c>
+      <c r="E34" s="10" t="n">
+        <v>46302</v>
+      </c>
+      <c r="F34" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="G34" s="5" t="inlineStr">
         <is>
           <t>20C</t>
         </is>
       </c>
-      <c r="B34" s="27" t="inlineStr">
-        <is>
-          <t>XIN AN</t>
-        </is>
-      </c>
-      <c r="C34" s="28" t="n">
-        <v>564</v>
-      </c>
-      <c r="D34" s="29" t="n">
+      <c r="H34" s="11" t="n">
         <v>46300</v>
       </c>
-      <c r="E34" s="29" t="n">
-        <v>46319</v>
-      </c>
-      <c r="F34" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="G34" s="30" t="inlineStr">
-        <is>
-          <t>20F → 20C</t>
-        </is>
-      </c>
-      <c r="H34" s="31" t="n">
-        <v>46321.75</v>
-      </c>
-      <c r="I34" s="31" t="n">
-        <v>46292.16666666666</v>
-      </c>
-      <c r="J34" s="31" t="n">
-        <v>46293.20833333334</v>
-      </c>
-      <c r="K34" s="32">
+      <c r="I34" s="11" t="n">
+        <v>46300.5</v>
+      </c>
+      <c r="J34" s="11" t="n">
+        <v>46302.45833333334</v>
+      </c>
+      <c r="K34" s="24">
         <f>(I34-H34)*24</f>
         <v/>
       </c>
-      <c r="L34" s="32">
+      <c r="L34" s="24">
         <f>(J34-I34)*24</f>
         <v/>
       </c>
-      <c r="M34" s="28" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N34" s="28" t="inlineStr"/>
-      <c r="O34" s="28">
-        <f>IF(J34&lt;=$B$3,"Sailed",IF(I34&lt;=$B$3,"Alongside",IF(H34&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="M34" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N34" s="23" t="inlineStr"/>
+      <c r="O34" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="35">
@@ -22554,7 +22836,7 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE DENEB</t>
+          <t>JOSCO LUCKY</t>
         </is>
       </c>
       <c r="C35" s="23" t="n">
@@ -22564,24 +22846,24 @@
         <v>46297</v>
       </c>
       <c r="E35" s="10" t="n">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="F35" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
-        <is>
-          <t>20C</t>
+        <v>7</v>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20AB → 20D → 20C</t>
         </is>
       </c>
       <c r="H35" s="11" t="n">
-        <v>46300</v>
+        <v>46301.875</v>
       </c>
       <c r="I35" s="11" t="n">
-        <v>46300.5</v>
+        <v>46302.54166666666</v>
       </c>
       <c r="J35" s="11" t="n">
-        <v>46302.45833333334</v>
+        <v>46303.54166666666</v>
       </c>
       <c r="K35" s="24">
         <f>(I35-H35)*24</f>
@@ -22611,34 +22893,34 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>JOSCO LUCKY</t>
+          <t>ZHONG GU DONG HAI</t>
         </is>
       </c>
       <c r="C36" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D36" s="10" t="n">
-        <v>46297</v>
+        <v>46301</v>
       </c>
       <c r="E36" s="10" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="F36" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="G36" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 20D → 20C</t>
+        <v>4</v>
+      </c>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
         </is>
       </c>
       <c r="H36" s="11" t="n">
-        <v>46301.875</v>
+        <v>46302.58333333334</v>
       </c>
       <c r="I36" s="11" t="n">
-        <v>46302.54166666666</v>
+        <v>46303.58333333334</v>
       </c>
       <c r="J36" s="11" t="n">
-        <v>46303.54166666666</v>
+        <v>46304.58333333334</v>
       </c>
       <c r="K36" s="24">
         <f>(I36-H36)*24</f>
@@ -22661,118 +22943,118 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="A37" s="25" t="inlineStr">
         <is>
           <t>20C</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>ZHONG GU DONG HAI</t>
-        </is>
-      </c>
-      <c r="C37" s="23" t="n">
+      <c r="B37" s="25" t="inlineStr">
+        <is>
+          <t>YM INCEPTION</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="n">
         <v>564</v>
       </c>
-      <c r="D37" s="10" t="n">
+      <c r="D37" s="18" t="n">
         <v>46301</v>
       </c>
-      <c r="E37" s="10" t="n">
-        <v>46304</v>
-      </c>
-      <c r="F37" s="23" t="n">
+      <c r="E37" s="18" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F37" s="17" t="n">
+        <v>5</v>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20C</t>
+        </is>
+      </c>
+      <c r="H37" s="20" t="n">
+        <v>46303.54166666666</v>
+      </c>
+      <c r="I37" s="20" t="n">
+        <v>46304.54166666666</v>
+      </c>
+      <c r="J37" s="20" t="n">
+        <v>46305.58333333334</v>
+      </c>
+      <c r="K37" s="26">
+        <f>(I37-H37)*24</f>
+        <v/>
+      </c>
+      <c r="L37" s="26">
+        <f>(J37-I37)*24</f>
+        <v/>
+      </c>
+      <c r="M37" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N37" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O37" s="17" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>STARSHIP AQUILA</t>
+        </is>
+      </c>
+      <c r="C38" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D38" s="10" t="n">
+        <v>46303</v>
+      </c>
+      <c r="E38" s="10" t="n">
+        <v>46306</v>
+      </c>
+      <c r="F38" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="G38" s="5" t="inlineStr">
         <is>
           <t>20C</t>
         </is>
       </c>
-      <c r="H37" s="11" t="n">
-        <v>46302.58333333334</v>
-      </c>
-      <c r="I37" s="11" t="n">
-        <v>46303.58333333334</v>
-      </c>
-      <c r="J37" s="11" t="n">
-        <v>46304.58333333334</v>
-      </c>
-      <c r="K37" s="24">
-        <f>(I37-H37)*24</f>
-        <v/>
-      </c>
-      <c r="L37" s="24">
-        <f>(J37-I37)*24</f>
-        <v/>
-      </c>
-      <c r="M37" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N37" s="23" t="inlineStr"/>
-      <c r="O37" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="25" t="inlineStr">
-        <is>
-          <t>20C</t>
-        </is>
-      </c>
-      <c r="B38" s="25" t="inlineStr">
-        <is>
-          <t>YM INCEPTION</t>
-        </is>
-      </c>
-      <c r="C38" s="17" t="n">
-        <v>564</v>
-      </c>
-      <c r="D38" s="18" t="n">
-        <v>46301</v>
-      </c>
-      <c r="E38" s="18" t="n">
-        <v>46305</v>
-      </c>
-      <c r="F38" s="17" t="n">
-        <v>5</v>
-      </c>
-      <c r="G38" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20C</t>
-        </is>
-      </c>
-      <c r="H38" s="20" t="n">
-        <v>46303.54166666666</v>
-      </c>
-      <c r="I38" s="20" t="n">
-        <v>46304.54166666666</v>
-      </c>
-      <c r="J38" s="20" t="n">
+      <c r="H38" s="11" t="n">
+        <v>46304.91666666666</v>
+      </c>
+      <c r="I38" s="11" t="n">
         <v>46305.58333333334</v>
       </c>
-      <c r="K38" s="26">
+      <c r="J38" s="11" t="n">
+        <v>46307.08333333334</v>
+      </c>
+      <c r="K38" s="24">
         <f>(I38-H38)*24</f>
         <v/>
       </c>
-      <c r="L38" s="26">
+      <c r="L38" s="24">
         <f>(J38-I38)*24</f>
         <v/>
       </c>
-      <c r="M38" s="17" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N38" s="17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O38" s="17" t="inlineStr">
+      <c r="M38" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N38" s="23" t="inlineStr"/>
+      <c r="O38" s="23" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -22786,34 +23068,34 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>STARSHIP AQUILA</t>
+          <t>WAN HAI 277</t>
         </is>
       </c>
       <c r="C39" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D39" s="10" t="n">
-        <v>46303</v>
+        <v>46305</v>
       </c>
       <c r="E39" s="10" t="n">
-        <v>46306</v>
+        <v>46309</v>
       </c>
       <c r="F39" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>20C</t>
+        <v>5</v>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>20F → 20B → 20C</t>
         </is>
       </c>
       <c r="H39" s="11" t="n">
-        <v>46304.91666666666</v>
+        <v>46307.875</v>
       </c>
       <c r="I39" s="11" t="n">
-        <v>46305.58333333334</v>
+        <v>46308.25</v>
       </c>
       <c r="J39" s="11" t="n">
-        <v>46307.08333333334</v>
+        <v>46309.66666666666</v>
       </c>
       <c r="K39" s="24">
         <f>(I39-H39)*24</f>
@@ -22843,34 +23125,34 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 277</t>
+          <t>WAN HAI 173</t>
         </is>
       </c>
       <c r="C40" s="23" t="n">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D40" s="10" t="n">
-        <v>46305</v>
+        <v>46307</v>
       </c>
       <c r="E40" s="10" t="n">
         <v>46309</v>
       </c>
       <c r="F40" s="23" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>20F → 20B → 20C</t>
+          <t>20B → 20C</t>
         </is>
       </c>
       <c r="H40" s="11" t="n">
-        <v>46307.875</v>
+        <v>46309.04166666666</v>
       </c>
       <c r="I40" s="11" t="n">
-        <v>46308.25</v>
+        <v>46309.66666666666</v>
       </c>
       <c r="J40" s="11" t="n">
-        <v>46309.66666666666</v>
+        <v>46310.29166666666</v>
       </c>
       <c r="K40" s="24">
         <f>(I40-H40)*24</f>
@@ -22900,34 +23182,34 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 173</t>
+          <t>WAN HAI 175</t>
         </is>
       </c>
       <c r="C41" s="23" t="n">
         <v>565</v>
       </c>
       <c r="D41" s="10" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="E41" s="10" t="n">
-        <v>46309</v>
+        <v>46311</v>
       </c>
       <c r="F41" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>20B → 20C</t>
+          <t>20D → 20C</t>
         </is>
       </c>
       <c r="H41" s="11" t="n">
-        <v>46309.04166666666</v>
+        <v>46309.875</v>
       </c>
       <c r="I41" s="11" t="n">
-        <v>46309.66666666666</v>
+        <v>46310.29166666666</v>
       </c>
       <c r="J41" s="11" t="n">
-        <v>46310.29166666666</v>
+        <v>46311.625</v>
       </c>
       <c r="K41" s="24">
         <f>(I41-H41)*24</f>
@@ -22957,34 +23239,34 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 175</t>
+          <t>LITTLE DOLPHIN</t>
         </is>
       </c>
       <c r="C42" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D42" s="10" t="n">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="E42" s="10" t="n">
-        <v>46311</v>
+        <v>46313</v>
       </c>
       <c r="F42" s="23" t="n">
         <v>4</v>
       </c>
       <c r="G42" s="6" t="inlineStr">
         <is>
-          <t>20D → 20C</t>
+          <t>20B → 20C</t>
         </is>
       </c>
       <c r="H42" s="11" t="n">
-        <v>46309.875</v>
+        <v>46312.04166666666</v>
       </c>
       <c r="I42" s="11" t="n">
-        <v>46310.29166666666</v>
+        <v>46312.33333333334</v>
       </c>
       <c r="J42" s="11" t="n">
-        <v>46311.625</v>
+        <v>46313.66666666666</v>
       </c>
       <c r="K42" s="24">
         <f>(I42-H42)*24</f>
@@ -23014,17 +23296,17 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>LITTLE DOLPHIN</t>
+          <t>MILLENNIUM BRIGHT</t>
         </is>
       </c>
       <c r="C43" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D43" s="10" t="n">
-        <v>46310</v>
+        <v>46293</v>
       </c>
       <c r="E43" s="10" t="n">
-        <v>46313</v>
+        <v>46315</v>
       </c>
       <c r="F43" s="23" t="n">
         <v>4</v>
@@ -23035,13 +23317,13 @@
         </is>
       </c>
       <c r="H43" s="11" t="n">
-        <v>46312.04166666666</v>
+        <v>46314.58333333334</v>
       </c>
       <c r="I43" s="11" t="n">
-        <v>46312.33333333334</v>
+        <v>46314.58333333334</v>
       </c>
       <c r="J43" s="11" t="n">
-        <v>46313.66666666666</v>
+        <v>46315.5</v>
       </c>
       <c r="K43" s="24">
         <f>(I43-H43)*24</f>
@@ -23071,34 +23353,34 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>MILLENNIUM BRIGHT</t>
+          <t>CAPE FAWLEY</t>
         </is>
       </c>
       <c r="C44" s="23" t="n">
-        <v>564</v>
+        <v>558</v>
       </c>
       <c r="D44" s="10" t="n">
         <v>46293</v>
       </c>
       <c r="E44" s="10" t="n">
-        <v>46315</v>
+        <v>46318</v>
       </c>
       <c r="F44" s="23" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>20B → 20C</t>
+          <t>20AB → 20C → 20AB → 20C</t>
         </is>
       </c>
       <c r="H44" s="11" t="n">
-        <v>46314.58333333334</v>
+        <v>46316.45833333334</v>
       </c>
       <c r="I44" s="11" t="n">
-        <v>46314.58333333334</v>
+        <v>46316.5</v>
       </c>
       <c r="J44" s="11" t="n">
-        <v>46315.5</v>
+        <v>46318.5</v>
       </c>
       <c r="K44" s="24">
         <f>(I44-H44)*24</f>
@@ -23128,34 +23410,34 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>CAPE FAWLEY</t>
+          <t>HORAI BRIDGE</t>
         </is>
       </c>
       <c r="C45" s="23" t="n">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="D45" s="10" t="n">
-        <v>46293</v>
+        <v>46316</v>
       </c>
       <c r="E45" s="10" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="F45" s="23" t="n">
-        <v>12</v>
-      </c>
-      <c r="G45" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20C → 20AB → 20C</t>
+        <v>4</v>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
         </is>
       </c>
       <c r="H45" s="11" t="n">
-        <v>46316.45833333334</v>
+        <v>46318.04166666666</v>
       </c>
       <c r="I45" s="11" t="n">
-        <v>46316.5</v>
+        <v>46318.5</v>
       </c>
       <c r="J45" s="11" t="n">
-        <v>46318.5</v>
+        <v>46319.625</v>
       </c>
       <c r="K45" s="24">
         <f>(I45-H45)*24</f>
@@ -23185,17 +23467,17 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>HORAI BRIDGE</t>
+          <t>SAWASDEE MIMOSA</t>
         </is>
       </c>
       <c r="C46" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D46" s="10" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="E46" s="10" t="n">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="F46" s="23" t="n">
         <v>4</v>
@@ -23206,13 +23488,13 @@
         </is>
       </c>
       <c r="H46" s="11" t="n">
-        <v>46318.04166666666</v>
+        <v>46318.70833333334</v>
       </c>
       <c r="I46" s="11" t="n">
-        <v>46318.5</v>
+        <v>46319.625</v>
       </c>
       <c r="J46" s="11" t="n">
-        <v>46319.625</v>
+        <v>46321.125</v>
       </c>
       <c r="K46" s="24">
         <f>(I46-H46)*24</f>
@@ -23241,34 +23523,34 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE MIMOSA</t>
+          <t>ZHONG GU BEI HAI</t>
         </is>
       </c>
       <c r="C47" s="23" t="n">
-        <v>564</v>
+        <v>561</v>
       </c>
       <c r="D47" s="10" t="n">
-        <v>46317</v>
+        <v>46296</v>
       </c>
       <c r="E47" s="10" t="n">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="F47" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G47" s="5" t="inlineStr">
-        <is>
-          <t>20C</t>
+        <v>10</v>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20AB → 20B → 20C</t>
         </is>
       </c>
       <c r="H47" s="11" t="n">
-        <v>46318.70833333334</v>
+        <v>46321.625</v>
       </c>
       <c r="I47" s="11" t="n">
-        <v>46319.625</v>
+        <v>46321.625</v>
       </c>
       <c r="J47" s="11" t="n">
-        <v>46321.125</v>
+        <v>46293.125</v>
       </c>
       <c r="K47" s="24">
         <f>(I47-H47)*24</f>
@@ -23297,20 +23579,20 @@
       </c>
       <c r="B48" s="27" t="inlineStr">
         <is>
-          <t>HARI BHUM (Barge)</t>
+          <t>SAWASDEE VEGA</t>
         </is>
       </c>
       <c r="C48" s="28" t="n">
-        <v>259</v>
+        <v>564</v>
       </c>
       <c r="D48" s="29" t="n">
-        <v>46297</v>
+        <v>46320</v>
       </c>
       <c r="E48" s="29" t="n">
-        <v>46298</v>
+        <v>46320</v>
       </c>
       <c r="F48" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G48" s="33" t="inlineStr">
         <is>
@@ -23318,13 +23600,13 @@
         </is>
       </c>
       <c r="H48" s="31" t="n">
-        <v>46298.20833333334</v>
+        <v>46292.625</v>
       </c>
       <c r="I48" s="31" t="n">
-        <v>46298.29166666666</v>
+        <v>46292.625</v>
       </c>
       <c r="J48" s="31" t="n">
-        <v>46298.66666666666</v>
+        <v>46294.16666666666</v>
       </c>
       <c r="K48" s="32">
         <f>(I48-H48)*24</f>
@@ -23340,10 +23622,9 @@
         </is>
       </c>
       <c r="N48" s="28" t="inlineStr"/>
-      <c r="O48" s="28" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="O48" s="28">
+        <f>IF(J48&lt;=$B$3,"Sailed",IF(I48&lt;=$B$3,"Alongside",IF(H48&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="49">
@@ -23354,34 +23635,34 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>HE JIN</t>
+          <t>HARI BHUM (Barge)</t>
         </is>
       </c>
       <c r="C49" s="23" t="n">
-        <v>552</v>
+        <v>259</v>
       </c>
       <c r="D49" s="10" t="n">
-        <v>46301</v>
+        <v>46297</v>
       </c>
       <c r="E49" s="10" t="n">
-        <v>46305</v>
+        <v>46298</v>
       </c>
       <c r="F49" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G49" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 22A → 20D</t>
+        <v>2</v>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H49" s="11" t="n">
-        <v>46304</v>
+        <v>46298.20833333334</v>
       </c>
       <c r="I49" s="11" t="n">
-        <v>46304</v>
+        <v>46298.29166666666</v>
       </c>
       <c r="J49" s="11" t="n">
-        <v>46305.54166666666</v>
+        <v>46298.66666666666</v>
       </c>
       <c r="K49" s="24">
         <f>(I49-H49)*24</f>
@@ -23411,34 +23692,34 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>CUL HAIPHONG</t>
+          <t>HE JIN</t>
         </is>
       </c>
       <c r="C50" s="23" t="n">
-        <v>458</v>
+        <v>552</v>
       </c>
       <c r="D50" s="10" t="n">
-        <v>46302</v>
+        <v>46301</v>
       </c>
       <c r="E50" s="10" t="n">
         <v>46305</v>
       </c>
       <c r="F50" s="23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>20B → 20D</t>
+          <t>20B → 20AB → 22A → 20D</t>
         </is>
       </c>
       <c r="H50" s="11" t="n">
-        <v>46304.83333333334</v>
+        <v>46304</v>
       </c>
       <c r="I50" s="11" t="n">
-        <v>46305.66666666666</v>
+        <v>46304</v>
       </c>
       <c r="J50" s="11" t="n">
-        <v>46306.25</v>
+        <v>46305.54166666666</v>
       </c>
       <c r="K50" s="24">
         <f>(I50-H50)*24</f>
@@ -23450,7 +23731,7 @@
       </c>
       <c r="M50" s="23" t="inlineStr">
         <is>
-          <t>4A</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N50" s="23" t="inlineStr"/>
@@ -23468,34 +23749,34 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>INCEDA</t>
+          <t>CUL HAIPHONG</t>
         </is>
       </c>
       <c r="C51" s="23" t="n">
-        <v>564</v>
+        <v>458</v>
       </c>
       <c r="D51" s="10" t="n">
-        <v>46303</v>
+        <v>46302</v>
       </c>
       <c r="E51" s="10" t="n">
-        <v>46307</v>
+        <v>46305</v>
       </c>
       <c r="F51" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
+        <v>4</v>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>20B → 20D</t>
         </is>
       </c>
       <c r="H51" s="11" t="n">
-        <v>46305.70833333334</v>
+        <v>46304.83333333334</v>
       </c>
       <c r="I51" s="11" t="n">
+        <v>46305.66666666666</v>
+      </c>
+      <c r="J51" s="11" t="n">
         <v>46306.25</v>
-      </c>
-      <c r="J51" s="11" t="n">
-        <v>46307.58333333334</v>
       </c>
       <c r="K51" s="24">
         <f>(I51-H51)*24</f>
@@ -23507,7 +23788,7 @@
       </c>
       <c r="M51" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>4A</t>
         </is>
       </c>
       <c r="N51" s="23" t="inlineStr"/>
@@ -23525,34 +23806,34 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE SUNRISE</t>
+          <t>INCEDA</t>
         </is>
       </c>
       <c r="C52" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D52" s="10" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="E52" s="10" t="n">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="F52" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="G52" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20D</t>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H52" s="11" t="n">
-        <v>46307.16666666666</v>
+        <v>46305.70833333334</v>
       </c>
       <c r="I52" s="11" t="n">
-        <v>46307.66666666666</v>
+        <v>46306.25</v>
       </c>
       <c r="J52" s="11" t="n">
-        <v>46309.20833333334</v>
+        <v>46307.58333333334</v>
       </c>
       <c r="K52" s="24">
         <f>(I52-H52)*24</f>
@@ -23582,34 +23863,34 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>KHUNA BHUM</t>
+          <t>SAWASDEE SUNRISE</t>
         </is>
       </c>
       <c r="C53" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D53" s="10" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="E53" s="10" t="n">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="F53" s="23" t="n">
         <v>5</v>
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20D</t>
+          <t>20F → 20D</t>
         </is>
       </c>
       <c r="H53" s="11" t="n">
-        <v>46308.45833333334</v>
+        <v>46307.16666666666</v>
       </c>
       <c r="I53" s="11" t="n">
+        <v>46307.66666666666</v>
+      </c>
+      <c r="J53" s="11" t="n">
         <v>46309.20833333334</v>
-      </c>
-      <c r="J53" s="11" t="n">
-        <v>46309.91666666666</v>
       </c>
       <c r="K53" s="24">
         <f>(I53-H53)*24</f>
@@ -23621,7 +23902,7 @@
       </c>
       <c r="M53" s="23" t="inlineStr">
         <is>
-          <t>7B</t>
+          <t>–</t>
         </is>
       </c>
       <c r="N53" s="23" t="inlineStr"/>
@@ -23639,34 +23920,34 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>SITC DALIAN</t>
+          <t>KHUNA BHUM</t>
         </is>
       </c>
       <c r="C54" s="23" t="n">
-        <v>470</v>
+        <v>564</v>
       </c>
       <c r="D54" s="10" t="n">
+        <v>46305</v>
+      </c>
+      <c r="E54" s="10" t="n">
         <v>46309</v>
       </c>
-      <c r="E54" s="10" t="n">
-        <v>46310</v>
-      </c>
       <c r="F54" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G54" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
+        <v>5</v>
+      </c>
+      <c r="G54" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20D</t>
         </is>
       </c>
       <c r="H54" s="11" t="n">
-        <v>46309.33333333334</v>
+        <v>46308.45833333334</v>
       </c>
       <c r="I54" s="11" t="n">
-        <v>46310.20833333334</v>
+        <v>46309.20833333334</v>
       </c>
       <c r="J54" s="11" t="n">
-        <v>46311.25</v>
+        <v>46309.91666666666</v>
       </c>
       <c r="K54" s="24">
         <f>(I54-H54)*24</f>
@@ -23678,7 +23959,7 @@
       </c>
       <c r="M54" s="23" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>7B</t>
         </is>
       </c>
       <c r="N54" s="23" t="inlineStr"/>
@@ -23696,20 +23977,20 @@
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 172</t>
+          <t>SITC DALIAN</t>
         </is>
       </c>
       <c r="C55" s="23" t="n">
-        <v>565</v>
+        <v>470</v>
       </c>
       <c r="D55" s="10" t="n">
         <v>46309</v>
       </c>
       <c r="E55" s="10" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="F55" s="23" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
@@ -23717,13 +23998,13 @@
         </is>
       </c>
       <c r="H55" s="11" t="n">
-        <v>46311.04166666666</v>
+        <v>46309.33333333334</v>
       </c>
       <c r="I55" s="11" t="n">
-        <v>46311.29166666666</v>
+        <v>46310.20833333334</v>
       </c>
       <c r="J55" s="11" t="n">
-        <v>46312.33333333334</v>
+        <v>46311.25</v>
       </c>
       <c r="K55" s="24">
         <f>(I55-H55)*24</f>
@@ -23753,34 +24034,34 @@
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>PUNNYA NAVEE</t>
+          <t>WAN HAI 172</t>
         </is>
       </c>
       <c r="C56" s="23" t="n">
-        <v>304</v>
+        <v>565</v>
       </c>
       <c r="D56" s="10" t="n">
+        <v>46309</v>
+      </c>
+      <c r="E56" s="10" t="n">
         <v>46311</v>
       </c>
-      <c r="E56" s="10" t="n">
-        <v>46312</v>
-      </c>
       <c r="F56" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="G56" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20D</t>
+        <v>3</v>
+      </c>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H56" s="11" t="n">
-        <v>46311.75</v>
+        <v>46311.04166666666</v>
       </c>
       <c r="I56" s="11" t="n">
-        <v>46312.125</v>
+        <v>46311.29166666666</v>
       </c>
       <c r="J56" s="11" t="n">
-        <v>46312.625</v>
+        <v>46312.33333333334</v>
       </c>
       <c r="K56" s="24">
         <f>(I56-H56)*24</f>
@@ -23810,34 +24091,34 @@
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>INFINITY</t>
+          <t>PUNNYA NAVEE</t>
         </is>
       </c>
       <c r="C57" s="23" t="n">
-        <v>565</v>
+        <v>304</v>
       </c>
       <c r="D57" s="10" t="n">
-        <v>46293</v>
+        <v>46311</v>
       </c>
       <c r="E57" s="10" t="n">
-        <v>46313</v>
+        <v>46312</v>
       </c>
       <c r="F57" s="23" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>20AB → 20C → 20D</t>
+          <t>20F → 20D</t>
         </is>
       </c>
       <c r="H57" s="11" t="n">
-        <v>46313</v>
+        <v>46311.75</v>
       </c>
       <c r="I57" s="11" t="n">
-        <v>46313.29166666666</v>
+        <v>46312.125</v>
       </c>
       <c r="J57" s="11" t="n">
-        <v>46314.375</v>
+        <v>46312.625</v>
       </c>
       <c r="K57" s="24">
         <f>(I57-H57)*24</f>
@@ -23867,34 +24148,34 @@
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>PUNNYA NAVEE (barge)</t>
+          <t>INFINITY</t>
         </is>
       </c>
       <c r="C58" s="23" t="n">
-        <v>304</v>
+        <v>565</v>
       </c>
       <c r="D58" s="10" t="n">
-        <v>46319</v>
+        <v>46293</v>
       </c>
       <c r="E58" s="10" t="n">
-        <v>46319</v>
+        <v>46313</v>
       </c>
       <c r="F58" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G58" s="5" t="inlineStr">
-        <is>
-          <t>20D</t>
+        <v>6</v>
+      </c>
+      <c r="G58" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20C → 20D</t>
         </is>
       </c>
       <c r="H58" s="11" t="n">
-        <v>46319.5</v>
+        <v>46313</v>
       </c>
       <c r="I58" s="11" t="n">
-        <v>46319.5</v>
+        <v>46313.29166666666</v>
       </c>
       <c r="J58" s="11" t="n">
-        <v>46319.95833333334</v>
+        <v>46314.375</v>
       </c>
       <c r="K58" s="24">
         <f>(I58-H58)*24</f>
@@ -23910,9 +24191,10 @@
         </is>
       </c>
       <c r="N58" s="23" t="inlineStr"/>
-      <c r="O58" s="23">
-        <f>IF(J58&lt;=$B$3,"Sailed",IF(I58&lt;=$B$3,"Alongside",IF(H58&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O58" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="59">
@@ -23923,11 +24205,11 @@
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>HARI BHUM (barge)</t>
+          <t>PUNNYA NAVEE (barge)</t>
         </is>
       </c>
       <c r="C59" s="23" t="n">
-        <v>259</v>
+        <v>304</v>
       </c>
       <c r="D59" s="10" t="n">
         <v>46319</v>
@@ -23944,13 +24226,13 @@
         </is>
       </c>
       <c r="H59" s="11" t="n">
-        <v>46319.91666666666</v>
+        <v>46319.5</v>
       </c>
       <c r="I59" s="11" t="n">
-        <v>46319.91666666666</v>
+        <v>46319.5</v>
       </c>
       <c r="J59" s="11" t="n">
-        <v>46320.29166666666</v>
+        <v>46319.95833333334</v>
       </c>
       <c r="K59" s="24">
         <f>(I59-H59)*24</f>
@@ -23966,9 +24248,10 @@
         </is>
       </c>
       <c r="N59" s="23" t="inlineStr"/>
-      <c r="O59" s="23">
-        <f>IF(J59&lt;=$B$3,"Sailed",IF(I59&lt;=$B$3,"Alongside",IF(H59&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O59" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="60">
@@ -23979,34 +24262,34 @@
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>KMTC BANGKOK</t>
+          <t>HARI BHUM (barge)</t>
         </is>
       </c>
       <c r="C60" s="23" t="n">
-        <v>565</v>
+        <v>259</v>
       </c>
       <c r="D60" s="10" t="n">
-        <v>46295</v>
+        <v>46319</v>
       </c>
       <c r="E60" s="10" t="n">
         <v>46319</v>
       </c>
       <c r="F60" s="23" t="n">
-        <v>7</v>
-      </c>
-      <c r="G60" s="6" t="inlineStr">
-        <is>
-          <t>20AB → 20F → 20D</t>
+        <v>1</v>
+      </c>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
         </is>
       </c>
       <c r="H60" s="11" t="n">
-        <v>46320.25</v>
+        <v>46319.91666666666</v>
       </c>
       <c r="I60" s="11" t="n">
-        <v>46320.25</v>
+        <v>46319.91666666666</v>
       </c>
       <c r="J60" s="11" t="n">
-        <v>46321.5</v>
+        <v>46320.29166666666</v>
       </c>
       <c r="K60" s="24">
         <f>(I60-H60)*24</f>
@@ -24022,127 +24305,122 @@
         </is>
       </c>
       <c r="N60" s="23" t="inlineStr"/>
-      <c r="O60" s="23">
-        <f>IF(J60&lt;=$B$3,"Sailed",IF(I60&lt;=$B$3,"Alongside",IF(H60&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O60" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="27" t="inlineStr">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>KMTC BANGKOK</t>
+        </is>
+      </c>
+      <c r="C61" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D61" s="10" t="n">
+        <v>46295</v>
+      </c>
+      <c r="E61" s="10" t="n">
+        <v>46320</v>
+      </c>
+      <c r="F61" s="23" t="n">
+        <v>8</v>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>20AB → 20F → 20D</t>
+        </is>
+      </c>
+      <c r="H61" s="11" t="n">
+        <v>46320.25</v>
+      </c>
+      <c r="I61" s="11" t="n">
+        <v>46320.25</v>
+      </c>
+      <c r="J61" s="11" t="n">
+        <v>46321.54166666666</v>
+      </c>
+      <c r="K61" s="24">
+        <f>(I61-H61)*24</f>
+        <v/>
+      </c>
+      <c r="L61" s="24">
+        <f>(J61-I61)*24</f>
+        <v/>
+      </c>
+      <c r="M61" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N61" s="23" t="inlineStr"/>
+      <c r="O61" s="23">
+        <f>IF(J61&lt;=$B$3,"Sailed",IF(I61&lt;=$B$3,"Alongside",IF(H61&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="27" t="inlineStr">
         <is>
           <t>20E</t>
         </is>
       </c>
-      <c r="B61" s="27" t="inlineStr">
-        <is>
-          <t>WAN HAI 278</t>
-        </is>
-      </c>
-      <c r="C61" s="28" t="n">
-        <v>564</v>
-      </c>
-      <c r="D61" s="29" t="n">
-        <v>46295</v>
-      </c>
-      <c r="E61" s="29" t="n">
-        <v>46300</v>
-      </c>
-      <c r="F61" s="28" t="n">
-        <v>6</v>
-      </c>
-      <c r="G61" s="30" t="inlineStr">
-        <is>
-          <t>20F → 20E</t>
-        </is>
-      </c>
-      <c r="H61" s="31" t="n">
-        <v>46297.75</v>
-      </c>
-      <c r="I61" s="31" t="n">
-        <v>46298.41666666666</v>
-      </c>
-      <c r="J61" s="31" t="n">
-        <v>46300.45833333334</v>
-      </c>
-      <c r="K61" s="32">
-        <f>(I61-H61)*24</f>
-        <v/>
-      </c>
-      <c r="L61" s="32">
-        <f>(J61-I61)*24</f>
-        <v/>
-      </c>
-      <c r="M61" s="28" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N61" s="28" t="inlineStr"/>
-      <c r="O61" s="28" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="25" t="inlineStr">
+      <c r="B62" s="27" t="inlineStr">
+        <is>
+          <t>KUO LONG</t>
+        </is>
+      </c>
+      <c r="C62" s="28" t="n">
+        <v>554</v>
+      </c>
+      <c r="D62" s="29" t="n">
+        <v>46320</v>
+      </c>
+      <c r="E62" s="29" t="n">
+        <v>46320</v>
+      </c>
+      <c r="F62" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="33" t="inlineStr">
         <is>
           <t>20E</t>
         </is>
       </c>
-      <c r="B62" s="25" t="inlineStr">
-        <is>
-          <t>MTT BANGKOK</t>
-        </is>
-      </c>
-      <c r="C62" s="17" t="n">
-        <v>564</v>
-      </c>
-      <c r="D62" s="18" t="n">
-        <v>46300</v>
-      </c>
-      <c r="E62" s="18" t="n">
-        <v>46316</v>
-      </c>
-      <c r="F62" s="17" t="n">
-        <v>8</v>
-      </c>
-      <c r="G62" s="6" t="inlineStr">
-        <is>
-          <t>20D → 20B → 20E</t>
-        </is>
-      </c>
-      <c r="H62" s="20" t="n">
-        <v>46315.625</v>
-      </c>
-      <c r="I62" s="20" t="n">
-        <v>46315.75</v>
-      </c>
-      <c r="J62" s="20" t="n">
-        <v>46316.83333333334</v>
-      </c>
-      <c r="K62" s="26">
+      <c r="H62" s="31" t="n">
+        <v>46292.125</v>
+      </c>
+      <c r="I62" s="31" t="n">
+        <v>46292.20833333334</v>
+      </c>
+      <c r="J62" s="31" t="n">
+        <v>46293.58333333334</v>
+      </c>
+      <c r="K62" s="32">
         <f>(I62-H62)*24</f>
         <v/>
       </c>
-      <c r="L62" s="26">
+      <c r="L62" s="32">
         <f>(J62-I62)*24</f>
         <v/>
       </c>
-      <c r="M62" s="17" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N62" s="17" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O62" s="17" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="M62" s="28" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N62" s="28" t="inlineStr"/>
+      <c r="O62" s="28">
+        <f>IF(J62&lt;=$B$3,"Sailed",IF(I62&lt;=$B$3,"Alongside",IF(H62&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="63">
@@ -24153,34 +24431,34 @@
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>SKY ORION</t>
+          <t>WAN HAI 278</t>
         </is>
       </c>
       <c r="C63" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D63" s="10" t="n">
-        <v>46315</v>
+        <v>46295</v>
       </c>
       <c r="E63" s="10" t="n">
-        <v>46318</v>
+        <v>46300</v>
       </c>
       <c r="F63" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G63" s="5" t="inlineStr">
-        <is>
-          <t>20E</t>
+        <v>6</v>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>20F → 20E</t>
         </is>
       </c>
       <c r="H63" s="11" t="n">
-        <v>46317.04166666666</v>
+        <v>46297.75</v>
       </c>
       <c r="I63" s="11" t="n">
-        <v>46317.54166666666</v>
+        <v>46298.41666666666</v>
       </c>
       <c r="J63" s="11" t="n">
-        <v>46319.04166666666</v>
+        <v>46300.45833333334</v>
       </c>
       <c r="K63" s="24">
         <f>(I63-H63)*24</f>
@@ -24203,59 +24481,64 @@
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="4" t="inlineStr">
+      <c r="A64" s="25" t="inlineStr">
         <is>
           <t>20E</t>
         </is>
       </c>
-      <c r="B64" s="4" t="inlineStr">
-        <is>
-          <t>YM IMAGE</t>
-        </is>
-      </c>
-      <c r="C64" s="23" t="n">
-        <v>565</v>
-      </c>
-      <c r="D64" s="10" t="n">
-        <v>46317</v>
-      </c>
-      <c r="E64" s="10" t="n">
-        <v>46319</v>
-      </c>
-      <c r="F64" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G64" s="5" t="inlineStr">
-        <is>
-          <t>20E</t>
-        </is>
-      </c>
-      <c r="H64" s="11" t="n">
-        <v>46318.25</v>
-      </c>
-      <c r="I64" s="11" t="n">
-        <v>46319.125</v>
-      </c>
-      <c r="J64" s="11" t="n">
-        <v>46320.04166666666</v>
-      </c>
-      <c r="K64" s="24">
+      <c r="B64" s="25" t="inlineStr">
+        <is>
+          <t>MTT BANGKOK</t>
+        </is>
+      </c>
+      <c r="C64" s="17" t="n">
+        <v>564</v>
+      </c>
+      <c r="D64" s="18" t="n">
+        <v>46300</v>
+      </c>
+      <c r="E64" s="18" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F64" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="G64" s="6" t="inlineStr">
+        <is>
+          <t>20D → 20B → 20E</t>
+        </is>
+      </c>
+      <c r="H64" s="20" t="n">
+        <v>46315.625</v>
+      </c>
+      <c r="I64" s="20" t="n">
+        <v>46315.75</v>
+      </c>
+      <c r="J64" s="20" t="n">
+        <v>46316.83333333334</v>
+      </c>
+      <c r="K64" s="26">
         <f>(I64-H64)*24</f>
         <v/>
       </c>
-      <c r="L64" s="24">
+      <c r="L64" s="26">
         <f>(J64-I64)*24</f>
         <v/>
       </c>
-      <c r="M64" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N64" s="23" t="inlineStr"/>
-      <c r="O64" s="23">
-        <f>IF(J64&lt;=$B$3,"Sailed",IF(I64&lt;=$B$3,"Alongside",IF(H64&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="M64" s="17" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N64" s="17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O64" s="17" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="65">
@@ -24266,34 +24549,34 @@
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 106</t>
+          <t>SKY ORION</t>
         </is>
       </c>
       <c r="C65" s="23" t="n">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D65" s="10" t="n">
-        <v>46317</v>
+        <v>46315</v>
       </c>
       <c r="E65" s="10" t="n">
-        <v>46319</v>
+        <v>46318</v>
       </c>
       <c r="F65" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G65" s="6" t="inlineStr">
-        <is>
-          <t>20F → 20E</t>
+        <v>4</v>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
         </is>
       </c>
       <c r="H65" s="11" t="n">
-        <v>46320.41666666666</v>
+        <v>46317.04166666666</v>
       </c>
       <c r="I65" s="11" t="n">
-        <v>46320.54166666666</v>
+        <v>46317.54166666666</v>
       </c>
       <c r="J65" s="11" t="n">
-        <v>46321.5</v>
+        <v>46319.04166666666</v>
       </c>
       <c r="K65" s="24">
         <f>(I65-H65)*24</f>
@@ -24309,63 +24592,64 @@
         </is>
       </c>
       <c r="N65" s="23" t="inlineStr"/>
-      <c r="O65" s="23">
-        <f>IF(J65&lt;=$B$3,"Sailed",IF(I65&lt;=$B$3,"Alongside",IF(H65&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O65" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="27" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="B66" s="27" t="inlineStr">
-        <is>
-          <t>XIN MING ZHOU 98</t>
-        </is>
-      </c>
-      <c r="C66" s="28" t="n">
-        <v>564</v>
-      </c>
-      <c r="D66" s="29" t="n">
-        <v>46297</v>
-      </c>
-      <c r="E66" s="29" t="n">
-        <v>46299</v>
-      </c>
-      <c r="F66" s="28" t="n">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>YM IMAGE</t>
+        </is>
+      </c>
+      <c r="C66" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D66" s="10" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E66" s="10" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F66" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="G66" s="33" t="inlineStr">
-        <is>
-          <t>20F</t>
-        </is>
-      </c>
-      <c r="H66" s="31" t="n">
-        <v>46299.375</v>
-      </c>
-      <c r="I66" s="31" t="n">
-        <v>46299.375</v>
-      </c>
-      <c r="J66" s="31" t="n">
-        <v>46300.375</v>
-      </c>
-      <c r="K66" s="32">
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="H66" s="11" t="n">
+        <v>46318.25</v>
+      </c>
+      <c r="I66" s="11" t="n">
+        <v>46319.125</v>
+      </c>
+      <c r="J66" s="11" t="n">
+        <v>46320.04166666666</v>
+      </c>
+      <c r="K66" s="24">
         <f>(I66-H66)*24</f>
         <v/>
       </c>
-      <c r="L66" s="32">
+      <c r="L66" s="24">
         <f>(J66-I66)*24</f>
         <v/>
       </c>
-      <c r="M66" s="28" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N66" s="28" t="inlineStr"/>
-      <c r="O66" s="28" t="inlineStr">
+      <c r="M66" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N66" s="23" t="inlineStr"/>
+      <c r="O66" s="23" t="inlineStr">
         <is>
           <t>Sailed</t>
         </is>
@@ -24374,39 +24658,39 @@
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>20F</t>
+          <t>20E</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE ATLANTIC</t>
+          <t>XIN MING ZHOU 106</t>
         </is>
       </c>
       <c r="C67" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D67" s="10" t="n">
-        <v>46300</v>
+        <v>46317</v>
       </c>
       <c r="E67" s="10" t="n">
-        <v>46306</v>
+        <v>46320</v>
       </c>
       <c r="F67" s="23" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
-          <t>20C → 20D → 20F</t>
+          <t>20F → 20E</t>
         </is>
       </c>
       <c r="H67" s="11" t="n">
-        <v>46302.83333333334</v>
+        <v>46320.41666666666</v>
       </c>
       <c r="I67" s="11" t="n">
-        <v>46304.625</v>
+        <v>46320.54166666666</v>
       </c>
       <c r="J67" s="11" t="n">
-        <v>46306.5</v>
+        <v>46321.5</v>
       </c>
       <c r="K67" s="24">
         <f>(I67-H67)*24</f>
@@ -24422,67 +24706,65 @@
         </is>
       </c>
       <c r="N67" s="23" t="inlineStr"/>
-      <c r="O67" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="O67" s="23">
+        <f>IF(J67&lt;=$B$3,"Sailed",IF(I67&lt;=$B$3,"Alongside",IF(H67&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="4" t="inlineStr">
+      <c r="A68" s="27" t="inlineStr">
         <is>
           <t>20F</t>
         </is>
       </c>
-      <c r="B68" s="4" t="inlineStr">
-        <is>
-          <t>JOSCO SHINE</t>
-        </is>
-      </c>
-      <c r="C68" s="23" t="n">
+      <c r="B68" s="27" t="inlineStr">
+        <is>
+          <t>WAN HAI 276</t>
+        </is>
+      </c>
+      <c r="C68" s="28" t="n">
         <v>564</v>
       </c>
-      <c r="D68" s="10" t="n">
-        <v>46304</v>
-      </c>
-      <c r="E68" s="10" t="n">
-        <v>46307</v>
-      </c>
-      <c r="F68" s="23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G68" s="6" t="inlineStr">
-        <is>
-          <t>20B → 20AB → 20F</t>
-        </is>
-      </c>
-      <c r="H68" s="11" t="n">
-        <v>46307.45833333334</v>
-      </c>
-      <c r="I68" s="11" t="n">
-        <v>46307.625</v>
-      </c>
-      <c r="J68" s="11" t="n">
-        <v>46308.25</v>
-      </c>
-      <c r="K68" s="24">
+      <c r="D68" s="29" t="n">
+        <v>46320</v>
+      </c>
+      <c r="E68" s="29" t="n">
+        <v>46320</v>
+      </c>
+      <c r="F68" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" s="33" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="H68" s="31" t="n">
+        <v>46292.66666666666</v>
+      </c>
+      <c r="I68" s="31" t="n">
+        <v>46292.66666666666</v>
+      </c>
+      <c r="J68" s="31" t="n">
+        <v>46294.16666666666</v>
+      </c>
+      <c r="K68" s="32">
         <f>(I68-H68)*24</f>
         <v/>
       </c>
-      <c r="L68" s="24">
+      <c r="L68" s="32">
         <f>(J68-I68)*24</f>
         <v/>
       </c>
-      <c r="M68" s="23" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="N68" s="23" t="inlineStr"/>
-      <c r="O68" s="23" t="inlineStr">
-        <is>
-          <t>Sailed</t>
-        </is>
+      <c r="M68" s="28" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N68" s="28" t="inlineStr"/>
+      <c r="O68" s="28">
+        <f>IF(J68&lt;=$B$3,"Sailed",IF(I68&lt;=$B$3,"Alongside",IF(H68&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
       </c>
     </row>
     <row r="69">
@@ -24493,20 +24775,20 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>SAWASDEE INCHEON</t>
+          <t>XIN MING ZHOU 98</t>
         </is>
       </c>
       <c r="C69" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D69" s="10" t="n">
-        <v>46307</v>
+        <v>46297</v>
       </c>
       <c r="E69" s="10" t="n">
-        <v>46310</v>
+        <v>46299</v>
       </c>
       <c r="F69" s="23" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
@@ -24514,13 +24796,13 @@
         </is>
       </c>
       <c r="H69" s="11" t="n">
-        <v>46308.625</v>
+        <v>46299.375</v>
       </c>
       <c r="I69" s="11" t="n">
-        <v>46309.25</v>
+        <v>46299.375</v>
       </c>
       <c r="J69" s="11" t="n">
-        <v>46311.25</v>
+        <v>46300.375</v>
       </c>
       <c r="K69" s="24">
         <f>(I69-H69)*24</f>
@@ -24550,34 +24832,34 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>INGENUITY</t>
+          <t>SAWASDEE ATLANTIC</t>
         </is>
       </c>
       <c r="C70" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D70" s="10" t="n">
-        <v>46310</v>
+        <v>46300</v>
       </c>
       <c r="E70" s="10" t="n">
-        <v>46312</v>
+        <v>46306</v>
       </c>
       <c r="F70" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="G70" s="5" t="inlineStr">
-        <is>
-          <t>20F</t>
+        <v>7</v>
+      </c>
+      <c r="G70" s="6" t="inlineStr">
+        <is>
+          <t>20C → 20D → 20F</t>
         </is>
       </c>
       <c r="H70" s="11" t="n">
-        <v>46311.95833333334</v>
+        <v>46302.83333333334</v>
       </c>
       <c r="I70" s="11" t="n">
-        <v>46312.33333333334</v>
+        <v>46304.625</v>
       </c>
       <c r="J70" s="11" t="n">
-        <v>46313.29166666666</v>
+        <v>46306.5</v>
       </c>
       <c r="K70" s="24">
         <f>(I70-H70)*24</f>
@@ -24607,34 +24889,34 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>XIN MING ZHOU 108</t>
+          <t>JOSCO SHINE</t>
         </is>
       </c>
       <c r="C71" s="23" t="n">
         <v>564</v>
       </c>
       <c r="D71" s="10" t="n">
-        <v>46310</v>
+        <v>46304</v>
       </c>
       <c r="E71" s="10" t="n">
-        <v>46314</v>
+        <v>46307</v>
       </c>
       <c r="F71" s="23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G71" s="6" t="inlineStr">
         <is>
-          <t>20B → 20F</t>
+          <t>20B → 20AB → 20F</t>
         </is>
       </c>
       <c r="H71" s="11" t="n">
-        <v>46312.41666666666</v>
+        <v>46307.45833333334</v>
       </c>
       <c r="I71" s="11" t="n">
-        <v>46313.33333333334</v>
+        <v>46307.625</v>
       </c>
       <c r="J71" s="11" t="n">
-        <v>46314.5</v>
+        <v>46308.25</v>
       </c>
       <c r="K71" s="24">
         <f>(I71-H71)*24</f>
@@ -24664,20 +24946,20 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>RENOWN</t>
+          <t>SAWASDEE INCHEON</t>
         </is>
       </c>
       <c r="C72" s="23" t="n">
-        <v>458</v>
+        <v>564</v>
       </c>
       <c r="D72" s="10" t="n">
-        <v>46315</v>
+        <v>46307</v>
       </c>
       <c r="E72" s="10" t="n">
-        <v>46317</v>
+        <v>46310</v>
       </c>
       <c r="F72" s="23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
@@ -24685,13 +24967,13 @@
         </is>
       </c>
       <c r="H72" s="11" t="n">
-        <v>46315.75</v>
+        <v>46308.625</v>
       </c>
       <c r="I72" s="11" t="n">
-        <v>46317.41666666666</v>
+        <v>46309.25</v>
       </c>
       <c r="J72" s="11" t="n">
-        <v>46318.375</v>
+        <v>46311.25</v>
       </c>
       <c r="K72" s="24">
         <f>(I72-H72)*24</f>
@@ -24721,34 +25003,34 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>WAN HAI 272</t>
+          <t>INGENUITY</t>
         </is>
       </c>
       <c r="C73" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D73" s="10" t="n">
-        <v>46315</v>
+        <v>46310</v>
       </c>
       <c r="E73" s="10" t="n">
-        <v>46319</v>
+        <v>46312</v>
       </c>
       <c r="F73" s="23" t="n">
-        <v>5</v>
-      </c>
-      <c r="G73" s="6" t="inlineStr">
-        <is>
-          <t>22A → 20F</t>
+        <v>3</v>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
         </is>
       </c>
       <c r="H73" s="11" t="n">
-        <v>46318.375</v>
+        <v>46311.95833333334</v>
       </c>
       <c r="I73" s="11" t="n">
-        <v>46318.375</v>
+        <v>46312.33333333334</v>
       </c>
       <c r="J73" s="11" t="n">
-        <v>46319.58333333334</v>
+        <v>46313.29166666666</v>
       </c>
       <c r="K73" s="24">
         <f>(I73-H73)*24</f>
@@ -24764,9 +25046,10 @@
         </is>
       </c>
       <c r="N73" s="23" t="inlineStr"/>
-      <c r="O73" s="23">
-        <f>IF(J73&lt;=$B$3,"Sailed",IF(I73&lt;=$B$3,"Alongside",IF(H73&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O73" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -24777,34 +25060,34 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>HEUNG A HOCHIMINH</t>
+          <t>XIN MING ZHOU 108</t>
         </is>
       </c>
       <c r="C74" s="23" t="n">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="D74" s="10" t="n">
-        <v>46317</v>
+        <v>46310</v>
       </c>
       <c r="E74" s="10" t="n">
-        <v>46319</v>
+        <v>46314</v>
       </c>
       <c r="F74" s="23" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G74" s="6" t="inlineStr">
         <is>
-          <t>20E → 20F</t>
+          <t>20B → 20F</t>
         </is>
       </c>
       <c r="H74" s="11" t="n">
-        <v>46320.58333333334</v>
+        <v>46312.41666666666</v>
       </c>
       <c r="I74" s="11" t="n">
-        <v>46320.625</v>
+        <v>46313.33333333334</v>
       </c>
       <c r="J74" s="11" t="n">
-        <v>46292.16666666666</v>
+        <v>46314.5</v>
       </c>
       <c r="K74" s="24">
         <f>(I74-H74)*24</f>
@@ -24820,20 +25103,191 @@
         </is>
       </c>
       <c r="N74" s="23" t="inlineStr"/>
-      <c r="O74" s="23">
-        <f>IF(J74&lt;=$B$3,"Sailed",IF(I74&lt;=$B$3,"Alongside",IF(H74&lt;=$B$3,"At anchorage","Expected")))</f>
-        <v/>
+      <c r="O74" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>RENOWN</t>
+        </is>
+      </c>
+      <c r="C75" s="23" t="n">
+        <v>458</v>
+      </c>
+      <c r="D75" s="10" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E75" s="10" t="n">
+        <v>46317</v>
+      </c>
+      <c r="F75" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="H75" s="11" t="n">
+        <v>46315.75</v>
+      </c>
+      <c r="I75" s="11" t="n">
+        <v>46317.41666666666</v>
+      </c>
+      <c r="J75" s="11" t="n">
+        <v>46318.375</v>
+      </c>
+      <c r="K75" s="24">
+        <f>(I75-H75)*24</f>
+        <v/>
+      </c>
+      <c r="L75" s="24">
+        <f>(J75-I75)*24</f>
+        <v/>
+      </c>
+      <c r="M75" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N75" s="23" t="inlineStr"/>
+      <c r="O75" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>69 vessels in total. Orange cells: marked on sheet, or the vessel changed berth.</t>
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>WAN HAI 272</t>
+        </is>
+      </c>
+      <c r="C76" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D76" s="10" t="n">
+        <v>46315</v>
+      </c>
+      <c r="E76" s="10" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F76" s="23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G76" s="6" t="inlineStr">
+        <is>
+          <t>22A → 20F</t>
+        </is>
+      </c>
+      <c r="H76" s="11" t="n">
+        <v>46318.375</v>
+      </c>
+      <c r="I76" s="11" t="n">
+        <v>46318.375</v>
+      </c>
+      <c r="J76" s="11" t="n">
+        <v>46319.58333333334</v>
+      </c>
+      <c r="K76" s="24">
+        <f>(I76-H76)*24</f>
+        <v/>
+      </c>
+      <c r="L76" s="24">
+        <f>(J76-I76)*24</f>
+        <v/>
+      </c>
+      <c r="M76" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N76" s="23" t="inlineStr"/>
+      <c r="O76" s="23" t="inlineStr">
+        <is>
+          <t>Sailed</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>HEUNG A HOCHIMINH</t>
+        </is>
+      </c>
+      <c r="C77" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D77" s="10" t="n">
+        <v>46317</v>
+      </c>
+      <c r="E77" s="10" t="n">
+        <v>46320</v>
+      </c>
+      <c r="F77" s="23" t="n">
+        <v>4</v>
+      </c>
+      <c r="G77" s="6" t="inlineStr">
+        <is>
+          <t>20E → 20F</t>
+        </is>
+      </c>
+      <c r="H77" s="11" t="n">
+        <v>46320.58333333334</v>
+      </c>
+      <c r="I77" s="11" t="n">
+        <v>46320.625</v>
+      </c>
+      <c r="J77" s="11" t="n">
+        <v>46292.16666666666</v>
+      </c>
+      <c r="K77" s="24">
+        <f>(I77-H77)*24</f>
+        <v/>
+      </c>
+      <c r="L77" s="24">
+        <f>(J77-I77)*24</f>
+        <v/>
+      </c>
+      <c r="M77" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="N77" s="23" t="inlineStr"/>
+      <c r="O77" s="23">
+        <f>IF(J77&lt;=$B$3,"Sailed",IF(I77&lt;=$B$3,"Alongside",IF(H77&lt;=$B$3,"At anchorage","Expected")))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>72 vessels in total. Orange cells: marked on sheet, or the vessel changed berth.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:O74"/>
+  <autoFilter ref="A5:O77"/>
   <mergeCells count="1">
     <mergeCell ref="A2:O2"/>
   </mergeCells>
@@ -25540,6 +25994,634 @@
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="F22:J22"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PAT Berth Window — Vessel List by Berth — Sheet dated 25 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Berth</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vessel</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>LOA (m)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>P.B</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>ETD</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Waiting for Berth (h)</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Hours Alongside</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Shift</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>KANWAY FORTUNE</t>
+        </is>
+      </c>
+      <c r="C4" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <v>46320.25</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>46320.625</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>46321.66666666666</v>
+      </c>
+      <c r="G4" s="24">
+        <f>(E4-D4)*24</f>
+        <v/>
+      </c>
+      <c r="H4" s="24">
+        <f>(F4-E4)*24</f>
+        <v/>
+      </c>
+      <c r="I4" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J4" s="23" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>20AB</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>KMTC TOKYO</t>
+        </is>
+      </c>
+      <c r="C5" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D5" s="11" t="n">
+        <v>46292.20833333334</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>46292.20833333334</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>46293.54166666666</v>
+      </c>
+      <c r="G5" s="24">
+        <f>(E5-D5)*24</f>
+        <v/>
+      </c>
+      <c r="H5" s="24">
+        <f>(F5-E5)*24</f>
+        <v/>
+      </c>
+      <c r="I5" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J5" s="23" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>ASL TAIPEIS</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D6" s="11" t="n">
+        <v>46320.25</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>46320.58333333334</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>46321.5</v>
+      </c>
+      <c r="G6" s="24">
+        <f>(E6-D6)*24</f>
+        <v/>
+      </c>
+      <c r="H6" s="24">
+        <f>(F6-E6)*24</f>
+        <v/>
+      </c>
+      <c r="I6" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J6" s="23" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>20B</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>XIN AN</t>
+        </is>
+      </c>
+      <c r="C7" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <v>46321.75</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>46292.16666666666</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>46293.20833333334</v>
+      </c>
+      <c r="G7" s="24">
+        <f>(E7-D7)*24</f>
+        <v/>
+      </c>
+      <c r="H7" s="24">
+        <f>(F7-E7)*24</f>
+        <v/>
+      </c>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J7" s="23" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE MIMOSA</t>
+        </is>
+      </c>
+      <c r="C8" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>46318.70833333334</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>46319.625</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>46321.125</v>
+      </c>
+      <c r="G8" s="24">
+        <f>(E8-D8)*24</f>
+        <v/>
+      </c>
+      <c r="H8" s="24">
+        <f>(F8-E8)*24</f>
+        <v/>
+      </c>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>ZHONG GU BEI HAI</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="n">
+        <v>561</v>
+      </c>
+      <c r="D9" s="11" t="n">
+        <v>46321.625</v>
+      </c>
+      <c r="E9" s="11" t="n">
+        <v>46321.625</v>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>46293.125</v>
+      </c>
+      <c r="G9" s="24">
+        <f>(E9-D9)*24</f>
+        <v/>
+      </c>
+      <c r="H9" s="24">
+        <f>(F9-E9)*24</f>
+        <v/>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J9" s="23" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>20C</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>M ODYSSEY</t>
+        </is>
+      </c>
+      <c r="C10" s="23" t="n">
+        <v>449</v>
+      </c>
+      <c r="D10" s="11" t="n">
+        <v>46293.125</v>
+      </c>
+      <c r="E10" s="11" t="n">
+        <v>46293.20833333334</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>46294.25</v>
+      </c>
+      <c r="G10" s="24">
+        <f>(E10-D10)*24</f>
+        <v/>
+      </c>
+      <c r="H10" s="24">
+        <f>(F10-E10)*24</f>
+        <v/>
+      </c>
+      <c r="I10" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>KMTC BANGKOK</t>
+        </is>
+      </c>
+      <c r="C11" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D11" s="11" t="n">
+        <v>46320.25</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>46320.25</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>46321.54166666666</v>
+      </c>
+      <c r="G11" s="24">
+        <f>(E11-D11)*24</f>
+        <v/>
+      </c>
+      <c r="H11" s="24">
+        <f>(F11-E11)*24</f>
+        <v/>
+      </c>
+      <c r="I11" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J11" s="23" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>20D</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>SAWASDEE VEGA</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D12" s="11" t="n">
+        <v>46292.625</v>
+      </c>
+      <c r="E12" s="11" t="n">
+        <v>46292.625</v>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>46294.16666666666</v>
+      </c>
+      <c r="G12" s="24">
+        <f>(E12-D12)*24</f>
+        <v/>
+      </c>
+      <c r="H12" s="24">
+        <f>(F12-E12)*24</f>
+        <v/>
+      </c>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J12" s="23" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>XIN MING ZHOU 106</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>46320.41666666666</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>46320.54166666666</v>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>46321.5</v>
+      </c>
+      <c r="G13" s="24">
+        <f>(E13-D13)*24</f>
+        <v/>
+      </c>
+      <c r="H13" s="24">
+        <f>(F13-E13)*24</f>
+        <v/>
+      </c>
+      <c r="I13" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J13" s="23" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>20E</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>KUO LONG</t>
+        </is>
+      </c>
+      <c r="C14" s="23" t="n">
+        <v>554</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>46292.125</v>
+      </c>
+      <c r="E14" s="11" t="n">
+        <v>46292.20833333334</v>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>46293.58333333334</v>
+      </c>
+      <c r="G14" s="24">
+        <f>(E14-D14)*24</f>
+        <v/>
+      </c>
+      <c r="H14" s="24">
+        <f>(F14-E14)*24</f>
+        <v/>
+      </c>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J14" s="23" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>HEUNG A HOCHIMINH</t>
+        </is>
+      </c>
+      <c r="C15" s="23" t="n">
+        <v>565</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>46320.58333333334</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>46320.625</v>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>46292.16666666666</v>
+      </c>
+      <c r="G15" s="24">
+        <f>(E15-D15)*24</f>
+        <v/>
+      </c>
+      <c r="H15" s="24">
+        <f>(F15-E15)*24</f>
+        <v/>
+      </c>
+      <c r="I15" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J15" s="23" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>20F</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>WAN HAI 276</t>
+        </is>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>564</v>
+      </c>
+      <c r="D16" s="11" t="n">
+        <v>46292.66666666666</v>
+      </c>
+      <c r="E16" s="11" t="n">
+        <v>46292.66666666666</v>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>46294.16666666666</v>
+      </c>
+      <c r="G16" s="24">
+        <f>(E16-D16)*24</f>
+        <v/>
+      </c>
+      <c r="H16" s="24">
+        <f>(F16-E16)*24</f>
+        <v/>
+      </c>
+      <c r="I16" s="23" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="J16" s="23" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="34" t="inlineStr">
+        <is>
+          <t>Berth &amp; gate notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Berth / Gate</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n"/>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>From</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>To</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Notice / change vs previous sheet</t>
+        </is>
+      </c>
+      <c r="G20" s="35" t="n"/>
+      <c r="H20" s="35" t="n"/>
+      <c r="I20" s="35" t="n"/>
+      <c r="J20" s="36" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="39" t="inlineStr">
+        <is>
+          <t>No notices on this sheet</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="F20:J20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>